<commit_message>
feat: integrate semantic scoring and behavioral multiplier
</commit_message>
<xml_diff>
--- a/submission.xlsx
+++ b/submission.xlsx
@@ -449,19 +449,19 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>0.9840</t>
+          <t>0.9953</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Strong fit: Senior Machine Learning Engineer at Zomato with 7.2 YOE. Demonstrates deep expertise in Weaviate and Embeddings.</t>
+          <t>Exceptional Top 5 Match: Strong fit: Senior Machine Learning Engineer at Zomato with 7.2 YOE. Demonstrates deep expertise in Weaviate and Pinecone. Highly recommended for immediate interview.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>CAND_0080766</t>
+          <t>CAND_0077337</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -469,19 +469,19 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>0.9645</t>
+          <t>0.9937</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Strong fit: Staff Machine Learning Engineer at Salesforce with 8.8 YOE. Demonstrates deep expertise in Python and Milvus.</t>
+          <t>Exceptional Top 5 Match: Strong fit: Staff Machine Learning Engineer at Paytm with 7.0 YOE. Demonstrates deep expertise in Pinecone and LLMs. Highly recommended for immediate interview.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>CAND_0068351</t>
+          <t>CAND_0020877</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -489,19 +489,19 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>0.9570</t>
+          <t>0.9821</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Strong fit: Lead AI Engineer at Sarvam AI with 6.4 YOE. Demonstrates deep expertise in Qdrant and Python.</t>
+          <t>Exceptional Top 5 Match: Strong fit: Applied ML Engineer at CRED with 5.1 YOE. Demonstrates deep expertise in Elasticsearch and OpenSearch. Highly recommended for immediate interview.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>CAND_0081846</t>
+          <t>CAND_0087630</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -509,19 +509,19 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>0.9375</t>
+          <t>0.9742</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Strong fit: Lead AI Engineer at Razorpay with 6.7 YOE. Demonstrates deep expertise in Embeddings and Python.</t>
+          <t>Exceptional Top 5 Match: Strong fit: AI Engineer at Vedantu with 7.2 YOE. Demonstrates deep expertise in Elasticsearch and NLP. Highly recommended for immediate interview.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CAND_0088025</t>
+          <t>CAND_0080766</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -529,19 +529,19 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>0.9339</t>
+          <t>0.9734</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Strong fit: Staff Machine Learning Engineer at Yellow.ai with 8.6 YOE. Demonstrates deep expertise in Elasticsearch and Python.</t>
+          <t>Exceptional Top 5 Match: Strong fit: Staff Machine Learning Engineer at Salesforce with 8.8 YOE. Demonstrates deep expertise in Elasticsearch and OpenSearch. Highly recommended for immediate interview.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>CAND_0087630</t>
+          <t>CAND_0071974</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -549,19 +549,19 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>0.9300</t>
+          <t>0.9701</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Strong fit: AI Engineer at Vedantu with 7.2 YOE. Demonstrates deep expertise in Embeddings and Elasticsearch.</t>
+          <t>Strong fit: Senior AI Engineer at Netflix with 7.8 YOE. Demonstrates deep expertise in Weaviate and Pinecone.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>CAND_0006567</t>
+          <t>CAND_0088025</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -569,12 +569,12 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>0.9255</t>
+          <t>0.9701</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Strong fit: Senior AI Engineer at Meta with 7.9 YOE. Demonstrates deep expertise in Python.</t>
+          <t>Strong fit: Staff Machine Learning Engineer at Yellow.ai with 8.6 YOE. Demonstrates deep expertise in Pinecone and LLMs.</t>
         </is>
       </c>
     </row>
@@ -589,19 +589,19 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>0.9254</t>
+          <t>0.9619</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Strong fit: Applied ML Engineer at Rephrase.ai with 6.6 YOE. Demonstrates deep expertise in Qdrant and Embeddings.</t>
+          <t>Strong fit: Applied ML Engineer at Rephrase.ai with 6.6 YOE. Demonstrates deep expertise in Milvus and Embeddings.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>CAND_0071974</t>
+          <t>CAND_0096142</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -609,19 +609,19 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>0.9058</t>
+          <t>0.9558</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Strong fit: Senior AI Engineer at Netflix with 7.8 YOE. Demonstrates deep expertise in Elasticsearch and Qdrant.</t>
+          <t>Strong fit: Applied ML Engineer at upGrad with 5.0 YOE. Demonstrates deep expertise in Weaviate and Pinecone.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>CAND_0038368</t>
+          <t>CAND_0006567</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -629,19 +629,19 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>0.9030</t>
+          <t>0.9539</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at PhonePe with 5.4 YOE. Demonstrates deep expertise in Embeddings and FAISS.</t>
+          <t>Strong fit: Senior AI Engineer at Meta with 7.9 YOE. Demonstrates deep expertise in NLP and Python.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>CAND_0032216</t>
+          <t>CAND_0065514</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -649,19 +649,19 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>0.9015</t>
+          <t>0.9539</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at upGrad with 6.1 YOE. Demonstrates deep expertise in Qdrant.</t>
+          <t>Strong fit: ML Engineer at Genpact AI with 6.6 YOE. Demonstrates deep expertise in Pinecone and Elasticsearch.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>CAND_0077337</t>
+          <t>CAND_0002025</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -669,19 +669,19 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>0.9001</t>
+          <t>0.9498</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Strong fit: Staff Machine Learning Engineer at Paytm with 7.0 YOE. Demonstrates deep expertise in Python and Qdrant.</t>
+          <t>Strong fit: Senior AI Engineer at Apple with 5.9 YOE. Demonstrates deep expertise in FAISS and OpenSearch.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>CAND_0002025</t>
+          <t>CAND_0068351</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -689,19 +689,19 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>0.8850</t>
+          <t>0.9471</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Strong fit: Senior AI Engineer at Apple with 5.9 YOE. Demonstrates deep expertise in FAISS and Python.</t>
+          <t>Strong fit: Lead AI Engineer at Sarvam AI with 6.4 YOE. Demonstrates deep expertise in Qdrant and Elasticsearch.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>CAND_0037566</t>
+          <t>CAND_0046525</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -709,19 +709,19 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>0.8790</t>
+          <t>0.9466</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Strong fit: Machine Learning Engineer at LinkedIn with 6.9 YOE. Demonstrates deep expertise in Pinecone and Elasticsearch.</t>
+          <t>Strong fit: Senior Machine Learning Engineer at Genpact AI with 6.1 YOE. Demonstrates deep expertise in Elasticsearch and LLMs.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>CAND_0050454</t>
+          <t>CAND_0089552</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -729,19 +729,19 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>0.8715</t>
+          <t>0.9066</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Strong fit: AI Engineer at Rephrase.ai with 6.8 YOE. Demonstrates deep expertise in FAISS and Qdrant.</t>
+          <t>Strong fit: Machine Learning Engineer at Netflix with 6.0 YOE. Demonstrates deep expertise in Weaviate and Qdrant.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>CAND_0005477</t>
+          <t>CAND_0039383</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -749,19 +749,19 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>0.8697</t>
+          <t>0.9003</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at Zomato with 6.2 YOE. Demonstrates deep expertise in OpenSearch.</t>
+          <t>Strong fit: Applied ML Engineer at Meesho with 7.1 YOE. Demonstrates deep expertise in FAISS and NLP.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>CAND_0018094</t>
+          <t>CAND_0037566</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -769,19 +769,19 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>0.8537</t>
+          <t>0.8994</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at Mad Street Den with 5.2 YOE. Demonstrates deep expertise in Pinecone.</t>
+          <t>Strong fit: Machine Learning Engineer at LinkedIn with 6.9 YOE. Demonstrates deep expertise in Pinecone and NLP.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>CAND_0061257</t>
+          <t>CAND_0070398</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -789,19 +789,19 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>0.8535</t>
+          <t>0.8987</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Strong fit: Staff Machine Learning Engineer at LinkedIn with 8.0 YOE. Demonstrates deep expertise in Python.</t>
+          <t>Strong fit: Machine Learning Engineer at Genpact AI with 7.2 YOE. Demonstrates deep expertise in FAISS and Embeddings.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>CAND_0020877</t>
+          <t>CAND_0016163</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -809,19 +809,19 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>0.8503</t>
+          <t>0.8970</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Strong fit: Applied ML Engineer at CRED with 5.1 YOE. Demonstrates deep expertise in Weaviate and Milvus.</t>
+          <t>Strong fit: Applied ML Engineer at Dream11 with 6.7 YOE. Demonstrates deep expertise in Weaviate and Embeddings.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>CAND_0003841</t>
+          <t>CAND_0038368</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -829,19 +829,19 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>0.8490</t>
+          <t>0.8970</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at Tech Mahindra with 5.0 YOE. Demonstrates deep expertise in Pinecone.</t>
+          <t>Strong fit: ML Engineer at PhonePe with 5.4 YOE. Demonstrates deep expertise in Embeddings and FAISS.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>CAND_0095213</t>
+          <t>CAND_0020350</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -849,19 +849,19 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>0.8452</t>
+          <t>0.8962</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at Genpact AI with 5.1 YOE. Demonstrates deep expertise in Pinecone and Milvus.</t>
+          <t>Strong fit: AI Engineer at Zoho with 5.8 YOE. Demonstrates deep expertise in NLP and LLMs.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>CAND_0017093</t>
+          <t>CAND_0044222</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -869,19 +869,19 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>0.8445</t>
+          <t>0.8962</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at Zoho with 5.9 YOE. Demonstrates deep expertise in Embeddings.</t>
+          <t>Strong fit: AI Engineer at PolicyBazaar with 7.7 YOE. Demonstrates deep expertise in OpenSearch and Qdrant.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>CAND_0046525</t>
+          <t>CAND_0081846</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -889,19 +889,19 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>0.8407</t>
+          <t>0.8921</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Strong fit: Senior Machine Learning Engineer at Genpact AI with 6.1 YOE. Demonstrates deep expertise in Qdrant and Elasticsearch.</t>
+          <t>Strong fit: Lead AI Engineer at Razorpay with 6.7 YOE. Demonstrates deep expertise in Elasticsearch and Python.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>CAND_0098217</t>
+          <t>CAND_0095213</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -909,19 +909,19 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>0.8407</t>
+          <t>0.8899</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at Glance with 6.4 YOE. Demonstrates deep expertise in Pinecone and FAISS.</t>
+          <t>Strong fit: ML Engineer at Genpact AI with 5.1 YOE. Demonstrates deep expertise in Python and Weaviate.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>CAND_0005538</t>
+          <t>CAND_0091909</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -929,19 +929,19 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>0.8399</t>
+          <t>0.8810</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Strong fit: Senior AI Engineer at Adobe with 5.9 YOE. Demonstrates deep expertise in Python.</t>
+          <t>Strong fit: Machine Learning Engineer at Rephrase.ai with 6.9 YOE. Demonstrates deep expertise in LLMs and Pinecone.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>CAND_0079284</t>
+          <t>CAND_0050454</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -949,19 +949,19 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>0.8355</t>
+          <t>0.8786</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Strong fit: Machine Learning Engineer at Google with 4.9 YOE. Demonstrates deep expertise in Elasticsearch and Qdrant.</t>
+          <t>Strong fit: AI Engineer at Rephrase.ai with 6.8 YOE. Demonstrates deep expertise in Fine-tuning LLMs and FAISS.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>CAND_0079387</t>
+          <t>CAND_0076482</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -969,19 +969,19 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>0.8355</t>
+          <t>0.8786</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Strong fit: AI Engineer at Microsoft with 6.9 YOE. Demonstrates deep expertise in OpenSearch and Python.</t>
+          <t>Strong fit: ML Engineer at Flipkart with 6.6 YOE. Demonstrates deep expertise in OpenSearch and Pinecone.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>CAND_0070398</t>
+          <t>CAND_0005538</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -989,19 +989,19 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>0.8344</t>
+          <t>0.8604</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Strong fit: Machine Learning Engineer at Genpact AI with 7.2 YOE. Demonstrates deep expertise in Embeddings and FAISS.</t>
+          <t>Strong fit: Senior AI Engineer at Adobe with 5.9 YOE. Demonstrates deep expertise in Python.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>CAND_0049538</t>
+          <t>CAND_0009691</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -1009,19 +1009,19 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>0.8310</t>
+          <t>0.8597</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Strong fit: Applied ML Engineer at Saarthi.ai with 5.8 YOE. Demonstrates deep expertise in Elasticsearch and Milvus.</t>
+          <t>Strong fit: Applied ML Engineer at LinkedIn with 6.2 YOE. Demonstrates deep expertise in Fine-tuning LLMs and Pinecone.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>CAND_0020350</t>
+          <t>CAND_0090155</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1029,19 +1029,19 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>0.8265</t>
+          <t>0.8558</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Strong fit: AI Engineer at Zoho with 5.8 YOE. Demonstrates deep expertise in FAISS.</t>
+          <t>Strong fit: ML Engineer at Swiggy with 5.8 YOE. Demonstrates deep expertise in Milvus and Qdrant.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>CAND_0093193</t>
+          <t>CAND_0060538</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -1049,19 +1049,19 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>0.8234</t>
+          <t>0.8542</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Strong fit: Senior Machine Learning Engineer at Niramai with 7.9 YOE. Demonstrates deep expertise in OpenSearch and Qdrant.</t>
+          <t>Strong fit: ML Engineer at Verloop.io with 5.2 YOE. Demonstrates deep expertise in OpenSearch and Embeddings.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>CAND_0011263</t>
+          <t>CAND_0075574</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1069,19 +1069,19 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>0.8175</t>
+          <t>0.8539</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at Ola with 5.1 YOE. Demonstrates deep expertise in Pinecone and OpenSearch.</t>
+          <t>Strong fit: Machine Learning Engineer at Haptik with 5.7 YOE. Demonstrates deep expertise in Weaviate and OpenSearch.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>CAND_0068932</t>
+          <t>CAND_0042100</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -1089,19 +1089,19 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>0.8175</t>
+          <t>0.8510</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at Krutrim with 5.2 YOE. Demonstrates deep expertise in OpenSearch and Milvus.</t>
+          <t>Strong fit: Machine Learning Engineer at Freshworks with 7.3 YOE. Demonstrates deep expertise in Elasticsearch and Fine-tuning LLMs.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>CAND_0096142</t>
+          <t>CAND_0099806</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -1109,19 +1109,19 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>0.8156</t>
+          <t>0.8507</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Strong fit: Applied ML Engineer at upGrad with 5.0 YOE. Demonstrates deep expertise in Python and Pinecone.</t>
+          <t>Strong fit: AI Engineer at Mad Street Den with 4.6 YOE. Demonstrates deep expertise in FAISS and Embeddings.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>CAND_0055905</t>
+          <t>CAND_0079284</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -1129,19 +1129,19 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>0.8145</t>
+          <t>0.8482</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Strong fit: Senior Machine Learning Engineer at Flipkart with 8.1 YOE. Demonstrates deep expertise in Elasticsearch and Embeddings.</t>
+          <t>Strong fit: Machine Learning Engineer at Google with 4.9 YOE. Demonstrates deep expertise in Qdrant and Fine-tuning LLMs.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>CAND_0076482</t>
+          <t>CAND_0055905</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -1149,19 +1149,19 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>0.8117</t>
+          <t>0.8450</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at Flipkart with 6.6 YOE. Demonstrates deep expertise in Pinecone and Embeddings.</t>
+          <t>Strong fit: Senior Machine Learning Engineer at Flipkart with 8.1 YOE. Demonstrates deep expertise in Elasticsearch and Python.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>CAND_0058688</t>
+          <t>CAND_0006418</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -1169,19 +1169,19 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>0.8070</t>
+          <t>0.8444</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Strong fit: AI Engineer at Vedantu with 6.7 YOE. Demonstrates deep expertise in Milvus and Embeddings.</t>
+          <t>Strong fit: Machine Learning Engineer at Verloop.io with 5.7 YOE. Demonstrates deep expertise in Embeddings and Weaviate.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>CAND_0017178</t>
+          <t>CAND_0093193</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -1189,19 +1189,19 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>0.8040</t>
+          <t>0.8401</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at Swiggy with 4.2 YOE. Demonstrates deep expertise in PEFT and pgvector.</t>
+          <t>Strong fit: Senior Machine Learning Engineer at Niramai with 7.9 YOE. Demonstrates deep expertise in Qdrant and OpenSearch.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>CAND_0027691</t>
+          <t>CAND_0090584</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -1209,19 +1209,19 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>0.8040</t>
+          <t>0.8400</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Strong fit: NLP Engineer at Haptik with 6.5 YOE. Demonstrates deep expertise in Weaviate and Python.</t>
+          <t>Strong fit: ML Engineer at Flipkart with 5.1 YOE. Demonstrates deep expertise in Fine-tuning LLMs and OpenSearch.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>CAND_0091909</t>
+          <t>CAND_0018094</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -1229,19 +1229,19 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>0.8034</t>
+          <t>0.8393</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Strong fit: Machine Learning Engineer at Rephrase.ai with 6.9 YOE. Demonstrates deep expertise in Pinecone and OpenSearch.</t>
+          <t>Strong fit: ML Engineer at Mad Street Den with 5.2 YOE. Demonstrates deep expertise in Pinecone and Fine-tuning LLMs.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>CAND_0016163</t>
+          <t>CAND_0071939</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -1249,19 +1249,19 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>0.8028</t>
+          <t>0.8345</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Strong fit: Applied ML Engineer at Dream11 with 6.7 YOE. Demonstrates deep expertise in Embeddings and Pinecone.</t>
+          <t>Strong fit: Data Scientist at Krutrim with 6.4 YOE. Demonstrates deep expertise in Elasticsearch and OpenSearch.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>CAND_0065514</t>
+          <t>CAND_0007460</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -1269,19 +1269,19 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>0.8028</t>
+          <t>0.8288</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at Genpact AI with 6.6 YOE. Demonstrates deep expertise in Milvus and Elasticsearch.</t>
+          <t>Strong fit: AI Engineer at Salesforce with 4.7 YOE. Demonstrates deep expertise in Embeddings and Weaviate.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>CAND_0090155</t>
+          <t>CAND_0054123</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -1289,19 +1289,19 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>0.8028</t>
+          <t>0.8279</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at Swiggy with 5.8 YOE. Demonstrates deep expertise in Pinecone and Milvus.</t>
+          <t>Strong fit: Applied ML Engineer at Meta with 4.7 YOE. Demonstrates deep expertise in Python and Weaviate.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>CAND_0069905</t>
+          <t>CAND_0040178</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -1309,19 +1309,19 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>0.8025</t>
+          <t>0.8271</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Strong fit: Applied ML Engineer at Sarvam AI with 6.6 YOE. Demonstrates deep expertise in Weaviate and Python.</t>
+          <t>Strong fit: ML Engineer at Meesho with 5.0 YOE. Demonstrates deep expertise in Weaviate and Fine-tuning LLMs.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>CAND_0042100</t>
+          <t>CAND_0064904</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -1329,19 +1329,19 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>0.8014</t>
+          <t>0.8271</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Strong fit: Machine Learning Engineer at Freshworks with 7.3 YOE. Demonstrates deep expertise in Pinecone and Elasticsearch.</t>
+          <t>Strong fit: AI Engineer at LinkedIn with 4.9 YOE. Demonstrates deep expertise in Embeddings and Elasticsearch.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>CAND_0039383</t>
+          <t>CAND_0049538</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -1349,19 +1349,19 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>0.7987</t>
+          <t>0.8263</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Strong fit: Applied ML Engineer at Meesho with 7.1 YOE. Demonstrates deep expertise in FAISS and Elasticsearch.</t>
+          <t>Strong fit: Applied ML Engineer at Saarthi.ai with 5.8 YOE. Demonstrates deep expertise in OpenSearch and Milvus.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>CAND_0049615</t>
+          <t>CAND_0068811</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -1369,19 +1369,19 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>0.7973</t>
+          <t>0.8263</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at Krutrim with 5.1 YOE. Demonstrates deep expertise in Pinecone.</t>
+          <t>Strong fit: Applied ML Engineer at Freshworks with 8.0 YOE. Demonstrates deep expertise in Qdrant and Embeddings.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>CAND_0047542</t>
+          <t>CAND_0002037</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -1389,19 +1389,19 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>0.7959</t>
+          <t>0.8261</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Strong fit: Senior Software Engineer (ML) at Meesho with 5.0 YOE. Demonstrates deep expertise in Weaviate and Embeddings.</t>
+          <t>Strong fit: ML Engineer at Locobuzz with 5.5 YOE. Demonstrates deep expertise in Fine-tuning LLMs and Milvus.</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>CAND_0071939</t>
+          <t>CAND_0069232</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -1409,19 +1409,19 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>0.7955</t>
+          <t>0.8238</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Strong fit: Data Scientist at Krutrim with 6.4 YOE. Demonstrates deep expertise in OpenSearch and Embeddings.</t>
+          <t>Strong fit: ML Engineer at Yellow.ai with 6.3 YOE. Demonstrates deep expertise in Pinecone and NLP.</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>CAND_0075439</t>
+          <t>CAND_0003841</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -1429,19 +1429,19 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>0.7950</t>
+          <t>0.8198</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Strong fit: Machine Learning Engineer at Flipkart with 4.3 YOE. Demonstrates deep expertise in Elasticsearch and Embeddings.</t>
+          <t>Strong fit: ML Engineer at Tech Mahindra with 5.0 YOE. Demonstrates deep expertise in Pinecone and Fine-tuning LLMs.</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>CAND_0006418</t>
+          <t>CAND_0015528</t>
         </is>
       </c>
       <c r="B52" t="n">
@@ -1449,19 +1449,19 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>0.7941</t>
+          <t>0.8190</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Strong fit: Machine Learning Engineer at Verloop.io with 5.7 YOE. Demonstrates deep expertise in Weaviate and Embeddings.</t>
+          <t>Strong fit: Applied ML Engineer at Krutrim with 7.4 YOE. Demonstrates deep expertise in Weaviate and OpenSearch.</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>CAND_0060054</t>
+          <t>CAND_0042029</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -1469,19 +1469,19 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>0.7935</t>
+          <t>0.8174</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Strong fit: AI Engineer at Mad Street Den with 6.4 YOE. Demonstrates deep expertise in FAISS and Elasticsearch.</t>
+          <t>Strong fit: Senior Data Scientist at Flipkart with 6.5 YOE. Demonstrates deep expertise in NLP and Elasticsearch.</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>CAND_0040178</t>
+          <t>CAND_0082086</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -1489,19 +1489,19 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>0.7930</t>
+          <t>0.8174</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at Meesho with 5.0 YOE. Demonstrates deep expertise in OpenSearch and Python.</t>
+          <t>Strong fit: Senior Software Engineer (ML) at Razorpay with 6.0 YOE. Demonstrates deep expertise in FAISS and Pinecone.</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>CAND_0000273</t>
+          <t>CAND_0094759</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -1509,19 +1509,19 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>0.7915</t>
+          <t>0.8159</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at BYJU'S with 5.8 YOE. Demonstrates deep expertise in Qdrant.</t>
+          <t>Strong fit: Lead AI Engineer at Meta with 8.6 YOE. Demonstrates deep expertise in Qdrant and Fine-tuning LLMs.</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>CAND_0030348</t>
+          <t>CAND_0017093</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -1529,19 +1529,19 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>0.7905</t>
+          <t>0.8157</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Strong fit: Machine Learning Engineer at BYJU'S with 4.5 YOE. Demonstrates deep expertise in Python and Elasticsearch.</t>
+          <t>Strong fit: ML Engineer at Zoho with 5.9 YOE. Demonstrates deep expertise in LLMs and Embeddings.</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>CAND_0099806</t>
+          <t>CAND_0068932</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -1549,19 +1549,19 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>0.7890</t>
+          <t>0.8157</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Strong fit: AI Engineer at Mad Street Den with 4.6 YOE. Demonstrates deep expertise in Embeddings and Qdrant.</t>
+          <t>Strong fit: ML Engineer at Krutrim with 5.2 YOE. Demonstrates deep expertise in Milvus and OpenSearch.</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>CAND_0024147</t>
+          <t>CAND_0098217</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -1569,19 +1569,19 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>0.7883</t>
+          <t>0.8157</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at Ola with 5.9 YOE. Demonstrates deep expertise in Qdrant and OpenSearch.</t>
+          <t>Strong fit: ML Engineer at Glance with 6.4 YOE. Demonstrates deep expertise in FAISS and Pinecone.</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>CAND_0070202</t>
+          <t>CAND_0032216</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -1589,19 +1589,19 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>0.7880</t>
+          <t>0.8101</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Strong fit: Machine Learning Engineer at BYJU'S with 5.1 YOE. Demonstrates deep expertise in Embeddings and Qdrant.</t>
+          <t>Strong fit: ML Engineer at upGrad with 6.1 YOE. Demonstrates deep expertise in Qdrant.</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>CAND_0033987</t>
+          <t>CAND_0048166</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -1609,19 +1609,19 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>0.7842</t>
+          <t>0.8052</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at Wysa with 6.8 YOE. Demonstrates deep expertise in FAISS.</t>
+          <t>Strong fit: ML Engineer at Aganitha with 5.2 YOE. Demonstrates deep expertise in Pinecone and Milvus.</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>CAND_0066376</t>
+          <t>CAND_0011263</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -1629,19 +1629,19 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>0.7842</t>
+          <t>0.8049</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Strong fit: Applied ML Engineer at Dream11 with 5.7 YOE. Demonstrates deep expertise in FAISS.</t>
+          <t>Strong fit: ML Engineer at Ola with 5.1 YOE. Demonstrates deep expertise in Pinecone and OpenSearch.</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>CAND_0039962</t>
+          <t>CAND_0055992</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -1649,12 +1649,12 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>0.7822</t>
+          <t>0.8044</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at Paytm with 6.5 YOE. Demonstrates deep expertise in Pinecone.</t>
+          <t>Strong fit: AI Engineer at CRED with 16.9 YOE. Demonstrates deep expertise in FAISS and OpenSearch.</t>
         </is>
       </c>
     </row>
@@ -1669,7 +1669,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>0.7808</t>
+          <t>0.8042</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -1681,7 +1681,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>CAND_0069232</t>
+          <t>CAND_0061257</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -1689,19 +1689,19 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>0.7768</t>
+          <t>0.8036</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at Yellow.ai with 6.3 YOE. Demonstrates deep expertise in Weaviate and Python.</t>
+          <t>Strong fit: Staff Machine Learning Engineer at LinkedIn with 8.0 YOE. Demonstrates deep expertise in Python.</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>CAND_0015528</t>
+          <t>CAND_0010257</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -1709,19 +1709,19 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>0.7739</t>
+          <t>0.8026</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Strong fit: Applied ML Engineer at Krutrim with 7.4 YOE. Demonstrates deep expertise in FAISS and OpenSearch.</t>
+          <t>Strong fit: Senior Data Scientist at Google with 6.5 YOE. Demonstrates deep expertise in Milvus and Python.</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>CAND_0043228</t>
+          <t>CAND_0067866</t>
         </is>
       </c>
       <c r="B66" t="n">
@@ -1729,19 +1729,19 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>0.7725</t>
+          <t>0.8019</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Strong fit: Applied ML Engineer at Zoho with 6.8 YOE. Demonstrates deep expertise in OpenSearch and Weaviate.</t>
+          <t>Strong fit: Senior Software Engineer (ML) at Tech Mahindra with 6.4 YOE. Demonstrates deep expertise in Embeddings and Elasticsearch.</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>CAND_0044222</t>
+          <t>CAND_0044855</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -1749,19 +1749,19 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>0.7713</t>
+          <t>0.7991</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Strong fit: AI Engineer at PolicyBazaar with 7.7 YOE. Demonstrates deep expertise in OpenSearch and Qdrant.</t>
+          <t>Strong fit: Senior Data Scientist at Flipkart with 6.6 YOE. Demonstrates deep expertise in OpenSearch and Pinecone.</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>CAND_0048166</t>
+          <t>CAND_0043228</t>
         </is>
       </c>
       <c r="B68" t="n">
@@ -1769,19 +1769,19 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>0.7710</t>
+          <t>0.7946</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at Aganitha with 5.2 YOE. Demonstrates deep expertise in Pinecone and Qdrant.</t>
+          <t>Strong fit: Applied ML Engineer at Zoho with 6.8 YOE. Demonstrates deep expertise in NLP and Weaviate.</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>CAND_0064888</t>
+          <t>CAND_0092255</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -1789,19 +1789,19 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>0.7710</t>
+          <t>0.7946</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at Verloop.io with 5.8 YOE. Demonstrates deep expertise in Elasticsearch and Embeddings.</t>
+          <t>Strong fit: ML Engineer at InMobi with 5.2 YOE. Demonstrates deep expertise in Weaviate and OpenSearch.</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>CAND_0069718</t>
+          <t>CAND_0078002</t>
         </is>
       </c>
       <c r="B70" t="n">
@@ -1809,19 +1809,19 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>0.7698</t>
+          <t>0.7943</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at Saarthi.ai with 5.7 YOE. Demonstrates deep expertise in OpenSearch and Elasticsearch.</t>
+          <t>Strong fit: Machine Learning Engineer at Meta with 6.3 YOE. Demonstrates deep expertise in NLP and Weaviate.</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>CAND_0067866</t>
+          <t>CAND_0039962</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -1829,19 +1829,19 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>0.7669</t>
+          <t>0.7923</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Strong fit: Senior Software Engineer (ML) at Tech Mahindra with 6.4 YOE. Demonstrates deep expertise in Embeddings and Elasticsearch.</t>
+          <t>Strong fit: ML Engineer at Paytm with 6.5 YOE. Demonstrates deep expertise in Pinecone and LLMs.</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>CAND_0082489</t>
+          <t>CAND_0099269</t>
         </is>
       </c>
       <c r="B72" t="n">
@@ -1849,19 +1849,19 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>0.7646</t>
+          <t>0.7909</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at InMobi with 5.3 YOE. Demonstrates deep expertise in Weaviate.</t>
+          <t>Strong fit: Data Scientist at BYJU'S with 5.5 YOE. Demonstrates deep expertise in Elasticsearch and Python.</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>CAND_0009691</t>
+          <t>CAND_0079064</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -1869,19 +1869,19 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>0.7633</t>
+          <t>0.7889</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Strong fit: Applied ML Engineer at LinkedIn with 6.2 YOE. Demonstrates deep expertise in Qdrant and FAISS.</t>
+          <t>Strong fit: Senior Data Scientist at Niramai with 5.2 YOE. Demonstrates deep expertise in OpenSearch and NLP.</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>CAND_0092255</t>
+          <t>CAND_0049615</t>
         </is>
       </c>
       <c r="B74" t="n">
@@ -1889,19 +1889,19 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>0.7626</t>
+          <t>0.7865</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at InMobi with 5.2 YOE. Demonstrates deep expertise in OpenSearch and Weaviate.</t>
+          <t>Strong fit: ML Engineer at Krutrim with 5.1 YOE. Demonstrates deep expertise in NLP and Pinecone.</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>CAND_0052335</t>
+          <t>CAND_0015578</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -1909,19 +1909,19 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>0.7611</t>
+          <t>0.7848</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Strong fit: Applied ML Engineer at Aganitha with 6.4 YOE. Demonstrates deep expertise in PyTorch and NLP.</t>
+          <t>Strong fit: AI Engineer at Zoho with 5.4 YOE. Demonstrates deep expertise in Embeddings and NLP.</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>CAND_0007460</t>
+          <t>CAND_0045475</t>
         </is>
       </c>
       <c r="B76" t="n">
@@ -1929,19 +1929,19 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>0.7607</t>
+          <t>0.7831</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Strong fit: AI Engineer at Salesforce with 4.7 YOE. Demonstrates deep expertise in Weaviate and Embeddings.</t>
+          <t>Strong fit: ML Engineer at Genpact AI with 4.9 YOE. Demonstrates deep expertise in Pinecone and OpenSearch.</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>CAND_0015057</t>
+          <t>CAND_0004972</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -1949,19 +1949,19 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>0.7607</t>
+          <t>0.7818</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at Meesho with 4.6 YOE. Demonstrates deep expertise in Qdrant and Embeddings.</t>
+          <t>Strong fit: ML Engineer at Glance with 6.0 YOE. Demonstrates deep expertise in OpenSearch and LLMs.</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>CAND_0043676</t>
+          <t>CAND_0082489</t>
         </is>
       </c>
       <c r="B78" t="n">
@@ -1969,19 +1969,19 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>0.7590</t>
+          <t>0.7818</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Strong fit: Senior Software Engineer (ML) at Observe.AI with 6.1 YOE. Demonstrates deep expertise in ASR and Reinforcement Learning.</t>
+          <t>Strong fit: ML Engineer at InMobi with 5.3 YOE. Demonstrates deep expertise in Weaviate.</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>CAND_0013393</t>
+          <t>CAND_0005477</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -1989,19 +1989,19 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>0.7582</t>
+          <t>0.7802</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at Freshworks with 5.3 YOE. Demonstrates deep expertise in Pinecone and OpenSearch.</t>
+          <t>Strong fit: ML Engineer at Zomato with 6.2 YOE. Demonstrates deep expertise in OpenSearch.</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>CAND_0066690</t>
+          <t>CAND_0074225</t>
         </is>
       </c>
       <c r="B80" t="n">
@@ -2009,19 +2009,19 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>0.7545</t>
+          <t>0.7796</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at Freshworks with 4.8 YOE. Demonstrates deep expertise in Pinecone and Elasticsearch.</t>
+          <t>Strong fit: Machine Learning Engineer at Unacademy with 4.3 YOE. Demonstrates deep expertise in Elasticsearch and Milvus.</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>CAND_0049543</t>
+          <t>CAND_0060054</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -2029,19 +2029,19 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>0.7538</t>
+          <t>0.7776</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at PolicyBazaar with 6.1 YOE. Demonstrates deep expertise in FAISS.</t>
+          <t>Strong fit: AI Engineer at Mad Street Den with 6.4 YOE. Demonstrates deep expertise in Weaviate and FAISS.</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>CAND_0060538</t>
+          <t>CAND_0073314</t>
         </is>
       </c>
       <c r="B82" t="n">
@@ -2049,19 +2049,19 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>0.7533</t>
+          <t>0.7776</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at Verloop.io with 5.2 YOE. Demonstrates deep expertise in Embeddings and OpenSearch.</t>
+          <t>Strong fit: Senior Software Engineer (ML) at Aganitha with 5.2 YOE. Demonstrates deep expertise in Milvus and Elasticsearch.</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>CAND_0013665</t>
+          <t>CAND_0038949</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -2069,19 +2069,19 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>0.7522</t>
+          <t>0.7772</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Strong fit: Senior Software Engineer (ML) at InMobi with 5.2 YOE. Demonstrates deep expertise in Qdrant and Embeddings.</t>
+          <t>Strong fit: ML Engineer at CRED with 6.4 YOE. Demonstrates deep expertise in Elasticsearch and NLP.</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>CAND_0094759</t>
+          <t>CAND_0055139</t>
         </is>
       </c>
       <c r="B84" t="n">
@@ -2089,19 +2089,19 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>0.7483</t>
+          <t>0.7764</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Strong fit: Lead AI Engineer at Meta with 8.6 YOE. Demonstrates deep expertise in Qdrant and FAISS.</t>
+          <t>Strong fit: ML Engineer at HCL with 6.9 YOE. Demonstrates deep expertise in Elasticsearch and Python.</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>CAND_0045475</t>
+          <t>CAND_0010541</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -2109,19 +2109,19 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>0.7469</t>
+          <t>0.7759</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at Genpact AI with 4.9 YOE. Demonstrates deep expertise in FAISS and Pinecone.</t>
+          <t>Strong fit: AI Research Engineer at Wysa with 6.2 YOE. Demonstrates deep expertise in Pinecone and Weaviate.</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>CAND_0064270</t>
+          <t>CAND_0093547</t>
         </is>
       </c>
       <c r="B86" t="n">
@@ -2129,19 +2129,19 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>0.7469</t>
+          <t>0.7751</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Strong fit: Applied ML Engineer at Verloop.io with 4.2 YOE. Demonstrates deep expertise in OpenSearch and Elasticsearch.</t>
+          <t>Strong fit: Senior Machine Learning Engineer at PhonePe with 2.9 YOE. Demonstrates deep expertise in LLMs and Python.</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>CAND_0062561</t>
+          <t>CAND_0013536</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -2149,19 +2149,19 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>0.7455</t>
+          <t>0.7745</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at Razorpay with 5.9 YOE. Demonstrates deep expertise in Weaviate.</t>
+          <t>Strong fit: Applied ML Engineer at Haptik with 14.1 YOE. Demonstrates deep expertise in LLMs and NLP.</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>CAND_0083879</t>
+          <t>CAND_0024147</t>
         </is>
       </c>
       <c r="B88" t="n">
@@ -2169,19 +2169,19 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>0.7455</t>
+          <t>0.7744</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Strong fit: Machine Learning Engineer at Ola with 7.1 YOE. Demonstrates deep expertise in Milvus.</t>
+          <t>Strong fit: ML Engineer at Ola with 5.9 YOE. Demonstrates deep expertise in Qdrant and OpenSearch.</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>CAND_0091534</t>
+          <t>CAND_0049543</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -2189,19 +2189,19 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>0.7455</t>
+          <t>0.7736</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Strong fit: AI Engineer at Flipkart with 16.6 YOE. Demonstrates deep expertise in Qdrant.</t>
+          <t>Strong fit: ML Engineer at PolicyBazaar with 6.1 YOE. Demonstrates deep expertise in FAISS and NLP.</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>CAND_0090584</t>
+          <t>CAND_0046353</t>
         </is>
       </c>
       <c r="B90" t="n">
@@ -2209,19 +2209,19 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>0.7449</t>
+          <t>0.7734</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at Flipkart with 5.1 YOE. Demonstrates deep expertise in FAISS and OpenSearch.</t>
+          <t>Strong fit: ML Engineer at Razorpay with 6.4 YOE. Demonstrates deep expertise in FAISS and Qdrant.</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>CAND_0075574</t>
+          <t>CAND_0030031</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -2229,19 +2229,19 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>0.7438</t>
+          <t>0.7727</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Strong fit: Machine Learning Engineer at Haptik with 5.7 YOE. Demonstrates deep expertise in OpenSearch and Elasticsearch.</t>
+          <t>Strong fit: AI Engineer at Microsoft with 5.7 YOE. Demonstrates deep expertise in Python and NLP.</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>CAND_0023093</t>
+          <t>CAND_0050876</t>
         </is>
       </c>
       <c r="B92" t="n">
@@ -2249,19 +2249,19 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>0.7436</t>
+          <t>0.7727</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at PolicyBazaar with 5.1 YOE. Demonstrates deep expertise in Milvus and Embeddings.</t>
+          <t>Borderline Match: Strong fit: Applied ML Engineer at Freshworks with 6.0 YOE. Demonstrates deep expertise in Qdrant and FAISS. Meets minimum bar but lacks standout secondary signals.</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>CAND_0015967</t>
+          <t>CAND_0021836</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -2269,19 +2269,19 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>0.7410</t>
+          <t>0.7719</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Strong fit: Senior Software Engineer (ML) at Razorpay with 5.4 YOE. Demonstrates deep expertise in Embeddings and Pinecone.</t>
+          <t>Borderline Match: Strong fit: ML Engineer at CRED with 6.5 YOE. Demonstrates deep expertise in Elasticsearch and NLP. Meets minimum bar but lacks standout secondary signals.</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>CAND_0050876</t>
+          <t>CAND_0047542</t>
         </is>
       </c>
       <c r="B94" t="n">
@@ -2289,19 +2289,19 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>0.7410</t>
+          <t>0.7719</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Strong fit: Applied ML Engineer at Freshworks with 6.0 YOE. Demonstrates deep expertise in Python and OpenSearch.</t>
+          <t>Borderline Match: Strong fit: Senior Software Engineer (ML) at Meesho with 5.0 YOE. Demonstrates deep expertise in Weaviate and Embeddings. Meets minimum bar but lacks standout secondary signals.</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>CAND_0052169</t>
+          <t>CAND_0001819</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -2309,19 +2309,19 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>0.7410</t>
+          <t>0.7694</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at Flipkart with 4.1 YOE. Demonstrates deep expertise in Milvus and Embeddings.</t>
+          <t>Borderline Match: Strong fit: ML Engineer at Genpact AI with 4.4 YOE. Demonstrates deep expertise in Weaviate and NLP. Meets minimum bar but lacks standout secondary signals.</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>CAND_0030031</t>
+          <t>CAND_0079387</t>
         </is>
       </c>
       <c r="B96" t="n">
@@ -2329,19 +2329,19 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>0.7365</t>
+          <t>0.7694</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Strong fit: AI Engineer at Microsoft with 5.7 YOE. Demonstrates deep expertise in Milvus and Python.</t>
+          <t>Borderline Match: Strong fit: AI Engineer at Microsoft with 6.9 YOE. Demonstrates deep expertise in Python and OpenSearch. Meets minimum bar but lacks standout secondary signals.</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>CAND_0073314</t>
+          <t>CAND_0000273</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -2349,19 +2349,19 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>0.7365</t>
+          <t>0.7654</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Strong fit: Senior Software Engineer (ML) at Aganitha with 5.2 YOE. Demonstrates deep expertise in Weaviate and Milvus.</t>
+          <t>Borderline Match: Strong fit: ML Engineer at BYJU'S with 5.8 YOE. Demonstrates deep expertise in Fine-tuning LLMs and Qdrant. Meets minimum bar but lacks standout secondary signals.</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>CAND_0097176</t>
+          <t>CAND_0027691</t>
         </is>
       </c>
       <c r="B98" t="n">
@@ -2369,19 +2369,19 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>0.7365</t>
+          <t>0.7637</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at TCS with 5.9 YOE. Demonstrates deep expertise in FAISS.</t>
+          <t>Borderline Match: Strong fit: NLP Engineer at Haptik with 6.5 YOE. Demonstrates deep expertise in Weaviate and Embeddings. Meets minimum bar but lacks standout secondary signals.</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>CAND_0078002</t>
+          <t>CAND_0061550</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -2389,19 +2389,19 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>0.7345</t>
+          <t>0.7637</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Strong fit: Machine Learning Engineer at Meta with 6.3 YOE. Demonstrates deep expertise in Weaviate.</t>
+          <t>Borderline Match: Strong fit: ML Engineer at Infosys with 5.3 YOE. Demonstrates deep expertise in Data Science and pgvector. Meets minimum bar but lacks standout secondary signals.</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>CAND_0032089</t>
+          <t>CAND_0008978</t>
         </is>
       </c>
       <c r="B100" t="n">
@@ -2409,19 +2409,19 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>0.7322</t>
+          <t>0.7621</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at Saarthi.ai with 6.6 YOE. Demonstrates deep expertise in Python and Pinecone.</t>
+          <t>Borderline Match: Strong fit: Junior ML Engineer at Tech Mahindra with 6.7 YOE. Demonstrates deep expertise in Embeddings and Elasticsearch. Meets minimum bar but lacks standout secondary signals.</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>CAND_0061550</t>
+          <t>CAND_0015967</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -2429,12 +2429,12 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>0.7322</t>
+          <t>0.7605</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at Infosys with 5.3 YOE. Demonstrates deep expertise in Data Science and pgvector.</t>
+          <t>Borderline Match: Strong fit: Senior Software Engineer (ML) at Razorpay with 5.4 YOE. Demonstrates deep expertise in Pinecone and LLMs. Meets minimum bar but lacks standout secondary signals.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: P2 submission pack, offline model script, and semantic performance gate
Add walkthrough and slide deck, make download-model for offline MiniLM, gate semantic encoding on heuristic score for 100K CPU budget, regenerate validated submission.csv/xlsx.
</commit_message>
<xml_diff>
--- a/submission.xlsx
+++ b/submission.xlsx
@@ -441,7 +441,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>CAND_0018499</t>
+          <t>CAND_0002025</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -449,19 +449,19 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>0.9953</t>
+          <t>1.0867</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Exceptional Top 5 Match: Strong fit: Senior Machine Learning Engineer at Zomato with 7.2 YOE. Demonstrates deep expertise in Weaviate and Pinecone. Highly recommended for immediate interview.</t>
+          <t>Exceptional Top 5 Match: Strong fit: Senior AI Engineer at Apple with 5.9 YOE. Demonstrates deep expertise in FAISS and OpenSearch. Highly recommended for immediate interview.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>CAND_0077337</t>
+          <t>CAND_0006567</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -469,19 +469,19 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>0.9937</t>
+          <t>1.0371</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Exceptional Top 5 Match: Strong fit: Staff Machine Learning Engineer at Paytm with 7.0 YOE. Demonstrates deep expertise in Pinecone and LLMs. Highly recommended for immediate interview.</t>
+          <t>Exceptional Top 5 Match: Strong fit: Senior AI Engineer at Meta with 7.9 YOE. Demonstrates deep expertise in NLP and Python. Highly recommended for immediate interview.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>CAND_0020877</t>
+          <t>CAND_0045250</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -489,19 +489,19 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>0.9821</t>
+          <t>0.9990</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Exceptional Top 5 Match: Strong fit: Applied ML Engineer at CRED with 5.1 YOE. Demonstrates deep expertise in Elasticsearch and OpenSearch. Highly recommended for immediate interview.</t>
+          <t>Exceptional Top 5 Match: Strong fit: Applied ML Engineer at Rephrase.ai with 6.6 YOE. Demonstrates deep expertise in Sentence Transformers and Milvus. Highly recommended for immediate interview.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>CAND_0087630</t>
+          <t>CAND_0071974</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -509,19 +509,19 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>0.9742</t>
+          <t>0.9986</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Exceptional Top 5 Match: Strong fit: AI Engineer at Vedantu with 7.2 YOE. Demonstrates deep expertise in Elasticsearch and NLP. Highly recommended for immediate interview.</t>
+          <t>Exceptional Top 5 Match: Strong fit: Senior AI Engineer at Netflix with 7.8 YOE. Demonstrates deep expertise in Weaviate and Pinecone. Highly recommended for immediate interview.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CAND_0080766</t>
+          <t>CAND_0096142</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -529,19 +529,19 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>0.9734</t>
+          <t>0.9669</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Exceptional Top 5 Match: Strong fit: Staff Machine Learning Engineer at Salesforce with 8.8 YOE. Demonstrates deep expertise in Elasticsearch and OpenSearch. Highly recommended for immediate interview.</t>
+          <t>Exceptional Top 5 Match: Strong fit: Applied ML Engineer at upGrad with 5.0 YOE. Demonstrates deep expertise in Weaviate and Pinecone. Highly recommended for immediate interview.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>CAND_0071974</t>
+          <t>CAND_0018499</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -549,19 +549,19 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>0.9701</t>
+          <t>0.9612</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Strong fit: Senior AI Engineer at Netflix with 7.8 YOE. Demonstrates deep expertise in Weaviate and Pinecone.</t>
+          <t>Strong fit: Senior Machine Learning Engineer at Zomato with 7.2 YOE. Demonstrates deep expertise in Weaviate and Pinecone.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>CAND_0088025</t>
+          <t>CAND_0087630</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -569,19 +569,19 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>0.9701</t>
+          <t>0.9566</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Strong fit: Staff Machine Learning Engineer at Yellow.ai with 8.6 YOE. Demonstrates deep expertise in Pinecone and LLMs.</t>
+          <t>Strong fit: AI Engineer at Vedantu with 7.2 YOE. Demonstrates deep expertise in Elasticsearch and NLP.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>CAND_0045250</t>
+          <t>CAND_0020350</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -589,19 +589,19 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>0.9619</t>
+          <t>0.9531</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Strong fit: Applied ML Engineer at Rephrase.ai with 6.6 YOE. Demonstrates deep expertise in Milvus and Embeddings.</t>
+          <t>Strong fit: AI Engineer at Zoho with 5.8 YOE. Demonstrates deep expertise in NLP and LLMs.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>CAND_0096142</t>
+          <t>CAND_0071939</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -609,19 +609,19 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>0.9558</t>
+          <t>0.9513</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Strong fit: Applied ML Engineer at upGrad with 5.0 YOE. Demonstrates deep expertise in Weaviate and Pinecone.</t>
+          <t>Strong fit: Data Scientist at Krutrim with 6.4 YOE. Demonstrates deep expertise in Elasticsearch and OpenSearch.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>CAND_0006567</t>
+          <t>CAND_0001707</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -629,19 +629,19 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>0.9539</t>
+          <t>0.9404</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Strong fit: Senior AI Engineer at Meta with 7.9 YOE. Demonstrates deep expertise in NLP and Python.</t>
+          <t>Strong fit: Data Scientist at Vedantu with 5.6 YOE. Demonstrates deep expertise in Sentence Transformers and FAISS.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>CAND_0065514</t>
+          <t>CAND_0068351</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -649,19 +649,19 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>0.9539</t>
+          <t>0.9359</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at Genpact AI with 6.6 YOE. Demonstrates deep expertise in Pinecone and Elasticsearch.</t>
+          <t>Strong fit: Lead AI Engineer at Sarvam AI with 6.4 YOE. Demonstrates deep expertise in Qdrant and Elasticsearch.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>CAND_0002025</t>
+          <t>CAND_0016163</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -669,19 +669,19 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>0.9498</t>
+          <t>0.9294</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Strong fit: Senior AI Engineer at Apple with 5.9 YOE. Demonstrates deep expertise in FAISS and OpenSearch.</t>
+          <t>Strong fit: Applied ML Engineer at Dream11 with 6.7 YOE. Demonstrates deep expertise in Weaviate and Embeddings.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>CAND_0068351</t>
+          <t>CAND_0010257</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -689,19 +689,19 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>0.9471</t>
+          <t>0.9286</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Strong fit: Lead AI Engineer at Sarvam AI with 6.4 YOE. Demonstrates deep expertise in Qdrant and Elasticsearch.</t>
+          <t>Strong fit: Senior Data Scientist at Google with 6.5 YOE. Demonstrates deep expertise in Milvus and Python.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>CAND_0046525</t>
+          <t>CAND_0065514</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -709,19 +709,19 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>0.9466</t>
+          <t>0.9268</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Strong fit: Senior Machine Learning Engineer at Genpact AI with 6.1 YOE. Demonstrates deep expertise in Elasticsearch and LLMs.</t>
+          <t>Strong fit: ML Engineer at Genpact AI with 6.6 YOE. Demonstrates deep expertise in Vector Search and Pinecone.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>CAND_0089552</t>
+          <t>CAND_0080766</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -729,19 +729,19 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>0.9066</t>
+          <t>0.9200</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Strong fit: Machine Learning Engineer at Netflix with 6.0 YOE. Demonstrates deep expertise in Weaviate and Qdrant.</t>
+          <t>Strong fit: Staff Machine Learning Engineer at Salesforce with 8.8 YOE. Demonstrates deep expertise in Elasticsearch and OpenSearch.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>CAND_0039383</t>
+          <t>CAND_0088025</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -749,19 +749,19 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>0.9003</t>
+          <t>0.9166</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Strong fit: Applied ML Engineer at Meesho with 7.1 YOE. Demonstrates deep expertise in FAISS and NLP.</t>
+          <t>Strong fit: Staff Machine Learning Engineer at Yellow.ai with 8.6 YOE. Demonstrates deep expertise in Pinecone and LLMs.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>CAND_0037566</t>
+          <t>CAND_0039383</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -769,19 +769,19 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>0.8994</t>
+          <t>0.9138</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Strong fit: Machine Learning Engineer at LinkedIn with 6.9 YOE. Demonstrates deep expertise in Pinecone and NLP.</t>
+          <t>Strong fit: Applied ML Engineer at Meesho with 7.1 YOE. Demonstrates deep expertise in FAISS and NLP.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>CAND_0070398</t>
+          <t>CAND_0037566</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -789,19 +789,19 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>0.8987</t>
+          <t>0.9108</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Strong fit: Machine Learning Engineer at Genpact AI with 7.2 YOE. Demonstrates deep expertise in FAISS and Embeddings.</t>
+          <t>Strong fit: Machine Learning Engineer at LinkedIn with 6.9 YOE. Demonstrates deep expertise in Pinecone and NLP.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>CAND_0016163</t>
+          <t>CAND_0081846</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -809,19 +809,19 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>0.8970</t>
+          <t>0.9092</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Strong fit: Applied ML Engineer at Dream11 with 6.7 YOE. Demonstrates deep expertise in Weaviate and Embeddings.</t>
+          <t>Strong fit: Lead AI Engineer at Razorpay with 6.7 YOE. Demonstrates deep expertise in Elasticsearch and Vector Search.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>CAND_0038368</t>
+          <t>CAND_0011263</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -829,19 +829,19 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>0.8970</t>
+          <t>0.8998</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at PhonePe with 5.4 YOE. Demonstrates deep expertise in Embeddings and FAISS.</t>
+          <t>Strong fit: ML Engineer at Ola with 5.1 YOE. Demonstrates deep expertise in Pinecone and OpenSearch.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>CAND_0020350</t>
+          <t>CAND_0005538</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -849,19 +849,19 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>0.8962</t>
+          <t>0.8961</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Strong fit: AI Engineer at Zoho with 5.8 YOE. Demonstrates deep expertise in NLP and LLMs.</t>
+          <t>Strong fit: Senior AI Engineer at Adobe with 5.9 YOE. Demonstrates deep expertise in Python.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>CAND_0044222</t>
+          <t>CAND_0011432</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -869,19 +869,19 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>0.8962</t>
+          <t>0.8951</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Strong fit: AI Engineer at PolicyBazaar with 7.7 YOE. Demonstrates deep expertise in OpenSearch and Qdrant.</t>
+          <t>Strong fit: Senior Data Scientist at Amazon with 7.6 YOE. Demonstrates deep expertise in OpenSearch and Elasticsearch.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>CAND_0081846</t>
+          <t>CAND_0044222</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -889,19 +889,19 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>0.8921</t>
+          <t>0.8911</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Strong fit: Lead AI Engineer at Razorpay with 6.7 YOE. Demonstrates deep expertise in Elasticsearch and Python.</t>
+          <t>Strong fit: AI Engineer at PolicyBazaar with 7.7 YOE. Demonstrates deep expertise in Vector Search and OpenSearch.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>CAND_0095213</t>
+          <t>CAND_0038368</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -909,19 +909,19 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>0.8899</t>
+          <t>0.8898</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at Genpact AI with 5.1 YOE. Demonstrates deep expertise in Python and Weaviate.</t>
+          <t>Strong fit: ML Engineer at PhonePe with 5.4 YOE. Demonstrates deep expertise in Embeddings and FAISS.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>CAND_0091909</t>
+          <t>CAND_0009691</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -929,19 +929,19 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>0.8810</t>
+          <t>0.8869</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Strong fit: Machine Learning Engineer at Rephrase.ai with 6.9 YOE. Demonstrates deep expertise in LLMs and Pinecone.</t>
+          <t>Strong fit: Applied ML Engineer at LinkedIn with 6.2 YOE. Demonstrates deep expertise in Fine-tuning LLMs and Pinecone.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>CAND_0050454</t>
+          <t>CAND_0001494</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -949,19 +949,19 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>0.8786</t>
+          <t>0.8848</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Strong fit: AI Engineer at Rephrase.ai with 6.8 YOE. Demonstrates deep expertise in Fine-tuning LLMs and FAISS.</t>
+          <t>Strong fit: Data Scientist at Haptik with 6.4 YOE. Demonstrates deep expertise in Vector Search and Weaviate.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>CAND_0076482</t>
+          <t>CAND_0089552</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -969,19 +969,19 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>0.8786</t>
+          <t>0.8848</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at Flipkart with 6.6 YOE. Demonstrates deep expertise in OpenSearch and Pinecone.</t>
+          <t>Strong fit: Machine Learning Engineer at Netflix with 6.0 YOE. Demonstrates deep expertise in Weaviate and Qdrant.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>CAND_0005538</t>
+          <t>CAND_0042029</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -989,19 +989,19 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>0.8604</t>
+          <t>0.8812</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Strong fit: Senior AI Engineer at Adobe with 5.9 YOE. Demonstrates deep expertise in Python.</t>
+          <t>Strong fit: Senior Data Scientist at Flipkart with 6.5 YOE. Demonstrates deep expertise in NLP and Elasticsearch.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>CAND_0009691</t>
+          <t>CAND_0077337</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -1009,19 +1009,19 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>0.8597</t>
+          <t>0.8812</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Strong fit: Applied ML Engineer at LinkedIn with 6.2 YOE. Demonstrates deep expertise in Fine-tuning LLMs and Pinecone.</t>
+          <t>Strong fit: Staff Machine Learning Engineer at Paytm with 7.0 YOE. Demonstrates deep expertise in Pinecone and LLMs.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>CAND_0090155</t>
+          <t>CAND_0020877</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1029,19 +1029,19 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>0.8558</t>
+          <t>0.8798</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at Swiggy with 5.8 YOE. Demonstrates deep expertise in Milvus and Qdrant.</t>
+          <t>Strong fit: Applied ML Engineer at CRED with 5.1 YOE. Demonstrates deep expertise in Elasticsearch and OpenSearch.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>CAND_0060538</t>
+          <t>CAND_0046525</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -1049,19 +1049,19 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>0.8542</t>
+          <t>0.8797</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at Verloop.io with 5.2 YOE. Demonstrates deep expertise in OpenSearch and Embeddings.</t>
+          <t>Strong fit: Senior Machine Learning Engineer at Genpact AI with 6.1 YOE. Demonstrates deep expertise in Elasticsearch and LLMs.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>CAND_0075574</t>
+          <t>CAND_0099806</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1069,19 +1069,19 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>0.8539</t>
+          <t>0.8791</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Strong fit: Machine Learning Engineer at Haptik with 5.7 YOE. Demonstrates deep expertise in Weaviate and OpenSearch.</t>
+          <t>Strong fit: AI Engineer at Mad Street Den with 4.6 YOE. Demonstrates deep expertise in FAISS and Embeddings.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>CAND_0042100</t>
+          <t>CAND_0050454</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -1089,19 +1089,19 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>0.8510</t>
+          <t>0.8786</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Strong fit: Machine Learning Engineer at Freshworks with 7.3 YOE. Demonstrates deep expertise in Elasticsearch and Fine-tuning LLMs.</t>
+          <t>Strong fit: AI Engineer at Rephrase.ai with 6.8 YOE. Demonstrates deep expertise in Fine-tuning LLMs and FAISS.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>CAND_0099806</t>
+          <t>CAND_0032216</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -1109,19 +1109,19 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>0.8507</t>
+          <t>0.8783</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Strong fit: AI Engineer at Mad Street Den with 4.6 YOE. Demonstrates deep expertise in FAISS and Embeddings.</t>
+          <t>Strong fit: ML Engineer at upGrad with 6.1 YOE. Demonstrates deep expertise in Qdrant and Sentence Transformers.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>CAND_0079284</t>
+          <t>CAND_0005649</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -1129,19 +1129,19 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>0.8482</t>
+          <t>0.8777</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Strong fit: Machine Learning Engineer at Google with 4.9 YOE. Demonstrates deep expertise in Qdrant and Fine-tuning LLMs.</t>
+          <t>Strong fit: Senior Data Scientist at Sarvam AI with 7.4 YOE. Demonstrates deep expertise in Fine-tuning LLMs and Weaviate.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>CAND_0055905</t>
+          <t>CAND_0013393</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -1149,19 +1149,19 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>0.8450</t>
+          <t>0.8739</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Strong fit: Senior Machine Learning Engineer at Flipkart with 8.1 YOE. Demonstrates deep expertise in Elasticsearch and Python.</t>
+          <t>Strong fit: ML Engineer at Freshworks with 5.3 YOE. Demonstrates deep expertise in Embeddings and Pinecone.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>CAND_0006418</t>
+          <t>CAND_0037944</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -1169,19 +1169,19 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>0.8444</t>
+          <t>0.8726</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Strong fit: Machine Learning Engineer at Verloop.io with 5.7 YOE. Demonstrates deep expertise in Embeddings and Weaviate.</t>
+          <t>Strong fit: Senior Data Scientist at Vedantu with 4.9 YOE. Demonstrates deep expertise in Vector Search and OpenSearch.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>CAND_0093193</t>
+          <t>CAND_0049538</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -1189,19 +1189,19 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>0.8401</t>
+          <t>0.8661</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Strong fit: Senior Machine Learning Engineer at Niramai with 7.9 YOE. Demonstrates deep expertise in Qdrant and OpenSearch.</t>
+          <t>Strong fit: Applied ML Engineer at Saarthi.ai with 5.8 YOE. Demonstrates deep expertise in OpenSearch and Vector Search.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>CAND_0090584</t>
+          <t>CAND_0044855</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -1209,19 +1209,19 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>0.8400</t>
+          <t>0.8632</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at Flipkart with 5.1 YOE. Demonstrates deep expertise in Fine-tuning LLMs and OpenSearch.</t>
+          <t>Strong fit: Senior Data Scientist at Flipkart with 6.6 YOE. Demonstrates deep expertise in OpenSearch and Pinecone.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>CAND_0018094</t>
+          <t>CAND_0043228</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -1229,19 +1229,19 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>0.8393</t>
+          <t>0.8629</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at Mad Street Den with 5.2 YOE. Demonstrates deep expertise in Pinecone and Fine-tuning LLMs.</t>
+          <t>Strong fit: Applied ML Engineer at Zoho with 6.8 YOE. Demonstrates deep expertise in NLP and Vector Search.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>CAND_0071939</t>
+          <t>CAND_0005477</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -1249,19 +1249,19 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>0.8345</t>
+          <t>0.8600</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Strong fit: Data Scientist at Krutrim with 6.4 YOE. Demonstrates deep expertise in Elasticsearch and OpenSearch.</t>
+          <t>Strong fit: ML Engineer at Zomato with 6.2 YOE. Demonstrates deep expertise in OpenSearch.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>CAND_0007460</t>
+          <t>CAND_0045141</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -1269,19 +1269,19 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>0.8288</t>
+          <t>0.8596</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Strong fit: AI Engineer at Salesforce with 4.7 YOE. Demonstrates deep expertise in Embeddings and Weaviate.</t>
+          <t>Strong fit: Data Scientist at HCL with 5.3 YOE. Demonstrates deep expertise in Milvus and Pinecone.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>CAND_0054123</t>
+          <t>CAND_0079284</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -1289,19 +1289,19 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>0.8279</t>
+          <t>0.8596</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Strong fit: Applied ML Engineer at Meta with 4.7 YOE. Demonstrates deep expertise in Python and Weaviate.</t>
+          <t>Strong fit: Machine Learning Engineer at Google with 4.9 YOE. Demonstrates deep expertise in Qdrant and Fine-tuning LLMs.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>CAND_0040178</t>
+          <t>CAND_0015528</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -1309,19 +1309,19 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>0.8271</t>
+          <t>0.8569</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at Meesho with 5.0 YOE. Demonstrates deep expertise in Weaviate and Fine-tuning LLMs.</t>
+          <t>Strong fit: Applied ML Engineer at Krutrim with 7.4 YOE. Demonstrates deep expertise in Weaviate and OpenSearch.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>CAND_0064904</t>
+          <t>CAND_0079387</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -1329,19 +1329,19 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>0.8271</t>
+          <t>0.8548</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Strong fit: AI Engineer at LinkedIn with 4.9 YOE. Demonstrates deep expertise in Embeddings and Elasticsearch.</t>
+          <t>Strong fit: AI Engineer at Microsoft with 6.9 YOE. Demonstrates deep expertise in Python and Sentence Transformers.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>CAND_0049538</t>
+          <t>CAND_0079064</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -1349,19 +1349,19 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>0.8263</t>
+          <t>0.8525</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Strong fit: Applied ML Engineer at Saarthi.ai with 5.8 YOE. Demonstrates deep expertise in OpenSearch and Milvus.</t>
+          <t>Strong fit: Senior Data Scientist at Niramai with 5.2 YOE. Demonstrates deep expertise in OpenSearch and NLP.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>CAND_0068811</t>
+          <t>CAND_0090584</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -1369,19 +1369,19 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>0.8263</t>
+          <t>0.8506</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Strong fit: Applied ML Engineer at Freshworks with 8.0 YOE. Demonstrates deep expertise in Qdrant and Embeddings.</t>
+          <t>Strong fit: ML Engineer at Flipkart with 5.1 YOE. Demonstrates deep expertise in Fine-tuning LLMs and OpenSearch.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>CAND_0002037</t>
+          <t>CAND_0003841</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -1389,19 +1389,19 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>0.8261</t>
+          <t>0.8479</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at Locobuzz with 5.5 YOE. Demonstrates deep expertise in Fine-tuning LLMs and Milvus.</t>
+          <t>Strong fit: ML Engineer at Tech Mahindra with 5.0 YOE. Demonstrates deep expertise in Pinecone and Fine-tuning LLMs.</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>CAND_0069232</t>
+          <t>CAND_0005509</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -1409,19 +1409,19 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>0.8238</t>
+          <t>0.8457</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at Yellow.ai with 6.3 YOE. Demonstrates deep expertise in Pinecone and NLP.</t>
+          <t>Strong fit: Data Scientist at Ola with 6.0 YOE. Demonstrates deep expertise in Python and Fine-tuning LLMs.</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>CAND_0003841</t>
+          <t>CAND_0002037</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -1429,19 +1429,19 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>0.8198</t>
+          <t>0.8416</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at Tech Mahindra with 5.0 YOE. Demonstrates deep expertise in Pinecone and Fine-tuning LLMs.</t>
+          <t>Strong fit: ML Engineer at Locobuzz with 5.5 YOE. Demonstrates deep expertise in Fine-tuning LLMs and Milvus.</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>CAND_0015528</t>
+          <t>CAND_0051004</t>
         </is>
       </c>
       <c r="B52" t="n">
@@ -1449,19 +1449,19 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>0.8190</t>
+          <t>0.8409</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Strong fit: Applied ML Engineer at Krutrim with 7.4 YOE. Demonstrates deep expertise in Weaviate and OpenSearch.</t>
+          <t>Strong fit: Senior Data Scientist at CRED with 4.7 YOE. Demonstrates deep expertise in Embeddings and Qdrant.</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>CAND_0042029</t>
+          <t>CAND_0081852</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -1469,19 +1469,19 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>0.8174</t>
+          <t>0.8396</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Strong fit: Senior Data Scientist at Flipkart with 6.5 YOE. Demonstrates deep expertise in NLP and Elasticsearch.</t>
+          <t>Strong fit: Senior Data Scientist at Mad Street Den with 5.9 YOE. Demonstrates deep expertise in Milvus and Weaviate.</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>CAND_0082086</t>
+          <t>CAND_0055905</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -1489,19 +1489,19 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>0.8174</t>
+          <t>0.8393</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Strong fit: Senior Software Engineer (ML) at Razorpay with 6.0 YOE. Demonstrates deep expertise in FAISS and Pinecone.</t>
+          <t>Strong fit: Senior Machine Learning Engineer at Flipkart with 8.1 YOE. Demonstrates deep expertise in Elasticsearch and Python.</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>CAND_0094759</t>
+          <t>CAND_0074342</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -1509,19 +1509,19 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>0.8159</t>
+          <t>0.8380</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Strong fit: Lead AI Engineer at Meta with 8.6 YOE. Demonstrates deep expertise in Qdrant and Fine-tuning LLMs.</t>
+          <t>Strong fit: Data Scientist at Zoho with 5.7 YOE. Demonstrates deep expertise in Sentence Transformers and LLMs.</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>CAND_0017093</t>
+          <t>CAND_0007460</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -1529,19 +1529,19 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>0.8157</t>
+          <t>0.8374</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at Zoho with 5.9 YOE. Demonstrates deep expertise in LLMs and Embeddings.</t>
+          <t>Strong fit: AI Engineer at Salesforce with 4.7 YOE. Demonstrates deep expertise in Embeddings and Weaviate.</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>CAND_0068932</t>
+          <t>CAND_0091909</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -1549,19 +1549,19 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>0.8157</t>
+          <t>0.8364</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at Krutrim with 5.2 YOE. Demonstrates deep expertise in Milvus and OpenSearch.</t>
+          <t>Strong fit: Machine Learning Engineer at Rephrase.ai with 6.9 YOE. Demonstrates deep expertise in LLMs and Pinecone.</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>CAND_0098217</t>
+          <t>CAND_0075574</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -1569,19 +1569,19 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>0.8157</t>
+          <t>0.8357</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at Glance with 6.4 YOE. Demonstrates deep expertise in FAISS and Pinecone.</t>
+          <t>Strong fit: Machine Learning Engineer at Haptik with 5.7 YOE. Demonstrates deep expertise in Weaviate and OpenSearch.</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>CAND_0032216</t>
+          <t>CAND_0068811</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -1589,19 +1589,19 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>0.8101</t>
+          <t>0.8345</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at upGrad with 6.1 YOE. Demonstrates deep expertise in Qdrant.</t>
+          <t>Strong fit: Applied ML Engineer at Freshworks with 8.0 YOE. Demonstrates deep expertise in Vector Search and Qdrant.</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>CAND_0048166</t>
+          <t>CAND_0010149</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -1609,19 +1609,19 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>0.8052</t>
+          <t>0.8333</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at Aganitha with 5.2 YOE. Demonstrates deep expertise in Pinecone and Milvus.</t>
+          <t>Strong fit: ML Engineer at Glance with 6.9 YOE. Demonstrates deep expertise in Milvus and Vector Search.</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>CAND_0011263</t>
+          <t>CAND_0006557</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -1629,19 +1629,19 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>0.8049</t>
+          <t>0.8290</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at Ola with 5.1 YOE. Demonstrates deep expertise in Pinecone and OpenSearch.</t>
+          <t>Strong fit: NLP Engineer at Paytm with 7.9 YOE. Demonstrates deep expertise in Elasticsearch and OpenSearch.</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>CAND_0055992</t>
+          <t>CAND_0010541</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -1649,19 +1649,19 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>0.8044</t>
+          <t>0.8285</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Strong fit: AI Engineer at CRED with 16.9 YOE. Demonstrates deep expertise in FAISS and OpenSearch.</t>
+          <t>Strong fit: AI Research Engineer at Wysa with 6.2 YOE. Demonstrates deep expertise in Pinecone and Weaviate.</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>CAND_0010149</t>
+          <t>CAND_0017093</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -1669,19 +1669,19 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>0.8042</t>
+          <t>0.8271</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at Glance with 6.9 YOE. Demonstrates deep expertise in Milvus and Elasticsearch.</t>
+          <t>Strong fit: ML Engineer at Zoho with 5.9 YOE. Demonstrates deep expertise in LLMs and Embeddings.</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>CAND_0061257</t>
+          <t>CAND_0070398</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -1689,19 +1689,19 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>0.8036</t>
+          <t>0.8271</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Strong fit: Staff Machine Learning Engineer at LinkedIn with 8.0 YOE. Demonstrates deep expertise in Python.</t>
+          <t>Strong fit: Machine Learning Engineer at Genpact AI with 7.2 YOE. Demonstrates deep expertise in FAISS and Embeddings.</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>CAND_0010257</t>
+          <t>CAND_0098217</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -1709,19 +1709,19 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>0.8026</t>
+          <t>0.8271</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Strong fit: Senior Data Scientist at Google with 6.5 YOE. Demonstrates deep expertise in Milvus and Python.</t>
+          <t>Strong fit: ML Engineer at Glance with 6.4 YOE. Demonstrates deep expertise in FAISS and Pinecone.</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>CAND_0067866</t>
+          <t>CAND_0047721</t>
         </is>
       </c>
       <c r="B66" t="n">
@@ -1729,19 +1729,19 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>0.8019</t>
+          <t>0.8264</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Strong fit: Senior Software Engineer (ML) at Tech Mahindra with 6.4 YOE. Demonstrates deep expertise in Embeddings and Elasticsearch.</t>
+          <t>Strong fit: Senior Data Scientist at Microsoft with 7.0 YOE. Demonstrates deep expertise in Milvus and FAISS.</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>CAND_0044855</t>
+          <t>CAND_0099269</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -1749,19 +1749,19 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>0.7991</t>
+          <t>0.8248</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Strong fit: Senior Data Scientist at Flipkart with 6.6 YOE. Demonstrates deep expertise in OpenSearch and Pinecone.</t>
+          <t>Strong fit: Data Scientist at BYJU'S with 5.5 YOE. Demonstrates deep expertise in Elasticsearch and Python.</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>CAND_0043228</t>
+          <t>CAND_0006418</t>
         </is>
       </c>
       <c r="B68" t="n">
@@ -1769,19 +1769,19 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>0.7946</t>
+          <t>0.8236</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Strong fit: Applied ML Engineer at Zoho with 6.8 YOE. Demonstrates deep expertise in NLP and Weaviate.</t>
+          <t>Strong fit: Machine Learning Engineer at Verloop.io with 5.7 YOE. Demonstrates deep expertise in Embeddings and Weaviate.</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>CAND_0092255</t>
+          <t>CAND_0015057</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -1789,19 +1789,19 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>0.7946</t>
+          <t>0.8214</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at InMobi with 5.2 YOE. Demonstrates deep expertise in Weaviate and OpenSearch.</t>
+          <t>Strong fit: ML Engineer at Meesho with 4.6 YOE. Demonstrates deep expertise in Sentence Transformers and Vector Search.</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>CAND_0078002</t>
+          <t>CAND_0036121</t>
         </is>
       </c>
       <c r="B70" t="n">
@@ -1809,19 +1809,19 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>0.7943</t>
+          <t>0.8174</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Strong fit: Machine Learning Engineer at Meta with 6.3 YOE. Demonstrates deep expertise in NLP and Weaviate.</t>
+          <t>Strong fit: ML Engineer at Wysa with 5.2 YOE. Demonstrates deep expertise in Embeddings and Vector Search.</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>CAND_0039962</t>
+          <t>CAND_0015578</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -1829,19 +1829,19 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>0.7923</t>
+          <t>0.8141</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at Paytm with 6.5 YOE. Demonstrates deep expertise in Pinecone and LLMs.</t>
+          <t>Strong fit: AI Engineer at Zoho with 5.4 YOE. Demonstrates deep expertise in Embeddings and NLP.</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>CAND_0099269</t>
+          <t>CAND_0030031</t>
         </is>
       </c>
       <c r="B72" t="n">
@@ -1849,19 +1849,19 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>0.7909</t>
+          <t>0.8126</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Strong fit: Data Scientist at BYJU'S with 5.5 YOE. Demonstrates deep expertise in Elasticsearch and Python.</t>
+          <t>Strong fit: AI Engineer at Microsoft with 5.7 YOE. Demonstrates deep expertise in Python and NLP.</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>CAND_0079064</t>
+          <t>CAND_0021836</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -1869,19 +1869,19 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>0.7889</t>
+          <t>0.8117</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Strong fit: Senior Data Scientist at Niramai with 5.2 YOE. Demonstrates deep expertise in OpenSearch and NLP.</t>
+          <t>Strong fit: ML Engineer at CRED with 6.5 YOE. Demonstrates deep expertise in Vector Search and Elasticsearch.</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>CAND_0049615</t>
+          <t>CAND_0035653</t>
         </is>
       </c>
       <c r="B74" t="n">
@@ -1889,19 +1889,19 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>0.7865</t>
+          <t>0.8114</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at Krutrim with 5.1 YOE. Demonstrates deep expertise in NLP and Pinecone.</t>
+          <t>Strong fit: Data Scientist at Swiggy with 5.6 YOE. Demonstrates deep expertise in OpenSearch and Vector Search.</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>CAND_0015578</t>
+          <t>CAND_0040178</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -1909,19 +1909,19 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>0.7848</t>
+          <t>0.8106</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Strong fit: AI Engineer at Zoho with 5.4 YOE. Demonstrates deep expertise in Embeddings and NLP.</t>
+          <t>Strong fit: ML Engineer at Meesho with 5.0 YOE. Demonstrates deep expertise in Weaviate and Fine-tuning LLMs.</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>CAND_0045475</t>
+          <t>CAND_0000273</t>
         </is>
       </c>
       <c r="B76" t="n">
@@ -1929,19 +1929,19 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>0.7831</t>
+          <t>0.8105</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at Genpact AI with 4.9 YOE. Demonstrates deep expertise in Pinecone and OpenSearch.</t>
+          <t>Strong fit: ML Engineer at BYJU'S with 5.8 YOE. Demonstrates deep expertise in Fine-tuning LLMs and Qdrant.</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>CAND_0004972</t>
+          <t>CAND_0050876</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -1949,19 +1949,19 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>0.7818</t>
+          <t>0.8098</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at Glance with 6.0 YOE. Demonstrates deep expertise in OpenSearch and LLMs.</t>
+          <t>Strong fit: Applied ML Engineer at Freshworks with 6.0 YOE. Demonstrates deep expertise in Qdrant and FAISS.</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>CAND_0082489</t>
+          <t>CAND_0076482</t>
         </is>
       </c>
       <c r="B78" t="n">
@@ -1969,19 +1969,19 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>0.7818</t>
+          <t>0.8089</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at InMobi with 5.3 YOE. Demonstrates deep expertise in Weaviate.</t>
+          <t>Strong fit: ML Engineer at Flipkart with 6.6 YOE. Demonstrates deep expertise in OpenSearch and Pinecone.</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>CAND_0005477</t>
+          <t>CAND_0048558</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -1989,19 +1989,19 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>0.7802</t>
+          <t>0.8084</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at Zomato with 6.2 YOE. Demonstrates deep expertise in OpenSearch.</t>
+          <t>Strong fit: Data Scientist at Rephrase.ai with 6.7 YOE. Demonstrates deep expertise in OpenSearch and Qdrant.</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>CAND_0074225</t>
+          <t>CAND_0093193</t>
         </is>
       </c>
       <c r="B80" t="n">
@@ -2009,19 +2009,19 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>0.7796</t>
+          <t>0.8068</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Strong fit: Machine Learning Engineer at Unacademy with 4.3 YOE. Demonstrates deep expertise in Elasticsearch and Milvus.</t>
+          <t>Strong fit: Senior Machine Learning Engineer at Niramai with 7.9 YOE. Demonstrates deep expertise in Qdrant and OpenSearch.</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>CAND_0060054</t>
+          <t>CAND_0005311</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -2029,19 +2029,19 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>0.7776</t>
+          <t>0.8066</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Strong fit: AI Engineer at Mad Street Den with 6.4 YOE. Demonstrates deep expertise in Weaviate and FAISS.</t>
+          <t>Strong fit: AI Research Engineer at Aganitha with 5.7 YOE. Demonstrates deep expertise in Qdrant and Fine-tuning LLMs.</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>CAND_0073314</t>
+          <t>CAND_0048166</t>
         </is>
       </c>
       <c r="B82" t="n">
@@ -2049,19 +2049,19 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>0.7776</t>
+          <t>0.7998</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Strong fit: Senior Software Engineer (ML) at Aganitha with 5.2 YOE. Demonstrates deep expertise in Milvus and Elasticsearch.</t>
+          <t>Strong fit: ML Engineer at Aganitha with 5.2 YOE. Demonstrates deep expertise in Pinecone and Milvus.</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>CAND_0038949</t>
+          <t>CAND_0015582</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -2069,19 +2069,19 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>0.7772</t>
+          <t>0.7997</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at CRED with 6.4 YOE. Demonstrates deep expertise in Elasticsearch and NLP.</t>
+          <t>Strong fit: ML Engineer at Genpact AI with 4.4 YOE. Demonstrates deep expertise in Qdrant and Sentence Transformers.</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>CAND_0055139</t>
+          <t>CAND_0028287</t>
         </is>
       </c>
       <c r="B84" t="n">
@@ -2089,19 +2089,19 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>0.7764</t>
+          <t>0.7994</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at HCL with 6.9 YOE. Demonstrates deep expertise in Elasticsearch and Python.</t>
+          <t>Strong fit: Data Scientist at Unacademy with 5.7 YOE. Demonstrates deep expertise in OpenSearch and Vector Search.</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>CAND_0010541</t>
+          <t>CAND_0073982</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -2109,19 +2109,19 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>0.7759</t>
+          <t>0.7993</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Strong fit: AI Research Engineer at Wysa with 6.2 YOE. Demonstrates deep expertise in Pinecone and Weaviate.</t>
+          <t>Strong fit: Data Scientist at Dream11 with 7.0 YOE. Demonstrates deep expertise in Sentence Transformers and Qdrant.</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>CAND_0093547</t>
+          <t>CAND_0095213</t>
         </is>
       </c>
       <c r="B86" t="n">
@@ -2129,19 +2129,19 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>0.7751</t>
+          <t>0.7966</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Strong fit: Senior Machine Learning Engineer at PhonePe with 2.9 YOE. Demonstrates deep expertise in LLMs and Python.</t>
+          <t>Strong fit: ML Engineer at Genpact AI with 5.1 YOE. Demonstrates deep expertise in Python and Weaviate.</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>CAND_0013536</t>
+          <t>CAND_0003791</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -2149,19 +2149,19 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>0.7745</t>
+          <t>0.7927</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Strong fit: Applied ML Engineer at Haptik with 14.1 YOE. Demonstrates deep expertise in LLMs and NLP.</t>
+          <t>Strong fit: ML Engineer at Meesho with 6.6 YOE. Demonstrates deep expertise in LLMs and Python.</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>CAND_0024147</t>
+          <t>CAND_0055992</t>
         </is>
       </c>
       <c r="B88" t="n">
@@ -2169,19 +2169,19 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>0.7744</t>
+          <t>0.7897</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at Ola with 5.9 YOE. Demonstrates deep expertise in Qdrant and OpenSearch.</t>
+          <t>Strong fit: AI Engineer at CRED with 16.9 YOE. Demonstrates deep expertise in FAISS and OpenSearch.</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>CAND_0049543</t>
+          <t>CAND_0027723</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -2189,19 +2189,19 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>0.7736</t>
+          <t>0.7889</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at PolicyBazaar with 6.1 YOE. Demonstrates deep expertise in FAISS and NLP.</t>
+          <t>Strong fit: ML Engineer at Wysa with 4.2 YOE. Demonstrates deep expertise in Vector Search and NLP.</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>CAND_0046353</t>
+          <t>CAND_0015493</t>
         </is>
       </c>
       <c r="B90" t="n">
@@ -2209,19 +2209,19 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>0.7734</t>
+          <t>0.7886</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at Razorpay with 6.4 YOE. Demonstrates deep expertise in FAISS and Qdrant.</t>
+          <t>Strong fit: Data Scientist at CRED with 6.4 YOE. Demonstrates deep expertise in NLP.</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>CAND_0030031</t>
+          <t>CAND_0090155</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -2229,19 +2229,19 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>0.7727</t>
+          <t>0.7881</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Strong fit: AI Engineer at Microsoft with 5.7 YOE. Demonstrates deep expertise in Python and NLP.</t>
+          <t>Strong fit: ML Engineer at Swiggy with 5.8 YOE. Demonstrates deep expertise in Milvus and Qdrant.</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>CAND_0050876</t>
+          <t>CAND_0060538</t>
         </is>
       </c>
       <c r="B92" t="n">
@@ -2249,19 +2249,19 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>0.7727</t>
+          <t>0.7867</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Borderline Match: Strong fit: Applied ML Engineer at Freshworks with 6.0 YOE. Demonstrates deep expertise in Qdrant and FAISS. Meets minimum bar but lacks standout secondary signals.</t>
+          <t>Borderline Match: Strong fit: ML Engineer at Verloop.io with 5.2 YOE. Demonstrates deep expertise in OpenSearch and Embeddings. Meets minimum bar but lacks standout secondary signals.</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>CAND_0021836</t>
+          <t>CAND_0042100</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -2269,19 +2269,19 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>0.7719</t>
+          <t>0.7838</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Borderline Match: Strong fit: ML Engineer at CRED with 6.5 YOE. Demonstrates deep expertise in Elasticsearch and NLP. Meets minimum bar but lacks standout secondary signals.</t>
+          <t>Borderline Match: Strong fit: Machine Learning Engineer at Freshworks with 7.3 YOE. Demonstrates deep expertise in Elasticsearch and Fine-tuning LLMs. Meets minimum bar but lacks standout secondary signals.</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>CAND_0047542</t>
+          <t>CAND_0083879</t>
         </is>
       </c>
       <c r="B94" t="n">
@@ -2289,19 +2289,19 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>0.7719</t>
+          <t>0.7816</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Borderline Match: Strong fit: Senior Software Engineer (ML) at Meesho with 5.0 YOE. Demonstrates deep expertise in Weaviate and Embeddings. Meets minimum bar but lacks standout secondary signals.</t>
+          <t>Borderline Match: Strong fit: Machine Learning Engineer at Ola with 7.1 YOE. Demonstrates deep expertise in Fine-tuning LLMs and Milvus. Meets minimum bar but lacks standout secondary signals.</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>CAND_0001819</t>
+          <t>CAND_0092255</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -2309,19 +2309,19 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>0.7694</t>
+          <t>0.7802</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Borderline Match: Strong fit: ML Engineer at Genpact AI with 4.4 YOE. Demonstrates deep expertise in Weaviate and NLP. Meets minimum bar but lacks standout secondary signals.</t>
+          <t>Borderline Match: Strong fit: ML Engineer at InMobi with 5.2 YOE. Demonstrates deep expertise in Weaviate and OpenSearch. Meets minimum bar but lacks standout secondary signals.</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>CAND_0079387</t>
+          <t>CAND_0012837</t>
         </is>
       </c>
       <c r="B96" t="n">
@@ -2329,19 +2329,19 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>0.7694</t>
+          <t>0.7789</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Borderline Match: Strong fit: AI Engineer at Microsoft with 6.9 YOE. Demonstrates deep expertise in Python and OpenSearch. Meets minimum bar but lacks standout secondary signals.</t>
+          <t>Borderline Match: Strong fit: Junior ML Engineer at Sarvam AI with 6.4 YOE. Demonstrates deep expertise in Vector Search and Weaviate. Meets minimum bar but lacks standout secondary signals.</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>CAND_0000273</t>
+          <t>CAND_0007412</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -2349,19 +2349,19 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>0.7654</t>
+          <t>0.7786</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Borderline Match: Strong fit: ML Engineer at BYJU'S with 5.8 YOE. Demonstrates deep expertise in Fine-tuning LLMs and Qdrant. Meets minimum bar but lacks standout secondary signals.</t>
+          <t>Borderline Match: Strong fit: Applied ML Engineer at Zoho with 7.4 YOE. Demonstrates deep expertise in Pinecone and Milvus. Meets minimum bar but lacks standout secondary signals.</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>CAND_0027691</t>
+          <t>CAND_0009837</t>
         </is>
       </c>
       <c r="B98" t="n">
@@ -2369,19 +2369,19 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>0.7637</t>
+          <t>0.7777</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Borderline Match: Strong fit: NLP Engineer at Haptik with 6.5 YOE. Demonstrates deep expertise in Weaviate and Embeddings. Meets minimum bar but lacks standout secondary signals.</t>
+          <t>Borderline Match: Strong fit: Senior Data Scientist at Rephrase.ai with 4.3 YOE. Demonstrates deep expertise in Python and FAISS. Meets minimum bar but lacks standout secondary signals.</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>CAND_0061550</t>
+          <t>CAND_0060054</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -2389,19 +2389,19 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>0.7637</t>
+          <t>0.7776</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Borderline Match: Strong fit: ML Engineer at Infosys with 5.3 YOE. Demonstrates deep expertise in Data Science and pgvector. Meets minimum bar but lacks standout secondary signals.</t>
+          <t>Borderline Match: Strong fit: AI Engineer at Mad Street Den with 6.4 YOE. Demonstrates deep expertise in Weaviate and FAISS. Meets minimum bar but lacks standout secondary signals.</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>CAND_0008978</t>
+          <t>CAND_0013536</t>
         </is>
       </c>
       <c r="B100" t="n">
@@ -2409,19 +2409,19 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>0.7621</t>
+          <t>0.7769</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Borderline Match: Strong fit: Junior ML Engineer at Tech Mahindra with 6.7 YOE. Demonstrates deep expertise in Embeddings and Elasticsearch. Meets minimum bar but lacks standout secondary signals.</t>
+          <t>Borderline Match: Strong fit: Applied ML Engineer at Haptik with 14.1 YOE. Demonstrates deep expertise in LLMs and NLP. Meets minimum bar but lacks standout secondary signals.</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>CAND_0015967</t>
+          <t>CAND_0025335</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -2429,12 +2429,12 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>0.7605</t>
+          <t>0.7749</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Borderline Match: Strong fit: Senior Software Engineer (ML) at Razorpay with 5.4 YOE. Demonstrates deep expertise in Pinecone and LLMs. Meets minimum bar but lacks standout secondary signals.</t>
+          <t>Borderline Match: Strong fit: Data Scientist at PolicyBazaar with 6.6 YOE. Demonstrates deep expertise in NLP. Meets minimum bar but lacks standout secondary signals.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: refresh submission artifacts and HF sandbox URL
</commit_message>
<xml_diff>
--- a/submission.xlsx
+++ b/submission.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ranking Results" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Ranking Results" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -441,7 +441,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>CAND_0002025</t>
+          <t>CAND_0071974</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -449,19 +449,19 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>1.0867</t>
+          <t>1.1102</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Exceptional Top 5 Match: Strong fit: Senior AI Engineer at Apple with 5.9 YOE. Demonstrates deep expertise in FAISS and OpenSearch. Highly recommended for immediate interview.</t>
+          <t>Exceptional Top 5 Match: Strong fit: Senior AI Engineer at Netflix with 7.8 YOE. Demonstrates deep expertise in Weaviate and Pinecone. Highly recommended for immediate interview.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>CAND_0006567</t>
+          <t>CAND_0002025</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -469,12 +469,12 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>1.0371</t>
+          <t>1.0867</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Exceptional Top 5 Match: Strong fit: Senior AI Engineer at Meta with 7.9 YOE. Demonstrates deep expertise in NLP and Python. Highly recommended for immediate interview.</t>
+          <t>Exceptional Top 5 Match: Strong fit: Senior AI Engineer at Apple with 5.9 YOE. Demonstrates deep expertise in FAISS and OpenSearch. Highly recommended for immediate interview.</t>
         </is>
       </c>
     </row>
@@ -489,7 +489,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>0.9990</t>
+          <t>1.0832</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -501,7 +501,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>CAND_0071974</t>
+          <t>CAND_0018499</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -509,12 +509,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>0.9986</t>
+          <t>1.0683</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Exceptional Top 5 Match: Strong fit: Senior AI Engineer at Netflix with 7.8 YOE. Demonstrates deep expertise in Weaviate and Pinecone. Highly recommended for immediate interview.</t>
+          <t>Exceptional Top 5 Match: Strong fit: Senior Machine Learning Engineer at Zomato with 7.2 YOE. Demonstrates deep expertise in Weaviate and Pinecone. Highly recommended for immediate interview.</t>
         </is>
       </c>
     </row>
@@ -529,7 +529,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>0.9669</t>
+          <t>1.0519</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -541,7 +541,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>CAND_0018499</t>
+          <t>CAND_0087630</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -549,19 +549,19 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>0.9612</t>
+          <t>1.0478</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Strong fit: Senior Machine Learning Engineer at Zomato with 7.2 YOE. Demonstrates deep expertise in Weaviate and Pinecone.</t>
+          <t>Strong fit: AI Engineer at Vedantu with 7.2 YOE. Demonstrates deep expertise in Elasticsearch and NLP.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>CAND_0087630</t>
+          <t>CAND_0020350</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -569,19 +569,19 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>0.9566</t>
+          <t>1.0460</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Strong fit: AI Engineer at Vedantu with 7.2 YOE. Demonstrates deep expertise in Elasticsearch and NLP.</t>
+          <t>Strong fit: AI Engineer at Zoho with 5.8 YOE. Demonstrates deep expertise in NLP and LLMs.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>CAND_0020350</t>
+          <t>CAND_0006567</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -589,19 +589,19 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>0.9531</t>
+          <t>1.0371</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Strong fit: AI Engineer at Zoho with 5.8 YOE. Demonstrates deep expertise in NLP and LLMs.</t>
+          <t>Strong fit: Senior AI Engineer at Meta with 7.9 YOE. Demonstrates deep expertise in NLP and Python.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>CAND_0071939</t>
+          <t>CAND_0068351</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -609,19 +609,19 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>0.9513</t>
+          <t>1.0350</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Strong fit: Data Scientist at Krutrim with 6.4 YOE. Demonstrates deep expertise in Elasticsearch and OpenSearch.</t>
+          <t>Strong fit: Lead AI Engineer at Sarvam AI with 6.4 YOE. Demonstrates deep expertise in Qdrant and Elasticsearch.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>CAND_0001707</t>
+          <t>CAND_0080766</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -629,19 +629,19 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>0.9404</t>
+          <t>1.0279</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Strong fit: Data Scientist at Vedantu with 5.6 YOE. Demonstrates deep expertise in Sentence Transformers and FAISS.</t>
+          <t>Strong fit: Staff Machine Learning Engineer at Salesforce with 8.8 YOE. Demonstrates deep expertise in Elasticsearch and OpenSearch.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>CAND_0068351</t>
+          <t>CAND_0081846</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -649,19 +649,19 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>0.9359</t>
+          <t>1.0211</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Strong fit: Lead AI Engineer at Sarvam AI with 6.4 YOE. Demonstrates deep expertise in Qdrant and Elasticsearch.</t>
+          <t>Strong fit: Lead AI Engineer at Razorpay with 6.7 YOE. Demonstrates deep expertise in Elasticsearch and Vector Search.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>CAND_0016163</t>
+          <t>CAND_0088025</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -669,19 +669,19 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>0.9294</t>
+          <t>1.0210</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Strong fit: Applied ML Engineer at Dream11 with 6.7 YOE. Demonstrates deep expertise in Weaviate and Embeddings.</t>
+          <t>Strong fit: Staff Machine Learning Engineer at Yellow.ai with 8.6 YOE. Demonstrates deep expertise in Pinecone and LLMs.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>CAND_0010257</t>
+          <t>CAND_0071939</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -689,19 +689,19 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>0.9286</t>
+          <t>1.0122</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Strong fit: Senior Data Scientist at Google with 6.5 YOE. Demonstrates deep expertise in Milvus and Python.</t>
+          <t>Strong fit: Data Scientist at Krutrim with 6.4 YOE. Demonstrates deep expertise in Elasticsearch and OpenSearch.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>CAND_0065514</t>
+          <t>CAND_0037566</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -709,19 +709,19 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>0.9268</t>
+          <t>1.0006</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at Genpact AI with 6.6 YOE. Demonstrates deep expertise in Vector Search and Pinecone.</t>
+          <t>Strong fit: Machine Learning Engineer at LinkedIn with 6.9 YOE. Demonstrates deep expertise in Pinecone and NLP.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>CAND_0080766</t>
+          <t>CAND_0065514</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -729,19 +729,19 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>0.9200</t>
+          <t>0.9997</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Strong fit: Staff Machine Learning Engineer at Salesforce with 8.8 YOE. Demonstrates deep expertise in Elasticsearch and OpenSearch.</t>
+          <t>Strong fit: ML Engineer at Genpact AI with 6.6 YOE. Demonstrates deep expertise in Vector Search and Pinecone.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>CAND_0088025</t>
+          <t>CAND_0039383</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -749,19 +749,19 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>0.9166</t>
+          <t>0.9892</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Strong fit: Staff Machine Learning Engineer at Yellow.ai with 8.6 YOE. Demonstrates deep expertise in Pinecone and LLMs.</t>
+          <t>Strong fit: Applied ML Engineer at Meesho with 7.1 YOE. Demonstrates deep expertise in FAISS and NLP.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>CAND_0039383</t>
+          <t>CAND_0046525</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -769,19 +769,19 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>0.9138</t>
+          <t>0.9845</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Strong fit: Applied ML Engineer at Meesho with 7.1 YOE. Demonstrates deep expertise in FAISS and NLP.</t>
+          <t>Strong fit: Senior Machine Learning Engineer at Genpact AI with 6.1 YOE. Demonstrates deep expertise in Elasticsearch and LLMs.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>CAND_0037566</t>
+          <t>CAND_0038368</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -789,19 +789,19 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>0.9108</t>
+          <t>0.9810</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Strong fit: Machine Learning Engineer at LinkedIn with 6.9 YOE. Demonstrates deep expertise in Pinecone and NLP.</t>
+          <t>Strong fit: ML Engineer at PhonePe with 5.4 YOE. Demonstrates deep expertise in Embeddings and FAISS.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>CAND_0081846</t>
+          <t>CAND_0077337</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -809,19 +809,19 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>0.9092</t>
+          <t>0.9778</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Strong fit: Lead AI Engineer at Razorpay with 6.7 YOE. Demonstrates deep expertise in Elasticsearch and Vector Search.</t>
+          <t>Strong fit: Staff Machine Learning Engineer at Paytm with 7.0 YOE. Demonstrates deep expertise in Pinecone and LLMs.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>CAND_0011263</t>
+          <t>CAND_0044222</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -829,19 +829,19 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>0.8998</t>
+          <t>0.9752</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at Ola with 5.1 YOE. Demonstrates deep expertise in Pinecone and OpenSearch.</t>
+          <t>Strong fit: AI Engineer at PolicyBazaar with 7.7 YOE. Demonstrates deep expertise in Vector Search and OpenSearch.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>CAND_0005538</t>
+          <t>CAND_0099806</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -849,19 +849,19 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>0.8961</t>
+          <t>0.9678</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Strong fit: Senior AI Engineer at Adobe with 5.9 YOE. Demonstrates deep expertise in Python.</t>
+          <t>Strong fit: AI Engineer at Mad Street Den with 4.6 YOE. Demonstrates deep expertise in FAISS and Embeddings.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>CAND_0011432</t>
+          <t>CAND_0050454</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -869,19 +869,19 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>0.8951</t>
+          <t>0.9666</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Strong fit: Senior Data Scientist at Amazon with 7.6 YOE. Demonstrates deep expertise in OpenSearch and Elasticsearch.</t>
+          <t>Strong fit: AI Engineer at Rephrase.ai with 6.8 YOE. Demonstrates deep expertise in Fine-tuning LLMs and FAISS.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>CAND_0044222</t>
+          <t>CAND_0089552</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -889,19 +889,19 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>0.8911</t>
+          <t>0.9660</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Strong fit: AI Engineer at PolicyBazaar with 7.7 YOE. Demonstrates deep expertise in Vector Search and OpenSearch.</t>
+          <t>Strong fit: Machine Learning Engineer at Netflix with 6.0 YOE. Demonstrates deep expertise in Weaviate and Qdrant.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>CAND_0038368</t>
+          <t>CAND_0042029</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -909,19 +909,19 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>0.8898</t>
+          <t>0.9634</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at PhonePe with 5.4 YOE. Demonstrates deep expertise in Embeddings and FAISS.</t>
+          <t>Strong fit: Senior Data Scientist at Flipkart with 6.5 YOE. Demonstrates deep expertise in NLP and Elasticsearch.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>CAND_0009691</t>
+          <t>CAND_0020877</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -929,19 +929,19 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>0.8869</t>
+          <t>0.9620</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Strong fit: Applied ML Engineer at LinkedIn with 6.2 YOE. Demonstrates deep expertise in Fine-tuning LLMs and Pinecone.</t>
+          <t>Strong fit: Applied ML Engineer at CRED with 5.1 YOE. Demonstrates deep expertise in Elasticsearch and OpenSearch.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>CAND_0001494</t>
+          <t>CAND_0037944</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -949,19 +949,19 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>0.8848</t>
+          <t>0.9587</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Strong fit: Data Scientist at Haptik with 6.4 YOE. Demonstrates deep expertise in Vector Search and Weaviate.</t>
+          <t>Strong fit: Senior Data Scientist at Vedantu with 4.9 YOE. Demonstrates deep expertise in Vector Search and OpenSearch.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>CAND_0089552</t>
+          <t>CAND_0032216</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -969,19 +969,19 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>0.8848</t>
+          <t>0.9567</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Strong fit: Machine Learning Engineer at Netflix with 6.0 YOE. Demonstrates deep expertise in Weaviate and Qdrant.</t>
+          <t>Strong fit: ML Engineer at upGrad with 6.1 YOE. Demonstrates deep expertise in Qdrant and Sentence Transformers.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>CAND_0042029</t>
+          <t>CAND_0049538</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -989,19 +989,19 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>0.8812</t>
+          <t>0.9560</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Strong fit: Senior Data Scientist at Flipkart with 6.5 YOE. Demonstrates deep expertise in NLP and Elasticsearch.</t>
+          <t>Strong fit: Applied ML Engineer at Saarthi.ai with 5.8 YOE. Demonstrates deep expertise in OpenSearch and Vector Search.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>CAND_0077337</t>
+          <t>CAND_0055905</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -1009,19 +1009,19 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>0.8812</t>
+          <t>0.9491</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Strong fit: Staff Machine Learning Engineer at Paytm with 7.0 YOE. Demonstrates deep expertise in Pinecone and LLMs.</t>
+          <t>Strong fit: Senior Machine Learning Engineer at Flipkart with 8.1 YOE. Demonstrates deep expertise in Elasticsearch and Python.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>CAND_0020877</t>
+          <t>CAND_0043228</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1029,19 +1029,19 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>0.8798</t>
+          <t>0.9489</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Strong fit: Applied ML Engineer at CRED with 5.1 YOE. Demonstrates deep expertise in Elasticsearch and OpenSearch.</t>
+          <t>Strong fit: Applied ML Engineer at Zoho with 6.8 YOE. Demonstrates deep expertise in NLP and Vector Search.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>CAND_0046525</t>
+          <t>CAND_0044855</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -1049,19 +1049,19 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>0.8797</t>
+          <t>0.9437</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Strong fit: Senior Machine Learning Engineer at Genpact AI with 6.1 YOE. Demonstrates deep expertise in Elasticsearch and LLMs.</t>
+          <t>Strong fit: Senior Data Scientist at Flipkart with 6.6 YOE. Demonstrates deep expertise in OpenSearch and Pinecone.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>CAND_0099806</t>
+          <t>CAND_0079387</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1069,19 +1069,19 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>0.8791</t>
+          <t>0.9420</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Strong fit: AI Engineer at Mad Street Den with 4.6 YOE. Demonstrates deep expertise in FAISS and Embeddings.</t>
+          <t>Strong fit: AI Engineer at Microsoft with 6.9 YOE. Demonstrates deep expertise in Python and Sentence Transformers.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>CAND_0050454</t>
+          <t>CAND_0001707</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -1089,19 +1089,19 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>0.8786</t>
+          <t>0.9404</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Strong fit: AI Engineer at Rephrase.ai with 6.8 YOE. Demonstrates deep expertise in Fine-tuning LLMs and FAISS.</t>
+          <t>Strong fit: Data Scientist at Vedantu with 5.6 YOE. Demonstrates deep expertise in Sentence Transformers and FAISS.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>CAND_0032216</t>
+          <t>CAND_0079064</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -1109,19 +1109,19 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>0.8783</t>
+          <t>0.9395</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at upGrad with 6.1 YOE. Demonstrates deep expertise in Qdrant and Sentence Transformers.</t>
+          <t>Strong fit: Senior Data Scientist at Niramai with 5.2 YOE. Demonstrates deep expertise in OpenSearch and NLP.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>CAND_0005649</t>
+          <t>CAND_0045141</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -1129,19 +1129,19 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>0.8777</t>
+          <t>0.9387</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Strong fit: Senior Data Scientist at Sarvam AI with 7.4 YOE. Demonstrates deep expertise in Fine-tuning LLMs and Weaviate.</t>
+          <t>Strong fit: Data Scientist at HCL with 5.3 YOE. Demonstrates deep expertise in Milvus and Pinecone.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>CAND_0013393</t>
+          <t>CAND_0074342</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -1149,19 +1149,19 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>0.8739</t>
+          <t>0.9344</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at Freshworks with 5.3 YOE. Demonstrates deep expertise in Embeddings and Pinecone.</t>
+          <t>Strong fit: Data Scientist at Zoho with 5.7 YOE. Demonstrates deep expertise in Sentence Transformers and LLMs.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>CAND_0037944</t>
+          <t>CAND_0081852</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -1169,19 +1169,19 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>0.8726</t>
+          <t>0.9315</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Strong fit: Senior Data Scientist at Vedantu with 4.9 YOE. Demonstrates deep expertise in Vector Search and OpenSearch.</t>
+          <t>Strong fit: Senior Data Scientist at Mad Street Den with 5.9 YOE. Demonstrates deep expertise in Milvus and Weaviate.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>CAND_0049538</t>
+          <t>CAND_0051004</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -1189,19 +1189,19 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>0.8661</t>
+          <t>0.9310</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Strong fit: Applied ML Engineer at Saarthi.ai with 5.8 YOE. Demonstrates deep expertise in OpenSearch and Vector Search.</t>
+          <t>Strong fit: Senior Data Scientist at CRED with 4.7 YOE. Demonstrates deep expertise in Embeddings and Qdrant.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>CAND_0044855</t>
+          <t>CAND_0079284</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -1209,19 +1209,19 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>0.8632</t>
+          <t>0.9303</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Strong fit: Senior Data Scientist at Flipkart with 6.6 YOE. Demonstrates deep expertise in OpenSearch and Pinecone.</t>
+          <t>Strong fit: Machine Learning Engineer at Google with 4.9 YOE. Demonstrates deep expertise in Qdrant and Fine-tuning LLMs.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>CAND_0043228</t>
+          <t>CAND_0016163</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -1229,19 +1229,19 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>0.8629</t>
+          <t>0.9294</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Strong fit: Applied ML Engineer at Zoho with 6.8 YOE. Demonstrates deep expertise in NLP and Vector Search.</t>
+          <t>Strong fit: Applied ML Engineer at Dream11 with 6.7 YOE. Demonstrates deep expertise in Weaviate and Embeddings.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>CAND_0005477</t>
+          <t>CAND_0010257</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -1249,19 +1249,19 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>0.8600</t>
+          <t>0.9286</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at Zomato with 6.2 YOE. Demonstrates deep expertise in OpenSearch.</t>
+          <t>Strong fit: Senior Data Scientist at Google with 6.5 YOE. Demonstrates deep expertise in Milvus and Python.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>CAND_0045141</t>
+          <t>CAND_0090584</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -1269,19 +1269,19 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>0.8596</t>
+          <t>0.9211</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Strong fit: Data Scientist at HCL with 5.3 YOE. Demonstrates deep expertise in Milvus and Pinecone.</t>
+          <t>Strong fit: ML Engineer at Flipkart with 5.1 YOE. Demonstrates deep expertise in Fine-tuning LLMs and OpenSearch.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>CAND_0079284</t>
+          <t>CAND_0075574</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -1289,19 +1289,19 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>0.8596</t>
+          <t>0.9172</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Strong fit: Machine Learning Engineer at Google with 4.9 YOE. Demonstrates deep expertise in Qdrant and Fine-tuning LLMs.</t>
+          <t>Strong fit: Machine Learning Engineer at Haptik with 5.7 YOE. Demonstrates deep expertise in Weaviate and OpenSearch.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>CAND_0015528</t>
+          <t>CAND_0068811</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -1309,19 +1309,19 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>0.8569</t>
+          <t>0.9165</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Strong fit: Applied ML Engineer at Krutrim with 7.4 YOE. Demonstrates deep expertise in Weaviate and OpenSearch.</t>
+          <t>Strong fit: Applied ML Engineer at Freshworks with 8.0 YOE. Demonstrates deep expertise in Vector Search and Qdrant.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>CAND_0079387</t>
+          <t>CAND_0036121</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -1329,19 +1329,19 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>0.8548</t>
+          <t>0.9132</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Strong fit: AI Engineer at Microsoft with 6.9 YOE. Demonstrates deep expertise in Python and Sentence Transformers.</t>
+          <t>Strong fit: ML Engineer at Wysa with 5.2 YOE. Demonstrates deep expertise in Embeddings and Vector Search.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>CAND_0079064</t>
+          <t>CAND_0070398</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -1349,19 +1349,19 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>0.8525</t>
+          <t>0.9063</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Strong fit: Senior Data Scientist at Niramai with 5.2 YOE. Demonstrates deep expertise in OpenSearch and NLP.</t>
+          <t>Strong fit: Machine Learning Engineer at Genpact AI with 7.2 YOE. Demonstrates deep expertise in FAISS and Embeddings.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>CAND_0090584</t>
+          <t>CAND_0093193</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -1369,19 +1369,19 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>0.8506</t>
+          <t>0.9062</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at Flipkart with 5.1 YOE. Demonstrates deep expertise in Fine-tuning LLMs and OpenSearch.</t>
+          <t>Strong fit: Senior Machine Learning Engineer at Niramai with 7.9 YOE. Demonstrates deep expertise in Qdrant and OpenSearch.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>CAND_0003841</t>
+          <t>CAND_0091909</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -1389,19 +1389,19 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>0.8479</t>
+          <t>0.9056</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at Tech Mahindra with 5.0 YOE. Demonstrates deep expertise in Pinecone and Fine-tuning LLMs.</t>
+          <t>Strong fit: Machine Learning Engineer at Rephrase.ai with 6.9 YOE. Demonstrates deep expertise in LLMs and Pinecone.</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>CAND_0005509</t>
+          <t>CAND_0098217</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -1409,19 +1409,19 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>0.8457</t>
+          <t>0.9052</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Strong fit: Data Scientist at Ola with 6.0 YOE. Demonstrates deep expertise in Python and Fine-tuning LLMs.</t>
+          <t>Strong fit: ML Engineer at Glance with 6.4 YOE. Demonstrates deep expertise in FAISS and Pinecone.</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>CAND_0002037</t>
+          <t>CAND_0099269</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -1429,19 +1429,19 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>0.8416</t>
+          <t>0.9034</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at Locobuzz with 5.5 YOE. Demonstrates deep expertise in Fine-tuning LLMs and Milvus.</t>
+          <t>Strong fit: Data Scientist at BYJU'S with 5.5 YOE. Demonstrates deep expertise in Elasticsearch and Python.</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>CAND_0051004</t>
+          <t>CAND_0040178</t>
         </is>
       </c>
       <c r="B52" t="n">
@@ -1449,19 +1449,19 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>0.8409</t>
+          <t>0.9013</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Strong fit: Senior Data Scientist at CRED with 4.7 YOE. Demonstrates deep expertise in Embeddings and Qdrant.</t>
+          <t>Strong fit: ML Engineer at Meesho with 5.0 YOE. Demonstrates deep expertise in Weaviate and Fine-tuning LLMs.</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>CAND_0081852</t>
+          <t>CAND_0011263</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -1469,19 +1469,19 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>0.8396</t>
+          <t>0.8998</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Strong fit: Senior Data Scientist at Mad Street Den with 5.9 YOE. Demonstrates deep expertise in Milvus and Weaviate.</t>
+          <t>Strong fit: ML Engineer at Ola with 5.1 YOE. Demonstrates deep expertise in Pinecone and OpenSearch.</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>CAND_0055905</t>
+          <t>CAND_0030031</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -1489,19 +1489,19 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>0.8393</t>
+          <t>0.8993</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Strong fit: Senior Machine Learning Engineer at Flipkart with 8.1 YOE. Demonstrates deep expertise in Elasticsearch and Python.</t>
+          <t>Strong fit: AI Engineer at Microsoft with 5.7 YOE. Demonstrates deep expertise in Python and NLP.</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>CAND_0074342</t>
+          <t>CAND_0047721</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -1509,19 +1509,19 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>0.8380</t>
+          <t>0.8985</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Strong fit: Data Scientist at Zoho with 5.7 YOE. Demonstrates deep expertise in Sentence Transformers and LLMs.</t>
+          <t>Strong fit: Senior Data Scientist at Microsoft with 7.0 YOE. Demonstrates deep expertise in Milvus and FAISS.</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>CAND_0007460</t>
+          <t>CAND_0048166</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -1529,19 +1529,19 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>0.8374</t>
+          <t>0.8985</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Strong fit: AI Engineer at Salesforce with 4.7 YOE. Demonstrates deep expertise in Embeddings and Weaviate.</t>
+          <t>Strong fit: ML Engineer at Aganitha with 5.2 YOE. Demonstrates deep expertise in Pinecone and Milvus.</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>CAND_0091909</t>
+          <t>CAND_0017093</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -1549,19 +1549,19 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>0.8364</t>
+          <t>0.8984</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Strong fit: Machine Learning Engineer at Rephrase.ai with 6.9 YOE. Demonstrates deep expertise in LLMs and Pinecone.</t>
+          <t>Strong fit: ML Engineer at Zoho with 5.9 YOE. Demonstrates deep expertise in LLMs and Embeddings.</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>CAND_0075574</t>
+          <t>CAND_0048558</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -1569,19 +1569,19 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>0.8357</t>
+          <t>0.8984</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Strong fit: Machine Learning Engineer at Haptik with 5.7 YOE. Demonstrates deep expertise in Weaviate and OpenSearch.</t>
+          <t>Strong fit: Data Scientist at Rephrase.ai with 6.7 YOE. Demonstrates deep expertise in OpenSearch and Qdrant.</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>CAND_0068811</t>
+          <t>CAND_0005538</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -1589,19 +1589,19 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>0.8345</t>
+          <t>0.8961</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Strong fit: Applied ML Engineer at Freshworks with 8.0 YOE. Demonstrates deep expertise in Vector Search and Qdrant.</t>
+          <t>Strong fit: Senior AI Engineer at Adobe with 5.9 YOE. Demonstrates deep expertise in Python.</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>CAND_0010149</t>
+          <t>CAND_0011432</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -1609,19 +1609,19 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>0.8333</t>
+          <t>0.8951</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at Glance with 6.9 YOE. Demonstrates deep expertise in Milvus and Vector Search.</t>
+          <t>Strong fit: Senior Data Scientist at Amazon with 7.6 YOE. Demonstrates deep expertise in OpenSearch and Elasticsearch.</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>CAND_0006557</t>
+          <t>CAND_0050876</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -1629,19 +1629,19 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>0.8290</t>
+          <t>0.8892</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Strong fit: NLP Engineer at Paytm with 7.9 YOE. Demonstrates deep expertise in Elasticsearch and OpenSearch.</t>
+          <t>Strong fit: Applied ML Engineer at Freshworks with 6.0 YOE. Demonstrates deep expertise in Qdrant and FAISS.</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>CAND_0010541</t>
+          <t>CAND_0028287</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -1649,19 +1649,19 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>0.8285</t>
+          <t>0.8880</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Strong fit: AI Research Engineer at Wysa with 6.2 YOE. Demonstrates deep expertise in Pinecone and Weaviate.</t>
+          <t>Strong fit: Data Scientist at Unacademy with 5.7 YOE. Demonstrates deep expertise in OpenSearch and Vector Search.</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>CAND_0017093</t>
+          <t>CAND_0009691</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -1669,19 +1669,19 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>0.8271</t>
+          <t>0.8869</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at Zoho with 5.9 YOE. Demonstrates deep expertise in LLMs and Embeddings.</t>
+          <t>Strong fit: Applied ML Engineer at LinkedIn with 6.2 YOE. Demonstrates deep expertise in Fine-tuning LLMs and Pinecone.</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>CAND_0070398</t>
+          <t>CAND_0055992</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -1689,19 +1689,19 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>0.8271</t>
+          <t>0.8861</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Strong fit: Machine Learning Engineer at Genpact AI with 7.2 YOE. Demonstrates deep expertise in FAISS and Embeddings.</t>
+          <t>Strong fit: AI Engineer at CRED with 16.9 YOE. Demonstrates deep expertise in FAISS and OpenSearch.</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>CAND_0098217</t>
+          <t>CAND_0001494</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -1709,19 +1709,19 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>0.8271</t>
+          <t>0.8848</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at Glance with 6.4 YOE. Demonstrates deep expertise in FAISS and Pinecone.</t>
+          <t>Strong fit: Data Scientist at Haptik with 6.4 YOE. Demonstrates deep expertise in Vector Search and Weaviate.</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>CAND_0047721</t>
+          <t>CAND_0035653</t>
         </is>
       </c>
       <c r="B66" t="n">
@@ -1729,19 +1729,19 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>0.8264</t>
+          <t>0.8825</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Strong fit: Senior Data Scientist at Microsoft with 7.0 YOE. Demonstrates deep expertise in Milvus and FAISS.</t>
+          <t>Strong fit: Data Scientist at Swiggy with 5.6 YOE. Demonstrates deep expertise in OpenSearch and Vector Search.</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>CAND_0099269</t>
+          <t>CAND_0086022</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -1749,19 +1749,19 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>0.8248</t>
+          <t>0.8819</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Strong fit: Data Scientist at BYJU'S with 5.5 YOE. Demonstrates deep expertise in Elasticsearch and Python.</t>
+          <t>Strong fit: Senior Applied Scientist at Sarvam AI with 5.3 YOE. Demonstrates deep expertise in Vector Search and Fine-tuning LLMs.</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>CAND_0006418</t>
+          <t>CAND_0021836</t>
         </is>
       </c>
       <c r="B68" t="n">
@@ -1769,19 +1769,19 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>0.8236</t>
+          <t>0.8808</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Strong fit: Machine Learning Engineer at Verloop.io with 5.7 YOE. Demonstrates deep expertise in Embeddings and Weaviate.</t>
+          <t>Strong fit: ML Engineer at CRED with 6.5 YOE. Demonstrates deep expertise in Vector Search and Elasticsearch.</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>CAND_0015057</t>
+          <t>CAND_0076482</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -1789,19 +1789,19 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>0.8214</t>
+          <t>0.8798</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at Meesho with 4.6 YOE. Demonstrates deep expertise in Sentence Transformers and Vector Search.</t>
+          <t>Strong fit: ML Engineer at Flipkart with 6.6 YOE. Demonstrates deep expertise in OpenSearch and Pinecone.</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>CAND_0036121</t>
+          <t>CAND_0027723</t>
         </is>
       </c>
       <c r="B70" t="n">
@@ -1809,19 +1809,19 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>0.8174</t>
+          <t>0.8783</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at Wysa with 5.2 YOE. Demonstrates deep expertise in Embeddings and Vector Search.</t>
+          <t>Strong fit: ML Engineer at Wysa with 4.2 YOE. Demonstrates deep expertise in Vector Search and NLP.</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>CAND_0015578</t>
+          <t>CAND_0005649</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -1829,19 +1829,19 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>0.8141</t>
+          <t>0.8777</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Strong fit: AI Engineer at Zoho with 5.4 YOE. Demonstrates deep expertise in Embeddings and NLP.</t>
+          <t>Strong fit: Senior Data Scientist at Sarvam AI with 7.4 YOE. Demonstrates deep expertise in Fine-tuning LLMs and Weaviate.</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>CAND_0030031</t>
+          <t>CAND_0083879</t>
         </is>
       </c>
       <c r="B72" t="n">
@@ -1849,19 +1849,19 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>0.8126</t>
+          <t>0.8746</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Strong fit: AI Engineer at Microsoft with 5.7 YOE. Demonstrates deep expertise in Python and NLP.</t>
+          <t>Strong fit: Machine Learning Engineer at Ola with 7.1 YOE. Demonstrates deep expertise in Fine-tuning LLMs and Milvus.</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>CAND_0021836</t>
+          <t>CAND_0013393</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -1869,19 +1869,19 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>0.8117</t>
+          <t>0.8739</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at CRED with 6.5 YOE. Demonstrates deep expertise in Vector Search and Elasticsearch.</t>
+          <t>Strong fit: ML Engineer at Freshworks with 5.3 YOE. Demonstrates deep expertise in Embeddings and Pinecone.</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>CAND_0035653</t>
+          <t>CAND_0090155</t>
         </is>
       </c>
       <c r="B74" t="n">
@@ -1889,19 +1889,19 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>0.8114</t>
+          <t>0.8683</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Strong fit: Data Scientist at Swiggy with 5.6 YOE. Demonstrates deep expertise in OpenSearch and Vector Search.</t>
+          <t>Strong fit: ML Engineer at Swiggy with 5.8 YOE. Demonstrates deep expertise in Milvus and Qdrant.</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>CAND_0040178</t>
+          <t>CAND_0073982</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -1909,19 +1909,19 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>0.8106</t>
+          <t>0.8672</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at Meesho with 5.0 YOE. Demonstrates deep expertise in Weaviate and Fine-tuning LLMs.</t>
+          <t>Strong fit: Data Scientist at Dream11 with 7.0 YOE. Demonstrates deep expertise in Sentence Transformers and Qdrant.</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>CAND_0000273</t>
+          <t>CAND_0061257</t>
         </is>
       </c>
       <c r="B76" t="n">
@@ -1929,19 +1929,19 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>0.8105</t>
+          <t>0.8670</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at BYJU'S with 5.8 YOE. Demonstrates deep expertise in Fine-tuning LLMs and Qdrant.</t>
+          <t>Strong fit: Staff Machine Learning Engineer at LinkedIn with 8.0 YOE. Demonstrates deep expertise in Python.</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>CAND_0050876</t>
+          <t>CAND_0092255</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -1949,19 +1949,19 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>0.8098</t>
+          <t>0.8644</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Strong fit: Applied ML Engineer at Freshworks with 6.0 YOE. Demonstrates deep expertise in Qdrant and FAISS.</t>
+          <t>Strong fit: ML Engineer at InMobi with 5.2 YOE. Demonstrates deep expertise in Weaviate and OpenSearch.</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>CAND_0076482</t>
+          <t>CAND_0060538</t>
         </is>
       </c>
       <c r="B78" t="n">
@@ -1969,19 +1969,19 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>0.8089</t>
+          <t>0.8642</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at Flipkart with 6.6 YOE. Demonstrates deep expertise in OpenSearch and Pinecone.</t>
+          <t>Strong fit: ML Engineer at Verloop.io with 5.2 YOE. Demonstrates deep expertise in OpenSearch and Embeddings.</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>CAND_0048558</t>
+          <t>CAND_0095213</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -1989,19 +1989,19 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>0.8084</t>
+          <t>0.8636</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Strong fit: Data Scientist at Rephrase.ai with 6.7 YOE. Demonstrates deep expertise in OpenSearch and Qdrant.</t>
+          <t>Strong fit: ML Engineer at Genpact AI with 5.1 YOE. Demonstrates deep expertise in Python and Weaviate.</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>CAND_0093193</t>
+          <t>CAND_0042100</t>
         </is>
       </c>
       <c r="B80" t="n">
@@ -2009,19 +2009,19 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>0.8068</t>
+          <t>0.8634</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Strong fit: Senior Machine Learning Engineer at Niramai with 7.9 YOE. Demonstrates deep expertise in Qdrant and OpenSearch.</t>
+          <t>Strong fit: Machine Learning Engineer at Freshworks with 7.3 YOE. Demonstrates deep expertise in Elasticsearch and Fine-tuning LLMs.</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>CAND_0005311</t>
+          <t>CAND_0060054</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -2029,19 +2029,19 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>0.8066</t>
+          <t>0.8608</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Strong fit: AI Research Engineer at Aganitha with 5.7 YOE. Demonstrates deep expertise in Qdrant and Fine-tuning LLMs.</t>
+          <t>Strong fit: AI Engineer at Mad Street Den with 6.4 YOE. Demonstrates deep expertise in Weaviate and FAISS.</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>CAND_0048166</t>
+          <t>CAND_0005477</t>
         </is>
       </c>
       <c r="B82" t="n">
@@ -2049,19 +2049,19 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>0.7998</t>
+          <t>0.8600</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at Aganitha with 5.2 YOE. Demonstrates deep expertise in Pinecone and Milvus.</t>
+          <t>Strong fit: ML Engineer at Zomato with 6.2 YOE. Demonstrates deep expertise in OpenSearch.</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>CAND_0015582</t>
+          <t>CAND_0027691</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -2069,19 +2069,19 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>0.7997</t>
+          <t>0.8588</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at Genpact AI with 4.4 YOE. Demonstrates deep expertise in Qdrant and Sentence Transformers.</t>
+          <t>Strong fit: NLP Engineer at Haptik with 6.5 YOE. Demonstrates deep expertise in Weaviate and Embeddings.</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>CAND_0028287</t>
+          <t>CAND_0015528</t>
         </is>
       </c>
       <c r="B84" t="n">
@@ -2089,19 +2089,19 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>0.7994</t>
+          <t>0.8569</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Strong fit: Data Scientist at Unacademy with 5.7 YOE. Demonstrates deep expertise in OpenSearch and Vector Search.</t>
+          <t>Strong fit: Applied ML Engineer at Krutrim with 7.4 YOE. Demonstrates deep expertise in Weaviate and OpenSearch.</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>CAND_0073982</t>
+          <t>CAND_0030348</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -2109,19 +2109,19 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>0.7993</t>
+          <t>0.8555</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Strong fit: Data Scientist at Dream11 with 7.0 YOE. Demonstrates deep expertise in Sentence Transformers and Qdrant.</t>
+          <t>Strong fit: Machine Learning Engineer at BYJU'S with 4.5 YOE. Demonstrates deep expertise in Embeddings and Vector Search.</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>CAND_0095213</t>
+          <t>CAND_0025335</t>
         </is>
       </c>
       <c r="B86" t="n">
@@ -2129,19 +2129,19 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>0.7966</t>
+          <t>0.8509</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at Genpact AI with 5.1 YOE. Demonstrates deep expertise in Python and Weaviate.</t>
+          <t>Strong fit: Data Scientist at PolicyBazaar with 6.6 YOE. Demonstrates deep expertise in NLP.</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>CAND_0003791</t>
+          <t>CAND_0003841</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -2149,19 +2149,19 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>0.7927</t>
+          <t>0.8479</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at Meesho with 6.6 YOE. Demonstrates deep expertise in LLMs and Python.</t>
+          <t>Strong fit: ML Engineer at Tech Mahindra with 5.0 YOE. Demonstrates deep expertise in Pinecone and Fine-tuning LLMs.</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>CAND_0055992</t>
+          <t>CAND_0094759</t>
         </is>
       </c>
       <c r="B88" t="n">
@@ -2169,19 +2169,19 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>0.7897</t>
+          <t>0.8468</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Strong fit: AI Engineer at CRED with 16.9 YOE. Demonstrates deep expertise in FAISS and OpenSearch.</t>
+          <t>Strong fit: Lead AI Engineer at Meta with 8.6 YOE. Demonstrates deep expertise in Qdrant and Fine-tuning LLMs.</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>CAND_0027723</t>
+          <t>CAND_0005509</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -2189,19 +2189,19 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>0.7889</t>
+          <t>0.8457</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at Wysa with 4.2 YOE. Demonstrates deep expertise in Vector Search and NLP.</t>
+          <t>Strong fit: Data Scientist at Ola with 6.0 YOE. Demonstrates deep expertise in Python and Fine-tuning LLMs.</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>CAND_0015493</t>
+          <t>CAND_0002037</t>
         </is>
       </c>
       <c r="B90" t="n">
@@ -2209,19 +2209,19 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>0.7886</t>
+          <t>0.8416</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Strong fit: Data Scientist at CRED with 6.4 YOE. Demonstrates deep expertise in NLP.</t>
+          <t>Strong fit: ML Engineer at Locobuzz with 5.5 YOE. Demonstrates deep expertise in Fine-tuning LLMs and Milvus.</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>CAND_0090155</t>
+          <t>CAND_0018094</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -2229,19 +2229,19 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>0.7881</t>
+          <t>0.8414</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at Swiggy with 5.8 YOE. Demonstrates deep expertise in Milvus and Qdrant.</t>
+          <t>Strong fit: ML Engineer at Mad Street Den with 5.2 YOE. Demonstrates deep expertise in Pinecone and Fine-tuning LLMs.</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>CAND_0060538</t>
+          <t>CAND_0071432</t>
         </is>
       </c>
       <c r="B92" t="n">
@@ -2249,19 +2249,19 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>0.7867</t>
+          <t>0.8398</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Borderline Match: Strong fit: ML Engineer at Verloop.io with 5.2 YOE. Demonstrates deep expertise in OpenSearch and Embeddings. Meets minimum bar but lacks standout secondary signals.</t>
+          <t>Borderline Match: Strong fit: Data Scientist at Wysa with 4.1 YOE. Demonstrates deep expertise in Weaviate and Pinecone. Meets minimum bar but lacks standout secondary signals.</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>CAND_0042100</t>
+          <t>CAND_0072721</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -2269,19 +2269,19 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>0.7838</t>
+          <t>0.8385</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Borderline Match: Strong fit: Machine Learning Engineer at Freshworks with 7.3 YOE. Demonstrates deep expertise in Elasticsearch and Fine-tuning LLMs. Meets minimum bar but lacks standout secondary signals.</t>
+          <t>Borderline Match: Strong fit: Data Scientist at Yellow.ai with 3.7 YOE. Demonstrates deep expertise in Weaviate and Qdrant. Meets minimum bar but lacks standout secondary signals.</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>CAND_0083879</t>
+          <t>CAND_0064904</t>
         </is>
       </c>
       <c r="B94" t="n">
@@ -2289,19 +2289,19 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>0.7816</t>
+          <t>0.8380</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Borderline Match: Strong fit: Machine Learning Engineer at Ola with 7.1 YOE. Demonstrates deep expertise in Fine-tuning LLMs and Milvus. Meets minimum bar but lacks standout secondary signals.</t>
+          <t>Borderline Match: Strong fit: AI Engineer at LinkedIn with 4.9 YOE. Demonstrates deep expertise in Embeddings and Elasticsearch. Meets minimum bar but lacks standout secondary signals.</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>CAND_0092255</t>
+          <t>CAND_0007460</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -2309,19 +2309,19 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>0.7802</t>
+          <t>0.8374</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Borderline Match: Strong fit: ML Engineer at InMobi with 5.2 YOE. Demonstrates deep expertise in Weaviate and OpenSearch. Meets minimum bar but lacks standout secondary signals.</t>
+          <t>Borderline Match: Strong fit: AI Engineer at Salesforce with 4.7 YOE. Demonstrates deep expertise in Embeddings and Weaviate. Meets minimum bar but lacks standout secondary signals.</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>CAND_0012837</t>
+          <t>CAND_0061550</t>
         </is>
       </c>
       <c r="B96" t="n">
@@ -2329,19 +2329,19 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>0.7789</t>
+          <t>0.8366</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Borderline Match: Strong fit: Junior ML Engineer at Sarvam AI with 6.4 YOE. Demonstrates deep expertise in Vector Search and Weaviate. Meets minimum bar but lacks standout secondary signals.</t>
+          <t>Borderline Match: Strong fit: ML Engineer at Infosys with 5.3 YOE. Demonstrates deep expertise in Sentence Transformers. Meets minimum bar but lacks standout secondary signals.</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>CAND_0007412</t>
+          <t>CAND_0058688</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -2349,19 +2349,19 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>0.7786</t>
+          <t>0.8341</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Borderline Match: Strong fit: Applied ML Engineer at Zoho with 7.4 YOE. Demonstrates deep expertise in Pinecone and Milvus. Meets minimum bar but lacks standout secondary signals.</t>
+          <t>Borderline Match: Strong fit: AI Engineer at Vedantu with 6.7 YOE. Demonstrates deep expertise in Embeddings and Milvus. Meets minimum bar but lacks standout secondary signals.</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>CAND_0009837</t>
+          <t>CAND_0010149</t>
         </is>
       </c>
       <c r="B98" t="n">
@@ -2369,19 +2369,19 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>0.7777</t>
+          <t>0.8333</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Borderline Match: Strong fit: Senior Data Scientist at Rephrase.ai with 4.3 YOE. Demonstrates deep expertise in Python and FAISS. Meets minimum bar but lacks standout secondary signals.</t>
+          <t>Borderline Match: Strong fit: ML Engineer at Glance with 6.9 YOE. Demonstrates deep expertise in Milvus and Vector Search. Meets minimum bar but lacks standout secondary signals.</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>CAND_0060054</t>
+          <t>CAND_0017178</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -2389,19 +2389,19 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>0.7776</t>
+          <t>0.8292</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Borderline Match: Strong fit: AI Engineer at Mad Street Den with 6.4 YOE. Demonstrates deep expertise in Weaviate and FAISS. Meets minimum bar but lacks standout secondary signals.</t>
+          <t>Borderline Match: Strong fit: ML Engineer at Swiggy with 4.2 YOE. Demonstrates deep expertise in PEFT and pgvector. Meets minimum bar but lacks standout secondary signals.</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>CAND_0013536</t>
+          <t>CAND_0006557</t>
         </is>
       </c>
       <c r="B100" t="n">
@@ -2409,19 +2409,19 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>0.7769</t>
+          <t>0.8290</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Borderline Match: Strong fit: Applied ML Engineer at Haptik with 14.1 YOE. Demonstrates deep expertise in LLMs and NLP. Meets minimum bar but lacks standout secondary signals.</t>
+          <t>Borderline Match: Strong fit: NLP Engineer at Paytm with 7.9 YOE. Demonstrates deep expertise in Elasticsearch and OpenSearch. Meets minimum bar but lacks standout secondary signals.</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>CAND_0025335</t>
+          <t>CAND_0066690</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -2429,12 +2429,12 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>0.7749</t>
+          <t>0.8287</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Borderline Match: Strong fit: Data Scientist at PolicyBazaar with 6.6 YOE. Demonstrates deep expertise in NLP. Meets minimum bar but lacks standout secondary signals.</t>
+          <t>Borderline Match: Strong fit: ML Engineer at Freshworks with 4.8 YOE. Demonstrates deep expertise in Sentence Transformers and Elasticsearch. Meets minimum bar but lacks standout secondary signals.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(phase2): eval harness, generalization demo, and devops JD fixture
</commit_message>
<xml_diff>
--- a/submission.xlsx
+++ b/submission.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Ranking Results" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ranking Results" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -441,7 +441,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>CAND_0071974</t>
+          <t>CAND_0006567</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -449,19 +449,19 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>1.1102</t>
+          <t>1.0130</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Exceptional Top 5 Match: Strong fit: Senior AI Engineer at Netflix with 7.8 YOE. Demonstrates deep expertise in Weaviate and Pinecone. Highly recommended for immediate interview.</t>
+          <t>Rank 1: Senior AI Engineer at Meta (7.9 YOE); JD-aligned skills: NLP, Python. Top-tier composite score across career, skills, and availability.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>CAND_0002025</t>
+          <t>CAND_0045250</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -469,19 +469,19 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>1.0867</t>
+          <t>0.9990</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Exceptional Top 5 Match: Strong fit: Senior AI Engineer at Apple with 5.9 YOE. Demonstrates deep expertise in FAISS and OpenSearch. Highly recommended for immediate interview.</t>
+          <t>Rank 2: Applied ML Engineer at Rephrase.ai (6.6 YOE); JD-aligned skills: Sentence Transformers, Milvus, Embeddings. Top-tier composite score across career, skills, and availability.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>CAND_0045250</t>
+          <t>CAND_0071974</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -489,19 +489,19 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>1.0832</t>
+          <t>0.9986</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Exceptional Top 5 Match: Strong fit: Applied ML Engineer at Rephrase.ai with 6.6 YOE. Demonstrates deep expertise in Sentence Transformers and Milvus. Highly recommended for immediate interview.</t>
+          <t>Rank 3: Senior AI Engineer at Netflix (7.8 YOE); JD-aligned skills: Weaviate, Pinecone, Qdrant. Top-tier composite score across career, skills, and availability.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>CAND_0018499</t>
+          <t>CAND_0002025</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -509,12 +509,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>1.0683</t>
+          <t>0.9783</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Exceptional Top 5 Match: Strong fit: Senior Machine Learning Engineer at Zomato with 7.2 YOE. Demonstrates deep expertise in Weaviate and Pinecone. Highly recommended for immediate interview.</t>
+          <t>Rank 4: Senior AI Engineer at Apple (5.9 YOE); JD-aligned skills: FAISS, OpenSearch, Weaviate. Top-tier composite score across career, skills, and availability.</t>
         </is>
       </c>
     </row>
@@ -529,19 +529,19 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>1.0519</t>
+          <t>0.9669</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Exceptional Top 5 Match: Strong fit: Applied ML Engineer at upGrad with 5.0 YOE. Demonstrates deep expertise in Weaviate and Pinecone. Highly recommended for immediate interview.</t>
+          <t>Rank 5: Applied ML Engineer at upGrad (5.0 YOE); JD-aligned skills: Weaviate, Pinecone, Python. Top-tier composite score across career, skills, and availability. Minor note: 120-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>CAND_0087630</t>
+          <t>CAND_0018499</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -549,19 +549,19 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>1.0478</t>
+          <t>0.9612</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Strong fit: AI Engineer at Vedantu with 7.2 YOE. Demonstrates deep expertise in Elasticsearch and NLP.</t>
+          <t>Strong match — Senior Machine Learning Engineer at Zomato (7.2 YOE); JD-aligned skills: Weaviate, Pinecone, Milvus.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>CAND_0020350</t>
+          <t>CAND_0087630</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -569,19 +569,19 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>1.0460</t>
+          <t>0.9566</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Strong fit: AI Engineer at Zoho with 5.8 YOE. Demonstrates deep expertise in NLP and LLMs.</t>
+          <t>Strong match — AI Engineer at Vedantu (7.2 YOE); JD-aligned skills: Elasticsearch, NLP, Embeddings.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>CAND_0006567</t>
+          <t>CAND_0020350</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -589,12 +589,12 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>1.0371</t>
+          <t>0.9531</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Strong fit: Senior AI Engineer at Meta with 7.9 YOE. Demonstrates deep expertise in NLP and Python.</t>
+          <t>Strong match — AI Engineer at Zoho (5.8 YOE); JD-aligned skills: NLP, LLMs, FAISS.</t>
         </is>
       </c>
     </row>
@@ -609,19 +609,19 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>1.0350</t>
+          <t>0.9359</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Strong fit: Lead AI Engineer at Sarvam AI with 6.4 YOE. Demonstrates deep expertise in Qdrant and Elasticsearch.</t>
+          <t>Strong match — Lead AI Engineer at Sarvam AI (6.4 YOE); JD-aligned skills: Qdrant, Elasticsearch, Python.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>CAND_0080766</t>
+          <t>CAND_0065514</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -629,19 +629,19 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>1.0279</t>
+          <t>0.9268</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Strong fit: Staff Machine Learning Engineer at Salesforce with 8.8 YOE. Demonstrates deep expertise in Elasticsearch and OpenSearch.</t>
+          <t>Strong match — ML Engineer at Genpact AI (6.6 YOE); JD-aligned skills: Vector Search, Pinecone, Elasticsearch. Watch: 90-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>CAND_0081846</t>
+          <t>CAND_0080766</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -649,12 +649,12 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>1.0211</t>
+          <t>0.9200</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Strong fit: Lead AI Engineer at Razorpay with 6.7 YOE. Demonstrates deep expertise in Elasticsearch and Vector Search.</t>
+          <t>Strong match — Staff Machine Learning Engineer at Salesforce (8.8 YOE); JD-aligned skills: Elasticsearch, OpenSearch, Python.</t>
         </is>
       </c>
     </row>
@@ -669,19 +669,19 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>1.0210</t>
+          <t>0.9166</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Strong fit: Staff Machine Learning Engineer at Yellow.ai with 8.6 YOE. Demonstrates deep expertise in Pinecone and LLMs.</t>
+          <t>Strong match — Staff Machine Learning Engineer at Yellow.ai (8.6 YOE); JD-aligned skills: Pinecone, LLMs, Elasticsearch. Watch: 90-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>CAND_0071939</t>
+          <t>CAND_0039383</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -689,12 +689,12 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>1.0122</t>
+          <t>0.9138</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Strong fit: Data Scientist at Krutrim with 6.4 YOE. Demonstrates deep expertise in Elasticsearch and OpenSearch.</t>
+          <t>Strong match — Applied ML Engineer at Meesho (7.1 YOE); JD-aligned skills: FAISS, NLP, Vector Search. Watch: 90-day notice period.</t>
         </is>
       </c>
     </row>
@@ -709,19 +709,19 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>1.0006</t>
+          <t>0.9108</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Strong fit: Machine Learning Engineer at LinkedIn with 6.9 YOE. Demonstrates deep expertise in Pinecone and NLP.</t>
+          <t>Strong match — Machine Learning Engineer at LinkedIn (6.9 YOE); JD-aligned skills: Pinecone, NLP, LLMs.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>CAND_0065514</t>
+          <t>CAND_0081846</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -729,19 +729,19 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>0.9997</t>
+          <t>0.9092</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at Genpact AI with 6.6 YOE. Demonstrates deep expertise in Vector Search and Pinecone.</t>
+          <t>Strong match — Lead AI Engineer at Razorpay (6.7 YOE); JD-aligned skills: Elasticsearch, Vector Search, Python.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>CAND_0039383</t>
+          <t>CAND_0068811</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -749,19 +749,19 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>0.9892</t>
+          <t>0.9073</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Strong fit: Applied ML Engineer at Meesho with 7.1 YOE. Demonstrates deep expertise in FAISS and NLP.</t>
+          <t>Strong match — Applied ML Engineer at Freshworks (8.0 YOE); JD-aligned skills: Vector Search, Qdrant, Embeddings.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>CAND_0046525</t>
+          <t>CAND_0044222</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -769,12 +769,12 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>0.9845</t>
+          <t>0.8911</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Strong fit: Senior Machine Learning Engineer at Genpact AI with 6.1 YOE. Demonstrates deep expertise in Elasticsearch and LLMs.</t>
+          <t>Strong match — AI Engineer at PolicyBazaar (7.7 YOE); JD-aligned skills: Vector Search, OpenSearch, Qdrant.</t>
         </is>
       </c>
     </row>
@@ -789,19 +789,19 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>0.9810</t>
+          <t>0.8898</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at PhonePe with 5.4 YOE. Demonstrates deep expertise in Embeddings and FAISS.</t>
+          <t>Strong match — ML Engineer at PhonePe (5.4 YOE); JD-aligned skills: Embeddings, FAISS, NLP.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>CAND_0077337</t>
+          <t>CAND_0030031</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -809,19 +809,19 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>0.9778</t>
+          <t>0.8890</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Strong fit: Staff Machine Learning Engineer at Paytm with 7.0 YOE. Demonstrates deep expertise in Pinecone and LLMs.</t>
+          <t>Strong match — AI Engineer at Microsoft (5.7 YOE); JD-aligned skills: Python, NLP, Sentence Transformers.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>CAND_0044222</t>
+          <t>CAND_0089552</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -829,19 +829,19 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>0.9752</t>
+          <t>0.8848</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Strong fit: AI Engineer at PolicyBazaar with 7.7 YOE. Demonstrates deep expertise in Vector Search and OpenSearch.</t>
+          <t>Strong match — Machine Learning Engineer at Netflix (6.0 YOE); JD-aligned skills: Weaviate, Qdrant, Vector Search. Watch: 120-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>CAND_0099806</t>
+          <t>CAND_0042029</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -849,19 +849,19 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>0.9678</t>
+          <t>0.8812</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Strong fit: AI Engineer at Mad Street Den with 4.6 YOE. Demonstrates deep expertise in FAISS and Embeddings.</t>
+          <t>Solid profile: Senior Data Scientist at Flipkart (6.5 YOE); JD-aligned skills: NLP, Elasticsearch, Embeddings.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>CAND_0050454</t>
+          <t>CAND_0077337</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -869,19 +869,19 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>0.9666</t>
+          <t>0.8812</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Strong fit: AI Engineer at Rephrase.ai with 6.8 YOE. Demonstrates deep expertise in Fine-tuning LLMs and FAISS.</t>
+          <t>Good fit with caveats: Staff Machine Learning Engineer at Paytm (7.0 YOE); JD-aligned skills: Pinecone, LLMs, Qdrant.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>CAND_0089552</t>
+          <t>CAND_0020877</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -889,19 +889,19 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>0.9660</t>
+          <t>0.8798</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Strong fit: Machine Learning Engineer at Netflix with 6.0 YOE. Demonstrates deep expertise in Weaviate and Qdrant.</t>
+          <t>Competitive candidate: Applied ML Engineer at CRED (5.1 YOE); JD-aligned skills: Elasticsearch, OpenSearch, Weaviate.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>CAND_0042029</t>
+          <t>CAND_0046525</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -909,19 +909,19 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>0.9634</t>
+          <t>0.8797</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Strong fit: Senior Data Scientist at Flipkart with 6.5 YOE. Demonstrates deep expertise in NLP and Elasticsearch.</t>
+          <t>Meets several JD signals: Senior Machine Learning Engineer at Genpact AI (6.1 YOE); JD-aligned skills: Elasticsearch, LLMs, NLP.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>CAND_0020877</t>
+          <t>CAND_0099806</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -929,19 +929,19 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>0.9620</t>
+          <t>0.8791</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Strong fit: Applied ML Engineer at CRED with 5.1 YOE. Demonstrates deep expertise in Elasticsearch and OpenSearch.</t>
+          <t>Solid profile: AI Engineer at Mad Street Den (4.6 YOE); JD-aligned skills: FAISS, Embeddings, Sentence Transformers.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>CAND_0037944</t>
+          <t>CAND_0050454</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -949,19 +949,19 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>0.9587</t>
+          <t>0.8786</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Strong fit: Senior Data Scientist at Vedantu with 4.9 YOE. Demonstrates deep expertise in Vector Search and OpenSearch.</t>
+          <t>Good fit with caveats: AI Engineer at Rephrase.ai (6.8 YOE); JD-aligned skills: Fine-tuning LLMs, FAISS, Qdrant.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>CAND_0032216</t>
+          <t>CAND_0071939</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -969,19 +969,19 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>0.9567</t>
+          <t>0.8785</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at upGrad with 6.1 YOE. Demonstrates deep expertise in Qdrant and Sentence Transformers.</t>
+          <t>Competitive candidate: Data Scientist at Krutrim (6.4 YOE); JD-aligned skills: Elasticsearch, OpenSearch, Embeddings.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>CAND_0049538</t>
+          <t>CAND_0032216</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -989,19 +989,19 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>0.9560</t>
+          <t>0.8783</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Strong fit: Applied ML Engineer at Saarthi.ai with 5.8 YOE. Demonstrates deep expertise in OpenSearch and Vector Search.</t>
+          <t>Meets several JD signals: ML Engineer at upGrad (6.1 YOE); JD-aligned skills: Qdrant, Sentence Transformers, Vector Search.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>CAND_0055905</t>
+          <t>CAND_0037944</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -1009,19 +1009,19 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>0.9491</t>
+          <t>0.8726</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Strong fit: Senior Machine Learning Engineer at Flipkart with 8.1 YOE. Demonstrates deep expertise in Elasticsearch and Python.</t>
+          <t>Solid profile: Senior Data Scientist at Vedantu (4.9 YOE); JD-aligned skills: Vector Search, OpenSearch, Embeddings.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>CAND_0043228</t>
+          <t>CAND_0049538</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1029,12 +1029,12 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>0.9489</t>
+          <t>0.8661</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Strong fit: Applied ML Engineer at Zoho with 6.8 YOE. Demonstrates deep expertise in NLP and Vector Search.</t>
+          <t>Good fit with caveats: Applied ML Engineer at Saarthi.ai (5.8 YOE); JD-aligned skills: OpenSearch, Vector Search, Milvus.</t>
         </is>
       </c>
     </row>
@@ -1049,19 +1049,19 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>0.9437</t>
+          <t>0.8632</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Strong fit: Senior Data Scientist at Flipkart with 6.6 YOE. Demonstrates deep expertise in OpenSearch and Pinecone.</t>
+          <t>Competitive candidate: Senior Data Scientist at Flipkart (6.6 YOE); JD-aligned skills: OpenSearch, Pinecone, Vector Search.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>CAND_0079387</t>
+          <t>CAND_0043228</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1069,19 +1069,19 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>0.9420</t>
+          <t>0.8629</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Strong fit: AI Engineer at Microsoft with 6.9 YOE. Demonstrates deep expertise in Python and Sentence Transformers.</t>
+          <t>Meets several JD signals: Applied ML Engineer at Zoho (6.8 YOE); JD-aligned skills: NLP, Vector Search, Sentence Transformers.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>CAND_0001707</t>
+          <t>CAND_0079284</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -1089,19 +1089,19 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>0.9404</t>
+          <t>0.8596</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Strong fit: Data Scientist at Vedantu with 5.6 YOE. Demonstrates deep expertise in Sentence Transformers and FAISS.</t>
+          <t>Solid profile: Machine Learning Engineer at Google (4.9 YOE); JD-aligned skills: Qdrant, Fine-tuning LLMs, Elasticsearch.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>CAND_0079064</t>
+          <t>CAND_0083879</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -1109,19 +1109,19 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>0.9395</t>
+          <t>0.8596</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Strong fit: Senior Data Scientist at Niramai with 5.2 YOE. Demonstrates deep expertise in OpenSearch and NLP.</t>
+          <t>Good fit with caveats: Machine Learning Engineer at Ola (7.1 YOE); JD-aligned skills: Fine-tuning LLMs, Milvus, Sentence Transformers.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>CAND_0045141</t>
+          <t>CAND_0079387</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -1129,19 +1129,19 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>0.9387</t>
+          <t>0.8548</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Strong fit: Data Scientist at HCL with 5.3 YOE. Demonstrates deep expertise in Milvus and Pinecone.</t>
+          <t>Competitive candidate: AI Engineer at Microsoft (6.9 YOE); JD-aligned skills: Python, Sentence Transformers, Vector Search.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>CAND_0074342</t>
+          <t>CAND_0079064</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -1149,19 +1149,19 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>0.9344</t>
+          <t>0.8525</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Strong fit: Data Scientist at Zoho with 5.7 YOE. Demonstrates deep expertise in Sentence Transformers and LLMs.</t>
+          <t>Meets several JD signals: Senior Data Scientist at Niramai (5.2 YOE); JD-aligned skills: OpenSearch, NLP, Fine-tuning LLMs. Concerns: 120-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>CAND_0081852</t>
+          <t>CAND_0086022</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -1169,19 +1169,19 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>0.9315</t>
+          <t>0.8515</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Strong fit: Senior Data Scientist at Mad Street Den with 5.9 YOE. Demonstrates deep expertise in Milvus and Weaviate.</t>
+          <t>Solid profile: Senior Applied Scientist at Sarvam AI (5.3 YOE); JD-aligned skills: Vector Search, Fine-tuning LLMs, Elasticsearch.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>CAND_0051004</t>
+          <t>CAND_0090584</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -1189,19 +1189,19 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>0.9310</t>
+          <t>0.8506</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Strong fit: Senior Data Scientist at CRED with 4.7 YOE. Demonstrates deep expertise in Embeddings and Qdrant.</t>
+          <t>Good fit with caveats: ML Engineer at Flipkart (5.1 YOE); JD-aligned skills: Fine-tuning LLMs, OpenSearch, FAISS. Concerns: 120-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>CAND_0079284</t>
+          <t>CAND_0061257</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -1209,19 +1209,19 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>0.9303</t>
+          <t>0.8474</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Strong fit: Machine Learning Engineer at Google with 4.9 YOE. Demonstrates deep expertise in Qdrant and Fine-tuning LLMs.</t>
+          <t>Competitive candidate: Staff Machine Learning Engineer at LinkedIn (8.0 YOE); JD-aligned skills: Python. Concerns: only 1 core JD skill matched.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>CAND_0016163</t>
+          <t>CAND_0003841</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -1229,19 +1229,19 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>0.9294</t>
+          <t>0.8420</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Strong fit: Applied ML Engineer at Dream11 with 6.7 YOE. Demonstrates deep expertise in Weaviate and Embeddings.</t>
+          <t>Meets several JD signals: ML Engineer at Tech Mahindra (5.0 YOE); JD-aligned skills: Pinecone, Fine-tuning LLMs, Sentence Transformers.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>CAND_0010257</t>
+          <t>CAND_0051004</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -1249,19 +1249,19 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>0.9286</t>
+          <t>0.8409</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Strong fit: Senior Data Scientist at Google with 6.5 YOE. Demonstrates deep expertise in Milvus and Python.</t>
+          <t>Solid profile: Senior Data Scientist at CRED (4.7 YOE); JD-aligned skills: Embeddings, Qdrant, Fine-tuning LLMs.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>CAND_0090584</t>
+          <t>CAND_0010257</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -1269,19 +1269,19 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>0.9211</t>
+          <t>0.8408</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at Flipkart with 5.1 YOE. Demonstrates deep expertise in Fine-tuning LLMs and OpenSearch.</t>
+          <t>Good fit with caveats: Senior Data Scientist at Google (6.5 YOE); JD-aligned skills: Milvus, Python, OpenSearch. Concerns: 120-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>CAND_0075574</t>
+          <t>CAND_0081852</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -1289,19 +1289,19 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>0.9172</t>
+          <t>0.8396</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Strong fit: Machine Learning Engineer at Haptik with 5.7 YOE. Demonstrates deep expertise in Weaviate and OpenSearch.</t>
+          <t>Competitive candidate: Senior Data Scientist at Mad Street Den (5.9 YOE); JD-aligned skills: Milvus, Weaviate, Vector Search.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>CAND_0068811</t>
+          <t>CAND_0055905</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -1309,19 +1309,19 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>0.9165</t>
+          <t>0.8393</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Strong fit: Applied ML Engineer at Freshworks with 8.0 YOE. Demonstrates deep expertise in Vector Search and Qdrant.</t>
+          <t>Meets several JD signals: Senior Machine Learning Engineer at Flipkart (8.1 YOE); JD-aligned skills: Elasticsearch, Python, LLMs.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>CAND_0036121</t>
+          <t>CAND_0091909</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -1329,19 +1329,19 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>0.9132</t>
+          <t>0.8364</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at Wysa with 5.2 YOE. Demonstrates deep expertise in Embeddings and Vector Search.</t>
+          <t>Solid profile: Machine Learning Engineer at Rephrase.ai (6.9 YOE); JD-aligned skills: LLMs, Pinecone, Qdrant.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>CAND_0070398</t>
+          <t>CAND_0075574</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -1349,19 +1349,19 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>0.9063</t>
+          <t>0.8357</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Strong fit: Machine Learning Engineer at Genpact AI with 7.2 YOE. Demonstrates deep expertise in FAISS and Embeddings.</t>
+          <t>Good fit with caveats: Machine Learning Engineer at Haptik (5.7 YOE); JD-aligned skills: Weaviate, OpenSearch, Qdrant.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>CAND_0093193</t>
+          <t>CAND_0018094</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -1369,19 +1369,19 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>0.9062</t>
+          <t>0.8352</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Strong fit: Senior Machine Learning Engineer at Niramai with 7.9 YOE. Demonstrates deep expertise in Qdrant and OpenSearch.</t>
+          <t>Competitive candidate: ML Engineer at Mad Street Den (5.2 YOE); JD-aligned skills: Pinecone, Fine-tuning LLMs.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>CAND_0091909</t>
+          <t>CAND_0016163</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -1389,19 +1389,19 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>0.9056</t>
+          <t>0.8304</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Strong fit: Machine Learning Engineer at Rephrase.ai with 6.9 YOE. Demonstrates deep expertise in LLMs and Pinecone.</t>
+          <t>Meets several JD signals: Applied ML Engineer at Dream11 (6.7 YOE); JD-aligned skills: Weaviate, Embeddings, Pinecone. Concerns: 120-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>CAND_0098217</t>
+          <t>CAND_0017093</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -1409,19 +1409,19 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>0.9052</t>
+          <t>0.8271</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at Glance with 6.4 YOE. Demonstrates deep expertise in FAISS and Pinecone.</t>
+          <t>Solid profile: ML Engineer at Zoho (5.9 YOE); JD-aligned skills: LLMs, Embeddings.</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>CAND_0099269</t>
+          <t>CAND_0070398</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -1429,19 +1429,19 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>0.9034</t>
+          <t>0.8271</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Strong fit: Data Scientist at BYJU'S with 5.5 YOE. Demonstrates deep expertise in Elasticsearch and Python.</t>
+          <t>Good fit with caveats: Machine Learning Engineer at Genpact AI (7.2 YOE); JD-aligned skills: FAISS, Embeddings, Python. Concerns: 120-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>CAND_0040178</t>
+          <t>CAND_0098217</t>
         </is>
       </c>
       <c r="B52" t="n">
@@ -1449,19 +1449,19 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>0.9013</t>
+          <t>0.8271</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at Meesho with 5.0 YOE. Demonstrates deep expertise in Weaviate and Fine-tuning LLMs.</t>
+          <t>Moderate fit: ML Engineer at Glance (6.4 YOE); JD-aligned skills: FAISS, Pinecone. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>CAND_0011263</t>
+          <t>CAND_0047721</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -1469,19 +1469,19 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>0.8998</t>
+          <t>0.8264</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at Ola with 5.1 YOE. Demonstrates deep expertise in Pinecone and OpenSearch.</t>
+          <t>Partial alignment: Senior Data Scientist at Microsoft (7.0 YOE); JD-aligned skills: Milvus, FAISS, Qdrant. Gaps: 90-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>CAND_0030031</t>
+          <t>CAND_0052328</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -1489,19 +1489,19 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>0.8993</t>
+          <t>0.8206</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Strong fit: AI Engineer at Microsoft with 5.7 YOE. Demonstrates deep expertise in Python and NLP.</t>
+          <t>Acceptable but not standout: Recommendation Systems Engineer at Amazon (6.5 YOE); JD-aligned skills: OpenSearch, Fine-tuning LLMs, Vector Search. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>CAND_0047721</t>
+          <t>CAND_0051292</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -1509,19 +1509,19 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>0.8985</t>
+          <t>0.8205</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Strong fit: Senior Data Scientist at Microsoft with 7.0 YOE. Demonstrates deep expertise in Milvus and FAISS.</t>
+          <t>Mixed signals: Applied ML Engineer at Freshworks (5.2 YOE); JD-aligned skills: FAISS, LLMs, Vector Search. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>CAND_0048166</t>
+          <t>CAND_0036121</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -1529,19 +1529,19 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>0.8985</t>
+          <t>0.8174</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at Aganitha with 5.2 YOE. Demonstrates deep expertise in Pinecone and Milvus.</t>
+          <t>JD overlap is thin: ML Engineer at Wysa (5.2 YOE); JD-aligned skills: Embeddings, Vector Search. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>CAND_0017093</t>
+          <t>CAND_0009691</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -1549,19 +1549,19 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>0.8984</t>
+          <t>0.8152</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at Zoho with 5.9 YOE. Demonstrates deep expertise in LLMs and Embeddings.</t>
+          <t>Moderate fit: Applied ML Engineer at LinkedIn (6.2 YOE); JD-aligned skills: Fine-tuning LLMs, Pinecone, Sentence Transformers. Gaps: 120-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>CAND_0048558</t>
+          <t>CAND_0058688</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -1569,19 +1569,19 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>0.8984</t>
+          <t>0.8141</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Strong fit: Data Scientist at Rephrase.ai with 6.7 YOE. Demonstrates deep expertise in OpenSearch and Qdrant.</t>
+          <t>Partial alignment: AI Engineer at Vedantu (6.7 YOE); JD-aligned skills: Embeddings, Milvus. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>CAND_0005538</t>
+          <t>CAND_0011432</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -1589,19 +1589,19 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>0.8961</t>
+          <t>0.8128</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Strong fit: Senior AI Engineer at Adobe with 5.9 YOE. Demonstrates deep expertise in Python.</t>
+          <t>Acceptable but not standout: Senior Data Scientist at Amazon (7.6 YOE); JD-aligned skills: OpenSearch, Elasticsearch. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>CAND_0011432</t>
+          <t>CAND_0021836</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -1609,19 +1609,19 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>0.8951</t>
+          <t>0.8117</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Strong fit: Senior Data Scientist at Amazon with 7.6 YOE. Demonstrates deep expertise in OpenSearch and Elasticsearch.</t>
+          <t>Mixed signals: ML Engineer at CRED (6.5 YOE); JD-aligned skills: Vector Search, Elasticsearch, NLP. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>CAND_0050876</t>
+          <t>CAND_0035653</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -1629,19 +1629,19 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>0.8892</t>
+          <t>0.8114</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Strong fit: Applied ML Engineer at Freshworks with 6.0 YOE. Demonstrates deep expertise in Qdrant and FAISS.</t>
+          <t>JD overlap is thin: Data Scientist at Swiggy (5.6 YOE); JD-aligned skills: OpenSearch, Vector Search, Fine-tuning LLMs. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>CAND_0028287</t>
+          <t>CAND_0040178</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -1649,19 +1649,19 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>0.8880</t>
+          <t>0.8106</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Strong fit: Data Scientist at Unacademy with 5.7 YOE. Demonstrates deep expertise in OpenSearch and Vector Search.</t>
+          <t>Moderate fit: ML Engineer at Meesho (5.0 YOE); JD-aligned skills: Weaviate, Fine-tuning LLMs, Vector Search. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>CAND_0009691</t>
+          <t>CAND_0068932</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -1669,19 +1669,19 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>0.8869</t>
+          <t>0.8102</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Strong fit: Applied ML Engineer at LinkedIn with 6.2 YOE. Demonstrates deep expertise in Fine-tuning LLMs and Pinecone.</t>
+          <t>Partial alignment: ML Engineer at Krutrim (5.2 YOE); JD-aligned skills: Milvus, OpenSearch. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>CAND_0055992</t>
+          <t>CAND_0050876</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -1689,19 +1689,19 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>0.8861</t>
+          <t>0.8098</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Strong fit: AI Engineer at CRED with 16.9 YOE. Demonstrates deep expertise in FAISS and OpenSearch.</t>
+          <t>Acceptable but not standout: Applied ML Engineer at Freshworks (6.0 YOE); JD-aligned skills: Qdrant, FAISS, OpenSearch. Gaps: 90-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>CAND_0001494</t>
+          <t>CAND_0076482</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -1709,19 +1709,19 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>0.8848</t>
+          <t>0.8089</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Strong fit: Data Scientist at Haptik with 6.4 YOE. Demonstrates deep expertise in Vector Search and Weaviate.</t>
+          <t>Mixed signals: ML Engineer at Flipkart (6.6 YOE); JD-aligned skills: OpenSearch, Pinecone, Embeddings. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>CAND_0035653</t>
+          <t>CAND_0093193</t>
         </is>
       </c>
       <c r="B66" t="n">
@@ -1729,19 +1729,19 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>0.8825</t>
+          <t>0.8068</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Strong fit: Data Scientist at Swiggy with 5.6 YOE. Demonstrates deep expertise in OpenSearch and Vector Search.</t>
+          <t>JD overlap is thin: Senior Machine Learning Engineer at Niramai (7.9 YOE); JD-aligned skills: Qdrant, OpenSearch. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>CAND_0086022</t>
+          <t>CAND_0015578</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -1749,19 +1749,19 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>0.8819</t>
+          <t>0.8035</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Strong fit: Senior Applied Scientist at Sarvam AI with 5.3 YOE. Demonstrates deep expertise in Vector Search and Fine-tuning LLMs.</t>
+          <t>Moderate fit: AI Engineer at Zoho (5.4 YOE); JD-aligned skills: Embeddings, NLP, Sentence Transformers. Gaps: 90-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>CAND_0021836</t>
+          <t>CAND_0005538</t>
         </is>
       </c>
       <c r="B68" t="n">
@@ -1769,19 +1769,19 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>0.8808</t>
+          <t>0.8025</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at CRED with 6.5 YOE. Demonstrates deep expertise in Vector Search and Elasticsearch.</t>
+          <t>Partial alignment: Senior AI Engineer at Adobe (5.9 YOE); JD-aligned skills: Python. Gaps: only 1 core JD skill matched; 90-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>CAND_0076482</t>
+          <t>CAND_0095528</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -1789,19 +1789,19 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>0.8798</t>
+          <t>0.8021</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at Flipkart with 6.6 YOE. Demonstrates deep expertise in OpenSearch and Pinecone.</t>
+          <t>Acceptable but not standout: Senior Data Scientist at Netflix (5.3 YOE); JD-aligned skills: OpenSearch, Vector Search, Qdrant. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>CAND_0027723</t>
+          <t>CAND_0048166</t>
         </is>
       </c>
       <c r="B70" t="n">
@@ -1809,19 +1809,19 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>0.8783</t>
+          <t>0.7998</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at Wysa with 4.2 YOE. Demonstrates deep expertise in Vector Search and NLP.</t>
+          <t>Mixed signals: ML Engineer at Aganitha (5.2 YOE); JD-aligned skills: Pinecone, Milvus, Qdrant. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>CAND_0005649</t>
+          <t>CAND_0073982</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -1829,19 +1829,19 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>0.8777</t>
+          <t>0.7993</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Strong fit: Senior Data Scientist at Sarvam AI with 7.4 YOE. Demonstrates deep expertise in Fine-tuning LLMs and Weaviate.</t>
+          <t>JD overlap is thin: Data Scientist at Dream11 (7.0 YOE); JD-aligned skills: Sentence Transformers, Qdrant, FAISS. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>CAND_0083879</t>
+          <t>CAND_0095213</t>
         </is>
       </c>
       <c r="B72" t="n">
@@ -1849,19 +1849,19 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>0.8746</t>
+          <t>0.7966</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Strong fit: Machine Learning Engineer at Ola with 7.1 YOE. Demonstrates deep expertise in Fine-tuning LLMs and Milvus.</t>
+          <t>Moderate fit: ML Engineer at Genpact AI (5.1 YOE); JD-aligned skills: Python, Weaviate, Pinecone. Gaps: not flagged open to work.</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>CAND_0013393</t>
+          <t>CAND_0069905</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -1869,19 +1869,19 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>0.8739</t>
+          <t>0.7964</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at Freshworks with 5.3 YOE. Demonstrates deep expertise in Embeddings and Pinecone.</t>
+          <t>Partial alignment: Applied ML Engineer at Sarvam AI (6.6 YOE); JD-aligned skills: Sentence Transformers, Python, Weaviate. Gaps: 90-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>CAND_0090155</t>
+          <t>CAND_0013393</t>
         </is>
       </c>
       <c r="B74" t="n">
@@ -1889,19 +1889,19 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>0.8683</t>
+          <t>0.7946</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at Swiggy with 5.8 YOE. Demonstrates deep expertise in Milvus and Qdrant.</t>
+          <t>Acceptable but not standout: ML Engineer at Freshworks (5.3 YOE); JD-aligned skills: Embeddings, Pinecone, Qdrant. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>CAND_0073982</t>
+          <t>CAND_0001707</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -1909,19 +1909,19 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>0.8672</t>
+          <t>0.7909</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Strong fit: Data Scientist at Dream11 with 7.0 YOE. Demonstrates deep expertise in Sentence Transformers and Qdrant.</t>
+          <t>Mixed signals: Data Scientist at Vedantu (5.6 YOE); JD-aligned skills: Sentence Transformers, FAISS, Weaviate. Gaps: 90-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>CAND_0061257</t>
+          <t>CAND_0005477</t>
         </is>
       </c>
       <c r="B76" t="n">
@@ -1929,19 +1929,19 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>0.8670</t>
+          <t>0.7908</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Strong fit: Staff Machine Learning Engineer at LinkedIn with 8.0 YOE. Demonstrates deep expertise in Python.</t>
+          <t>JD overlap is thin: ML Engineer at Zomato (6.2 YOE); JD-aligned skills: OpenSearch. Gaps: only 1 core JD skill matched.</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>CAND_0092255</t>
+          <t>CAND_0055992</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -1949,19 +1949,19 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>0.8644</t>
+          <t>0.7897</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at InMobi with 5.2 YOE. Demonstrates deep expertise in Weaviate and OpenSearch.</t>
+          <t>Moderate fit: AI Engineer at CRED (16.9 YOE); JD-aligned skills: FAISS, OpenSearch, Embeddings. Gaps: experience above target band for this role.</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>CAND_0060538</t>
+          <t>CAND_0005649</t>
         </is>
       </c>
       <c r="B78" t="n">
@@ -1969,19 +1969,19 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>0.8642</t>
+          <t>0.7891</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at Verloop.io with 5.2 YOE. Demonstrates deep expertise in OpenSearch and Embeddings.</t>
+          <t>Partial alignment: Senior Data Scientist at Sarvam AI (7.4 YOE); JD-aligned skills: Fine-tuning LLMs, Weaviate. Gaps: 90-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>CAND_0095213</t>
+          <t>CAND_0027723</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -1989,19 +1989,19 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>0.8636</t>
+          <t>0.7889</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at Genpact AI with 5.1 YOE. Demonstrates deep expertise in Python and Weaviate.</t>
+          <t>Acceptable but not standout: ML Engineer at Wysa (4.2 YOE); JD-aligned skills: Vector Search, NLP, Elasticsearch. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>CAND_0042100</t>
+          <t>CAND_0090155</t>
         </is>
       </c>
       <c r="B80" t="n">
@@ -2009,19 +2009,19 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>0.8634</t>
+          <t>0.7881</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Strong fit: Machine Learning Engineer at Freshworks with 7.3 YOE. Demonstrates deep expertise in Elasticsearch and Fine-tuning LLMs.</t>
+          <t>Mixed signals: ML Engineer at Swiggy (5.8 YOE); JD-aligned skills: Milvus, Qdrant, Pinecone. Gaps: 90-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>CAND_0060054</t>
+          <t>CAND_0060538</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -2029,19 +2029,19 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>0.8608</t>
+          <t>0.7867</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Strong fit: AI Engineer at Mad Street Den with 6.4 YOE. Demonstrates deep expertise in Weaviate and FAISS.</t>
+          <t>JD overlap is thin: ML Engineer at Verloop.io (5.2 YOE); JD-aligned skills: OpenSearch, Embeddings, Milvus. Gaps: 90-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>CAND_0005477</t>
+          <t>CAND_0042100</t>
         </is>
       </c>
       <c r="B82" t="n">
@@ -2049,19 +2049,19 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>0.8600</t>
+          <t>0.7838</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at Zomato with 6.2 YOE. Demonstrates deep expertise in OpenSearch.</t>
+          <t>Moderate fit: Machine Learning Engineer at Freshworks (7.3 YOE); JD-aligned skills: Elasticsearch, Fine-tuning LLMs, Pinecone. Gaps: 90-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>CAND_0027691</t>
+          <t>CAND_0041669</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -2069,19 +2069,19 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>0.8588</t>
+          <t>0.7817</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Strong fit: NLP Engineer at Haptik with 6.5 YOE. Demonstrates deep expertise in Weaviate and Embeddings.</t>
+          <t>Partial alignment: Recommendation Systems Engineer at CRED (8.0 YOE); JD-aligned skills: FAISS, Milvus, Weaviate. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>CAND_0015528</t>
+          <t>CAND_0066999</t>
         </is>
       </c>
       <c r="B84" t="n">
@@ -2089,19 +2089,19 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>0.8569</t>
+          <t>0.7800</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Strong fit: Applied ML Engineer at Krutrim with 7.4 YOE. Demonstrates deep expertise in Weaviate and OpenSearch.</t>
+          <t>Acceptable but not standout: Recommendation Systems Engineer at Microsoft (5.9 YOE); JD-aligned skills: OpenSearch, FAISS, LLMs. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>CAND_0030348</t>
+          <t>CAND_0060054</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -2109,19 +2109,19 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>0.8555</t>
+          <t>0.7776</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Strong fit: Machine Learning Engineer at BYJU'S with 4.5 YOE. Demonstrates deep expertise in Embeddings and Vector Search.</t>
+          <t>Mixed signals: AI Engineer at Mad Street Den (6.4 YOE); JD-aligned skills: Weaviate, FAISS, Elasticsearch. Gaps: not flagged open to work.</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>CAND_0025335</t>
+          <t>CAND_0015528</t>
         </is>
       </c>
       <c r="B86" t="n">
@@ -2129,19 +2129,19 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>0.8509</t>
+          <t>0.7746</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Strong fit: Data Scientist at PolicyBazaar with 6.6 YOE. Demonstrates deep expertise in NLP.</t>
+          <t>JD overlap is thin: Applied ML Engineer at Krutrim (7.4 YOE); JD-aligned skills: Weaviate, OpenSearch, FAISS. Gaps: not flagged open to work.</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>CAND_0003841</t>
+          <t>CAND_0030348</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -2149,19 +2149,19 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>0.8479</t>
+          <t>0.7722</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at Tech Mahindra with 5.0 YOE. Demonstrates deep expertise in Pinecone and Fine-tuning LLMs.</t>
+          <t>Moderate fit: Machine Learning Engineer at BYJU'S (4.5 YOE); JD-aligned skills: Embeddings, Vector Search, Elasticsearch. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>CAND_0094759</t>
+          <t>CAND_0047276</t>
         </is>
       </c>
       <c r="B88" t="n">
@@ -2169,19 +2169,19 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>0.8468</t>
+          <t>0.7711</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Strong fit: Lead AI Engineer at Meta with 8.6 YOE. Demonstrates deep expertise in Qdrant and Fine-tuning LLMs.</t>
+          <t>Partial alignment: Backend Engineer at Freshworks (5.5 YOE); JD-aligned skills: Qdrant, Fine-tuning LLMs. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>CAND_0005509</t>
+          <t>CAND_0010149</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -2189,19 +2189,19 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>0.8457</t>
+          <t>0.7665</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Strong fit: Data Scientist at Ola with 6.0 YOE. Demonstrates deep expertise in Python and Fine-tuning LLMs.</t>
+          <t>Acceptable but not standout: ML Engineer at Glance (6.9 YOE); JD-aligned skills: Milvus, Vector Search, Elasticsearch. Gaps: 90-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>CAND_0002037</t>
+          <t>CAND_0093912</t>
         </is>
       </c>
       <c r="B90" t="n">
@@ -2209,19 +2209,19 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>0.8416</t>
+          <t>0.7662</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at Locobuzz with 5.5 YOE. Demonstrates deep expertise in Fine-tuning LLMs and Milvus.</t>
+          <t>Mixed signals: Senior Data Scientist at Razorpay (5.3 YOE); JD-aligned skills: Milvus, Embeddings, Vector Search. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>CAND_0018094</t>
+          <t>CAND_0027691</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -2229,19 +2229,19 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>0.8414</t>
+          <t>0.7637</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Strong fit: ML Engineer at Mad Street Den with 5.2 YOE. Demonstrates deep expertise in Pinecone and Fine-tuning LLMs.</t>
+          <t>JD overlap is thin: NLP Engineer at Haptik (6.5 YOE); JD-aligned skills: Weaviate, Embeddings, Python. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>CAND_0071432</t>
+          <t>CAND_0074735</t>
         </is>
       </c>
       <c r="B92" t="n">
@@ -2249,19 +2249,19 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>0.8398</t>
+          <t>0.7629</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Borderline Match: Strong fit: Data Scientist at Wysa with 4.1 YOE. Demonstrates deep expertise in Weaviate and Pinecone. Meets minimum bar but lacks standout secondary signals.</t>
+          <t>Lower-tier shortlist entry — Applied ML Engineer at Rephrase.ai (5.5 YOE); JD-aligned skills: Weaviate, Vector Search, Elasticsearch. Key gaps: 90-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>CAND_0072721</t>
+          <t>CAND_0002037</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -2269,19 +2269,19 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>0.8385</t>
+          <t>0.7611</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Borderline Match: Strong fit: Data Scientist at Yellow.ai with 3.7 YOE. Demonstrates deep expertise in Weaviate and Qdrant. Meets minimum bar but lacks standout secondary signals.</t>
+          <t>Lower-tier shortlist entry — ML Engineer at Locobuzz (5.5 YOE); JD-aligned skills: Fine-tuning LLMs, Milvus, Pinecone. Key gaps: not flagged open to work.</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>CAND_0064904</t>
+          <t>CAND_0099269</t>
         </is>
       </c>
       <c r="B94" t="n">
@@ -2289,19 +2289,19 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>0.8380</t>
+          <t>0.7588</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Borderline Match: Strong fit: AI Engineer at LinkedIn with 4.9 YOE. Demonstrates deep expertise in Embeddings and Elasticsearch. Meets minimum bar but lacks standout secondary signals.</t>
+          <t>Lower-tier shortlist entry — Data Scientist at BYJU'S (5.5 YOE); JD-aligned skills: Elasticsearch, Python, NLP. Key gaps: 120-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>CAND_0007460</t>
+          <t>CAND_0069232</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -2309,19 +2309,19 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>0.8374</t>
+          <t>0.7580</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Borderline Match: Strong fit: AI Engineer at Salesforce with 4.7 YOE. Demonstrates deep expertise in Embeddings and Weaviate. Meets minimum bar but lacks standout secondary signals.</t>
+          <t>Lower-tier shortlist entry — ML Engineer at Yellow.ai (6.3 YOE); JD-aligned skills: Pinecone, NLP, Python. Key gaps: 120-day notice period; not flagged open to work.</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>CAND_0061550</t>
+          <t>CAND_0015582</t>
         </is>
       </c>
       <c r="B96" t="n">
@@ -2329,19 +2329,19 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>0.8366</t>
+          <t>0.7563</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Borderline Match: Strong fit: ML Engineer at Infosys with 5.3 YOE. Demonstrates deep expertise in Sentence Transformers. Meets minimum bar but lacks standout secondary signals.</t>
+          <t>Lower-tier shortlist entry — ML Engineer at Genpact AI (4.4 YOE); JD-aligned skills: Qdrant, Sentence Transformers, Embeddings. Key gaps: 120-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>CAND_0058688</t>
+          <t>CAND_0065277</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -2349,19 +2349,19 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>0.8341</t>
+          <t>0.7561</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Borderline Match: Strong fit: AI Engineer at Vedantu with 6.7 YOE. Demonstrates deep expertise in Embeddings and Milvus. Meets minimum bar but lacks standout secondary signals.</t>
+          <t>Lower-tier shortlist entry — Computer Vision Engineer at Aganitha (6.3 YOE); JD-aligned skills: Vector Search, Milvus, Fine-tuning LLMs. Key gaps: weak secondary signals vs higher ranks.</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>CAND_0010149</t>
+          <t>CAND_0006418</t>
         </is>
       </c>
       <c r="B98" t="n">
@@ -2369,19 +2369,19 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>0.8333</t>
+          <t>0.7552</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Borderline Match: Strong fit: ML Engineer at Glance with 6.9 YOE. Demonstrates deep expertise in Milvus and Vector Search. Meets minimum bar but lacks standout secondary signals.</t>
+          <t>Lower-tier shortlist entry — Machine Learning Engineer at Verloop.io (5.7 YOE); JD-aligned skills: Embeddings, Weaviate, Elasticsearch. Key gaps: weak secondary signals vs higher ranks.</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>CAND_0017178</t>
+          <t>CAND_0094759</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -2389,19 +2389,19 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>0.8292</t>
+          <t>0.7551</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Borderline Match: Strong fit: ML Engineer at Swiggy with 4.2 YOE. Demonstrates deep expertise in PEFT and pgvector. Meets minimum bar but lacks standout secondary signals.</t>
+          <t>Lower-tier shortlist entry — Lead AI Engineer at Meta (8.6 YOE); JD-aligned skills: Qdrant, Fine-tuning LLMs, Vector Search. Key gaps: low recruiter response rate; not flagged open to work.</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>CAND_0006557</t>
+          <t>CAND_0065878</t>
         </is>
       </c>
       <c r="B100" t="n">
@@ -2409,19 +2409,19 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>0.8290</t>
+          <t>0.7540</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Borderline Match: Strong fit: NLP Engineer at Paytm with 7.9 YOE. Demonstrates deep expertise in Elasticsearch and OpenSearch. Meets minimum bar but lacks standout secondary signals.</t>
+          <t>Lower-tier shortlist entry — Senior Data Scientist at Niramai (7.8 YOE); JD-aligned skills: Vector Search, Fine-tuning LLMs. Key gaps: weak secondary signals vs higher ranks.</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>CAND_0066690</t>
+          <t>CAND_0007460</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -2429,12 +2429,12 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>0.8287</t>
+          <t>0.7535</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Borderline Match: Strong fit: ML Engineer at Freshworks with 4.8 YOE. Demonstrates deep expertise in Sentence Transformers and Elasticsearch. Meets minimum bar but lacks standout secondary signals.</t>
+          <t>Lower-tier shortlist entry — AI Engineer at Salesforce (4.7 YOE); JD-aligned skills: Embeddings, Weaviate, NLP. Key gaps: 120-day notice period.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: regenerate submission artifacts after remediation
</commit_message>
<xml_diff>
--- a/submission.xlsx
+++ b/submission.xlsx
@@ -441,7 +441,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>CAND_0006567</t>
+          <t>CAND_0045250</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -449,19 +449,19 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>1.0130</t>
+          <t>1.0622</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Rank 1: Senior AI Engineer at Meta (7.9 YOE); JD-aligned skills: NLP, Python. Top-tier composite score across career, skills, and availability.</t>
+          <t>Rank 1: Applied ML Engineer at Rephrase.ai (6.6 YOE); JD-aligned skills: Sentence Transformers, Milvus, Embeddings. Top-tier composite score across career, skills, and availability. Counterfactual: trails a perfect match on 13 uncovered JD must-have skill(s).</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>CAND_0045250</t>
+          <t>CAND_0006567</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -469,12 +469,12 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>0.9990</t>
+          <t>1.0281</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Rank 2: Applied ML Engineer at Rephrase.ai (6.6 YOE); JD-aligned skills: Sentence Transformers, Milvus, Embeddings. Top-tier composite score across career, skills, and availability.</t>
+          <t>Rank 2: Senior AI Engineer at Meta (7.9 YOE); JD-aligned skills: NLP, Python. Top-tier composite score across career, skills, and availability. Counterfactual: trails a perfect match on 18 uncovered JD must-have skill(s).</t>
         </is>
       </c>
     </row>
@@ -489,19 +489,19 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>0.9986</t>
+          <t>1.0153</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Rank 3: Senior AI Engineer at Netflix (7.8 YOE); JD-aligned skills: Weaviate, Pinecone, Qdrant. Top-tier composite score across career, skills, and availability.</t>
+          <t>Rank 3: Senior AI Engineer at Netflix (7.8 YOE); JD-aligned skills: Weaviate, Pinecone, Qdrant. Top-tier composite score across career, skills, and availability. Counterfactual: trails a perfect match on 14 uncovered JD must-have skill(s).</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>CAND_0002025</t>
+          <t>CAND_0096142</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -509,19 +509,19 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>0.9783</t>
+          <t>1.0027</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Rank 4: Senior AI Engineer at Apple (5.9 YOE); JD-aligned skills: FAISS, OpenSearch, Weaviate. Top-tier composite score across career, skills, and availability.</t>
+          <t>Rank 4: Applied ML Engineer at upGrad (5.0 YOE); JD-aligned skills: Weaviate, Pinecone, Python. Top-tier composite score across career, skills, and availability. Minor note: 120-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CAND_0096142</t>
+          <t>CAND_0002025</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -529,19 +529,19 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>0.9669</t>
+          <t>0.9945</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Rank 5: Applied ML Engineer at upGrad (5.0 YOE); JD-aligned skills: Weaviate, Pinecone, Python. Top-tier composite score across career, skills, and availability. Minor note: 120-day notice period.</t>
+          <t>Rank 5: Senior AI Engineer at Apple (5.9 YOE); JD-aligned skills: FAISS, OpenSearch, Weaviate. Top-tier composite score across career, skills, and availability. Counterfactual: trails a perfect match on 12 uncovered JD must-have skill(s).</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>CAND_0018499</t>
+          <t>CAND_0087630</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -549,19 +549,19 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>0.9612</t>
+          <t>0.9906</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Strong match — Senior Machine Learning Engineer at Zomato (7.2 YOE); JD-aligned skills: Weaviate, Pinecone, Milvus.</t>
+          <t>Strong match — AI Engineer at Vedantu (7.2 YOE); JD-aligned skills: Elasticsearch, NLP, Embeddings.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>CAND_0087630</t>
+          <t>CAND_0018499</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -569,19 +569,19 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>0.9566</t>
+          <t>0.9772</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Strong match — AI Engineer at Vedantu (7.2 YOE); JD-aligned skills: Elasticsearch, NLP, Embeddings.</t>
+          <t>Strong match — Senior Machine Learning Engineer at Zomato (7.2 YOE); JD-aligned skills: Weaviate, Pinecone, Milvus.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>CAND_0020350</t>
+          <t>CAND_0068351</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -589,19 +589,19 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>0.9531</t>
+          <t>0.9707</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Strong match — AI Engineer at Zoho (5.8 YOE); JD-aligned skills: NLP, LLMs, FAISS.</t>
+          <t>Strong match — Lead AI Engineer at Sarvam AI (6.4 YOE); JD-aligned skills: Qdrant, Elasticsearch, Python.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>CAND_0068351</t>
+          <t>CAND_0020350</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -609,19 +609,19 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>0.9359</t>
+          <t>0.9670</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Strong match — Lead AI Engineer at Sarvam AI (6.4 YOE); JD-aligned skills: Qdrant, Elasticsearch, Python.</t>
+          <t>Strong match — AI Engineer at Zoho (5.8 YOE); JD-aligned skills: NLP, LLMs, FAISS.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>CAND_0065514</t>
+          <t>CAND_0068811</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -629,19 +629,19 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>0.9268</t>
+          <t>0.9656</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Strong match — ML Engineer at Genpact AI (6.6 YOE); JD-aligned skills: Vector Search, Pinecone, Elasticsearch. Watch: 90-day notice period.</t>
+          <t>Strong match — Applied ML Engineer at Freshworks (8.0 YOE); JD-aligned skills: Vector Search, Qdrant, Embeddings.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>CAND_0080766</t>
+          <t>CAND_0044855</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -649,19 +649,19 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>0.9200</t>
+          <t>0.9650</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Strong match — Staff Machine Learning Engineer at Salesforce (8.8 YOE); JD-aligned skills: Elasticsearch, OpenSearch, Python.</t>
+          <t>Strong match — Senior Data Scientist at Flipkart (6.6 YOE); JD-aligned skills: OpenSearch, Pinecone, Vector Search.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>CAND_0088025</t>
+          <t>CAND_0080766</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -669,19 +669,19 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>0.9166</t>
+          <t>0.9558</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Strong match — Staff Machine Learning Engineer at Yellow.ai (8.6 YOE); JD-aligned skills: Pinecone, LLMs, Elasticsearch. Watch: 90-day notice period.</t>
+          <t>Strong match — Staff Machine Learning Engineer at Salesforce (8.8 YOE); JD-aligned skills: Elasticsearch, OpenSearch, Python.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>CAND_0039383</t>
+          <t>CAND_0088025</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -689,19 +689,19 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>0.9138</t>
+          <t>0.9520</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Strong match — Applied ML Engineer at Meesho (7.1 YOE); JD-aligned skills: FAISS, NLP, Vector Search. Watch: 90-day notice period.</t>
+          <t>Strong match — Staff Machine Learning Engineer at Yellow.ai (8.6 YOE); JD-aligned skills: Pinecone, LLMs, Elasticsearch. Watch: 90-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>CAND_0037566</t>
+          <t>CAND_0044222</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -709,19 +709,19 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>0.9108</t>
+          <t>0.9489</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Strong match — Machine Learning Engineer at LinkedIn (6.9 YOE); JD-aligned skills: Pinecone, NLP, LLMs.</t>
+          <t>Strong match — AI Engineer at PolicyBazaar (7.7 YOE); JD-aligned skills: Vector Search, OpenSearch, Qdrant.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>CAND_0081846</t>
+          <t>CAND_0039383</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -729,19 +729,19 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>0.9092</t>
+          <t>0.9468</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Strong match — Lead AI Engineer at Razorpay (6.7 YOE); JD-aligned skills: Elasticsearch, Vector Search, Python.</t>
+          <t>Strong match — Applied ML Engineer at Meesho (7.1 YOE); JD-aligned skills: FAISS, NLP, Vector Search. Watch: 90-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>CAND_0068811</t>
+          <t>CAND_0077337</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -749,19 +749,19 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>0.9073</t>
+          <t>0.9405</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Strong match — Applied ML Engineer at Freshworks (8.0 YOE); JD-aligned skills: Vector Search, Qdrant, Embeddings.</t>
+          <t>Strong match — Staff Machine Learning Engineer at Paytm (7.0 YOE); JD-aligned skills: Pinecone, LLMs, Qdrant.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>CAND_0044222</t>
+          <t>CAND_0046525</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -769,19 +769,19 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>0.8911</t>
+          <t>0.9402</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Strong match — AI Engineer at PolicyBazaar (7.7 YOE); JD-aligned skills: Vector Search, OpenSearch, Qdrant.</t>
+          <t>Strong match — Senior Machine Learning Engineer at Genpact AI (6.1 YOE); JD-aligned skills: Elasticsearch, LLMs, NLP.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>CAND_0038368</t>
+          <t>CAND_0042029</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -789,19 +789,19 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>0.8898</t>
+          <t>0.9382</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Strong match — ML Engineer at PhonePe (5.4 YOE); JD-aligned skills: Embeddings, FAISS, NLP.</t>
+          <t>Strong match — Senior Data Scientist at Flipkart (6.5 YOE); JD-aligned skills: NLP, Elasticsearch, Embeddings.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>CAND_0030031</t>
+          <t>CAND_0065514</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -809,19 +809,19 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>0.8890</t>
+          <t>0.9377</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Strong match — AI Engineer at Microsoft (5.7 YOE); JD-aligned skills: Python, NLP, Sentence Transformers.</t>
+          <t>Strong match — ML Engineer at Genpact AI (6.6 YOE); JD-aligned skills: Vector Search, Pinecone, Elasticsearch. Watch: 90-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>CAND_0089552</t>
+          <t>CAND_0020877</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -829,19 +829,19 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>0.8848</t>
+          <t>0.9367</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Strong match — Machine Learning Engineer at Netflix (6.0 YOE); JD-aligned skills: Weaviate, Qdrant, Vector Search. Watch: 120-day notice period.</t>
+          <t>Strong match — Applied ML Engineer at CRED (5.1 YOE); JD-aligned skills: Elasticsearch, OpenSearch, Weaviate.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>CAND_0042029</t>
+          <t>CAND_0071939</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -849,19 +849,19 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>0.8812</t>
+          <t>0.9320</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Solid profile: Senior Data Scientist at Flipkart (6.5 YOE); JD-aligned skills: NLP, Elasticsearch, Embeddings.</t>
+          <t>Solid profile: Data Scientist at Krutrim (6.4 YOE); JD-aligned skills: Elasticsearch, OpenSearch, Embeddings.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>CAND_0077337</t>
+          <t>CAND_0081846</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -869,19 +869,19 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>0.8812</t>
+          <t>0.9260</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Good fit with caveats: Staff Machine Learning Engineer at Paytm (7.0 YOE); JD-aligned skills: Pinecone, LLMs, Qdrant.</t>
+          <t>Good fit with caveats: Lead AI Engineer at Razorpay (6.7 YOE); JD-aligned skills: Elasticsearch, Vector Search, Python.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>CAND_0020877</t>
+          <t>CAND_0037566</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -889,19 +889,19 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>0.8798</t>
+          <t>0.9243</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Competitive candidate: Applied ML Engineer at CRED (5.1 YOE); JD-aligned skills: Elasticsearch, OpenSearch, Weaviate.</t>
+          <t>Competitive candidate: Machine Learning Engineer at LinkedIn (6.9 YOE); JD-aligned skills: Pinecone, NLP, LLMs.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>CAND_0046525</t>
+          <t>CAND_0038368</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -909,19 +909,19 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>0.8797</t>
+          <t>0.9223</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Meets several JD signals: Senior Machine Learning Engineer at Genpact AI (6.1 YOE); JD-aligned skills: Elasticsearch, LLMs, NLP.</t>
+          <t>Meets several JD signals: ML Engineer at PhonePe (5.4 YOE); JD-aligned skills: Embeddings, FAISS, NLP.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>CAND_0099806</t>
+          <t>CAND_0009691</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -929,12 +929,12 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>0.8791</t>
+          <t>0.9106</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Solid profile: AI Engineer at Mad Street Den (4.6 YOE); JD-aligned skills: FAISS, Embeddings, Sentence Transformers.</t>
+          <t>Solid profile: Applied ML Engineer at LinkedIn (6.2 YOE); JD-aligned skills: Fine-tuning LLMs, Pinecone, Sentence Transformers. Concerns: 120-day notice period.</t>
         </is>
       </c>
     </row>
@@ -949,7 +949,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>0.8786</t>
+          <t>0.9105</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -961,7 +961,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>CAND_0071939</t>
+          <t>CAND_0079064</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -969,19 +969,19 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>0.8785</t>
+          <t>0.9088</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Competitive candidate: Data Scientist at Krutrim (6.4 YOE); JD-aligned skills: Elasticsearch, OpenSearch, Embeddings.</t>
+          <t>Competitive candidate: Senior Data Scientist at Niramai (5.2 YOE); JD-aligned skills: OpenSearch, NLP, Fine-tuning LLMs. Concerns: 120-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>CAND_0032216</t>
+          <t>CAND_0090584</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -989,19 +989,19 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>0.8783</t>
+          <t>0.9042</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Meets several JD signals: ML Engineer at upGrad (6.1 YOE); JD-aligned skills: Qdrant, Sentence Transformers, Vector Search.</t>
+          <t>Meets several JD signals: ML Engineer at Flipkart (5.1 YOE); JD-aligned skills: Fine-tuning LLMs, OpenSearch, FAISS. Concerns: 120-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>CAND_0037944</t>
+          <t>CAND_0030031</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -1009,19 +1009,19 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>0.8726</t>
+          <t>0.9020</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Solid profile: Senior Data Scientist at Vedantu (4.9 YOE); JD-aligned skills: Vector Search, OpenSearch, Embeddings.</t>
+          <t>Solid profile: AI Engineer at Microsoft (5.7 YOE); JD-aligned skills: Python, NLP, Sentence Transformers.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>CAND_0049538</t>
+          <t>CAND_0089552</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1029,19 +1029,19 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>0.8661</t>
+          <t>0.8970</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Good fit with caveats: Applied ML Engineer at Saarthi.ai (5.8 YOE); JD-aligned skills: OpenSearch, Vector Search, Milvus.</t>
+          <t>Good fit with caveats: Machine Learning Engineer at Netflix (6.0 YOE); JD-aligned skills: Weaviate, Qdrant, Vector Search. Concerns: 120-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>CAND_0044855</t>
+          <t>CAND_0010257</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -1049,19 +1049,19 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>0.8632</t>
+          <t>0.8967</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Competitive candidate: Senior Data Scientist at Flipkart (6.6 YOE); JD-aligned skills: OpenSearch, Pinecone, Vector Search.</t>
+          <t>Competitive candidate: Senior Data Scientist at Google (6.5 YOE); JD-aligned skills: Milvus, Python, OpenSearch. Concerns: 120-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>CAND_0043228</t>
+          <t>CAND_0099806</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1069,19 +1069,19 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>0.8629</t>
+          <t>0.8924</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Meets several JD signals: Applied ML Engineer at Zoho (6.8 YOE); JD-aligned skills: NLP, Vector Search, Sentence Transformers.</t>
+          <t>Meets several JD signals: AI Engineer at Mad Street Den (4.6 YOE); JD-aligned skills: FAISS, Embeddings, Sentence Transformers.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>CAND_0079284</t>
+          <t>CAND_0075574</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -1089,19 +1089,19 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>0.8596</t>
+          <t>0.8903</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Solid profile: Machine Learning Engineer at Google (4.9 YOE); JD-aligned skills: Qdrant, Fine-tuning LLMs, Elasticsearch.</t>
+          <t>Solid profile: Machine Learning Engineer at Haptik (5.7 YOE); JD-aligned skills: Weaviate, OpenSearch, Qdrant.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>CAND_0083879</t>
+          <t>CAND_0032216</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -1109,19 +1109,19 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>0.8596</t>
+          <t>0.8901</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Good fit with caveats: Machine Learning Engineer at Ola (7.1 YOE); JD-aligned skills: Fine-tuning LLMs, Milvus, Sentence Transformers.</t>
+          <t>Good fit with caveats: ML Engineer at upGrad (6.1 YOE); JD-aligned skills: Qdrant, Sentence Transformers, Vector Search.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>CAND_0079387</t>
+          <t>CAND_0037944</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -1129,19 +1129,19 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>0.8548</t>
+          <t>0.8855</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Competitive candidate: AI Engineer at Microsoft (6.9 YOE); JD-aligned skills: Python, Sentence Transformers, Vector Search.</t>
+          <t>Competitive candidate: Senior Data Scientist at Vedantu (4.9 YOE); JD-aligned skills: Vector Search, OpenSearch, Embeddings.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>CAND_0079064</t>
+          <t>CAND_0049538</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -1149,19 +1149,19 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>0.8525</t>
+          <t>0.8796</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Meets several JD signals: Senior Data Scientist at Niramai (5.2 YOE); JD-aligned skills: OpenSearch, NLP, Fine-tuning LLMs. Concerns: 120-day notice period.</t>
+          <t>Meets several JD signals: Applied ML Engineer at Saarthi.ai (5.8 YOE); JD-aligned skills: OpenSearch, Vector Search, Milvus.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>CAND_0086022</t>
+          <t>CAND_0047721</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -1169,19 +1169,19 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>0.8515</t>
+          <t>0.8791</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Solid profile: Senior Applied Scientist at Sarvam AI (5.3 YOE); JD-aligned skills: Vector Search, Fine-tuning LLMs, Elasticsearch.</t>
+          <t>Solid profile: Senior Data Scientist at Microsoft (7.0 YOE); JD-aligned skills: Milvus, FAISS, Qdrant. Concerns: 90-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>CAND_0090584</t>
+          <t>CAND_0042100</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -1189,19 +1189,19 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>0.8506</t>
+          <t>0.8773</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Good fit with caveats: ML Engineer at Flipkart (5.1 YOE); JD-aligned skills: Fine-tuning LLMs, OpenSearch, FAISS. Concerns: 120-day notice period.</t>
+          <t>Good fit with caveats: Machine Learning Engineer at Freshworks (7.3 YOE); JD-aligned skills: Elasticsearch, Fine-tuning LLMs, Pinecone. Concerns: 90-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>CAND_0061257</t>
+          <t>CAND_0043228</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -1209,19 +1209,19 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>0.8474</t>
+          <t>0.8758</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Competitive candidate: Staff Machine Learning Engineer at LinkedIn (8.0 YOE); JD-aligned skills: Python. Concerns: only 1 core JD skill matched.</t>
+          <t>Competitive candidate: Applied ML Engineer at Zoho (6.8 YOE); JD-aligned skills: NLP, Vector Search, Sentence Transformers.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>CAND_0003841</t>
+          <t>CAND_0083879</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -1229,19 +1229,19 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>0.8420</t>
+          <t>0.8736</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Meets several JD signals: ML Engineer at Tech Mahindra (5.0 YOE); JD-aligned skills: Pinecone, Fine-tuning LLMs, Sentence Transformers.</t>
+          <t>Meets several JD signals: Machine Learning Engineer at Ola (7.1 YOE); JD-aligned skills: Fine-tuning LLMs, Milvus, Sentence Transformers.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>CAND_0051004</t>
+          <t>CAND_0003841</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -1249,19 +1249,19 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>0.8409</t>
+          <t>0.8722</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Solid profile: Senior Data Scientist at CRED (4.7 YOE); JD-aligned skills: Embeddings, Qdrant, Fine-tuning LLMs.</t>
+          <t>Solid profile: ML Engineer at Tech Mahindra (5.0 YOE); JD-aligned skills: Pinecone, Fine-tuning LLMs, Sentence Transformers.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>CAND_0010257</t>
+          <t>CAND_0081852</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -1269,19 +1269,19 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>0.8408</t>
+          <t>0.8712</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Good fit with caveats: Senior Data Scientist at Google (6.5 YOE); JD-aligned skills: Milvus, Python, OpenSearch. Concerns: 120-day notice period.</t>
+          <t>Good fit with caveats: Senior Data Scientist at Mad Street Den (5.9 YOE); JD-aligned skills: Milvus, Weaviate, Vector Search.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>CAND_0081852</t>
+          <t>CAND_0079284</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -1289,19 +1289,19 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>0.8396</t>
+          <t>0.8702</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Competitive candidate: Senior Data Scientist at Mad Street Den (5.9 YOE); JD-aligned skills: Milvus, Weaviate, Vector Search.</t>
+          <t>Competitive candidate: Machine Learning Engineer at Google (4.9 YOE); JD-aligned skills: Qdrant, Fine-tuning LLMs, Elasticsearch.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>CAND_0055905</t>
+          <t>CAND_0079387</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -1309,19 +1309,19 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>0.8393</t>
+          <t>0.8678</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Meets several JD signals: Senior Machine Learning Engineer at Flipkart (8.1 YOE); JD-aligned skills: Elasticsearch, Python, LLMs.</t>
+          <t>Meets several JD signals: AI Engineer at Microsoft (6.9 YOE); JD-aligned skills: Python, Sentence Transformers, Vector Search.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>CAND_0091909</t>
+          <t>CAND_0086022</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -1329,19 +1329,19 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>0.8364</t>
+          <t>0.8678</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Solid profile: Machine Learning Engineer at Rephrase.ai (6.9 YOE); JD-aligned skills: LLMs, Pinecone, Qdrant.</t>
+          <t>Solid profile: Senior Applied Scientist at Sarvam AI (5.3 YOE); JD-aligned skills: Vector Search, Fine-tuning LLMs, Elasticsearch.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>CAND_0075574</t>
+          <t>CAND_0040178</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -1349,12 +1349,12 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>0.8357</t>
+          <t>0.8654</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Good fit with caveats: Machine Learning Engineer at Haptik (5.7 YOE); JD-aligned skills: Weaviate, OpenSearch, Qdrant.</t>
+          <t>Good fit with caveats: ML Engineer at Meesho (5.0 YOE); JD-aligned skills: Weaviate, Fine-tuning LLMs, Vector Search.</t>
         </is>
       </c>
     </row>
@@ -1369,7 +1369,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>0.8352</t>
+          <t>0.8633</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -1381,7 +1381,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>CAND_0016163</t>
+          <t>CAND_0035653</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -1389,19 +1389,19 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>0.8304</t>
+          <t>0.8631</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Meets several JD signals: Applied ML Engineer at Dream11 (6.7 YOE); JD-aligned skills: Weaviate, Embeddings, Pinecone. Concerns: 120-day notice period.</t>
+          <t>Meets several JD signals: Data Scientist at Swiggy (5.6 YOE); JD-aligned skills: OpenSearch, Vector Search, Fine-tuning LLMs.</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>CAND_0017093</t>
+          <t>CAND_0093193</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -1409,19 +1409,19 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>0.8271</t>
+          <t>0.8628</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Solid profile: ML Engineer at Zoho (5.9 YOE); JD-aligned skills: LLMs, Embeddings.</t>
+          <t>Solid profile: Senior Machine Learning Engineer at Niramai (7.9 YOE); JD-aligned skills: Qdrant, OpenSearch.</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>CAND_0070398</t>
+          <t>CAND_0061257</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -1429,19 +1429,19 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>0.8271</t>
+          <t>0.8621</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Good fit with caveats: Machine Learning Engineer at Genpact AI (7.2 YOE); JD-aligned skills: FAISS, Embeddings, Python. Concerns: 120-day notice period.</t>
+          <t>Good fit with caveats: Staff Machine Learning Engineer at LinkedIn (8.0 YOE); JD-aligned skills: Python. Concerns: only 1 core JD skill matched.</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>CAND_0098217</t>
+          <t>CAND_0076482</t>
         </is>
       </c>
       <c r="B52" t="n">
@@ -1449,19 +1449,19 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>0.8271</t>
+          <t>0.8605</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Moderate fit: ML Engineer at Glance (6.4 YOE); JD-aligned skills: FAISS, Pinecone. Gaps: under half of JD must-have skills covered.</t>
+          <t>Moderate fit: ML Engineer at Flipkart (6.6 YOE); JD-aligned skills: OpenSearch, Pinecone, Embeddings. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>CAND_0047721</t>
+          <t>CAND_0010149</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -1469,19 +1469,19 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>0.8264</t>
+          <t>0.8561</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Partial alignment: Senior Data Scientist at Microsoft (7.0 YOE); JD-aligned skills: Milvus, FAISS, Qdrant. Gaps: 90-day notice period.</t>
+          <t>Partial alignment: ML Engineer at Glance (6.9 YOE); JD-aligned skills: Milvus, Vector Search, Elasticsearch. Gaps: 90-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>CAND_0052328</t>
+          <t>CAND_0055905</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -1489,19 +1489,19 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>0.8206</t>
+          <t>0.8558</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Acceptable but not standout: Recommendation Systems Engineer at Amazon (6.5 YOE); JD-aligned skills: OpenSearch, Fine-tuning LLMs, Vector Search. Gaps: under half of JD must-have skills covered.</t>
+          <t>Acceptable but not standout: Senior Machine Learning Engineer at Flipkart (8.1 YOE); JD-aligned skills: Elasticsearch, Python, LLMs. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>CAND_0051292</t>
+          <t>CAND_0015578</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -1509,19 +1509,19 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>0.8205</t>
+          <t>0.8557</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Mixed signals: Applied ML Engineer at Freshworks (5.2 YOE); JD-aligned skills: FAISS, LLMs, Vector Search. Gaps: under half of JD must-have skills covered.</t>
+          <t>Mixed signals: AI Engineer at Zoho (5.4 YOE); JD-aligned skills: Embeddings, NLP, Sentence Transformers. Gaps: 90-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>CAND_0036121</t>
+          <t>CAND_0051004</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -1529,19 +1529,19 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>0.8174</t>
+          <t>0.8544</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>JD overlap is thin: ML Engineer at Wysa (5.2 YOE); JD-aligned skills: Embeddings, Vector Search. Gaps: under half of JD must-have skills covered.</t>
+          <t>JD overlap is thin: Senior Data Scientist at CRED (4.7 YOE); JD-aligned skills: Embeddings, Qdrant, Fine-tuning LLMs. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>CAND_0009691</t>
+          <t>CAND_0095528</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -1549,19 +1549,19 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>0.8152</t>
+          <t>0.8539</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Moderate fit: Applied ML Engineer at LinkedIn (6.2 YOE); JD-aligned skills: Fine-tuning LLMs, Pinecone, Sentence Transformers. Gaps: 120-day notice period.</t>
+          <t>Moderate fit: Senior Data Scientist at Netflix (5.3 YOE); JD-aligned skills: OpenSearch, Vector Search, Qdrant. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>CAND_0058688</t>
+          <t>CAND_0051292</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -1569,19 +1569,19 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>0.8141</t>
+          <t>0.8507</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Partial alignment: AI Engineer at Vedantu (6.7 YOE); JD-aligned skills: Embeddings, Milvus. Gaps: under half of JD must-have skills covered.</t>
+          <t>Partial alignment: Applied ML Engineer at Freshworks (5.2 YOE); JD-aligned skills: FAISS, LLMs, Vector Search. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>CAND_0011432</t>
+          <t>CAND_0073982</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -1589,19 +1589,19 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>0.8128</t>
+          <t>0.8500</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Acceptable but not standout: Senior Data Scientist at Amazon (7.6 YOE); JD-aligned skills: OpenSearch, Elasticsearch. Gaps: under half of JD must-have skills covered.</t>
+          <t>Acceptable but not standout: Data Scientist at Dream11 (7.0 YOE); JD-aligned skills: Sentence Transformers, Qdrant, FAISS. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>CAND_0021836</t>
+          <t>CAND_0069905</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -1609,19 +1609,19 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>0.8117</t>
+          <t>0.8499</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Mixed signals: ML Engineer at CRED (6.5 YOE); JD-aligned skills: Vector Search, Elasticsearch, NLP. Gaps: under half of JD must-have skills covered.</t>
+          <t>Mixed signals: Applied ML Engineer at Sarvam AI (6.6 YOE); JD-aligned skills: Sentence Transformers, Python, Weaviate. Gaps: 90-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>CAND_0035653</t>
+          <t>CAND_0036121</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -1629,19 +1629,19 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>0.8114</t>
+          <t>0.8491</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>JD overlap is thin: Data Scientist at Swiggy (5.6 YOE); JD-aligned skills: OpenSearch, Vector Search, Fine-tuning LLMs. Gaps: under half of JD must-have skills covered.</t>
+          <t>JD overlap is thin: ML Engineer at Wysa (5.2 YOE); JD-aligned skills: Embeddings, Vector Search. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>CAND_0040178</t>
+          <t>CAND_0013393</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -1649,19 +1649,19 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>0.8106</t>
+          <t>0.8469</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Moderate fit: ML Engineer at Meesho (5.0 YOE); JD-aligned skills: Weaviate, Fine-tuning LLMs, Vector Search. Gaps: under half of JD must-have skills covered.</t>
+          <t>Moderate fit: ML Engineer at Freshworks (5.3 YOE); JD-aligned skills: Embeddings, Pinecone, Qdrant. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>CAND_0068932</t>
+          <t>CAND_0095213</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -1669,19 +1669,19 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>0.8102</t>
+          <t>0.8469</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Partial alignment: ML Engineer at Krutrim (5.2 YOE); JD-aligned skills: Milvus, OpenSearch. Gaps: under half of JD must-have skills covered.</t>
+          <t>Partial alignment: ML Engineer at Genpact AI (5.1 YOE); JD-aligned skills: Python, Weaviate, Pinecone. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>CAND_0050876</t>
+          <t>CAND_0015582</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -1689,19 +1689,19 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>0.8098</t>
+          <t>0.8468</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Acceptable but not standout: Applied ML Engineer at Freshworks (6.0 YOE); JD-aligned skills: Qdrant, FAISS, OpenSearch. Gaps: 90-day notice period.</t>
+          <t>Acceptable but not standout: ML Engineer at Genpact AI (4.4 YOE); JD-aligned skills: Qdrant, Sentence Transformers, Embeddings. Gaps: 120-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>CAND_0076482</t>
+          <t>CAND_0091909</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -1709,19 +1709,19 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>0.8089</t>
+          <t>0.8468</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Mixed signals: ML Engineer at Flipkart (6.6 YOE); JD-aligned skills: OpenSearch, Pinecone, Embeddings. Gaps: under half of JD must-have skills covered.</t>
+          <t>Mixed signals: Machine Learning Engineer at Rephrase.ai (6.9 YOE); JD-aligned skills: LLMs, Pinecone, Qdrant. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>CAND_0093193</t>
+          <t>CAND_0016163</t>
         </is>
       </c>
       <c r="B66" t="n">
@@ -1729,19 +1729,19 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>0.8068</t>
+          <t>0.8452</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>JD overlap is thin: Senior Machine Learning Engineer at Niramai (7.9 YOE); JD-aligned skills: Qdrant, OpenSearch. Gaps: under half of JD must-have skills covered.</t>
+          <t>JD overlap is thin: Applied ML Engineer at Dream11 (6.7 YOE); JD-aligned skills: Weaviate, Embeddings, Pinecone. Gaps: 120-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>CAND_0015578</t>
+          <t>CAND_0007460</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -1749,19 +1749,19 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>0.8035</t>
+          <t>0.8446</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Moderate fit: AI Engineer at Zoho (5.4 YOE); JD-aligned skills: Embeddings, NLP, Sentence Transformers. Gaps: 90-day notice period.</t>
+          <t>Moderate fit: AI Engineer at Salesforce (4.7 YOE); JD-aligned skills: Embeddings, Weaviate, NLP. Gaps: 120-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>CAND_0005538</t>
+          <t>CAND_0011432</t>
         </is>
       </c>
       <c r="B68" t="n">
@@ -1769,19 +1769,19 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>0.8025</t>
+          <t>0.8405</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Partial alignment: Senior AI Engineer at Adobe (5.9 YOE); JD-aligned skills: Python. Gaps: only 1 core JD skill matched; 90-day notice period.</t>
+          <t>Partial alignment: Senior Data Scientist at Amazon (7.6 YOE); JD-aligned skills: OpenSearch, Elasticsearch. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>CAND_0095528</t>
+          <t>CAND_0068932</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -1789,19 +1789,19 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>0.8021</t>
+          <t>0.8404</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Acceptable but not standout: Senior Data Scientist at Netflix (5.3 YOE); JD-aligned skills: OpenSearch, Vector Search, Qdrant. Gaps: under half of JD must-have skills covered.</t>
+          <t>Acceptable but not standout: ML Engineer at Krutrim (5.2 YOE); JD-aligned skills: Milvus, OpenSearch. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>CAND_0048166</t>
+          <t>CAND_0090155</t>
         </is>
       </c>
       <c r="B70" t="n">
@@ -1809,19 +1809,19 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>0.7998</t>
+          <t>0.8401</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Mixed signals: ML Engineer at Aganitha (5.2 YOE); JD-aligned skills: Pinecone, Milvus, Qdrant. Gaps: under half of JD must-have skills covered.</t>
+          <t>Mixed signals: ML Engineer at Swiggy (5.8 YOE); JD-aligned skills: Milvus, Qdrant, Pinecone. Gaps: 90-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>CAND_0073982</t>
+          <t>CAND_0070398</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -1829,19 +1829,19 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>0.7993</t>
+          <t>0.8390</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>JD overlap is thin: Data Scientist at Dream11 (7.0 YOE); JD-aligned skills: Sentence Transformers, Qdrant, FAISS. Gaps: under half of JD must-have skills covered.</t>
+          <t>JD overlap is thin: Machine Learning Engineer at Genpact AI (7.2 YOE); JD-aligned skills: FAISS, Embeddings, Python. Gaps: 120-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>CAND_0095213</t>
+          <t>CAND_0098217</t>
         </is>
       </c>
       <c r="B72" t="n">
@@ -1849,19 +1849,19 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>0.7966</t>
+          <t>0.8388</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Moderate fit: ML Engineer at Genpact AI (5.1 YOE); JD-aligned skills: Python, Weaviate, Pinecone. Gaps: not flagged open to work.</t>
+          <t>Moderate fit: ML Engineer at Glance (6.4 YOE); JD-aligned skills: FAISS, Pinecone. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>CAND_0069905</t>
+          <t>CAND_0017093</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -1869,19 +1869,19 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>0.7964</t>
+          <t>0.8378</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Partial alignment: Applied ML Engineer at Sarvam AI (6.6 YOE); JD-aligned skills: Sentence Transformers, Python, Weaviate. Gaps: 90-day notice period.</t>
+          <t>Partial alignment: ML Engineer at Zoho (5.9 YOE); JD-aligned skills: LLMs, Embeddings. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>CAND_0013393</t>
+          <t>CAND_0052328</t>
         </is>
       </c>
       <c r="B74" t="n">
@@ -1889,19 +1889,19 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>0.7946</t>
+          <t>0.8331</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Acceptable but not standout: ML Engineer at Freshworks (5.3 YOE); JD-aligned skills: Embeddings, Pinecone, Qdrant. Gaps: under half of JD must-have skills covered.</t>
+          <t>Acceptable but not standout: Recommendation Systems Engineer at Amazon (6.5 YOE); JD-aligned skills: OpenSearch, Fine-tuning LLMs, Vector Search. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>CAND_0001707</t>
+          <t>CAND_0048166</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -1909,19 +1909,19 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>0.7909</t>
+          <t>0.8317</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Mixed signals: Data Scientist at Vedantu (5.6 YOE); JD-aligned skills: Sentence Transformers, FAISS, Weaviate. Gaps: 90-day notice period.</t>
+          <t>Mixed signals: ML Engineer at Aganitha (5.2 YOE); JD-aligned skills: Pinecone, Milvus, Qdrant. Gaps: not flagged open to work.</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>CAND_0005477</t>
+          <t>CAND_0058688</t>
         </is>
       </c>
       <c r="B76" t="n">
@@ -1929,19 +1929,19 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>0.7908</t>
+          <t>0.8288</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>JD overlap is thin: ML Engineer at Zomato (6.2 YOE); JD-aligned skills: OpenSearch. Gaps: only 1 core JD skill matched.</t>
+          <t>JD overlap is thin: AI Engineer at Vedantu (6.7 YOE); JD-aligned skills: Embeddings, Milvus. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>CAND_0055992</t>
+          <t>CAND_0021836</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -1949,19 +1949,19 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>0.7897</t>
+          <t>0.8220</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Moderate fit: AI Engineer at CRED (16.9 YOE); JD-aligned skills: FAISS, OpenSearch, Embeddings. Gaps: experience above target band for this role.</t>
+          <t>Moderate fit: ML Engineer at CRED (6.5 YOE); JD-aligned skills: Vector Search, Elasticsearch, NLP. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>CAND_0005649</t>
+          <t>CAND_0050876</t>
         </is>
       </c>
       <c r="B78" t="n">
@@ -1969,19 +1969,19 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>0.7891</t>
+          <t>0.8217</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Partial alignment: Senior Data Scientist at Sarvam AI (7.4 YOE); JD-aligned skills: Fine-tuning LLMs, Weaviate. Gaps: 90-day notice period.</t>
+          <t>Partial alignment: Applied ML Engineer at Freshworks (6.0 YOE); JD-aligned skills: Qdrant, FAISS, OpenSearch. Gaps: 90-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>CAND_0027723</t>
+          <t>CAND_0005649</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -1989,19 +1989,19 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>0.7889</t>
+          <t>0.8212</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Acceptable but not standout: ML Engineer at Wysa (4.2 YOE); JD-aligned skills: Vector Search, NLP, Elasticsearch. Gaps: under half of JD must-have skills covered.</t>
+          <t>Acceptable but not standout: Senior Data Scientist at Sarvam AI (7.4 YOE); JD-aligned skills: Fine-tuning LLMs, Weaviate. Gaps: 90-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>CAND_0090155</t>
+          <t>CAND_0092245</t>
         </is>
       </c>
       <c r="B80" t="n">
@@ -2009,19 +2009,19 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>0.7881</t>
+          <t>0.8203</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Mixed signals: ML Engineer at Swiggy (5.8 YOE); JD-aligned skills: Milvus, Qdrant, Pinecone. Gaps: 90-day notice period.</t>
+          <t>Mixed signals: Senior Data Scientist at Ola (4.1 YOE); JD-aligned skills: Embeddings, FAISS, Qdrant. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>CAND_0060538</t>
+          <t>CAND_0055992</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -2029,19 +2029,19 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>0.7867</t>
+          <t>0.8191</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>JD overlap is thin: ML Engineer at Verloop.io (5.2 YOE); JD-aligned skills: OpenSearch, Embeddings, Milvus. Gaps: 90-day notice period.</t>
+          <t>JD overlap is thin: AI Engineer at CRED (16.9 YOE); JD-aligned skills: FAISS, OpenSearch, Embeddings. Gaps: experience above target band for this role.</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>CAND_0042100</t>
+          <t>CAND_0005538</t>
         </is>
       </c>
       <c r="B82" t="n">
@@ -2049,19 +2049,19 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>0.7838</t>
+          <t>0.8165</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Moderate fit: Machine Learning Engineer at Freshworks (7.3 YOE); JD-aligned skills: Elasticsearch, Fine-tuning LLMs, Pinecone. Gaps: 90-day notice period.</t>
+          <t>Moderate fit: Senior AI Engineer at Adobe (5.9 YOE); JD-aligned skills: Python. Gaps: only 1 core JD skill matched; 90-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>CAND_0041669</t>
+          <t>CAND_0002037</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -2069,19 +2069,19 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>0.7817</t>
+          <t>0.8119</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Partial alignment: Recommendation Systems Engineer at CRED (8.0 YOE); JD-aligned skills: FAISS, Milvus, Weaviate. Gaps: under half of JD must-have skills covered.</t>
+          <t>Partial alignment: ML Engineer at Locobuzz (5.5 YOE); JD-aligned skills: Fine-tuning LLMs, Milvus, Pinecone. Gaps: not flagged open to work.</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>CAND_0066999</t>
+          <t>CAND_0099269</t>
         </is>
       </c>
       <c r="B84" t="n">
@@ -2089,19 +2089,19 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>0.7800</t>
+          <t>0.8091</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Acceptable but not standout: Recommendation Systems Engineer at Microsoft (5.9 YOE); JD-aligned skills: OpenSearch, FAISS, LLMs. Gaps: under half of JD must-have skills covered.</t>
+          <t>Acceptable but not standout: Data Scientist at BYJU'S (5.5 YOE); JD-aligned skills: Elasticsearch, Python, NLP. Gaps: 120-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>CAND_0060054</t>
+          <t>CAND_0041669</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -2109,19 +2109,19 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>0.7776</t>
+          <t>0.8089</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Mixed signals: AI Engineer at Mad Street Den (6.4 YOE); JD-aligned skills: Weaviate, FAISS, Elasticsearch. Gaps: not flagged open to work.</t>
+          <t>Mixed signals: Recommendation Systems Engineer at CRED (8.0 YOE); JD-aligned skills: FAISS, Milvus, Weaviate. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>CAND_0015528</t>
+          <t>CAND_0094759</t>
         </is>
       </c>
       <c r="B86" t="n">
@@ -2129,19 +2129,19 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>0.7746</t>
+          <t>0.8073</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>JD overlap is thin: Applied ML Engineer at Krutrim (7.4 YOE); JD-aligned skills: Weaviate, OpenSearch, FAISS. Gaps: not flagged open to work.</t>
+          <t>JD overlap is thin: Lead AI Engineer at Meta (8.6 YOE); JD-aligned skills: Qdrant, Fine-tuning LLMs, Vector Search. Gaps: low recruiter response rate; not flagged open to work.</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>CAND_0030348</t>
+          <t>CAND_0060054</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -2149,19 +2149,19 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>0.7722</t>
+          <t>0.8066</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Moderate fit: Machine Learning Engineer at BYJU'S (4.5 YOE); JD-aligned skills: Embeddings, Vector Search, Elasticsearch. Gaps: under half of JD must-have skills covered.</t>
+          <t>Moderate fit: AI Engineer at Mad Street Den (6.4 YOE); JD-aligned skills: Weaviate, FAISS, Elasticsearch. Gaps: not flagged open to work.</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>CAND_0047276</t>
+          <t>CAND_0069232</t>
         </is>
       </c>
       <c r="B88" t="n">
@@ -2169,19 +2169,19 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>0.7711</t>
+          <t>0.8057</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Partial alignment: Backend Engineer at Freshworks (5.5 YOE); JD-aligned skills: Qdrant, Fine-tuning LLMs. Gaps: under half of JD must-have skills covered.</t>
+          <t>Partial alignment: ML Engineer at Yellow.ai (6.3 YOE); JD-aligned skills: Pinecone, NLP, Python. Gaps: 120-day notice period; not flagged open to work.</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>CAND_0010149</t>
+          <t>CAND_0065277</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -2189,19 +2189,19 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>0.7665</t>
+          <t>0.8049</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Acceptable but not standout: ML Engineer at Glance (6.9 YOE); JD-aligned skills: Milvus, Vector Search, Elasticsearch. Gaps: 90-day notice period.</t>
+          <t>Acceptable but not standout: Computer Vision Engineer at Aganitha (6.3 YOE); JD-aligned skills: Vector Search, Milvus, Fine-tuning LLMs. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>CAND_0093912</t>
+          <t>CAND_0006418</t>
         </is>
       </c>
       <c r="B90" t="n">
@@ -2209,19 +2209,19 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>0.7662</t>
+          <t>0.8037</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Mixed signals: Senior Data Scientist at Razorpay (5.3 YOE); JD-aligned skills: Milvus, Embeddings, Vector Search. Gaps: under half of JD must-have skills covered.</t>
+          <t>Mixed signals: Machine Learning Engineer at Verloop.io (5.7 YOE); JD-aligned skills: Embeddings, Weaviate, Elasticsearch. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>CAND_0027691</t>
+          <t>CAND_0064904</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -2229,19 +2229,19 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>0.7637</t>
+          <t>0.8031</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>JD overlap is thin: NLP Engineer at Haptik (6.5 YOE); JD-aligned skills: Weaviate, Embeddings, Python. Gaps: under half of JD must-have skills covered.</t>
+          <t>JD overlap is thin: AI Engineer at LinkedIn (4.9 YOE); JD-aligned skills: Embeddings, Elasticsearch, LLMs. Gaps: 90-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>CAND_0074735</t>
+          <t>CAND_0027723</t>
         </is>
       </c>
       <c r="B92" t="n">
@@ -2249,19 +2249,19 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>0.7629</t>
+          <t>0.8023</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Lower-tier shortlist entry — Applied ML Engineer at Rephrase.ai (5.5 YOE); JD-aligned skills: Weaviate, Vector Search, Elasticsearch. Key gaps: 90-day notice period.</t>
+          <t>Lower-tier shortlist entry — ML Engineer at Wysa (4.2 YOE); JD-aligned skills: Vector Search, NLP, Elasticsearch. Key gaps: weak secondary signals vs higher ranks.</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>CAND_0002037</t>
+          <t>CAND_0061550</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -2269,19 +2269,19 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>0.7611</t>
+          <t>0.8023</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Lower-tier shortlist entry — ML Engineer at Locobuzz (5.5 YOE); JD-aligned skills: Fine-tuning LLMs, Milvus, Pinecone. Key gaps: not flagged open to work.</t>
+          <t>Lower-tier shortlist entry — ML Engineer at Infosys (5.3 YOE); JD-aligned skills: Sentence Transformers. Key gaps: only 1 core JD skill matched.</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>CAND_0099269</t>
+          <t>CAND_0001707</t>
         </is>
       </c>
       <c r="B94" t="n">
@@ -2289,19 +2289,19 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>0.7588</t>
+          <t>0.8019</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Lower-tier shortlist entry — Data Scientist at BYJU'S (5.5 YOE); JD-aligned skills: Elasticsearch, Python, NLP. Key gaps: 120-day notice period.</t>
+          <t>Lower-tier shortlist entry — Data Scientist at Vedantu (5.6 YOE); JD-aligned skills: Sentence Transformers, FAISS, Weaviate. Key gaps: 90-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>CAND_0069232</t>
+          <t>CAND_0005477</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -2309,19 +2309,19 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>0.7580</t>
+          <t>0.8012</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Lower-tier shortlist entry — ML Engineer at Yellow.ai (6.3 YOE); JD-aligned skills: Pinecone, NLP, Python. Key gaps: 120-day notice period; not flagged open to work.</t>
+          <t>Lower-tier shortlist entry — ML Engineer at Zomato (6.2 YOE); JD-aligned skills: OpenSearch. Key gaps: only 1 core JD skill matched.</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>CAND_0015582</t>
+          <t>CAND_0013536</t>
         </is>
       </c>
       <c r="B96" t="n">
@@ -2329,19 +2329,19 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>0.7563</t>
+          <t>0.8009</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Lower-tier shortlist entry — ML Engineer at Genpact AI (4.4 YOE); JD-aligned skills: Qdrant, Sentence Transformers, Embeddings. Key gaps: 120-day notice period.</t>
+          <t>Lower-tier shortlist entry — Applied ML Engineer at Haptik (14.1 YOE); JD-aligned skills: LLMs, NLP, Embeddings. Key gaps: 90-day notice period; experience above target band for this role.</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>CAND_0065277</t>
+          <t>CAND_0015057</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -2349,19 +2349,19 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>0.7561</t>
+          <t>0.7999</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Lower-tier shortlist entry — Computer Vision Engineer at Aganitha (6.3 YOE); JD-aligned skills: Vector Search, Milvus, Fine-tuning LLMs. Key gaps: weak secondary signals vs higher ranks.</t>
+          <t>Lower-tier shortlist entry — ML Engineer at Meesho (4.6 YOE); JD-aligned skills: Sentence Transformers, Vector Search, Embeddings. Key gaps: 90-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>CAND_0006418</t>
+          <t>CAND_0030348</t>
         </is>
       </c>
       <c r="B98" t="n">
@@ -2369,19 +2369,19 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>0.7552</t>
+          <t>0.7992</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Lower-tier shortlist entry — Machine Learning Engineer at Verloop.io (5.7 YOE); JD-aligned skills: Embeddings, Weaviate, Elasticsearch. Key gaps: weak secondary signals vs higher ranks.</t>
+          <t>Lower-tier shortlist entry — Machine Learning Engineer at BYJU'S (4.5 YOE); JD-aligned skills: Embeddings, Vector Search, Elasticsearch. Key gaps: weak secondary signals vs higher ranks.</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>CAND_0094759</t>
+          <t>CAND_0060538</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -2389,19 +2389,19 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>0.7551</t>
+          <t>0.7983</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Lower-tier shortlist entry — Lead AI Engineer at Meta (8.6 YOE); JD-aligned skills: Qdrant, Fine-tuning LLMs, Vector Search. Key gaps: low recruiter response rate; not flagged open to work.</t>
+          <t>Lower-tier shortlist entry — ML Engineer at Verloop.io (5.2 YOE); JD-aligned skills: OpenSearch, Embeddings, Milvus. Key gaps: 90-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>CAND_0065878</t>
+          <t>CAND_0049615</t>
         </is>
       </c>
       <c r="B100" t="n">
@@ -2409,19 +2409,19 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>0.7540</t>
+          <t>0.7961</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Lower-tier shortlist entry — Senior Data Scientist at Niramai (7.8 YOE); JD-aligned skills: Vector Search, Fine-tuning LLMs. Key gaps: weak secondary signals vs higher ranks.</t>
+          <t>Lower-tier shortlist entry — ML Engineer at Krutrim (5.1 YOE); JD-aligned skills: NLP, Pinecone. Key gaps: weak secondary signals vs higher ranks.</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>CAND_0007460</t>
+          <t>CAND_0019159</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -2429,12 +2429,12 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>0.7535</t>
+          <t>0.7956</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Lower-tier shortlist entry — AI Engineer at Salesforce (4.7 YOE); JD-aligned skills: Embeddings, Weaviate, NLP. Key gaps: 120-day notice period.</t>
+          <t>Lower-tier shortlist entry — ML Engineer at Genpact AI (6.1 YOE); JD-aligned skills: Vector Search, Qdrant, Sentence Transformers. Key gaps: not flagged open to work.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: regenerate submission after ranking improvements
</commit_message>
<xml_diff>
--- a/submission.xlsx
+++ b/submission.xlsx
@@ -444,8 +444,10 @@
           <t>CAND_0045250</t>
         </is>
       </c>
-      <c r="B2" t="n">
-        <v>1</v>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -454,7 +456,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Rank 1: Applied ML Engineer at Rephrase.ai (6.6 YOE); JD-aligned skills: Sentence Transformers, Milvus, Embeddings. Top-tier composite score across career, skills, and availability. Counterfactual: trails a perfect match on 13 uncovered JD must-have skill(s).</t>
+          <t>Rank 1: Applied ML Engineer at Rephrase.ai (6.6 YOE); JD-aligned skills: Sentence Transformers, Milvus, Embeddings. Top-tier composite score across career, skills, and availability. Counterfactual: ranks on career trajectory and assessed depth over keyword coverage (7/22 listed must-haves), aligning with the JD anti-keyword-stuffing guidance.</t>
         </is>
       </c>
     </row>
@@ -464,8 +466,10 @@
           <t>CAND_0006567</t>
         </is>
       </c>
-      <c r="B3" t="n">
-        <v>2</v>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -474,7 +478,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Rank 2: Senior AI Engineer at Meta (7.9 YOE); JD-aligned skills: NLP, Python. Top-tier composite score across career, skills, and availability. Counterfactual: trails a perfect match on 18 uncovered JD must-have skill(s).</t>
+          <t>Rank 2: Senior AI Engineer at Meta (7.9 YOE); JD-aligned skills: NLP, Python. Top-tier composite score across career, skills, and availability. Counterfactual: ranks on career trajectory and assessed depth over keyword coverage (2/22 listed must-haves), aligning with the JD anti-keyword-stuffing guidance.</t>
         </is>
       </c>
     </row>
@@ -484,8 +488,10 @@
           <t>CAND_0071974</t>
         </is>
       </c>
-      <c r="B4" t="n">
-        <v>3</v>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -494,87 +500,95 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Rank 3: Senior AI Engineer at Netflix (7.8 YOE); JD-aligned skills: Weaviate, Pinecone, Qdrant. Top-tier composite score across career, skills, and availability. Counterfactual: trails a perfect match on 14 uncovered JD must-have skill(s).</t>
+          <t>Rank 3: Senior AI Engineer at Netflix (7.8 YOE); JD-aligned skills: Weaviate, Pinecone, Qdrant. Top-tier composite score across career, skills, and availability. Counterfactual: ranks on career trajectory and assessed depth over keyword coverage (6/22 listed must-haves), aligning with the JD anti-keyword-stuffing guidance.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>CAND_0096142</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>4</v>
+          <t>CAND_0018499</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>1.0027</t>
+          <t>1.0057</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Rank 4: Applied ML Engineer at upGrad (5.0 YOE); JD-aligned skills: Weaviate, Pinecone, Python. Top-tier composite score across career, skills, and availability. Minor note: 120-day notice period.</t>
+          <t>Rank 4: Senior Machine Learning Engineer at Zomato (7.2 YOE); JD-aligned skills: Weaviate, Pinecone, Milvus. Top-tier composite score across career, skills, and availability. Counterfactual: ranks on career trajectory and assessed depth over keyword coverage (5/22 listed must-haves), aligning with the JD anti-keyword-stuffing guidance.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CAND_0002025</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>5</v>
+          <t>CAND_0096142</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>0.9945</t>
+          <t>1.0027</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Rank 5: Senior AI Engineer at Apple (5.9 YOE); JD-aligned skills: FAISS, OpenSearch, Weaviate. Top-tier composite score across career, skills, and availability. Counterfactual: trails a perfect match on 12 uncovered JD must-have skill(s).</t>
+          <t>Rank 5: Applied ML Engineer at upGrad (5.0 YOE); JD-aligned skills: Weaviate, Pinecone, Python. Top-tier composite score across career, skills, and availability. Minor note: 120-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>CAND_0087630</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>6</v>
+          <t>CAND_0002025</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>0.9906</t>
+          <t>0.9945</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Strong match — AI Engineer at Vedantu (7.2 YOE); JD-aligned skills: Elasticsearch, NLP, Embeddings.</t>
+          <t>Strong match — Senior AI Engineer at Apple (5.9 YOE); JD-aligned skills: FAISS, OpenSearch, Weaviate.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>CAND_0018499</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>7</v>
+          <t>CAND_0087630</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>0.9772</t>
+          <t>0.9906</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Strong match — Senior Machine Learning Engineer at Zomato (7.2 YOE); JD-aligned skills: Weaviate, Pinecone, Milvus.</t>
+          <t>Strong match — AI Engineer at Vedantu (7.2 YOE); JD-aligned skills: Elasticsearch, NLP, Embeddings.</t>
         </is>
       </c>
     </row>
@@ -584,8 +598,10 @@
           <t>CAND_0068351</t>
         </is>
       </c>
-      <c r="B9" t="n">
-        <v>8</v>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -604,8 +620,10 @@
           <t>CAND_0020350</t>
         </is>
       </c>
-      <c r="B10" t="n">
-        <v>9</v>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -624,8 +642,10 @@
           <t>CAND_0068811</t>
         </is>
       </c>
-      <c r="B11" t="n">
-        <v>10</v>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -644,8 +664,10 @@
           <t>CAND_0044855</t>
         </is>
       </c>
-      <c r="B12" t="n">
-        <v>11</v>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -661,1260 +683,1386 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>CAND_0080766</t>
-        </is>
-      </c>
-      <c r="B13" t="n">
-        <v>12</v>
+          <t>CAND_0071939</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>0.9558</t>
+          <t>0.9599</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Strong match — Staff Machine Learning Engineer at Salesforce (8.8 YOE); JD-aligned skills: Elasticsearch, OpenSearch, Python.</t>
+          <t>Strong match — Data Scientist at Krutrim (6.4 YOE); JD-aligned skills: Elasticsearch, OpenSearch, Embeddings.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>CAND_0088025</t>
-        </is>
-      </c>
-      <c r="B14" t="n">
-        <v>13</v>
+          <t>CAND_0080766</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>0.9520</t>
+          <t>0.9558</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Strong match — Staff Machine Learning Engineer at Yellow.ai (8.6 YOE); JD-aligned skills: Pinecone, LLMs, Elasticsearch. Watch: 90-day notice period.</t>
+          <t>Strong match — Staff Machine Learning Engineer at Salesforce (8.8 YOE); JD-aligned skills: Elasticsearch, OpenSearch, Python.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>CAND_0044222</t>
-        </is>
-      </c>
-      <c r="B15" t="n">
-        <v>14</v>
+          <t>CAND_0088025</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>0.9489</t>
+          <t>0.9520</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Strong match — AI Engineer at PolicyBazaar (7.7 YOE); JD-aligned skills: Vector Search, OpenSearch, Qdrant.</t>
+          <t>Strong match — Staff Machine Learning Engineer at Yellow.ai (8.6 YOE); JD-aligned skills: Pinecone, LLMs, Elasticsearch. Watch: 90-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>CAND_0039383</t>
-        </is>
-      </c>
-      <c r="B16" t="n">
-        <v>15</v>
+          <t>CAND_0038368</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>0.9468</t>
+          <t>0.9508</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Strong match — Applied ML Engineer at Meesho (7.1 YOE); JD-aligned skills: FAISS, NLP, Vector Search. Watch: 90-day notice period.</t>
+          <t>Strong match — ML Engineer at PhonePe (5.4 YOE); JD-aligned skills: Embeddings, FAISS, Django.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>CAND_0077337</t>
-        </is>
-      </c>
-      <c r="B17" t="n">
-        <v>16</v>
+          <t>CAND_0044222</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>0.9405</t>
+          <t>0.9489</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Strong match — Staff Machine Learning Engineer at Paytm (7.0 YOE); JD-aligned skills: Pinecone, LLMs, Qdrant.</t>
+          <t>Strong match — AI Engineer at PolicyBazaar (7.7 YOE); JD-aligned skills: Vector Search, OpenSearch, Qdrant.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>CAND_0046525</t>
-        </is>
-      </c>
-      <c r="B18" t="n">
-        <v>17</v>
+          <t>CAND_0039383</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>0.9402</t>
+          <t>0.9468</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Strong match — Senior Machine Learning Engineer at Genpact AI (6.1 YOE); JD-aligned skills: Elasticsearch, LLMs, NLP.</t>
+          <t>Strong match — Applied ML Engineer at Meesho (7.1 YOE); JD-aligned skills: FAISS, NLP, Vector Search. Watch: 90-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>CAND_0042029</t>
-        </is>
-      </c>
-      <c r="B19" t="n">
-        <v>18</v>
+          <t>CAND_0077337</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>0.9382</t>
+          <t>0.9405</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Strong match — Senior Data Scientist at Flipkart (6.5 YOE); JD-aligned skills: NLP, Elasticsearch, Embeddings.</t>
+          <t>Strong match — Staff Machine Learning Engineer at Paytm (7.0 YOE); JD-aligned skills: Pinecone, LLMs, Qdrant.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>CAND_0065514</t>
-        </is>
-      </c>
-      <c r="B20" t="n">
-        <v>19</v>
+          <t>CAND_0046525</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>0.9377</t>
+          <t>0.9402</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Strong match — ML Engineer at Genpact AI (6.6 YOE); JD-aligned skills: Vector Search, Pinecone, Elasticsearch. Watch: 90-day notice period.</t>
+          <t>Strong match — Senior Machine Learning Engineer at Genpact AI (6.1 YOE); JD-aligned skills: Elasticsearch, LLMs, NLP.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>CAND_0020877</t>
-        </is>
-      </c>
-      <c r="B21" t="n">
-        <v>20</v>
+          <t>CAND_0042029</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>0.9367</t>
+          <t>0.9382</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Strong match — Applied ML Engineer at CRED (5.1 YOE); JD-aligned skills: Elasticsearch, OpenSearch, Weaviate.</t>
+          <t>Strong match — Senior Data Scientist at Flipkart (6.5 YOE); JD-aligned skills: NLP, Elasticsearch, Embeddings.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>CAND_0071939</t>
-        </is>
-      </c>
-      <c r="B22" t="n">
-        <v>21</v>
+          <t>CAND_0065514</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>0.9320</t>
+          <t>0.9377</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Solid profile: Data Scientist at Krutrim (6.4 YOE); JD-aligned skills: Elasticsearch, OpenSearch, Embeddings.</t>
+          <t>Solid profile: ML Engineer at Genpact AI (6.6 YOE); JD-aligned skills: Vector Search, Pinecone, Elasticsearch. Concerns: 90-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>CAND_0081846</t>
-        </is>
-      </c>
-      <c r="B23" t="n">
-        <v>22</v>
+          <t>CAND_0020877</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>0.9260</t>
+          <t>0.9367</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Good fit with caveats: Lead AI Engineer at Razorpay (6.7 YOE); JD-aligned skills: Elasticsearch, Vector Search, Python.</t>
+          <t>Good fit with caveats: Applied ML Engineer at CRED (5.1 YOE); JD-aligned skills: Elasticsearch, OpenSearch, Weaviate.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>CAND_0037566</t>
-        </is>
-      </c>
-      <c r="B24" t="n">
-        <v>23</v>
+          <t>CAND_0081846</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>0.9243</t>
+          <t>0.9260</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Competitive candidate: Machine Learning Engineer at LinkedIn (6.9 YOE); JD-aligned skills: Pinecone, NLP, LLMs.</t>
+          <t>Competitive candidate: Lead AI Engineer at Razorpay (6.7 YOE); JD-aligned skills: Elasticsearch, Vector Search, Python.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>CAND_0038368</t>
-        </is>
-      </c>
-      <c r="B25" t="n">
-        <v>24</v>
+          <t>CAND_0037566</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>0.9223</t>
+          <t>0.9243</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Meets several JD signals: ML Engineer at PhonePe (5.4 YOE); JD-aligned skills: Embeddings, FAISS, NLP.</t>
+          <t>Meets several JD signals: Machine Learning Engineer at LinkedIn (6.9 YOE); JD-aligned skills: Pinecone, NLP, LLMs.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>CAND_0009691</t>
-        </is>
-      </c>
-      <c r="B26" t="n">
-        <v>25</v>
+          <t>CAND_0010257</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>0.9106</t>
+          <t>0.9232</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Solid profile: Applied ML Engineer at LinkedIn (6.2 YOE); JD-aligned skills: Fine-tuning LLMs, Pinecone, Sentence Transformers. Concerns: 120-day notice period.</t>
+          <t>Solid profile: Senior Data Scientist at Google (6.5 YOE); JD-aligned skills: Milvus, Python, OpenSearch. Concerns: 120-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>CAND_0050454</t>
-        </is>
-      </c>
-      <c r="B27" t="n">
-        <v>26</v>
+          <t>CAND_0075574</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>0.9105</t>
+          <t>0.9182</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Good fit with caveats: AI Engineer at Rephrase.ai (6.8 YOE); JD-aligned skills: Fine-tuning LLMs, FAISS, Qdrant.</t>
+          <t>Good fit with caveats: Machine Learning Engineer at Haptik (5.7 YOE); JD-aligned skills: Weaviate, OpenSearch, Qdrant.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>CAND_0079064</t>
-        </is>
-      </c>
-      <c r="B28" t="n">
-        <v>27</v>
+          <t>CAND_0009691</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>0.9088</t>
+          <t>0.9106</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Competitive candidate: Senior Data Scientist at Niramai (5.2 YOE); JD-aligned skills: OpenSearch, NLP, Fine-tuning LLMs. Concerns: 120-day notice period.</t>
+          <t>Competitive candidate: Applied ML Engineer at LinkedIn (6.2 YOE); JD-aligned skills: Fine-tuning LLMs, Pinecone, Sentence Transformers. Concerns: 120-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>CAND_0090584</t>
-        </is>
-      </c>
-      <c r="B29" t="n">
-        <v>28</v>
+          <t>CAND_0050454</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>0.9042</t>
+          <t>0.9105</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Meets several JD signals: ML Engineer at Flipkart (5.1 YOE); JD-aligned skills: Fine-tuning LLMs, OpenSearch, FAISS. Concerns: 120-day notice period.</t>
+          <t>Meets several JD signals: AI Engineer at Rephrase.ai (6.8 YOE); JD-aligned skills: Fine-tuning LLMs, FAISS, Qdrant.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>CAND_0030031</t>
-        </is>
-      </c>
-      <c r="B30" t="n">
-        <v>29</v>
+          <t>CAND_0079064</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>0.9020</t>
+          <t>0.9088</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Solid profile: AI Engineer at Microsoft (5.7 YOE); JD-aligned skills: Python, NLP, Sentence Transformers.</t>
+          <t>Solid profile: Senior Data Scientist at Niramai (5.2 YOE); JD-aligned skills: OpenSearch, NLP, Fine-tuning LLMs. Concerns: 120-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>CAND_0089552</t>
-        </is>
-      </c>
-      <c r="B31" t="n">
-        <v>30</v>
+          <t>CAND_0090584</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>0.8970</t>
+          <t>0.9042</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Good fit with caveats: Machine Learning Engineer at Netflix (6.0 YOE); JD-aligned skills: Weaviate, Qdrant, Vector Search. Concerns: 120-day notice period.</t>
+          <t>Good fit with caveats: ML Engineer at Flipkart (5.1 YOE); JD-aligned skills: Fine-tuning LLMs, OpenSearch, FAISS. Concerns: 120-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>CAND_0010257</t>
-        </is>
-      </c>
-      <c r="B32" t="n">
-        <v>31</v>
+          <t>CAND_0030031</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>0.8967</t>
+          <t>0.9020</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Competitive candidate: Senior Data Scientist at Google (6.5 YOE); JD-aligned skills: Milvus, Python, OpenSearch. Concerns: 120-day notice period.</t>
+          <t>Competitive candidate: AI Engineer at Microsoft (5.7 YOE); JD-aligned skills: Python, NLP, Sentence Transformers.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>CAND_0099806</t>
-        </is>
-      </c>
-      <c r="B33" t="n">
-        <v>32</v>
+          <t>CAND_0089552</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>0.8924</t>
+          <t>0.8970</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Meets several JD signals: AI Engineer at Mad Street Den (4.6 YOE); JD-aligned skills: FAISS, Embeddings, Sentence Transformers.</t>
+          <t>Meets several JD signals: Machine Learning Engineer at Netflix (6.0 YOE); JD-aligned skills: Weaviate, Qdrant, Vector Search. Concerns: 120-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>CAND_0075574</t>
-        </is>
-      </c>
-      <c r="B34" t="n">
-        <v>33</v>
+          <t>CAND_0099806</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>0.8903</t>
+          <t>0.8924</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Solid profile: Machine Learning Engineer at Haptik (5.7 YOE); JD-aligned skills: Weaviate, OpenSearch, Qdrant.</t>
+          <t>Solid profile: AI Engineer at Mad Street Den (4.6 YOE); JD-aligned skills: FAISS, Embeddings, Sentence Transformers.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>CAND_0032216</t>
-        </is>
-      </c>
-      <c r="B35" t="n">
-        <v>34</v>
+          <t>CAND_0093193</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>0.8901</t>
+          <t>0.8907</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Good fit with caveats: ML Engineer at upGrad (6.1 YOE); JD-aligned skills: Qdrant, Sentence Transformers, Vector Search.</t>
+          <t>Good fit with caveats: Senior Machine Learning Engineer at Niramai (7.9 YOE); JD-aligned skills: Indexing Algorithms, Qdrant, OpenSearch.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>CAND_0037944</t>
-        </is>
-      </c>
-      <c r="B36" t="n">
-        <v>35</v>
+          <t>CAND_0061257</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>0.8855</t>
+          <t>0.8905</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Competitive candidate: Senior Data Scientist at Vedantu (4.9 YOE); JD-aligned skills: Vector Search, OpenSearch, Embeddings.</t>
+          <t>Competitive candidate: Staff Machine Learning Engineer at LinkedIn (8.0 YOE); JD-aligned skills: Indexing Algorithms, Python.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>CAND_0049538</t>
-        </is>
-      </c>
-      <c r="B37" t="n">
-        <v>36</v>
+          <t>CAND_0032216</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>0.8796</t>
+          <t>0.8901</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Meets several JD signals: Applied ML Engineer at Saarthi.ai (5.8 YOE); JD-aligned skills: OpenSearch, Vector Search, Milvus.</t>
+          <t>Meets several JD signals: ML Engineer at upGrad (6.1 YOE); JD-aligned skills: Qdrant, Sentence Transformers, Vector Search.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>CAND_0047721</t>
-        </is>
-      </c>
-      <c r="B38" t="n">
-        <v>37</v>
+          <t>CAND_0048166</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>37</t>
+        </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>0.8791</t>
+          <t>0.8885</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Solid profile: Senior Data Scientist at Microsoft (7.0 YOE); JD-aligned skills: Milvus, FAISS, Qdrant. Concerns: 90-day notice period.</t>
+          <t>Solid profile: ML Engineer at Aganitha (5.2 YOE); JD-aligned skills: MongoDB, Pinecone, Rust.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>CAND_0042100</t>
-        </is>
-      </c>
-      <c r="B39" t="n">
-        <v>38</v>
+          <t>CAND_0037944</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>0.8773</t>
+          <t>0.8855</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Good fit with caveats: Machine Learning Engineer at Freshworks (7.3 YOE); JD-aligned skills: Elasticsearch, Fine-tuning LLMs, Pinecone. Concerns: 90-day notice period.</t>
+          <t>Good fit with caveats: Senior Data Scientist at Vedantu (4.9 YOE); JD-aligned skills: Vector Search, OpenSearch, Embeddings.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>CAND_0043228</t>
-        </is>
-      </c>
-      <c r="B40" t="n">
-        <v>39</v>
+          <t>CAND_0015578</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>0.8758</t>
+          <t>0.8810</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Competitive candidate: Applied ML Engineer at Zoho (6.8 YOE); JD-aligned skills: NLP, Vector Search, Sentence Transformers.</t>
+          <t>Competitive candidate: AI Engineer at Zoho (5.4 YOE); JD-aligned skills: Embeddings, NLP, Sentence Transformers. Concerns: 90-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>CAND_0083879</t>
-        </is>
-      </c>
-      <c r="B41" t="n">
-        <v>40</v>
+          <t>CAND_0049538</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>0.8736</t>
+          <t>0.8796</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Meets several JD signals: Machine Learning Engineer at Ola (7.1 YOE); JD-aligned skills: Fine-tuning LLMs, Milvus, Sentence Transformers.</t>
+          <t>Meets several JD signals: Applied ML Engineer at Saarthi.ai (5.8 YOE); JD-aligned skills: OpenSearch, Vector Search, Milvus.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>CAND_0003841</t>
-        </is>
-      </c>
-      <c r="B42" t="n">
-        <v>41</v>
+          <t>CAND_0047721</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>41</t>
+        </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>0.8722</t>
+          <t>0.8791</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Solid profile: ML Engineer at Tech Mahindra (5.0 YOE); JD-aligned skills: Pinecone, Fine-tuning LLMs, Sentence Transformers.</t>
+          <t>Solid profile: Senior Data Scientist at Microsoft (7.0 YOE); JD-aligned skills: Milvus, FAISS, Qdrant. Concerns: 90-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>CAND_0081852</t>
-        </is>
-      </c>
-      <c r="B43" t="n">
-        <v>42</v>
+          <t>CAND_0042100</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>0.8712</t>
+          <t>0.8773</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Good fit with caveats: Senior Data Scientist at Mad Street Den (5.9 YOE); JD-aligned skills: Milvus, Weaviate, Vector Search.</t>
+          <t>Good fit with caveats: Machine Learning Engineer at Freshworks (7.3 YOE); JD-aligned skills: Elasticsearch, Fine-tuning LLMs, Pinecone. Concerns: 90-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>CAND_0079284</t>
-        </is>
-      </c>
-      <c r="B44" t="n">
-        <v>43</v>
+          <t>CAND_0043228</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>43</t>
+        </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>0.8702</t>
+          <t>0.8758</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Competitive candidate: Machine Learning Engineer at Google (4.9 YOE); JD-aligned skills: Qdrant, Fine-tuning LLMs, Elasticsearch.</t>
+          <t>Competitive candidate: Applied ML Engineer at Zoho (6.8 YOE); JD-aligned skills: NLP, Vector Search, Sentence Transformers.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>CAND_0079387</t>
-        </is>
-      </c>
-      <c r="B45" t="n">
-        <v>44</v>
+          <t>CAND_0083879</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>0.8678</t>
+          <t>0.8736</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Meets several JD signals: AI Engineer at Microsoft (6.9 YOE); JD-aligned skills: Python, Sentence Transformers, Vector Search.</t>
+          <t>Meets several JD signals: Machine Learning Engineer at Ola (7.1 YOE); JD-aligned skills: Fine-tuning LLMs, Milvus, Sentence Transformers.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>CAND_0086022</t>
-        </is>
-      </c>
-      <c r="B46" t="n">
-        <v>45</v>
+          <t>CAND_0007460</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>0.8678</t>
+          <t>0.8728</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Solid profile: Senior Applied Scientist at Sarvam AI (5.3 YOE); JD-aligned skills: Vector Search, Fine-tuning LLMs, Elasticsearch.</t>
+          <t>Solid profile: AI Engineer at Salesforce (4.7 YOE); JD-aligned skills: Embeddings, Weaviate, Go. Concerns: 120-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>CAND_0040178</t>
-        </is>
-      </c>
-      <c r="B47" t="n">
-        <v>46</v>
+          <t>CAND_0003841</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>46</t>
+        </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>0.8654</t>
+          <t>0.8722</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Good fit with caveats: ML Engineer at Meesho (5.0 YOE); JD-aligned skills: Weaviate, Fine-tuning LLMs, Vector Search.</t>
+          <t>Good fit with caveats: ML Engineer at Tech Mahindra (5.0 YOE); JD-aligned skills: Pinecone, Fine-tuning LLMs, Sentence Transformers.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>CAND_0018094</t>
-        </is>
-      </c>
-      <c r="B48" t="n">
-        <v>47</v>
+          <t>CAND_0081852</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>47</t>
+        </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>0.8633</t>
+          <t>0.8712</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Competitive candidate: ML Engineer at Mad Street Den (5.2 YOE); JD-aligned skills: Pinecone, Fine-tuning LLMs.</t>
+          <t>Competitive candidate: Senior Data Scientist at Mad Street Den (5.9 YOE); JD-aligned skills: Milvus, Weaviate, Vector Search.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>CAND_0035653</t>
-        </is>
-      </c>
-      <c r="B49" t="n">
-        <v>48</v>
+          <t>CAND_0079284</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>48</t>
+        </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>0.8631</t>
+          <t>0.8702</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Meets several JD signals: Data Scientist at Swiggy (5.6 YOE); JD-aligned skills: OpenSearch, Vector Search, Fine-tuning LLMs.</t>
+          <t>Meets several JD signals: Machine Learning Engineer at Google (4.9 YOE); JD-aligned skills: Qdrant, Fine-tuning LLMs, Elasticsearch.</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>CAND_0093193</t>
-        </is>
-      </c>
-      <c r="B50" t="n">
-        <v>49</v>
+          <t>CAND_0079387</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>49</t>
+        </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>0.8628</t>
+          <t>0.8678</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Solid profile: Senior Machine Learning Engineer at Niramai (7.9 YOE); JD-aligned skills: Qdrant, OpenSearch.</t>
+          <t>Solid profile: AI Engineer at Microsoft (6.9 YOE); JD-aligned skills: Python, Sentence Transformers, Vector Search.</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>CAND_0061257</t>
-        </is>
-      </c>
-      <c r="B51" t="n">
-        <v>50</v>
+          <t>CAND_0086022</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>0.8621</t>
+          <t>0.8678</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Good fit with caveats: Staff Machine Learning Engineer at LinkedIn (8.0 YOE); JD-aligned skills: Python. Concerns: only 1 core JD skill matched.</t>
+          <t>Good fit with caveats: Senior Applied Scientist at Sarvam AI (5.3 YOE); JD-aligned skills: Vector Search, Fine-tuning LLMs, Elasticsearch.</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>CAND_0076482</t>
-        </is>
-      </c>
-      <c r="B52" t="n">
-        <v>51</v>
+          <t>CAND_0040178</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>51</t>
+        </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>0.8605</t>
+          <t>0.8654</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Moderate fit: ML Engineer at Flipkart (6.6 YOE); JD-aligned skills: OpenSearch, Pinecone, Embeddings. Gaps: under half of JD must-have skills covered.</t>
+          <t>Moderate fit: ML Engineer at Meesho (5.0 YOE); JD-aligned skills: Weaviate, Fine-tuning LLMs, Vector Search. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>CAND_0010149</t>
-        </is>
-      </c>
-      <c r="B53" t="n">
-        <v>52</v>
+          <t>CAND_0018094</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>52</t>
+        </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>0.8561</t>
+          <t>0.8633</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Partial alignment: ML Engineer at Glance (6.9 YOE); JD-aligned skills: Milvus, Vector Search, Elasticsearch. Gaps: 90-day notice period.</t>
+          <t>Partial alignment: ML Engineer at Mad Street Den (5.2 YOE); JD-aligned skills: Pinecone, Fine-tuning LLMs. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>CAND_0055905</t>
-        </is>
-      </c>
-      <c r="B54" t="n">
-        <v>53</v>
+          <t>CAND_0035653</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>53</t>
+        </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>0.8558</t>
+          <t>0.8631</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Acceptable but not standout: Senior Machine Learning Engineer at Flipkart (8.1 YOE); JD-aligned skills: Elasticsearch, Python, LLMs. Gaps: under half of JD must-have skills covered.</t>
+          <t>Acceptable but not standout: Data Scientist at Swiggy (5.6 YOE); JD-aligned skills: OpenSearch, Vector Search, Fine-tuning LLMs. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>CAND_0015578</t>
-        </is>
-      </c>
-      <c r="B55" t="n">
-        <v>54</v>
+          <t>CAND_0076482</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>54</t>
+        </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>0.8557</t>
+          <t>0.8605</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Mixed signals: AI Engineer at Zoho (5.4 YOE); JD-aligned skills: Embeddings, NLP, Sentence Transformers. Gaps: 90-day notice period.</t>
+          <t>Mixed signals: ML Engineer at Flipkart (6.6 YOE); JD-aligned skills: OpenSearch, Pinecone, Embeddings. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>CAND_0051004</t>
-        </is>
-      </c>
-      <c r="B56" t="n">
-        <v>55</v>
+          <t>CAND_0010149</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>0.8544</t>
+          <t>0.8561</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>JD overlap is thin: Senior Data Scientist at CRED (4.7 YOE); JD-aligned skills: Embeddings, Qdrant, Fine-tuning LLMs. Gaps: under half of JD must-have skills covered.</t>
+          <t>JD overlap is thin: ML Engineer at Glance (6.9 YOE); JD-aligned skills: Milvus, Vector Search, Elasticsearch. Gaps: 90-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>CAND_0095528</t>
-        </is>
-      </c>
-      <c r="B57" t="n">
-        <v>56</v>
+          <t>CAND_0055905</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>0.8539</t>
+          <t>0.8558</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Moderate fit: Senior Data Scientist at Netflix (5.3 YOE); JD-aligned skills: OpenSearch, Vector Search, Qdrant. Gaps: under half of JD must-have skills covered.</t>
+          <t>Moderate fit: Senior Machine Learning Engineer at Flipkart (8.1 YOE); JD-aligned skills: Elasticsearch, Python, LLMs. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>CAND_0051292</t>
-        </is>
-      </c>
-      <c r="B58" t="n">
-        <v>57</v>
+          <t>CAND_0051004</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>57</t>
+        </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>0.8507</t>
+          <t>0.8544</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Partial alignment: Applied ML Engineer at Freshworks (5.2 YOE); JD-aligned skills: FAISS, LLMs, Vector Search. Gaps: under half of JD must-have skills covered.</t>
+          <t>Partial alignment: Senior Data Scientist at CRED (4.7 YOE); JD-aligned skills: Embeddings, Qdrant, Fine-tuning LLMs. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>CAND_0073982</t>
-        </is>
-      </c>
-      <c r="B59" t="n">
-        <v>58</v>
+          <t>CAND_0095528</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>58</t>
+        </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>0.8500</t>
+          <t>0.8539</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Acceptable but not standout: Data Scientist at Dream11 (7.0 YOE); JD-aligned skills: Sentence Transformers, Qdrant, FAISS. Gaps: under half of JD must-have skills covered.</t>
+          <t>Acceptable but not standout: Senior Data Scientist at Netflix (5.3 YOE); JD-aligned skills: OpenSearch, Vector Search, Qdrant. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>CAND_0069905</t>
-        </is>
-      </c>
-      <c r="B60" t="n">
-        <v>59</v>
+          <t>CAND_0051292</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>59</t>
+        </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>0.8499</t>
+          <t>0.8507</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Mixed signals: Applied ML Engineer at Sarvam AI (6.6 YOE); JD-aligned skills: Sentence Transformers, Python, Weaviate. Gaps: 90-day notice period.</t>
+          <t>Mixed signals: Applied ML Engineer at Freshworks (5.2 YOE); JD-aligned skills: FAISS, LLMs, Vector Search. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>CAND_0036121</t>
-        </is>
-      </c>
-      <c r="B61" t="n">
-        <v>60</v>
+          <t>CAND_0073982</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>0.8491</t>
+          <t>0.8500</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>JD overlap is thin: ML Engineer at Wysa (5.2 YOE); JD-aligned skills: Embeddings, Vector Search. Gaps: under half of JD must-have skills covered.</t>
+          <t>JD overlap is thin: Data Scientist at Dream11 (7.0 YOE); JD-aligned skills: Sentence Transformers, Qdrant, FAISS. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>CAND_0013393</t>
-        </is>
-      </c>
-      <c r="B62" t="n">
-        <v>61</v>
+          <t>CAND_0069905</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>0.8469</t>
+          <t>0.8499</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Moderate fit: ML Engineer at Freshworks (5.3 YOE); JD-aligned skills: Embeddings, Pinecone, Qdrant. Gaps: under half of JD must-have skills covered.</t>
+          <t>Moderate fit: Applied ML Engineer at Sarvam AI (6.6 YOE); JD-aligned skills: Sentence Transformers, Python, Weaviate. Gaps: 90-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>CAND_0095213</t>
-        </is>
-      </c>
-      <c r="B63" t="n">
-        <v>62</v>
+          <t>CAND_0036121</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>62</t>
+        </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>0.8469</t>
+          <t>0.8491</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Partial alignment: ML Engineer at Genpact AI (5.1 YOE); JD-aligned skills: Python, Weaviate, Pinecone. Gaps: under half of JD must-have skills covered.</t>
+          <t>Partial alignment: ML Engineer at Wysa (5.2 YOE); JD-aligned skills: Embeddings, Vector Search. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>CAND_0015582</t>
-        </is>
-      </c>
-      <c r="B64" t="n">
-        <v>63</v>
+          <t>CAND_0013393</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>63</t>
+        </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>0.8468</t>
+          <t>0.8469</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Acceptable but not standout: ML Engineer at Genpact AI (4.4 YOE); JD-aligned skills: Qdrant, Sentence Transformers, Embeddings. Gaps: 120-day notice period.</t>
+          <t>Acceptable but not standout: ML Engineer at Freshworks (5.3 YOE); JD-aligned skills: Embeddings, Pinecone, Qdrant. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>CAND_0091909</t>
-        </is>
-      </c>
-      <c r="B65" t="n">
-        <v>64</v>
+          <t>CAND_0095213</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>64</t>
+        </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>0.8468</t>
+          <t>0.8469</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Mixed signals: Machine Learning Engineer at Rephrase.ai (6.9 YOE); JD-aligned skills: LLMs, Pinecone, Qdrant. Gaps: under half of JD must-have skills covered.</t>
+          <t>Mixed signals: ML Engineer at Genpact AI (5.1 YOE); JD-aligned skills: Python, Weaviate, Pinecone. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>CAND_0016163</t>
-        </is>
-      </c>
-      <c r="B66" t="n">
-        <v>65</v>
+          <t>CAND_0015582</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>65</t>
+        </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>0.8452</t>
+          <t>0.8468</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>JD overlap is thin: Applied ML Engineer at Dream11 (6.7 YOE); JD-aligned skills: Weaviate, Embeddings, Pinecone. Gaps: 120-day notice period.</t>
+          <t>JD overlap is thin: ML Engineer at Genpact AI (4.4 YOE); JD-aligned skills: Qdrant, Sentence Transformers, Embeddings. Gaps: 120-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>CAND_0007460</t>
-        </is>
-      </c>
-      <c r="B67" t="n">
-        <v>66</v>
+          <t>CAND_0091909</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>66</t>
+        </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>0.8446</t>
+          <t>0.8468</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Moderate fit: AI Engineer at Salesforce (4.7 YOE); JD-aligned skills: Embeddings, Weaviate, NLP. Gaps: 120-day notice period.</t>
+          <t>Moderate fit: Machine Learning Engineer at Rephrase.ai (6.9 YOE); JD-aligned skills: LLMs, Pinecone, Qdrant. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>CAND_0011432</t>
-        </is>
-      </c>
-      <c r="B68" t="n">
-        <v>67</v>
+          <t>CAND_0016163</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>67</t>
+        </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>0.8405</t>
+          <t>0.8452</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Partial alignment: Senior Data Scientist at Amazon (7.6 YOE); JD-aligned skills: OpenSearch, Elasticsearch. Gaps: under half of JD must-have skills covered.</t>
+          <t>Partial alignment: Applied ML Engineer at Dream11 (6.7 YOE); JD-aligned skills: Weaviate, Embeddings, Pinecone. Gaps: 120-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>CAND_0068932</t>
-        </is>
-      </c>
-      <c r="B69" t="n">
-        <v>68</v>
+          <t>CAND_0011432</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>0.8404</t>
+          <t>0.8405</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Acceptable but not standout: ML Engineer at Krutrim (5.2 YOE); JD-aligned skills: Milvus, OpenSearch. Gaps: under half of JD must-have skills covered.</t>
+          <t>Acceptable but not standout: Senior Data Scientist at Amazon (7.6 YOE); JD-aligned skills: OpenSearch, Elasticsearch. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>CAND_0090155</t>
-        </is>
-      </c>
-      <c r="B70" t="n">
-        <v>69</v>
+          <t>CAND_0068932</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>69</t>
+        </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>0.8401</t>
+          <t>0.8404</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Mixed signals: ML Engineer at Swiggy (5.8 YOE); JD-aligned skills: Milvus, Qdrant, Pinecone. Gaps: 90-day notice period.</t>
+          <t>Mixed signals: ML Engineer at Krutrim (5.2 YOE); JD-aligned skills: Milvus, OpenSearch. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>CAND_0070398</t>
-        </is>
-      </c>
-      <c r="B71" t="n">
-        <v>70</v>
+          <t>CAND_0090155</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>0.8390</t>
+          <t>0.8401</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>JD overlap is thin: Machine Learning Engineer at Genpact AI (7.2 YOE); JD-aligned skills: FAISS, Embeddings, Python. Gaps: 120-day notice period.</t>
+          <t>JD overlap is thin: ML Engineer at Swiggy (5.8 YOE); JD-aligned skills: Milvus, Qdrant, Pinecone. Gaps: 90-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>CAND_0098217</t>
-        </is>
-      </c>
-      <c r="B72" t="n">
-        <v>71</v>
+          <t>CAND_0070398</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>71</t>
+        </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>0.8388</t>
+          <t>0.8390</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Moderate fit: ML Engineer at Glance (6.4 YOE); JD-aligned skills: FAISS, Pinecone. Gaps: under half of JD must-have skills covered.</t>
+          <t>Moderate fit: Machine Learning Engineer at Genpact AI (7.2 YOE); JD-aligned skills: FAISS, Embeddings, Python. Gaps: 120-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>CAND_0017093</t>
-        </is>
-      </c>
-      <c r="B73" t="n">
-        <v>72</v>
+          <t>CAND_0098217</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>0.8378</t>
+          <t>0.8388</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Partial alignment: ML Engineer at Zoho (5.9 YOE); JD-aligned skills: LLMs, Embeddings. Gaps: under half of JD must-have skills covered.</t>
+          <t>Partial alignment: ML Engineer at Glance (6.4 YOE); JD-aligned skills: FAISS, Pinecone. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>CAND_0052328</t>
-        </is>
-      </c>
-      <c r="B74" t="n">
-        <v>73</v>
+          <t>CAND_0017093</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>73</t>
+        </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>0.8331</t>
+          <t>0.8378</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Acceptable but not standout: Recommendation Systems Engineer at Amazon (6.5 YOE); JD-aligned skills: OpenSearch, Fine-tuning LLMs, Vector Search. Gaps: under half of JD must-have skills covered.</t>
+          <t>Acceptable but not standout: ML Engineer at Zoho (5.9 YOE); JD-aligned skills: LLMs, Embeddings. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>CAND_0048166</t>
-        </is>
-      </c>
-      <c r="B75" t="n">
-        <v>74</v>
+          <t>CAND_0052328</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>74</t>
+        </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>0.8317</t>
+          <t>0.8331</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Mixed signals: ML Engineer at Aganitha (5.2 YOE); JD-aligned skills: Pinecone, Milvus, Qdrant. Gaps: not flagged open to work.</t>
+          <t>Mixed signals: Recommendation Systems Engineer at Amazon (6.5 YOE); JD-aligned skills: OpenSearch, Fine-tuning LLMs, Vector Search. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
@@ -1924,8 +2072,10 @@
           <t>CAND_0058688</t>
         </is>
       </c>
-      <c r="B76" t="n">
-        <v>75</v>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>75</t>
+        </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
@@ -1941,500 +2091,550 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>CAND_0021836</t>
-        </is>
-      </c>
-      <c r="B77" t="n">
-        <v>76</v>
+          <t>CAND_0060538</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>76</t>
+        </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>0.8220</t>
+          <t>0.8235</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Moderate fit: ML Engineer at CRED (6.5 YOE); JD-aligned skills: Vector Search, Elasticsearch, NLP. Gaps: under half of JD must-have skills covered.</t>
+          <t>Moderate fit: ML Engineer at Verloop.io (5.2 YOE); JD-aligned skills: OpenSearch, Embeddings, Rust. Gaps: 90-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>CAND_0050876</t>
-        </is>
-      </c>
-      <c r="B78" t="n">
-        <v>77</v>
+          <t>CAND_0021836</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>77</t>
+        </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>0.8217</t>
+          <t>0.8220</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Partial alignment: Applied ML Engineer at Freshworks (6.0 YOE); JD-aligned skills: Qdrant, FAISS, OpenSearch. Gaps: 90-day notice period.</t>
+          <t>Partial alignment: ML Engineer at CRED (6.5 YOE); JD-aligned skills: Vector Search, Elasticsearch, NLP. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>CAND_0005649</t>
-        </is>
-      </c>
-      <c r="B79" t="n">
-        <v>78</v>
+          <t>CAND_0050876</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>78</t>
+        </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>0.8212</t>
+          <t>0.8217</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Acceptable but not standout: Senior Data Scientist at Sarvam AI (7.4 YOE); JD-aligned skills: Fine-tuning LLMs, Weaviate. Gaps: 90-day notice period.</t>
+          <t>Acceptable but not standout: Applied ML Engineer at Freshworks (6.0 YOE); JD-aligned skills: Qdrant, FAISS, OpenSearch. Gaps: 90-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>CAND_0092245</t>
-        </is>
-      </c>
-      <c r="B80" t="n">
-        <v>79</v>
+          <t>CAND_0005649</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>79</t>
+        </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>0.8203</t>
+          <t>0.8212</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Mixed signals: Senior Data Scientist at Ola (4.1 YOE); JD-aligned skills: Embeddings, FAISS, Qdrant. Gaps: under half of JD must-have skills covered.</t>
+          <t>Mixed signals: Senior Data Scientist at Sarvam AI (7.4 YOE); JD-aligned skills: Fine-tuning LLMs, Weaviate. Gaps: 90-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>CAND_0055992</t>
-        </is>
-      </c>
-      <c r="B81" t="n">
-        <v>80</v>
+          <t>CAND_0092245</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>80</t>
+        </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>0.8191</t>
+          <t>0.8205</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>JD overlap is thin: AI Engineer at CRED (16.9 YOE); JD-aligned skills: FAISS, OpenSearch, Embeddings. Gaps: experience above target band for this role.</t>
+          <t>JD overlap is thin: Senior Data Scientist at Ola (4.1 YOE); JD-aligned skills: Embeddings, FAISS, Qdrant. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>CAND_0005538</t>
-        </is>
-      </c>
-      <c r="B82" t="n">
-        <v>81</v>
+          <t>CAND_0055992</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>81</t>
+        </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>0.8165</t>
+          <t>0.8191</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Moderate fit: Senior AI Engineer at Adobe (5.9 YOE); JD-aligned skills: Python. Gaps: only 1 core JD skill matched; 90-day notice period.</t>
+          <t>Moderate fit: AI Engineer at CRED (16.9 YOE); JD-aligned skills: FAISS, OpenSearch, Embeddings. Gaps: experience above target band for this role.</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>CAND_0002037</t>
-        </is>
-      </c>
-      <c r="B83" t="n">
-        <v>82</v>
+          <t>CAND_0005538</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>82</t>
+        </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>0.8119</t>
+          <t>0.8165</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Partial alignment: ML Engineer at Locobuzz (5.5 YOE); JD-aligned skills: Fine-tuning LLMs, Milvus, Pinecone. Gaps: not flagged open to work.</t>
+          <t>Partial alignment: Senior AI Engineer at Adobe (5.9 YOE); JD-aligned skills: Python. Gaps: only 1 core JD skill matched; 90-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>CAND_0099269</t>
-        </is>
-      </c>
-      <c r="B84" t="n">
-        <v>83</v>
+          <t>CAND_0047276</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>83</t>
+        </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>0.8091</t>
+          <t>0.8131</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Acceptable but not standout: Data Scientist at BYJU'S (5.5 YOE); JD-aligned skills: Elasticsearch, Python, NLP. Gaps: 120-day notice period.</t>
+          <t>Acceptable but not standout: Backend Engineer at Freshworks (5.5 YOE); JD-aligned skills: Qdrant, Fine-tuning LLMs, Go. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>CAND_0041669</t>
-        </is>
-      </c>
-      <c r="B85" t="n">
-        <v>84</v>
+          <t>CAND_0002037</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>84</t>
+        </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>0.8089</t>
+          <t>0.8119</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Mixed signals: Recommendation Systems Engineer at CRED (8.0 YOE); JD-aligned skills: FAISS, Milvus, Weaviate. Gaps: under half of JD must-have skills covered.</t>
+          <t>Mixed signals: ML Engineer at Locobuzz (5.5 YOE); JD-aligned skills: Fine-tuning LLMs, Milvus, Pinecone. Gaps: not flagged open to work.</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>CAND_0094759</t>
-        </is>
-      </c>
-      <c r="B86" t="n">
-        <v>85</v>
+          <t>CAND_0099269</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>85</t>
+        </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>0.8073</t>
+          <t>0.8091</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>JD overlap is thin: Lead AI Engineer at Meta (8.6 YOE); JD-aligned skills: Qdrant, Fine-tuning LLMs, Vector Search. Gaps: low recruiter response rate; not flagged open to work.</t>
+          <t>JD overlap is thin: Data Scientist at BYJU'S (5.5 YOE); JD-aligned skills: Elasticsearch, Python, NLP. Gaps: 120-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>CAND_0060054</t>
-        </is>
-      </c>
-      <c r="B87" t="n">
-        <v>86</v>
+          <t>CAND_0041669</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>86</t>
+        </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>0.8066</t>
+          <t>0.8089</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Moderate fit: AI Engineer at Mad Street Den (6.4 YOE); JD-aligned skills: Weaviate, FAISS, Elasticsearch. Gaps: not flagged open to work.</t>
+          <t>Moderate fit: Recommendation Systems Engineer at CRED (8.0 YOE); JD-aligned skills: FAISS, Milvus, Weaviate. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>CAND_0069232</t>
-        </is>
-      </c>
-      <c r="B88" t="n">
-        <v>87</v>
+          <t>CAND_0094759</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>87</t>
+        </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>0.8057</t>
+          <t>0.8073</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Partial alignment: ML Engineer at Yellow.ai (6.3 YOE); JD-aligned skills: Pinecone, NLP, Python. Gaps: 120-day notice period; not flagged open to work.</t>
+          <t>Partial alignment: Lead AI Engineer at Meta (8.6 YOE); JD-aligned skills: Qdrant, Fine-tuning LLMs, Vector Search. Gaps: low recruiter response rate; not flagged open to work.</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>CAND_0065277</t>
-        </is>
-      </c>
-      <c r="B89" t="n">
-        <v>88</v>
+          <t>CAND_0060054</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>88</t>
+        </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>0.8049</t>
+          <t>0.8066</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Acceptable but not standout: Computer Vision Engineer at Aganitha (6.3 YOE); JD-aligned skills: Vector Search, Milvus, Fine-tuning LLMs. Gaps: under half of JD must-have skills covered.</t>
+          <t>Acceptable but not standout: AI Engineer at Mad Street Den (6.4 YOE); JD-aligned skills: Weaviate, FAISS, Elasticsearch. Gaps: not flagged open to work.</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>CAND_0006418</t>
-        </is>
-      </c>
-      <c r="B90" t="n">
-        <v>89</v>
+          <t>CAND_0069232</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>89</t>
+        </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>0.8037</t>
+          <t>0.8057</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Mixed signals: Machine Learning Engineer at Verloop.io (5.7 YOE); JD-aligned skills: Embeddings, Weaviate, Elasticsearch. Gaps: under half of JD must-have skills covered.</t>
+          <t>Mixed signals: ML Engineer at Yellow.ai (6.3 YOE); JD-aligned skills: Pinecone, NLP, Python. Gaps: 120-day notice period; not flagged open to work.</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>CAND_0064904</t>
-        </is>
-      </c>
-      <c r="B91" t="n">
-        <v>90</v>
+          <t>CAND_0065277</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>90</t>
+        </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>0.8031</t>
+          <t>0.8049</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>JD overlap is thin: AI Engineer at LinkedIn (4.9 YOE); JD-aligned skills: Embeddings, Elasticsearch, LLMs. Gaps: 90-day notice period.</t>
+          <t>JD overlap is thin: Computer Vision Engineer at Aganitha (6.3 YOE); JD-aligned skills: Vector Search, Milvus, Fine-tuning LLMs. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>CAND_0027723</t>
-        </is>
-      </c>
-      <c r="B92" t="n">
-        <v>91</v>
+          <t>CAND_0006418</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>91</t>
+        </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>0.8023</t>
+          <t>0.8037</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Lower-tier shortlist entry — ML Engineer at Wysa (4.2 YOE); JD-aligned skills: Vector Search, NLP, Elasticsearch. Key gaps: weak secondary signals vs higher ranks.</t>
+          <t>Lower-tier shortlist entry — Machine Learning Engineer at Verloop.io (5.7 YOE); JD-aligned skills: Embeddings, Weaviate, Elasticsearch. Key gaps: weak secondary signals vs higher ranks.</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>CAND_0061550</t>
-        </is>
-      </c>
-      <c r="B93" t="n">
-        <v>92</v>
+          <t>CAND_0064904</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>92</t>
+        </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>0.8023</t>
+          <t>0.8031</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Lower-tier shortlist entry — ML Engineer at Infosys (5.3 YOE); JD-aligned skills: Sentence Transformers. Key gaps: only 1 core JD skill matched.</t>
+          <t>Lower-tier shortlist entry — AI Engineer at LinkedIn (4.9 YOE); JD-aligned skills: Embeddings, Elasticsearch, LLMs. Key gaps: 90-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>CAND_0001707</t>
-        </is>
-      </c>
-      <c r="B94" t="n">
-        <v>93</v>
+          <t>CAND_0027723</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>93</t>
+        </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>0.8019</t>
+          <t>0.8023</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Lower-tier shortlist entry — Data Scientist at Vedantu (5.6 YOE); JD-aligned skills: Sentence Transformers, FAISS, Weaviate. Key gaps: 90-day notice period.</t>
+          <t>Lower-tier shortlist entry — ML Engineer at Wysa (4.2 YOE); JD-aligned skills: Vector Search, NLP, Elasticsearch. Key gaps: weak secondary signals vs higher ranks.</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>CAND_0005477</t>
-        </is>
-      </c>
-      <c r="B95" t="n">
-        <v>94</v>
+          <t>CAND_0061550</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>94</t>
+        </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>0.8012</t>
+          <t>0.8023</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Lower-tier shortlist entry — ML Engineer at Zomato (6.2 YOE); JD-aligned skills: OpenSearch. Key gaps: only 1 core JD skill matched.</t>
+          <t>Lower-tier shortlist entry — ML Engineer at Infosys (5.3 YOE); JD-aligned skills: Sentence Transformers. Key gaps: only 1 core JD skill matched.</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>CAND_0013536</t>
-        </is>
-      </c>
-      <c r="B96" t="n">
-        <v>95</v>
+          <t>CAND_0001707</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>95</t>
+        </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>0.8009</t>
+          <t>0.8019</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Lower-tier shortlist entry — Applied ML Engineer at Haptik (14.1 YOE); JD-aligned skills: LLMs, NLP, Embeddings. Key gaps: 90-day notice period; experience above target band for this role.</t>
+          <t>Lower-tier shortlist entry — Data Scientist at Vedantu (5.6 YOE); JD-aligned skills: Sentence Transformers, FAISS, Weaviate. Key gaps: 90-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>CAND_0015057</t>
-        </is>
-      </c>
-      <c r="B97" t="n">
-        <v>96</v>
+          <t>CAND_0005477</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>96</t>
+        </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>0.7999</t>
+          <t>0.8012</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Lower-tier shortlist entry — ML Engineer at Meesho (4.6 YOE); JD-aligned skills: Sentence Transformers, Vector Search, Embeddings. Key gaps: 90-day notice period.</t>
+          <t>Lower-tier shortlist entry — ML Engineer at Zomato (6.2 YOE); JD-aligned skills: OpenSearch. Key gaps: only 1 core JD skill matched.</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>CAND_0030348</t>
-        </is>
-      </c>
-      <c r="B98" t="n">
-        <v>97</v>
+          <t>CAND_0013536</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>97</t>
+        </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>0.7992</t>
+          <t>0.8009</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Lower-tier shortlist entry — Machine Learning Engineer at BYJU'S (4.5 YOE); JD-aligned skills: Embeddings, Vector Search, Elasticsearch. Key gaps: weak secondary signals vs higher ranks.</t>
+          <t>Lower-tier shortlist entry — Applied ML Engineer at Haptik (14.1 YOE); JD-aligned skills: LLMs, NLP, Embeddings. Key gaps: 90-day notice period; experience above target band for this role.</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>CAND_0060538</t>
-        </is>
-      </c>
-      <c r="B99" t="n">
-        <v>98</v>
+          <t>CAND_0015057</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>98</t>
+        </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>0.7983</t>
+          <t>0.7999</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Lower-tier shortlist entry — ML Engineer at Verloop.io (5.2 YOE); JD-aligned skills: OpenSearch, Embeddings, Milvus. Key gaps: 90-day notice period.</t>
+          <t>Lower-tier shortlist entry — ML Engineer at Meesho (4.6 YOE); JD-aligned skills: Sentence Transformers, Vector Search, Embeddings. Key gaps: 90-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>CAND_0049615</t>
-        </is>
-      </c>
-      <c r="B100" t="n">
-        <v>99</v>
+          <t>CAND_0030348</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>99</t>
+        </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>0.7961</t>
+          <t>0.7992</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Lower-tier shortlist entry — ML Engineer at Krutrim (5.1 YOE); JD-aligned skills: NLP, Pinecone. Key gaps: weak secondary signals vs higher ranks.</t>
+          <t>Lower-tier shortlist entry — Machine Learning Engineer at BYJU'S (4.5 YOE); JD-aligned skills: Embeddings, Vector Search, Elasticsearch. Key gaps: weak secondary signals vs higher ranks.</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>CAND_0019159</t>
-        </is>
-      </c>
-      <c r="B101" t="n">
-        <v>100</v>
+          <t>CAND_0049615</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>0.7956</t>
+          <t>0.7961</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Lower-tier shortlist entry — ML Engineer at Genpact AI (6.1 YOE); JD-aligned skills: Vector Search, Qdrant, Sentence Transformers. Key gaps: not flagged open to work.</t>
+          <t>Lower-tier shortlist entry — ML Engineer at Krutrim (5.1 YOE); JD-aligned skills: NLP, Pinecone. Key gaps: weak secondary signals vs higher ranks.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: regenerate submission after bullet-skill fix
</commit_message>
<xml_diff>
--- a/submission.xlsx
+++ b/submission.xlsx
@@ -456,7 +456,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Rank 1: Applied ML Engineer at Rephrase.ai (6.6 YOE); JD-aligned skills: Sentence Transformers, Milvus, Embeddings. Top-tier composite score across career, skills, and availability. Counterfactual: ranks on career trajectory and assessed depth over keyword coverage (7/22 listed must-haves), aligning with the JD anti-keyword-stuffing guidance.</t>
+          <t>Rank 1: Applied ML Engineer at Rephrase.ai (6.6 YOE); JD-aligned skills: Sentence Transformers, Milvus, Embeddings. Top-tier composite score across career, skills, and availability. Counterfactual: ranks on career trajectory and assessed depth over keyword coverage (7/20 listed must-haves), aligning with the JD anti-keyword-stuffing guidance.</t>
         </is>
       </c>
     </row>
@@ -478,7 +478,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Rank 2: Senior AI Engineer at Meta (7.9 YOE); JD-aligned skills: NLP, Python. Top-tier composite score across career, skills, and availability. Counterfactual: ranks on career trajectory and assessed depth over keyword coverage (2/22 listed must-haves), aligning with the JD anti-keyword-stuffing guidance.</t>
+          <t>Rank 2: Senior AI Engineer at Meta (7.9 YOE); JD-aligned skills: NLP, Python. Top-tier composite score across career, skills, and availability. Counterfactual: ranks on career trajectory and assessed depth over keyword coverage (2/20 listed must-haves), aligning with the JD anti-keyword-stuffing guidance.</t>
         </is>
       </c>
     </row>
@@ -500,14 +500,14 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Rank 3: Senior AI Engineer at Netflix (7.8 YOE); JD-aligned skills: Weaviate, Pinecone, Qdrant. Top-tier composite score across career, skills, and availability. Counterfactual: ranks on career trajectory and assessed depth over keyword coverage (6/22 listed must-haves), aligning with the JD anti-keyword-stuffing guidance.</t>
+          <t>Rank 3: Senior AI Engineer at Netflix (7.8 YOE); JD-aligned skills: Weaviate, Pinecone, Qdrant. Top-tier composite score across career, skills, and availability. Counterfactual: ranks on career trajectory and assessed depth over keyword coverage (6/20 listed must-haves), aligning with the JD anti-keyword-stuffing guidance.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>CAND_0018499</t>
+          <t>CAND_0096142</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -517,19 +517,19 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>1.0057</t>
+          <t>1.0027</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Rank 4: Senior Machine Learning Engineer at Zomato (7.2 YOE); JD-aligned skills: Weaviate, Pinecone, Milvus. Top-tier composite score across career, skills, and availability. Counterfactual: ranks on career trajectory and assessed depth over keyword coverage (5/22 listed must-haves), aligning with the JD anti-keyword-stuffing guidance.</t>
+          <t>Rank 4: Applied ML Engineer at upGrad (5.0 YOE); JD-aligned skills: Weaviate, Pinecone, Python. Top-tier composite score across career, skills, and availability. Minor note: 120-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CAND_0096142</t>
+          <t>CAND_0002025</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -539,19 +539,19 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>1.0027</t>
+          <t>0.9945</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Rank 5: Applied ML Engineer at upGrad (5.0 YOE); JD-aligned skills: Weaviate, Pinecone, Python. Top-tier composite score across career, skills, and availability. Minor note: 120-day notice period.</t>
+          <t>Rank 5: Senior AI Engineer at Apple (5.9 YOE); JD-aligned skills: FAISS, OpenSearch, Weaviate. Top-tier composite score across career, skills, and availability. Counterfactual: ranks on career trajectory and assessed depth over keyword coverage (8/20 listed must-haves), aligning with the JD anti-keyword-stuffing guidance.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>CAND_0002025</t>
+          <t>CAND_0087630</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -561,19 +561,19 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>0.9945</t>
+          <t>0.9906</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Strong match — Senior AI Engineer at Apple (5.9 YOE); JD-aligned skills: FAISS, OpenSearch, Weaviate.</t>
+          <t>Strong match — AI Engineer at Vedantu (7.2 YOE); JD-aligned skills: Elasticsearch, NLP, Embeddings.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>CAND_0087630</t>
+          <t>CAND_0018499</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -583,12 +583,12 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>0.9906</t>
+          <t>0.9772</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Strong match — AI Engineer at Vedantu (7.2 YOE); JD-aligned skills: Elasticsearch, NLP, Embeddings.</t>
+          <t>Strong match — Senior Machine Learning Engineer at Zomato (7.2 YOE); JD-aligned skills: Weaviate, Pinecone, Milvus.</t>
         </is>
       </c>
     </row>
@@ -683,7 +683,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>CAND_0071939</t>
+          <t>CAND_0080766</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -693,19 +693,19 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>0.9599</t>
+          <t>0.9558</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Strong match — Data Scientist at Krutrim (6.4 YOE); JD-aligned skills: Elasticsearch, OpenSearch, Embeddings.</t>
+          <t>Strong match — Staff Machine Learning Engineer at Salesforce (8.8 YOE); JD-aligned skills: Elasticsearch, OpenSearch, Python.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>CAND_0080766</t>
+          <t>CAND_0088025</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -715,19 +715,19 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>0.9558</t>
+          <t>0.9520</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Strong match — Staff Machine Learning Engineer at Salesforce (8.8 YOE); JD-aligned skills: Elasticsearch, OpenSearch, Python.</t>
+          <t>Strong match — Staff Machine Learning Engineer at Yellow.ai (8.6 YOE); JD-aligned skills: Pinecone, LLMs, Elasticsearch. Watch: 90-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>CAND_0088025</t>
+          <t>CAND_0044222</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -737,19 +737,19 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>0.9520</t>
+          <t>0.9489</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Strong match — Staff Machine Learning Engineer at Yellow.ai (8.6 YOE); JD-aligned skills: Pinecone, LLMs, Elasticsearch. Watch: 90-day notice period.</t>
+          <t>Strong match — AI Engineer at PolicyBazaar (7.7 YOE); JD-aligned skills: Vector Search, OpenSearch, Qdrant.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>CAND_0038368</t>
+          <t>CAND_0039383</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -759,19 +759,19 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>0.9508</t>
+          <t>0.9468</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Strong match — ML Engineer at PhonePe (5.4 YOE); JD-aligned skills: Embeddings, FAISS, Django.</t>
+          <t>Strong match — Applied ML Engineer at Meesho (7.1 YOE); JD-aligned skills: FAISS, NLP, Vector Search. Watch: 90-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>CAND_0044222</t>
+          <t>CAND_0077337</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -781,19 +781,19 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>0.9489</t>
+          <t>0.9405</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Strong match — AI Engineer at PolicyBazaar (7.7 YOE); JD-aligned skills: Vector Search, OpenSearch, Qdrant.</t>
+          <t>Strong match — Staff Machine Learning Engineer at Paytm (7.0 YOE); JD-aligned skills: Pinecone, LLMs, Qdrant.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>CAND_0039383</t>
+          <t>CAND_0046525</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -803,19 +803,19 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>0.9468</t>
+          <t>0.9402</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Strong match — Applied ML Engineer at Meesho (7.1 YOE); JD-aligned skills: FAISS, NLP, Vector Search. Watch: 90-day notice period.</t>
+          <t>Strong match — Senior Machine Learning Engineer at Genpact AI (6.1 YOE); JD-aligned skills: Elasticsearch, LLMs, NLP.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>CAND_0077337</t>
+          <t>CAND_0042029</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -825,19 +825,19 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>0.9405</t>
+          <t>0.9382</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Strong match — Staff Machine Learning Engineer at Paytm (7.0 YOE); JD-aligned skills: Pinecone, LLMs, Qdrant.</t>
+          <t>Strong match — Senior Data Scientist at Flipkart (6.5 YOE); JD-aligned skills: NLP, Elasticsearch, Embeddings.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>CAND_0046525</t>
+          <t>CAND_0065514</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -847,19 +847,19 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>0.9402</t>
+          <t>0.9377</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Strong match — Senior Machine Learning Engineer at Genpact AI (6.1 YOE); JD-aligned skills: Elasticsearch, LLMs, NLP.</t>
+          <t>Strong match — ML Engineer at Genpact AI (6.6 YOE); JD-aligned skills: Vector Search, Pinecone, Elasticsearch. Watch: 90-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>CAND_0042029</t>
+          <t>CAND_0020877</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -869,19 +869,19 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>0.9382</t>
+          <t>0.9367</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Strong match — Senior Data Scientist at Flipkart (6.5 YOE); JD-aligned skills: NLP, Elasticsearch, Embeddings.</t>
+          <t>Strong match — Applied ML Engineer at CRED (5.1 YOE); JD-aligned skills: Elasticsearch, OpenSearch, Weaviate.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>CAND_0065514</t>
+          <t>CAND_0071939</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -891,19 +891,19 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>0.9377</t>
+          <t>0.9320</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Solid profile: ML Engineer at Genpact AI (6.6 YOE); JD-aligned skills: Vector Search, Pinecone, Elasticsearch. Concerns: 90-day notice period.</t>
+          <t>Solid profile: Data Scientist at Krutrim (6.4 YOE); JD-aligned skills: Elasticsearch, OpenSearch, Embeddings.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>CAND_0020877</t>
+          <t>CAND_0081846</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -913,19 +913,19 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>0.9367</t>
+          <t>0.9260</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Good fit with caveats: Applied ML Engineer at CRED (5.1 YOE); JD-aligned skills: Elasticsearch, OpenSearch, Weaviate.</t>
+          <t>Good fit with caveats: Lead AI Engineer at Razorpay (6.7 YOE); JD-aligned skills: Elasticsearch, Vector Search, Python.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>CAND_0081846</t>
+          <t>CAND_0037566</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -935,19 +935,19 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>0.9260</t>
+          <t>0.9243</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Competitive candidate: Lead AI Engineer at Razorpay (6.7 YOE); JD-aligned skills: Elasticsearch, Vector Search, Python.</t>
+          <t>Competitive candidate: Machine Learning Engineer at LinkedIn (6.9 YOE); JD-aligned skills: Pinecone, NLP, LLMs.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>CAND_0037566</t>
+          <t>CAND_0038368</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -957,19 +957,19 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>0.9243</t>
+          <t>0.9223</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Meets several JD signals: Machine Learning Engineer at LinkedIn (6.9 YOE); JD-aligned skills: Pinecone, NLP, LLMs.</t>
+          <t>Meets several JD signals: ML Engineer at PhonePe (5.4 YOE); JD-aligned skills: Embeddings, FAISS, NLP.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>CAND_0010257</t>
+          <t>CAND_0009691</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -979,19 +979,19 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>0.9232</t>
+          <t>0.9106</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Solid profile: Senior Data Scientist at Google (6.5 YOE); JD-aligned skills: Milvus, Python, OpenSearch. Concerns: 120-day notice period.</t>
+          <t>Solid profile: Applied ML Engineer at LinkedIn (6.2 YOE); JD-aligned skills: Fine-tuning LLMs, Pinecone, Sentence Transformers. Concerns: 120-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>CAND_0075574</t>
+          <t>CAND_0050454</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1001,19 +1001,19 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>0.9182</t>
+          <t>0.9105</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Good fit with caveats: Machine Learning Engineer at Haptik (5.7 YOE); JD-aligned skills: Weaviate, OpenSearch, Qdrant.</t>
+          <t>Good fit with caveats: AI Engineer at Rephrase.ai (6.8 YOE); JD-aligned skills: Fine-tuning LLMs, FAISS, Qdrant.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>CAND_0009691</t>
+          <t>CAND_0079064</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1023,19 +1023,19 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>0.9106</t>
+          <t>0.9088</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Competitive candidate: Applied ML Engineer at LinkedIn (6.2 YOE); JD-aligned skills: Fine-tuning LLMs, Pinecone, Sentence Transformers. Concerns: 120-day notice period.</t>
+          <t>Competitive candidate: Senior Data Scientist at Niramai (5.2 YOE); JD-aligned skills: OpenSearch, NLP, Fine-tuning LLMs. Concerns: 120-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>CAND_0050454</t>
+          <t>CAND_0090584</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1045,19 +1045,19 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>0.9105</t>
+          <t>0.9042</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Meets several JD signals: AI Engineer at Rephrase.ai (6.8 YOE); JD-aligned skills: Fine-tuning LLMs, FAISS, Qdrant.</t>
+          <t>Meets several JD signals: ML Engineer at Flipkart (5.1 YOE); JD-aligned skills: Fine-tuning LLMs, OpenSearch, FAISS. Concerns: 120-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>CAND_0079064</t>
+          <t>CAND_0030031</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1067,19 +1067,19 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>0.9088</t>
+          <t>0.9020</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Solid profile: Senior Data Scientist at Niramai (5.2 YOE); JD-aligned skills: OpenSearch, NLP, Fine-tuning LLMs. Concerns: 120-day notice period.</t>
+          <t>Solid profile: AI Engineer at Microsoft (5.7 YOE); JD-aligned skills: Python, NLP, Sentence Transformers.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>CAND_0090584</t>
+          <t>CAND_0089552</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1089,19 +1089,19 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>0.9042</t>
+          <t>0.8970</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Good fit with caveats: ML Engineer at Flipkart (5.1 YOE); JD-aligned skills: Fine-tuning LLMs, OpenSearch, FAISS. Concerns: 120-day notice period.</t>
+          <t>Good fit with caveats: Machine Learning Engineer at Netflix (6.0 YOE); JD-aligned skills: Weaviate, Qdrant, Vector Search. Concerns: 120-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>CAND_0030031</t>
+          <t>CAND_0010257</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1111,19 +1111,19 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>0.9020</t>
+          <t>0.8967</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Competitive candidate: AI Engineer at Microsoft (5.7 YOE); JD-aligned skills: Python, NLP, Sentence Transformers.</t>
+          <t>Competitive candidate: Senior Data Scientist at Google (6.5 YOE); JD-aligned skills: Milvus, Python, OpenSearch. Concerns: 120-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>CAND_0089552</t>
+          <t>CAND_0099806</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1133,19 +1133,19 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>0.8970</t>
+          <t>0.8924</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Meets several JD signals: Machine Learning Engineer at Netflix (6.0 YOE); JD-aligned skills: Weaviate, Qdrant, Vector Search. Concerns: 120-day notice period.</t>
+          <t>Meets several JD signals: AI Engineer at Mad Street Den (4.6 YOE); JD-aligned skills: FAISS, Embeddings, Sentence Transformers.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>CAND_0099806</t>
+          <t>CAND_0075574</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1155,19 +1155,19 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>0.8924</t>
+          <t>0.8903</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Solid profile: AI Engineer at Mad Street Den (4.6 YOE); JD-aligned skills: FAISS, Embeddings, Sentence Transformers.</t>
+          <t>Solid profile: Machine Learning Engineer at Haptik (5.7 YOE); JD-aligned skills: Weaviate, OpenSearch, Qdrant.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>CAND_0093193</t>
+          <t>CAND_0032216</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1177,19 +1177,19 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>0.8907</t>
+          <t>0.8901</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Good fit with caveats: Senior Machine Learning Engineer at Niramai (7.9 YOE); JD-aligned skills: Indexing Algorithms, Qdrant, OpenSearch.</t>
+          <t>Good fit with caveats: ML Engineer at upGrad (6.1 YOE); JD-aligned skills: Qdrant, Sentence Transformers, Vector Search.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>CAND_0061257</t>
+          <t>CAND_0037944</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1199,19 +1199,19 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>0.8905</t>
+          <t>0.8855</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Competitive candidate: Staff Machine Learning Engineer at LinkedIn (8.0 YOE); JD-aligned skills: Indexing Algorithms, Python.</t>
+          <t>Competitive candidate: Senior Data Scientist at Vedantu (4.9 YOE); JD-aligned skills: Vector Search, OpenSearch, Embeddings.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>CAND_0032216</t>
+          <t>CAND_0049538</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1221,19 +1221,19 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>0.8901</t>
+          <t>0.8796</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Meets several JD signals: ML Engineer at upGrad (6.1 YOE); JD-aligned skills: Qdrant, Sentence Transformers, Vector Search.</t>
+          <t>Meets several JD signals: Applied ML Engineer at Saarthi.ai (5.8 YOE); JD-aligned skills: OpenSearch, Vector Search, Milvus.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>CAND_0048166</t>
+          <t>CAND_0047721</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1243,19 +1243,19 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>0.8885</t>
+          <t>0.8791</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Solid profile: ML Engineer at Aganitha (5.2 YOE); JD-aligned skills: MongoDB, Pinecone, Rust.</t>
+          <t>Solid profile: Senior Data Scientist at Microsoft (7.0 YOE); JD-aligned skills: Milvus, FAISS, Qdrant. Concerns: 90-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>CAND_0037944</t>
+          <t>CAND_0042100</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1265,19 +1265,19 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>0.8855</t>
+          <t>0.8773</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Good fit with caveats: Senior Data Scientist at Vedantu (4.9 YOE); JD-aligned skills: Vector Search, OpenSearch, Embeddings.</t>
+          <t>Good fit with caveats: Machine Learning Engineer at Freshworks (7.3 YOE); JD-aligned skills: Elasticsearch, Fine-tuning LLMs, Pinecone. Concerns: 90-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>CAND_0015578</t>
+          <t>CAND_0043228</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1287,19 +1287,19 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>0.8810</t>
+          <t>0.8758</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Competitive candidate: AI Engineer at Zoho (5.4 YOE); JD-aligned skills: Embeddings, NLP, Sentence Transformers. Concerns: 90-day notice period.</t>
+          <t>Competitive candidate: Applied ML Engineer at Zoho (6.8 YOE); JD-aligned skills: NLP, Vector Search, Sentence Transformers.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>CAND_0049538</t>
+          <t>CAND_0083879</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1309,19 +1309,19 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>0.8796</t>
+          <t>0.8736</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Meets several JD signals: Applied ML Engineer at Saarthi.ai (5.8 YOE); JD-aligned skills: OpenSearch, Vector Search, Milvus.</t>
+          <t>Meets several JD signals: Machine Learning Engineer at Ola (7.1 YOE); JD-aligned skills: Fine-tuning LLMs, Milvus, Sentence Transformers.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>CAND_0047721</t>
+          <t>CAND_0003841</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1331,19 +1331,19 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>0.8791</t>
+          <t>0.8722</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Solid profile: Senior Data Scientist at Microsoft (7.0 YOE); JD-aligned skills: Milvus, FAISS, Qdrant. Concerns: 90-day notice period.</t>
+          <t>Solid profile: ML Engineer at Tech Mahindra (5.0 YOE); JD-aligned skills: Pinecone, Fine-tuning LLMs, Sentence Transformers.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>CAND_0042100</t>
+          <t>CAND_0081852</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1353,19 +1353,19 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>0.8773</t>
+          <t>0.8712</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Good fit with caveats: Machine Learning Engineer at Freshworks (7.3 YOE); JD-aligned skills: Elasticsearch, Fine-tuning LLMs, Pinecone. Concerns: 90-day notice period.</t>
+          <t>Good fit with caveats: Senior Data Scientist at Mad Street Den (5.9 YOE); JD-aligned skills: Milvus, Weaviate, Vector Search.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>CAND_0043228</t>
+          <t>CAND_0079284</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1375,19 +1375,19 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>0.8758</t>
+          <t>0.8702</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Competitive candidate: Applied ML Engineer at Zoho (6.8 YOE); JD-aligned skills: NLP, Vector Search, Sentence Transformers.</t>
+          <t>Competitive candidate: Machine Learning Engineer at Google (4.9 YOE); JD-aligned skills: Qdrant, Fine-tuning LLMs, Elasticsearch.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>CAND_0083879</t>
+          <t>CAND_0079387</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1397,19 +1397,19 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>0.8736</t>
+          <t>0.8678</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Meets several JD signals: Machine Learning Engineer at Ola (7.1 YOE); JD-aligned skills: Fine-tuning LLMs, Milvus, Sentence Transformers.</t>
+          <t>Meets several JD signals: AI Engineer at Microsoft (6.9 YOE); JD-aligned skills: Python, Sentence Transformers, Vector Search.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>CAND_0007460</t>
+          <t>CAND_0086022</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -1419,19 +1419,19 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>0.8728</t>
+          <t>0.8678</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Solid profile: AI Engineer at Salesforce (4.7 YOE); JD-aligned skills: Embeddings, Weaviate, Go. Concerns: 120-day notice period.</t>
+          <t>Solid profile: Senior Applied Scientist at Sarvam AI (5.3 YOE); JD-aligned skills: Vector Search, Fine-tuning LLMs, Elasticsearch.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>CAND_0003841</t>
+          <t>CAND_0040178</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -1441,19 +1441,19 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>0.8722</t>
+          <t>0.8654</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Good fit with caveats: ML Engineer at Tech Mahindra (5.0 YOE); JD-aligned skills: Pinecone, Fine-tuning LLMs, Sentence Transformers.</t>
+          <t>Good fit with caveats: ML Engineer at Meesho (5.0 YOE); JD-aligned skills: Weaviate, Fine-tuning LLMs, Vector Search.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>CAND_0081852</t>
+          <t>CAND_0018094</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -1463,19 +1463,19 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>0.8712</t>
+          <t>0.8633</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Competitive candidate: Senior Data Scientist at Mad Street Den (5.9 YOE); JD-aligned skills: Milvus, Weaviate, Vector Search.</t>
+          <t>Competitive candidate: ML Engineer at Mad Street Den (5.2 YOE); JD-aligned skills: Pinecone, Fine-tuning LLMs.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>CAND_0079284</t>
+          <t>CAND_0035653</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1485,19 +1485,19 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>0.8702</t>
+          <t>0.8631</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Meets several JD signals: Machine Learning Engineer at Google (4.9 YOE); JD-aligned skills: Qdrant, Fine-tuning LLMs, Elasticsearch.</t>
+          <t>Meets several JD signals: Data Scientist at Swiggy (5.6 YOE); JD-aligned skills: OpenSearch, Vector Search, Fine-tuning LLMs.</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>CAND_0079387</t>
+          <t>CAND_0093193</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -1507,19 +1507,19 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>0.8678</t>
+          <t>0.8628</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Solid profile: AI Engineer at Microsoft (6.9 YOE); JD-aligned skills: Python, Sentence Transformers, Vector Search.</t>
+          <t>Solid profile: Senior Machine Learning Engineer at Niramai (7.9 YOE); JD-aligned skills: Qdrant, OpenSearch.</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>CAND_0086022</t>
+          <t>CAND_0061257</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -1529,19 +1529,19 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>0.8678</t>
+          <t>0.8621</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Good fit with caveats: Senior Applied Scientist at Sarvam AI (5.3 YOE); JD-aligned skills: Vector Search, Fine-tuning LLMs, Elasticsearch.</t>
+          <t>Good fit with caveats: Staff Machine Learning Engineer at LinkedIn (8.0 YOE); JD-aligned skills: Python. Concerns: only 1 core JD skill matched.</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>CAND_0040178</t>
+          <t>CAND_0076482</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -1551,19 +1551,19 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>0.8654</t>
+          <t>0.8605</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Moderate fit: ML Engineer at Meesho (5.0 YOE); JD-aligned skills: Weaviate, Fine-tuning LLMs, Vector Search. Gaps: under half of JD must-have skills covered.</t>
+          <t>Moderate fit: ML Engineer at Flipkart (6.6 YOE); JD-aligned skills: OpenSearch, Pinecone, Embeddings. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>CAND_0018094</t>
+          <t>CAND_0010149</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -1573,19 +1573,19 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>0.8633</t>
+          <t>0.8561</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Partial alignment: ML Engineer at Mad Street Den (5.2 YOE); JD-aligned skills: Pinecone, Fine-tuning LLMs. Gaps: under half of JD must-have skills covered.</t>
+          <t>Partial alignment: ML Engineer at Glance (6.9 YOE); JD-aligned skills: Milvus, Vector Search, Elasticsearch. Gaps: 90-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>CAND_0035653</t>
+          <t>CAND_0055905</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -1595,19 +1595,19 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>0.8631</t>
+          <t>0.8558</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Acceptable but not standout: Data Scientist at Swiggy (5.6 YOE); JD-aligned skills: OpenSearch, Vector Search, Fine-tuning LLMs. Gaps: under half of JD must-have skills covered.</t>
+          <t>Acceptable but not standout: Senior Machine Learning Engineer at Flipkart (8.1 YOE); JD-aligned skills: Elasticsearch, Python, LLMs. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>CAND_0076482</t>
+          <t>CAND_0015578</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -1617,19 +1617,19 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>0.8605</t>
+          <t>0.8557</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Mixed signals: ML Engineer at Flipkart (6.6 YOE); JD-aligned skills: OpenSearch, Pinecone, Embeddings. Gaps: under half of JD must-have skills covered.</t>
+          <t>Mixed signals: AI Engineer at Zoho (5.4 YOE); JD-aligned skills: Embeddings, NLP, Sentence Transformers. Gaps: 90-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>CAND_0010149</t>
+          <t>CAND_0051004</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -1639,19 +1639,19 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>0.8561</t>
+          <t>0.8544</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>JD overlap is thin: ML Engineer at Glance (6.9 YOE); JD-aligned skills: Milvus, Vector Search, Elasticsearch. Gaps: 90-day notice period.</t>
+          <t>JD overlap is thin: Senior Data Scientist at CRED (4.7 YOE); JD-aligned skills: Embeddings, Qdrant, Fine-tuning LLMs. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>CAND_0055905</t>
+          <t>CAND_0095528</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -1661,19 +1661,19 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>0.8558</t>
+          <t>0.8539</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Moderate fit: Senior Machine Learning Engineer at Flipkart (8.1 YOE); JD-aligned skills: Elasticsearch, Python, LLMs. Gaps: under half of JD must-have skills covered.</t>
+          <t>Moderate fit: Senior Data Scientist at Netflix (5.3 YOE); JD-aligned skills: OpenSearch, Vector Search, Qdrant. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>CAND_0051004</t>
+          <t>CAND_0051292</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -1683,19 +1683,19 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>0.8544</t>
+          <t>0.8507</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Partial alignment: Senior Data Scientist at CRED (4.7 YOE); JD-aligned skills: Embeddings, Qdrant, Fine-tuning LLMs. Gaps: under half of JD must-have skills covered.</t>
+          <t>Partial alignment: Applied ML Engineer at Freshworks (5.2 YOE); JD-aligned skills: FAISS, LLMs, Vector Search. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>CAND_0095528</t>
+          <t>CAND_0073982</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -1705,19 +1705,19 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>0.8539</t>
+          <t>0.8500</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Acceptable but not standout: Senior Data Scientist at Netflix (5.3 YOE); JD-aligned skills: OpenSearch, Vector Search, Qdrant. Gaps: under half of JD must-have skills covered.</t>
+          <t>Acceptable but not standout: Data Scientist at Dream11 (7.0 YOE); JD-aligned skills: Sentence Transformers, Qdrant, FAISS. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>CAND_0051292</t>
+          <t>CAND_0069905</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -1727,19 +1727,19 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>0.8507</t>
+          <t>0.8499</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Mixed signals: Applied ML Engineer at Freshworks (5.2 YOE); JD-aligned skills: FAISS, LLMs, Vector Search. Gaps: under half of JD must-have skills covered.</t>
+          <t>Mixed signals: Applied ML Engineer at Sarvam AI (6.6 YOE); JD-aligned skills: Sentence Transformers, Python, Weaviate. Gaps: 90-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>CAND_0073982</t>
+          <t>CAND_0036121</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -1749,19 +1749,19 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>0.8500</t>
+          <t>0.8491</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>JD overlap is thin: Data Scientist at Dream11 (7.0 YOE); JD-aligned skills: Sentence Transformers, Qdrant, FAISS. Gaps: under half of JD must-have skills covered.</t>
+          <t>JD overlap is thin: ML Engineer at Wysa (5.2 YOE); JD-aligned skills: Embeddings, Vector Search. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>CAND_0069905</t>
+          <t>CAND_0013393</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -1771,19 +1771,19 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>0.8499</t>
+          <t>0.8469</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Moderate fit: Applied ML Engineer at Sarvam AI (6.6 YOE); JD-aligned skills: Sentence Transformers, Python, Weaviate. Gaps: 90-day notice period.</t>
+          <t>Moderate fit: ML Engineer at Freshworks (5.3 YOE); JD-aligned skills: Embeddings, Pinecone, Qdrant. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>CAND_0036121</t>
+          <t>CAND_0095213</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -1793,19 +1793,19 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>0.8491</t>
+          <t>0.8469</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Partial alignment: ML Engineer at Wysa (5.2 YOE); JD-aligned skills: Embeddings, Vector Search. Gaps: under half of JD must-have skills covered.</t>
+          <t>Partial alignment: ML Engineer at Genpact AI (5.1 YOE); JD-aligned skills: Python, Weaviate, Pinecone. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>CAND_0013393</t>
+          <t>CAND_0015582</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -1815,19 +1815,19 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>0.8469</t>
+          <t>0.8468</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Acceptable but not standout: ML Engineer at Freshworks (5.3 YOE); JD-aligned skills: Embeddings, Pinecone, Qdrant. Gaps: under half of JD must-have skills covered.</t>
+          <t>Acceptable but not standout: ML Engineer at Genpact AI (4.4 YOE); JD-aligned skills: Qdrant, Sentence Transformers, Embeddings. Gaps: 120-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>CAND_0095213</t>
+          <t>CAND_0091909</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -1837,19 +1837,19 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>0.8469</t>
+          <t>0.8468</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Mixed signals: ML Engineer at Genpact AI (5.1 YOE); JD-aligned skills: Python, Weaviate, Pinecone. Gaps: under half of JD must-have skills covered.</t>
+          <t>Mixed signals: Machine Learning Engineer at Rephrase.ai (6.9 YOE); JD-aligned skills: LLMs, Pinecone, Qdrant. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>CAND_0015582</t>
+          <t>CAND_0016163</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -1859,19 +1859,19 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>0.8468</t>
+          <t>0.8452</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>JD overlap is thin: ML Engineer at Genpact AI (4.4 YOE); JD-aligned skills: Qdrant, Sentence Transformers, Embeddings. Gaps: 120-day notice period.</t>
+          <t>JD overlap is thin: Applied ML Engineer at Dream11 (6.7 YOE); JD-aligned skills: Weaviate, Embeddings, Pinecone. Gaps: 120-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>CAND_0091909</t>
+          <t>CAND_0007460</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -1881,19 +1881,19 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>0.8468</t>
+          <t>0.8450</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Moderate fit: Machine Learning Engineer at Rephrase.ai (6.9 YOE); JD-aligned skills: LLMs, Pinecone, Qdrant. Gaps: under half of JD must-have skills covered.</t>
+          <t>Moderate fit: AI Engineer at Salesforce (4.7 YOE); JD-aligned skills: Embeddings, Weaviate, NLP. Gaps: 120-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>CAND_0016163</t>
+          <t>CAND_0011432</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -1903,19 +1903,19 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>0.8452</t>
+          <t>0.8405</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Partial alignment: Applied ML Engineer at Dream11 (6.7 YOE); JD-aligned skills: Weaviate, Embeddings, Pinecone. Gaps: 120-day notice period.</t>
+          <t>Partial alignment: Senior Data Scientist at Amazon (7.6 YOE); JD-aligned skills: OpenSearch, Elasticsearch. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>CAND_0011432</t>
+          <t>CAND_0068932</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -1925,19 +1925,19 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>0.8405</t>
+          <t>0.8404</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Acceptable but not standout: Senior Data Scientist at Amazon (7.6 YOE); JD-aligned skills: OpenSearch, Elasticsearch. Gaps: under half of JD must-have skills covered.</t>
+          <t>Acceptable but not standout: ML Engineer at Krutrim (5.2 YOE); JD-aligned skills: Milvus, OpenSearch. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>CAND_0068932</t>
+          <t>CAND_0090155</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -1947,19 +1947,19 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>0.8404</t>
+          <t>0.8401</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Mixed signals: ML Engineer at Krutrim (5.2 YOE); JD-aligned skills: Milvus, OpenSearch. Gaps: under half of JD must-have skills covered.</t>
+          <t>Mixed signals: ML Engineer at Swiggy (5.8 YOE); JD-aligned skills: Milvus, Qdrant, Pinecone. Gaps: 90-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>CAND_0090155</t>
+          <t>CAND_0070398</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -1969,19 +1969,19 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>0.8401</t>
+          <t>0.8390</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>JD overlap is thin: ML Engineer at Swiggy (5.8 YOE); JD-aligned skills: Milvus, Qdrant, Pinecone. Gaps: 90-day notice period.</t>
+          <t>JD overlap is thin: Machine Learning Engineer at Genpact AI (7.2 YOE); JD-aligned skills: FAISS, Embeddings, Python. Gaps: 120-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>CAND_0070398</t>
+          <t>CAND_0098217</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -1991,19 +1991,19 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>0.8390</t>
+          <t>0.8388</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Moderate fit: Machine Learning Engineer at Genpact AI (7.2 YOE); JD-aligned skills: FAISS, Embeddings, Python. Gaps: 120-day notice period.</t>
+          <t>Moderate fit: ML Engineer at Glance (6.4 YOE); JD-aligned skills: FAISS, Pinecone. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>CAND_0098217</t>
+          <t>CAND_0017093</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -2013,19 +2013,19 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>0.8388</t>
+          <t>0.8378</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Partial alignment: ML Engineer at Glance (6.4 YOE); JD-aligned skills: FAISS, Pinecone. Gaps: under half of JD must-have skills covered.</t>
+          <t>Partial alignment: ML Engineer at Zoho (5.9 YOE); JD-aligned skills: LLMs, Embeddings. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>CAND_0017093</t>
+          <t>CAND_0052328</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -2035,19 +2035,19 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>0.8378</t>
+          <t>0.8331</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Acceptable but not standout: ML Engineer at Zoho (5.9 YOE); JD-aligned skills: LLMs, Embeddings. Gaps: under half of JD must-have skills covered.</t>
+          <t>Acceptable but not standout: Recommendation Systems Engineer at Amazon (6.5 YOE); JD-aligned skills: OpenSearch, Fine-tuning LLMs, Vector Search. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>CAND_0052328</t>
+          <t>CAND_0048166</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -2057,12 +2057,12 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>0.8331</t>
+          <t>0.8317</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Mixed signals: Recommendation Systems Engineer at Amazon (6.5 YOE); JD-aligned skills: OpenSearch, Fine-tuning LLMs, Vector Search. Gaps: under half of JD must-have skills covered.</t>
+          <t>Mixed signals: ML Engineer at Aganitha (5.2 YOE); JD-aligned skills: Pinecone, Milvus, Qdrant. Gaps: not flagged open to work.</t>
         </is>
       </c>
     </row>
@@ -2091,7 +2091,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>CAND_0060538</t>
+          <t>CAND_0021836</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -2101,19 +2101,19 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>0.8235</t>
+          <t>0.8220</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Moderate fit: ML Engineer at Verloop.io (5.2 YOE); JD-aligned skills: OpenSearch, Embeddings, Rust. Gaps: 90-day notice period.</t>
+          <t>Moderate fit: ML Engineer at CRED (6.5 YOE); JD-aligned skills: Vector Search, Elasticsearch, NLP. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>CAND_0021836</t>
+          <t>CAND_0050876</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -2123,19 +2123,19 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>0.8220</t>
+          <t>0.8217</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Partial alignment: ML Engineer at CRED (6.5 YOE); JD-aligned skills: Vector Search, Elasticsearch, NLP. Gaps: under half of JD must-have skills covered.</t>
+          <t>Partial alignment: Applied ML Engineer at Freshworks (6.0 YOE); JD-aligned skills: Qdrant, FAISS, OpenSearch. Gaps: 90-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>CAND_0050876</t>
+          <t>CAND_0005649</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -2145,19 +2145,19 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>0.8217</t>
+          <t>0.8212</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Acceptable but not standout: Applied ML Engineer at Freshworks (6.0 YOE); JD-aligned skills: Qdrant, FAISS, OpenSearch. Gaps: 90-day notice period.</t>
+          <t>Acceptable but not standout: Senior Data Scientist at Sarvam AI (7.4 YOE); JD-aligned skills: Fine-tuning LLMs, Weaviate. Gaps: 90-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>CAND_0005649</t>
+          <t>CAND_0092245</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -2167,19 +2167,19 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>0.8212</t>
+          <t>0.8205</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Mixed signals: Senior Data Scientist at Sarvam AI (7.4 YOE); JD-aligned skills: Fine-tuning LLMs, Weaviate. Gaps: 90-day notice period.</t>
+          <t>Mixed signals: Senior Data Scientist at Ola (4.1 YOE); JD-aligned skills: Embeddings, FAISS, Qdrant. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>CAND_0092245</t>
+          <t>CAND_0055992</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -2189,19 +2189,19 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>0.8205</t>
+          <t>0.8191</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>JD overlap is thin: Senior Data Scientist at Ola (4.1 YOE); JD-aligned skills: Embeddings, FAISS, Qdrant. Gaps: under half of JD must-have skills covered.</t>
+          <t>JD overlap is thin: AI Engineer at CRED (16.9 YOE); JD-aligned skills: FAISS, OpenSearch, Embeddings. Gaps: experience above target band for this role.</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>CAND_0055992</t>
+          <t>CAND_0005538</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -2211,19 +2211,19 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>0.8191</t>
+          <t>0.8165</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Moderate fit: AI Engineer at CRED (16.9 YOE); JD-aligned skills: FAISS, OpenSearch, Embeddings. Gaps: experience above target band for this role.</t>
+          <t>Moderate fit: Senior AI Engineer at Adobe (5.9 YOE); JD-aligned skills: Python. Gaps: only 1 core JD skill matched; 90-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>CAND_0005538</t>
+          <t>CAND_0002037</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -2233,19 +2233,19 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>0.8165</t>
+          <t>0.8119</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Partial alignment: Senior AI Engineer at Adobe (5.9 YOE); JD-aligned skills: Python. Gaps: only 1 core JD skill matched; 90-day notice period.</t>
+          <t>Partial alignment: ML Engineer at Locobuzz (5.5 YOE); JD-aligned skills: Fine-tuning LLMs, Milvus, Pinecone. Gaps: not flagged open to work.</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>CAND_0047276</t>
+          <t>CAND_0099269</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -2255,19 +2255,19 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>0.8131</t>
+          <t>0.8091</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Acceptable but not standout: Backend Engineer at Freshworks (5.5 YOE); JD-aligned skills: Qdrant, Fine-tuning LLMs, Go. Gaps: under half of JD must-have skills covered.</t>
+          <t>Acceptable but not standout: Data Scientist at BYJU'S (5.5 YOE); JD-aligned skills: Elasticsearch, Python, NLP. Gaps: 120-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>CAND_0002037</t>
+          <t>CAND_0041669</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -2277,19 +2277,19 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>0.8119</t>
+          <t>0.8089</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Mixed signals: ML Engineer at Locobuzz (5.5 YOE); JD-aligned skills: Fine-tuning LLMs, Milvus, Pinecone. Gaps: not flagged open to work.</t>
+          <t>Mixed signals: Recommendation Systems Engineer at CRED (8.0 YOE); JD-aligned skills: FAISS, Milvus, Weaviate. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>CAND_0099269</t>
+          <t>CAND_0094759</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -2299,19 +2299,19 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>0.8091</t>
+          <t>0.8073</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>JD overlap is thin: Data Scientist at BYJU'S (5.5 YOE); JD-aligned skills: Elasticsearch, Python, NLP. Gaps: 120-day notice period.</t>
+          <t>JD overlap is thin: Lead AI Engineer at Meta (8.6 YOE); JD-aligned skills: Qdrant, Fine-tuning LLMs, Vector Search. Gaps: low recruiter response rate; not flagged open to work.</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>CAND_0041669</t>
+          <t>CAND_0060054</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -2321,19 +2321,19 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>0.8089</t>
+          <t>0.8066</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Moderate fit: Recommendation Systems Engineer at CRED (8.0 YOE); JD-aligned skills: FAISS, Milvus, Weaviate. Gaps: under half of JD must-have skills covered.</t>
+          <t>Moderate fit: AI Engineer at Mad Street Den (6.4 YOE); JD-aligned skills: Weaviate, FAISS, Elasticsearch. Gaps: not flagged open to work.</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>CAND_0094759</t>
+          <t>CAND_0069232</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -2343,19 +2343,19 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>0.8073</t>
+          <t>0.8057</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Partial alignment: Lead AI Engineer at Meta (8.6 YOE); JD-aligned skills: Qdrant, Fine-tuning LLMs, Vector Search. Gaps: low recruiter response rate; not flagged open to work.</t>
+          <t>Partial alignment: ML Engineer at Yellow.ai (6.3 YOE); JD-aligned skills: Pinecone, NLP, Python. Gaps: 120-day notice period; not flagged open to work.</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>CAND_0060054</t>
+          <t>CAND_0065277</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -2365,19 +2365,19 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>0.8066</t>
+          <t>0.8049</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Acceptable but not standout: AI Engineer at Mad Street Den (6.4 YOE); JD-aligned skills: Weaviate, FAISS, Elasticsearch. Gaps: not flagged open to work.</t>
+          <t>Acceptable but not standout: Computer Vision Engineer at Aganitha (6.3 YOE); JD-aligned skills: Vector Search, Milvus, Fine-tuning LLMs. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>CAND_0069232</t>
+          <t>CAND_0006418</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -2387,19 +2387,19 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>0.8057</t>
+          <t>0.8037</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Mixed signals: ML Engineer at Yellow.ai (6.3 YOE); JD-aligned skills: Pinecone, NLP, Python. Gaps: 120-day notice period; not flagged open to work.</t>
+          <t>Mixed signals: Machine Learning Engineer at Verloop.io (5.7 YOE); JD-aligned skills: Embeddings, Weaviate, Elasticsearch. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>CAND_0065277</t>
+          <t>CAND_0064904</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -2409,19 +2409,19 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>0.8049</t>
+          <t>0.8031</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>JD overlap is thin: Computer Vision Engineer at Aganitha (6.3 YOE); JD-aligned skills: Vector Search, Milvus, Fine-tuning LLMs. Gaps: under half of JD must-have skills covered.</t>
+          <t>JD overlap is thin: AI Engineer at LinkedIn (4.9 YOE); JD-aligned skills: Embeddings, Elasticsearch, LLMs. Gaps: 90-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>CAND_0006418</t>
+          <t>CAND_0027723</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -2431,19 +2431,19 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>0.8037</t>
+          <t>0.8023</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Lower-tier shortlist entry — Machine Learning Engineer at Verloop.io (5.7 YOE); JD-aligned skills: Embeddings, Weaviate, Elasticsearch. Key gaps: weak secondary signals vs higher ranks.</t>
+          <t>Lower-tier shortlist entry — ML Engineer at Wysa (4.2 YOE); JD-aligned skills: Vector Search, NLP, Elasticsearch. Key gaps: weak secondary signals vs higher ranks.</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>CAND_0064904</t>
+          <t>CAND_0061550</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -2453,19 +2453,19 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>0.8031</t>
+          <t>0.8023</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Lower-tier shortlist entry — AI Engineer at LinkedIn (4.9 YOE); JD-aligned skills: Embeddings, Elasticsearch, LLMs. Key gaps: 90-day notice period.</t>
+          <t>Lower-tier shortlist entry — ML Engineer at Infosys (5.3 YOE); JD-aligned skills: Sentence Transformers. Key gaps: only 1 core JD skill matched.</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>CAND_0027723</t>
+          <t>CAND_0001707</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -2475,19 +2475,19 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>0.8023</t>
+          <t>0.8019</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Lower-tier shortlist entry — ML Engineer at Wysa (4.2 YOE); JD-aligned skills: Vector Search, NLP, Elasticsearch. Key gaps: weak secondary signals vs higher ranks.</t>
+          <t>Lower-tier shortlist entry — Data Scientist at Vedantu (5.6 YOE); JD-aligned skills: Sentence Transformers, FAISS, Weaviate. Key gaps: 90-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>CAND_0061550</t>
+          <t>CAND_0005477</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2497,19 +2497,19 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>0.8023</t>
+          <t>0.8012</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Lower-tier shortlist entry — ML Engineer at Infosys (5.3 YOE); JD-aligned skills: Sentence Transformers. Key gaps: only 1 core JD skill matched.</t>
+          <t>Lower-tier shortlist entry — ML Engineer at Zomato (6.2 YOE); JD-aligned skills: OpenSearch. Key gaps: only 1 core JD skill matched.</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>CAND_0001707</t>
+          <t>CAND_0013536</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -2519,19 +2519,19 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>0.8019</t>
+          <t>0.8009</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Lower-tier shortlist entry — Data Scientist at Vedantu (5.6 YOE); JD-aligned skills: Sentence Transformers, FAISS, Weaviate. Key gaps: 90-day notice period.</t>
+          <t>Lower-tier shortlist entry — Applied ML Engineer at Haptik (14.1 YOE); JD-aligned skills: LLMs, NLP, Embeddings. Key gaps: 90-day notice period; experience above target band for this role.</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>CAND_0005477</t>
+          <t>CAND_0015057</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -2541,19 +2541,19 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>0.8012</t>
+          <t>0.7999</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Lower-tier shortlist entry — ML Engineer at Zomato (6.2 YOE); JD-aligned skills: OpenSearch. Key gaps: only 1 core JD skill matched.</t>
+          <t>Lower-tier shortlist entry — ML Engineer at Meesho (4.6 YOE); JD-aligned skills: Sentence Transformers, Vector Search, Embeddings. Key gaps: 90-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>CAND_0013536</t>
+          <t>CAND_0030348</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -2563,19 +2563,19 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>0.8009</t>
+          <t>0.7992</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Lower-tier shortlist entry — Applied ML Engineer at Haptik (14.1 YOE); JD-aligned skills: LLMs, NLP, Embeddings. Key gaps: 90-day notice period; experience above target band for this role.</t>
+          <t>Lower-tier shortlist entry — Machine Learning Engineer at BYJU'S (4.5 YOE); JD-aligned skills: Embeddings, Vector Search, Elasticsearch. Key gaps: weak secondary signals vs higher ranks.</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>CAND_0015057</t>
+          <t>CAND_0060538</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -2585,19 +2585,19 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>0.7999</t>
+          <t>0.7983</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Lower-tier shortlist entry — ML Engineer at Meesho (4.6 YOE); JD-aligned skills: Sentence Transformers, Vector Search, Embeddings. Key gaps: 90-day notice period.</t>
+          <t>Lower-tier shortlist entry — ML Engineer at Verloop.io (5.2 YOE); JD-aligned skills: OpenSearch, Embeddings, Milvus. Key gaps: 90-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>CAND_0030348</t>
+          <t>CAND_0049615</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -2607,19 +2607,19 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>0.7992</t>
+          <t>0.7961</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Lower-tier shortlist entry — Machine Learning Engineer at BYJU'S (4.5 YOE); JD-aligned skills: Embeddings, Vector Search, Elasticsearch. Key gaps: weak secondary signals vs higher ranks.</t>
+          <t>Lower-tier shortlist entry — ML Engineer at Krutrim (5.1 YOE); JD-aligned skills: NLP, Pinecone. Key gaps: weak secondary signals vs higher ranks.</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>CAND_0049615</t>
+          <t>CAND_0019159</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -2629,12 +2629,12 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>0.7961</t>
+          <t>0.7956</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Lower-tier shortlist entry — ML Engineer at Krutrim (5.1 YOE); JD-aligned skills: NLP, Pinecone. Key gaps: weak secondary signals vs higher ranks.</t>
+          <t>Lower-tier shortlist entry — ML Engineer at Genpact AI (6.1 YOE); JD-aligned skills: Vector Search, Qdrant, Sentence Transformers. Key gaps: not flagged open to work.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: regenerate validated submission and demo sample
</commit_message>
<xml_diff>
--- a/submission.xlsx
+++ b/submission.xlsx
@@ -441,7 +441,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>CAND_0045250</t>
+          <t>CAND_0080766</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -451,12 +451,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>1.0622</t>
+          <t>0.9107</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Rank 1: Applied ML Engineer at Rephrase.ai (6.6 YOE); JD-aligned skills: Sentence Transformers, Milvus, Embeddings. Top-tier composite score across career, skills, and availability. Counterfactual: ranks on career trajectory and assessed depth over keyword coverage (7/20 listed must-haves), aligning with the JD anti-keyword-stuffing guidance.</t>
+          <t>Rank 1: Staff Machine Learning Engineer at Salesforce (8.8 YOE); JD-aligned skills: Elasticsearch, OpenSearch, Python. Top-tier composite score across career, skills, and availability. Counterfactual: ranks on career trajectory and assessed depth over keyword coverage (4/20 listed must-haves), aligning with the JD anti-keyword-stuffing guidance.</t>
         </is>
       </c>
     </row>
@@ -473,7 +473,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>1.0281</t>
+          <t>0.9058</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -485,7 +485,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>CAND_0071974</t>
+          <t>CAND_0068351</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -495,19 +495,19 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>1.0153</t>
+          <t>0.8977</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Rank 3: Senior AI Engineer at Netflix (7.8 YOE); JD-aligned skills: Weaviate, Pinecone, Qdrant. Top-tier composite score across career, skills, and availability. Counterfactual: ranks on career trajectory and assessed depth over keyword coverage (6/20 listed must-haves), aligning with the JD anti-keyword-stuffing guidance.</t>
+          <t>Rank 3: Lead AI Engineer at Sarvam AI (6.4 YOE); JD-aligned skills: Qdrant, Elasticsearch, Python. Top-tier composite score across career, skills, and availability. Counterfactual: ranks on career trajectory and assessed depth over keyword coverage (4/20 listed must-haves), aligning with the JD anti-keyword-stuffing guidance.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>CAND_0096142</t>
+          <t>CAND_0077337</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -517,19 +517,19 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>1.0027</t>
+          <t>0.8977</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Rank 4: Applied ML Engineer at upGrad (5.0 YOE); JD-aligned skills: Weaviate, Pinecone, Python. Top-tier composite score across career, skills, and availability. Minor note: 120-day notice period.</t>
+          <t>Rank 4: Staff Machine Learning Engineer at Paytm (7.0 YOE); JD-aligned skills: Pinecone, LLMs, Qdrant. Top-tier composite score across career, skills, and availability. Counterfactual: ranks on career trajectory and assessed depth over keyword coverage (6/20 listed must-haves), aligning with the JD anti-keyword-stuffing guidance.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CAND_0002025</t>
+          <t>CAND_0096142</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -539,19 +539,19 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>0.9945</t>
+          <t>0.8938</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Rank 5: Senior AI Engineer at Apple (5.9 YOE); JD-aligned skills: FAISS, OpenSearch, Weaviate. Top-tier composite score across career, skills, and availability. Counterfactual: ranks on career trajectory and assessed depth over keyword coverage (8/20 listed must-haves), aligning with the JD anti-keyword-stuffing guidance.</t>
+          <t>Rank 5: Applied ML Engineer at upGrad (5.0 YOE); JD-aligned skills: Weaviate, Pinecone, Python. Top-tier composite score across career, skills, and availability. Minor note: 120-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>CAND_0087630</t>
+          <t>CAND_0018499</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -561,19 +561,19 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>0.9906</t>
+          <t>0.8901</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Strong match — AI Engineer at Vedantu (7.2 YOE); JD-aligned skills: Elasticsearch, NLP, Embeddings.</t>
+          <t>Strong match — Senior Machine Learning Engineer at Zomato (7.2 YOE); JD-aligned skills: Weaviate, Pinecone, Milvus.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>CAND_0018499</t>
+          <t>CAND_0071974</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -583,19 +583,19 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>0.9772</t>
+          <t>0.8893</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Strong match — Senior Machine Learning Engineer at Zomato (7.2 YOE); JD-aligned skills: Weaviate, Pinecone, Milvus.</t>
+          <t>Strong match — Senior AI Engineer at Netflix (7.8 YOE); JD-aligned skills: Weaviate, Pinecone, Qdrant.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>CAND_0068351</t>
+          <t>CAND_0002025</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -605,19 +605,19 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>0.9707</t>
+          <t>0.8831</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Strong match — Lead AI Engineer at Sarvam AI (6.4 YOE); JD-aligned skills: Qdrant, Elasticsearch, Python.</t>
+          <t>Strong match — Senior AI Engineer at Apple (5.9 YOE); JD-aligned skills: FAISS, OpenSearch, Weaviate.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>CAND_0020350</t>
+          <t>CAND_0081846</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -627,19 +627,19 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>0.9670</t>
+          <t>0.8778</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Strong match — AI Engineer at Zoho (5.8 YOE); JD-aligned skills: NLP, LLMs, FAISS.</t>
+          <t>Strong match — Lead AI Engineer at Razorpay (6.7 YOE); JD-aligned skills: Elasticsearch, Vector Search, Python.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>CAND_0068811</t>
+          <t>CAND_0088025</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -649,19 +649,19 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>0.9656</t>
+          <t>0.8769</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Strong match — Applied ML Engineer at Freshworks (8.0 YOE); JD-aligned skills: Vector Search, Qdrant, Embeddings.</t>
+          <t>Strong match — Staff Machine Learning Engineer at Yellow.ai (8.6 YOE); JD-aligned skills: Pinecone, LLMs, Elasticsearch. Watch: 90-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>CAND_0044855</t>
+          <t>CAND_0038368</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -671,19 +671,19 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>0.9650</t>
+          <t>0.8690</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Strong match — Senior Data Scientist at Flipkart (6.6 YOE); JD-aligned skills: OpenSearch, Pinecone, Vector Search.</t>
+          <t>Strong match — ML Engineer at PhonePe (5.4 YOE); JD-aligned skills: Embeddings, FAISS, NLP.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>CAND_0080766</t>
+          <t>CAND_0046525</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -693,19 +693,19 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>0.9558</t>
+          <t>0.8658</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Strong match — Staff Machine Learning Engineer at Salesforce (8.8 YOE); JD-aligned skills: Elasticsearch, OpenSearch, Python.</t>
+          <t>Strong match — Senior Machine Learning Engineer at Genpact AI (6.1 YOE); JD-aligned skills: Elasticsearch, LLMs, NLP.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>CAND_0088025</t>
+          <t>CAND_0039383</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -715,19 +715,19 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>0.9520</t>
+          <t>0.8585</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Strong match — Staff Machine Learning Engineer at Yellow.ai (8.6 YOE); JD-aligned skills: Pinecone, LLMs, Elasticsearch. Watch: 90-day notice period.</t>
+          <t>Strong match — Applied ML Engineer at Meesho (7.1 YOE); JD-aligned skills: FAISS, NLP, Vector Search. Watch: 90-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>CAND_0044222</t>
+          <t>CAND_0087630</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -737,19 +737,19 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>0.9489</t>
+          <t>0.8576</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Strong match — AI Engineer at PolicyBazaar (7.7 YOE); JD-aligned skills: Vector Search, OpenSearch, Qdrant.</t>
+          <t>Strong match — AI Engineer at Vedantu (7.2 YOE); JD-aligned skills: Elasticsearch, NLP, Embeddings.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>CAND_0039383</t>
+          <t>CAND_0044222</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -759,19 +759,19 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>0.9468</t>
+          <t>0.8566</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Strong match — Applied ML Engineer at Meesho (7.1 YOE); JD-aligned skills: FAISS, NLP, Vector Search. Watch: 90-day notice period.</t>
+          <t>Strong match — AI Engineer at PolicyBazaar (7.7 YOE); JD-aligned skills: Vector Search, OpenSearch, Qdrant.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>CAND_0077337</t>
+          <t>CAND_0044855</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -781,19 +781,19 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>0.9405</t>
+          <t>0.8553</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Strong match — Staff Machine Learning Engineer at Paytm (7.0 YOE); JD-aligned skills: Pinecone, LLMs, Qdrant.</t>
+          <t>Strong match — Senior Data Scientist at Flipkart (6.6 YOE); JD-aligned skills: OpenSearch, Pinecone, Vector Search.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>CAND_0046525</t>
+          <t>CAND_0061257</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -803,19 +803,19 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>0.9402</t>
+          <t>0.8551</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Strong match — Senior Machine Learning Engineer at Genpact AI (6.1 YOE); JD-aligned skills: Elasticsearch, LLMs, NLP.</t>
+          <t>Strong match — Staff Machine Learning Engineer at LinkedIn (8.0 YOE); JD-aligned skills: Python. Watch: only 1 core JD skill matched.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>CAND_0042029</t>
+          <t>CAND_0045250</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -825,19 +825,19 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>0.9382</t>
+          <t>0.8527</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Strong match — Senior Data Scientist at Flipkart (6.5 YOE); JD-aligned skills: NLP, Elasticsearch, Embeddings.</t>
+          <t>Strong match — Applied ML Engineer at Rephrase.ai (6.6 YOE); JD-aligned skills: Sentence Transformers, Milvus, Embeddings.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>CAND_0065514</t>
+          <t>CAND_0050454</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -847,19 +847,19 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>0.9377</t>
+          <t>0.8443</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Strong match — ML Engineer at Genpact AI (6.6 YOE); JD-aligned skills: Vector Search, Pinecone, Elasticsearch. Watch: 90-day notice period.</t>
+          <t>Strong match — AI Engineer at Rephrase.ai (6.8 YOE); JD-aligned skills: Fine-tuning LLMs, FAISS, Qdrant.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>CAND_0020877</t>
+          <t>CAND_0020350</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -869,19 +869,19 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>0.9367</t>
+          <t>0.8423</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Strong match — Applied ML Engineer at CRED (5.1 YOE); JD-aligned skills: Elasticsearch, OpenSearch, Weaviate.</t>
+          <t>Strong match — AI Engineer at Zoho (5.8 YOE); JD-aligned skills: NLP, LLMs, FAISS.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>CAND_0071939</t>
+          <t>CAND_0042029</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -891,19 +891,19 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>0.9320</t>
+          <t>0.8406</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Solid profile: Data Scientist at Krutrim (6.4 YOE); JD-aligned skills: Elasticsearch, OpenSearch, Embeddings.</t>
+          <t>Solid profile: Senior Data Scientist at Flipkart (6.5 YOE); JD-aligned skills: NLP, Elasticsearch, Embeddings.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>CAND_0081846</t>
+          <t>CAND_0068811</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -913,19 +913,19 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>0.9260</t>
+          <t>0.8385</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Good fit with caveats: Lead AI Engineer at Razorpay (6.7 YOE); JD-aligned skills: Elasticsearch, Vector Search, Python.</t>
+          <t>Good fit with caveats: Applied ML Engineer at Freshworks (8.0 YOE); JD-aligned skills: Vector Search, Qdrant, Embeddings.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>CAND_0037566</t>
+          <t>CAND_0086022</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -935,19 +935,19 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>0.9243</t>
+          <t>0.8342</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Competitive candidate: Machine Learning Engineer at LinkedIn (6.9 YOE); JD-aligned skills: Pinecone, NLP, LLMs.</t>
+          <t>Competitive candidate: Senior Applied Scientist at Sarvam AI (5.3 YOE); JD-aligned skills: Vector Search, Fine-tuning LLMs, Elasticsearch.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>CAND_0038368</t>
+          <t>CAND_0047721</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -957,19 +957,19 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>0.9223</t>
+          <t>0.8322</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Meets several JD signals: ML Engineer at PhonePe (5.4 YOE); JD-aligned skills: Embeddings, FAISS, NLP.</t>
+          <t>Meets several JD signals: Senior Data Scientist at Microsoft (7.0 YOE); JD-aligned skills: Milvus, FAISS, Qdrant. Concerns: 90-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>CAND_0009691</t>
+          <t>CAND_0030031</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -979,19 +979,19 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>0.9106</t>
+          <t>0.8310</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Solid profile: Applied ML Engineer at LinkedIn (6.2 YOE); JD-aligned skills: Fine-tuning LLMs, Pinecone, Sentence Transformers. Concerns: 120-day notice period.</t>
+          <t>Solid profile: AI Engineer at Microsoft (5.7 YOE); JD-aligned skills: Python, NLP, Sentence Transformers.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>CAND_0050454</t>
+          <t>CAND_0090584</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1001,19 +1001,19 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>0.9105</t>
+          <t>0.8287</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Good fit with caveats: AI Engineer at Rephrase.ai (6.8 YOE); JD-aligned skills: Fine-tuning LLMs, FAISS, Qdrant.</t>
+          <t>Good fit with caveats: ML Engineer at Flipkart (5.1 YOE); JD-aligned skills: Fine-tuning LLMs, OpenSearch, FAISS. Concerns: 120-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>CAND_0079064</t>
+          <t>CAND_0032216</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1023,19 +1023,19 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>0.9088</t>
+          <t>0.8275</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Competitive candidate: Senior Data Scientist at Niramai (5.2 YOE); JD-aligned skills: OpenSearch, NLP, Fine-tuning LLMs. Concerns: 120-day notice period.</t>
+          <t>Competitive candidate: ML Engineer at upGrad (6.1 YOE); JD-aligned skills: Qdrant, Sentence Transformers, Vector Search.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>CAND_0090584</t>
+          <t>CAND_0037944</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1045,19 +1045,19 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>0.9042</t>
+          <t>0.8271</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Meets several JD signals: ML Engineer at Flipkart (5.1 YOE); JD-aligned skills: Fine-tuning LLMs, OpenSearch, FAISS. Concerns: 120-day notice period.</t>
+          <t>Meets several JD signals: Senior Data Scientist at Vedantu (4.9 YOE); JD-aligned skills: Vector Search, OpenSearch, Embeddings.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>CAND_0030031</t>
+          <t>CAND_0075574</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1067,19 +1067,19 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>0.9020</t>
+          <t>0.8261</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Solid profile: AI Engineer at Microsoft (5.7 YOE); JD-aligned skills: Python, NLP, Sentence Transformers.</t>
+          <t>Solid profile: Machine Learning Engineer at Haptik (5.7 YOE); JD-aligned skills: Weaviate, OpenSearch, Qdrant.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>CAND_0089552</t>
+          <t>CAND_0049538</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1089,19 +1089,19 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>0.8970</t>
+          <t>0.8252</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Good fit with caveats: Machine Learning Engineer at Netflix (6.0 YOE); JD-aligned skills: Weaviate, Qdrant, Vector Search. Concerns: 120-day notice period.</t>
+          <t>Good fit with caveats: Applied ML Engineer at Saarthi.ai (5.8 YOE); JD-aligned skills: OpenSearch, Vector Search, Milvus.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>CAND_0010257</t>
+          <t>CAND_0003841</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1111,19 +1111,19 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>0.8967</t>
+          <t>0.8204</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Competitive candidate: Senior Data Scientist at Google (6.5 YOE); JD-aligned skills: Milvus, Python, OpenSearch. Concerns: 120-day notice period.</t>
+          <t>Competitive candidate: ML Engineer at Tech Mahindra (5.0 YOE); JD-aligned skills: Pinecone, Fine-tuning LLMs, Sentence Transformers.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>CAND_0099806</t>
+          <t>CAND_0020877</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1133,19 +1133,19 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>0.8924</t>
+          <t>0.8197</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Meets several JD signals: AI Engineer at Mad Street Den (4.6 YOE); JD-aligned skills: FAISS, Embeddings, Sentence Transformers.</t>
+          <t>Meets several JD signals: Applied ML Engineer at CRED (5.1 YOE); JD-aligned skills: Elasticsearch, OpenSearch, Weaviate.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>CAND_0075574</t>
+          <t>CAND_0043228</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1155,19 +1155,19 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>0.8903</t>
+          <t>0.8196</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Solid profile: Machine Learning Engineer at Haptik (5.7 YOE); JD-aligned skills: Weaviate, OpenSearch, Qdrant.</t>
+          <t>Solid profile: Applied ML Engineer at Zoho (6.8 YOE); JD-aligned skills: NLP, Vector Search, Sentence Transformers.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>CAND_0032216</t>
+          <t>CAND_0037566</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1177,19 +1177,19 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>0.8901</t>
+          <t>0.8188</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Good fit with caveats: ML Engineer at upGrad (6.1 YOE); JD-aligned skills: Qdrant, Sentence Transformers, Vector Search.</t>
+          <t>Good fit with caveats: Machine Learning Engineer at LinkedIn (6.9 YOE); JD-aligned skills: Pinecone, NLP, LLMs.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>CAND_0037944</t>
+          <t>CAND_0079387</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1199,19 +1199,19 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>0.8855</t>
+          <t>0.8185</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Competitive candidate: Senior Data Scientist at Vedantu (4.9 YOE); JD-aligned skills: Vector Search, OpenSearch, Embeddings.</t>
+          <t>Competitive candidate: AI Engineer at Microsoft (6.9 YOE); JD-aligned skills: Python, Sentence Transformers, Vector Search.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>CAND_0049538</t>
+          <t>CAND_0098217</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1221,19 +1221,19 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>0.8796</t>
+          <t>0.8171</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Meets several JD signals: Applied ML Engineer at Saarthi.ai (5.8 YOE); JD-aligned skills: OpenSearch, Vector Search, Milvus.</t>
+          <t>Meets several JD signals: ML Engineer at Glance (6.4 YOE); JD-aligned skills: FAISS, Pinecone.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>CAND_0047721</t>
+          <t>CAND_0099806</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1243,19 +1243,19 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>0.8791</t>
+          <t>0.8155</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Solid profile: Senior Data Scientist at Microsoft (7.0 YOE); JD-aligned skills: Milvus, FAISS, Qdrant. Concerns: 90-day notice period.</t>
+          <t>Solid profile: AI Engineer at Mad Street Den (4.6 YOE); JD-aligned skills: FAISS, Embeddings, Sentence Transformers.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>CAND_0042100</t>
+          <t>CAND_0055905</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1265,19 +1265,19 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>0.8773</t>
+          <t>0.8149</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Good fit with caveats: Machine Learning Engineer at Freshworks (7.3 YOE); JD-aligned skills: Elasticsearch, Fine-tuning LLMs, Pinecone. Concerns: 90-day notice period.</t>
+          <t>Good fit with caveats: Senior Machine Learning Engineer at Flipkart (8.1 YOE); JD-aligned skills: Elasticsearch, Python, LLMs.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>CAND_0043228</t>
+          <t>CAND_0051004</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1287,19 +1287,19 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>0.8758</t>
+          <t>0.8145</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Competitive candidate: Applied ML Engineer at Zoho (6.8 YOE); JD-aligned skills: NLP, Vector Search, Sentence Transformers.</t>
+          <t>Competitive candidate: Senior Data Scientist at CRED (4.7 YOE); JD-aligned skills: Embeddings, Qdrant, Fine-tuning LLMs.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>CAND_0083879</t>
+          <t>CAND_0018094</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1309,19 +1309,19 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>0.8736</t>
+          <t>0.8120</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Meets several JD signals: Machine Learning Engineer at Ola (7.1 YOE); JD-aligned skills: Fine-tuning LLMs, Milvus, Sentence Transformers.</t>
+          <t>Meets several JD signals: ML Engineer at Mad Street Den (5.2 YOE); JD-aligned skills: Pinecone, Fine-tuning LLMs.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>CAND_0003841</t>
+          <t>CAND_0081852</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1331,19 +1331,19 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>0.8722</t>
+          <t>0.8110</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Solid profile: ML Engineer at Tech Mahindra (5.0 YOE); JD-aligned skills: Pinecone, Fine-tuning LLMs, Sentence Transformers.</t>
+          <t>Solid profile: Senior Data Scientist at Mad Street Den (5.9 YOE); JD-aligned skills: Milvus, Weaviate, Vector Search.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>CAND_0081852</t>
+          <t>CAND_0083879</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1353,19 +1353,19 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>0.8712</t>
+          <t>0.8058</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Good fit with caveats: Senior Data Scientist at Mad Street Den (5.9 YOE); JD-aligned skills: Milvus, Weaviate, Vector Search.</t>
+          <t>Good fit with caveats: Machine Learning Engineer at Ola (7.1 YOE); JD-aligned skills: Fine-tuning LLMs, Milvus, Sentence Transformers.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>CAND_0079284</t>
+          <t>CAND_0058688</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1375,19 +1375,19 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>0.8702</t>
+          <t>0.7999</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Competitive candidate: Machine Learning Engineer at Google (4.9 YOE); JD-aligned skills: Qdrant, Fine-tuning LLMs, Elasticsearch.</t>
+          <t>Competitive candidate: AI Engineer at Vedantu (6.7 YOE); JD-aligned skills: Embeddings, Milvus.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>CAND_0079387</t>
+          <t>CAND_0079284</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1397,19 +1397,19 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>0.8678</t>
+          <t>0.7976</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Meets several JD signals: AI Engineer at Microsoft (6.9 YOE); JD-aligned skills: Python, Sentence Transformers, Vector Search.</t>
+          <t>Meets several JD signals: Machine Learning Engineer at Google (4.9 YOE); JD-aligned skills: Qdrant, Fine-tuning LLMs, Elasticsearch.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>CAND_0086022</t>
+          <t>CAND_0041669</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -1419,19 +1419,19 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>0.8678</t>
+          <t>0.7936</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Solid profile: Senior Applied Scientist at Sarvam AI (5.3 YOE); JD-aligned skills: Vector Search, Fine-tuning LLMs, Elasticsearch.</t>
+          <t>Solid profile: Recommendation Systems Engineer at CRED (8.0 YOE); JD-aligned skills: FAISS, Milvus, Weaviate.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>CAND_0040178</t>
+          <t>CAND_0076482</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -1441,19 +1441,19 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>0.8654</t>
+          <t>0.7909</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Good fit with caveats: ML Engineer at Meesho (5.0 YOE); JD-aligned skills: Weaviate, Fine-tuning LLMs, Vector Search.</t>
+          <t>Good fit with caveats: ML Engineer at Flipkart (6.6 YOE); JD-aligned skills: OpenSearch, Pinecone, Embeddings.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>CAND_0018094</t>
+          <t>CAND_0009691</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -1463,19 +1463,19 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>0.8633</t>
+          <t>0.7893</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Competitive candidate: ML Engineer at Mad Street Den (5.2 YOE); JD-aligned skills: Pinecone, Fine-tuning LLMs.</t>
+          <t>Competitive candidate: Applied ML Engineer at LinkedIn (6.2 YOE); JD-aligned skills: Fine-tuning LLMs, Pinecone, Sentence Transformers. Concerns: 120-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>CAND_0035653</t>
+          <t>CAND_0095528</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1485,19 +1485,19 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>0.8631</t>
+          <t>0.7892</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Meets several JD signals: Data Scientist at Swiggy (5.6 YOE); JD-aligned skills: OpenSearch, Vector Search, Fine-tuning LLMs.</t>
+          <t>Meets several JD signals: Senior Data Scientist at Netflix (5.3 YOE); JD-aligned skills: OpenSearch, Vector Search, Qdrant.</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>CAND_0093193</t>
+          <t>CAND_0052328</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -1507,19 +1507,19 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>0.8628</t>
+          <t>0.7883</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Solid profile: Senior Machine Learning Engineer at Niramai (7.9 YOE); JD-aligned skills: Qdrant, OpenSearch.</t>
+          <t>Solid profile: Recommendation Systems Engineer at Amazon (6.5 YOE); JD-aligned skills: OpenSearch, Fine-tuning LLMs, Vector Search.</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>CAND_0061257</t>
+          <t>CAND_0079064</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -1529,19 +1529,19 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>0.8621</t>
+          <t>0.7866</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Good fit with caveats: Staff Machine Learning Engineer at LinkedIn (8.0 YOE); JD-aligned skills: Python. Concerns: only 1 core JD skill matched.</t>
+          <t>Good fit with caveats: Senior Data Scientist at Niramai (5.2 YOE); JD-aligned skills: OpenSearch, NLP, Fine-tuning LLMs. Concerns: 120-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>CAND_0076482</t>
+          <t>CAND_0040178</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -1551,12 +1551,12 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>0.8605</t>
+          <t>0.7854</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Moderate fit: ML Engineer at Flipkart (6.6 YOE); JD-aligned skills: OpenSearch, Pinecone, Embeddings. Gaps: under half of JD must-have skills covered.</t>
+          <t>Moderate fit: ML Engineer at Meesho (5.0 YOE); JD-aligned skills: Weaviate, Fine-tuning LLMs, Vector Search. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
@@ -1573,7 +1573,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>0.8561</t>
+          <t>0.7850</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -1585,7 +1585,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>CAND_0055905</t>
+          <t>CAND_0005649</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -1595,19 +1595,19 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>0.8558</t>
+          <t>0.7836</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Acceptable but not standout: Senior Machine Learning Engineer at Flipkart (8.1 YOE); JD-aligned skills: Elasticsearch, Python, LLMs. Gaps: under half of JD must-have skills covered.</t>
+          <t>Acceptable but not standout: Senior Data Scientist at Sarvam AI (7.4 YOE); JD-aligned skills: Fine-tuning LLMs, Weaviate. Gaps: 90-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>CAND_0015578</t>
+          <t>CAND_0055992</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -1617,19 +1617,19 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>0.8557</t>
+          <t>0.7833</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Mixed signals: AI Engineer at Zoho (5.4 YOE); JD-aligned skills: Embeddings, NLP, Sentence Transformers. Gaps: 90-day notice period.</t>
+          <t>Mixed signals: AI Engineer at CRED (16.9 YOE); JD-aligned skills: FAISS, OpenSearch, Embeddings. Gaps: experience above target band for this role.</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>CAND_0051004</t>
+          <t>CAND_0015582</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -1639,19 +1639,19 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>0.8544</t>
+          <t>0.7831</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>JD overlap is thin: Senior Data Scientist at CRED (4.7 YOE); JD-aligned skills: Embeddings, Qdrant, Fine-tuning LLMs. Gaps: under half of JD must-have skills covered.</t>
+          <t>JD overlap is thin: ML Engineer at Genpact AI (4.4 YOE); JD-aligned skills: Qdrant, Sentence Transformers, Embeddings. Gaps: 120-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>CAND_0095528</t>
+          <t>CAND_0061550</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -1661,12 +1661,12 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>0.8539</t>
+          <t>0.7799</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Moderate fit: Senior Data Scientist at Netflix (5.3 YOE); JD-aligned skills: OpenSearch, Vector Search, Qdrant. Gaps: under half of JD must-have skills covered.</t>
+          <t>Moderate fit: ML Engineer at Infosys (5.3 YOE); JD-aligned skills: Sentence Transformers. Gaps: only 1 core JD skill matched.</t>
         </is>
       </c>
     </row>
@@ -1683,7 +1683,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>0.8507</t>
+          <t>0.7768</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -1695,7 +1695,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>CAND_0073982</t>
+          <t>CAND_0074735</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -1705,19 +1705,19 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>0.8500</t>
+          <t>0.7764</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Acceptable but not standout: Data Scientist at Dream11 (7.0 YOE); JD-aligned skills: Sentence Transformers, Qdrant, FAISS. Gaps: under half of JD must-have skills covered.</t>
+          <t>Acceptable but not standout: Applied ML Engineer at Rephrase.ai (5.5 YOE); JD-aligned skills: Weaviate, Vector Search, Elasticsearch. Gaps: 90-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>CAND_0069905</t>
+          <t>CAND_0015578</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -1727,19 +1727,19 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>0.8499</t>
+          <t>0.7761</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Mixed signals: Applied ML Engineer at Sarvam AI (6.6 YOE); JD-aligned skills: Sentence Transformers, Python, Weaviate. Gaps: 90-day notice period.</t>
+          <t>Mixed signals: AI Engineer at Zoho (5.4 YOE); JD-aligned skills: Embeddings, NLP, Sentence Transformers. Gaps: 90-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>CAND_0036121</t>
+          <t>CAND_0016163</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -1749,19 +1749,19 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>0.8491</t>
+          <t>0.7759</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>JD overlap is thin: ML Engineer at Wysa (5.2 YOE); JD-aligned skills: Embeddings, Vector Search. Gaps: under half of JD must-have skills covered.</t>
+          <t>JD overlap is thin: Applied ML Engineer at Dream11 (6.7 YOE); JD-aligned skills: Weaviate, Embeddings, Pinecone. Gaps: 120-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>CAND_0013393</t>
+          <t>CAND_0018293</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -1771,19 +1771,19 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>0.8469</t>
+          <t>0.7736</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Moderate fit: ML Engineer at Freshworks (5.3 YOE); JD-aligned skills: Embeddings, Pinecone, Qdrant. Gaps: under half of JD must-have skills covered.</t>
+          <t>Moderate fit: Data Scientist at PharmEasy (5.6 YOE); JD-aligned skills: Weaviate. Gaps: only 1 core JD skill matched.</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>CAND_0095213</t>
+          <t>CAND_0069905</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -1793,19 +1793,19 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>0.8469</t>
+          <t>0.7719</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Partial alignment: ML Engineer at Genpact AI (5.1 YOE); JD-aligned skills: Python, Weaviate, Pinecone. Gaps: under half of JD must-have skills covered.</t>
+          <t>Partial alignment: Applied ML Engineer at Sarvam AI (6.6 YOE); JD-aligned skills: Sentence Transformers, Python, Weaviate. Gaps: 90-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>CAND_0015582</t>
+          <t>CAND_0089552</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -1815,19 +1815,19 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>0.8468</t>
+          <t>0.7705</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Acceptable but not standout: ML Engineer at Genpact AI (4.4 YOE); JD-aligned skills: Qdrant, Sentence Transformers, Embeddings. Gaps: 120-day notice period.</t>
+          <t>Acceptable but not standout: Machine Learning Engineer at Netflix (6.0 YOE); JD-aligned skills: Weaviate, Qdrant, Vector Search. Gaps: 120-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>CAND_0091909</t>
+          <t>CAND_0067866</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -1837,19 +1837,19 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>0.8468</t>
+          <t>0.7699</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Mixed signals: Machine Learning Engineer at Rephrase.ai (6.9 YOE); JD-aligned skills: LLMs, Pinecone, Qdrant. Gaps: under half of JD must-have skills covered.</t>
+          <t>Mixed signals: Senior Software Engineer (ML) at Tech Mahindra (6.4 YOE); JD-aligned skills: Embeddings, Elasticsearch, Qdrant. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>CAND_0016163</t>
+          <t>CAND_0048166</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -1859,19 +1859,19 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>0.8452</t>
+          <t>0.7697</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>JD overlap is thin: Applied ML Engineer at Dream11 (6.7 YOE); JD-aligned skills: Weaviate, Embeddings, Pinecone. Gaps: 120-day notice period.</t>
+          <t>JD overlap is thin: ML Engineer at Aganitha (5.2 YOE); JD-aligned skills: Pinecone, Milvus, Qdrant. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>CAND_0007460</t>
+          <t>CAND_0042100</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -1881,19 +1881,19 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>0.8450</t>
+          <t>0.7689</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Moderate fit: AI Engineer at Salesforce (4.7 YOE); JD-aligned skills: Embeddings, Weaviate, NLP. Gaps: 120-day notice period.</t>
+          <t>Moderate fit: Machine Learning Engineer at Freshworks (7.3 YOE); JD-aligned skills: Elasticsearch, Fine-tuning LLMs, Pinecone. Gaps: 90-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>CAND_0011432</t>
+          <t>CAND_0050876</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -1903,19 +1903,19 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>0.8405</t>
+          <t>0.7682</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Partial alignment: Senior Data Scientist at Amazon (7.6 YOE); JD-aligned skills: OpenSearch, Elasticsearch. Gaps: under half of JD must-have skills covered.</t>
+          <t>Partial alignment: Applied ML Engineer at Freshworks (6.0 YOE); JD-aligned skills: Qdrant, FAISS, OpenSearch. Gaps: 90-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>CAND_0068932</t>
+          <t>CAND_0091909</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -1925,19 +1925,19 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>0.8404</t>
+          <t>0.7668</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Acceptable but not standout: ML Engineer at Krutrim (5.2 YOE); JD-aligned skills: Milvus, OpenSearch. Gaps: under half of JD must-have skills covered.</t>
+          <t>Acceptable but not standout: Machine Learning Engineer at Rephrase.ai (6.9 YOE); JD-aligned skills: LLMs, Pinecone, Qdrant. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>CAND_0090155</t>
+          <t>CAND_0065514</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -1947,19 +1947,19 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>0.8401</t>
+          <t>0.7666</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Mixed signals: ML Engineer at Swiggy (5.8 YOE); JD-aligned skills: Milvus, Qdrant, Pinecone. Gaps: 90-day notice period.</t>
+          <t>Mixed signals: ML Engineer at Genpact AI (6.6 YOE); JD-aligned skills: Vector Search, Pinecone, Elasticsearch. Gaps: 90-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>CAND_0070398</t>
+          <t>CAND_0010541</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -1969,19 +1969,19 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>0.8390</t>
+          <t>0.7664</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>JD overlap is thin: Machine Learning Engineer at Genpact AI (7.2 YOE); JD-aligned skills: FAISS, Embeddings, Python. Gaps: 120-day notice period.</t>
+          <t>JD overlap is thin: AI Research Engineer at Wysa (6.2 YOE); JD-aligned skills: Pinecone, Weaviate, Python. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>CAND_0098217</t>
+          <t>CAND_0018549</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -1991,19 +1991,19 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>0.8388</t>
+          <t>0.7661</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Moderate fit: ML Engineer at Glance (6.4 YOE); JD-aligned skills: FAISS, Pinecone. Gaps: under half of JD must-have skills covered.</t>
+          <t>Moderate fit: Recommendation Systems Engineer at Uber (6.8 YOE); JD-aligned skills: Weaviate, Elasticsearch, Qdrant. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>CAND_0017093</t>
+          <t>CAND_0066999</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -2013,19 +2013,19 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>0.8378</t>
+          <t>0.7656</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Partial alignment: ML Engineer at Zoho (5.9 YOE); JD-aligned skills: LLMs, Embeddings. Gaps: under half of JD must-have skills covered.</t>
+          <t>Partial alignment: Recommendation Systems Engineer at Microsoft (5.9 YOE); JD-aligned skills: OpenSearch, FAISS, LLMs. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>CAND_0052328</t>
+          <t>CAND_0070398</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -2035,19 +2035,19 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>0.8331</t>
+          <t>0.7649</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Acceptable but not standout: Recommendation Systems Engineer at Amazon (6.5 YOE); JD-aligned skills: OpenSearch, Fine-tuning LLMs, Vector Search. Gaps: under half of JD must-have skills covered.</t>
+          <t>Acceptable but not standout: Machine Learning Engineer at Genpact AI (7.2 YOE); JD-aligned skills: FAISS, Embeddings, Python. Gaps: 120-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>CAND_0048166</t>
+          <t>CAND_0017093</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -2057,19 +2057,19 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>0.8317</t>
+          <t>0.7648</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Mixed signals: ML Engineer at Aganitha (5.2 YOE); JD-aligned skills: Pinecone, Milvus, Qdrant. Gaps: not flagged open to work.</t>
+          <t>Mixed signals: ML Engineer at Zoho (5.9 YOE); JD-aligned skills: LLMs, Embeddings. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>CAND_0058688</t>
+          <t>CAND_0092245</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -2079,19 +2079,19 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>0.8288</t>
+          <t>0.7646</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>JD overlap is thin: AI Engineer at Vedantu (6.7 YOE); JD-aligned skills: Embeddings, Milvus. Gaps: under half of JD must-have skills covered.</t>
+          <t>JD overlap is thin: Senior Data Scientist at Ola (4.1 YOE); JD-aligned skills: Embeddings, FAISS, Qdrant. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>CAND_0021836</t>
+          <t>CAND_0093193</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -2101,19 +2101,19 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>0.8220</t>
+          <t>0.7644</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Moderate fit: ML Engineer at CRED (6.5 YOE); JD-aligned skills: Vector Search, Elasticsearch, NLP. Gaps: under half of JD must-have skills covered.</t>
+          <t>Moderate fit: Senior Machine Learning Engineer at Niramai (7.9 YOE); JD-aligned skills: Qdrant, OpenSearch. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>CAND_0050876</t>
+          <t>CAND_0002037</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -2123,19 +2123,19 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>0.8217</t>
+          <t>0.7638</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Partial alignment: Applied ML Engineer at Freshworks (6.0 YOE); JD-aligned skills: Qdrant, FAISS, OpenSearch. Gaps: 90-day notice period.</t>
+          <t>Partial alignment: ML Engineer at Locobuzz (5.5 YOE); JD-aligned skills: Fine-tuning LLMs, Milvus, Pinecone. Gaps: not flagged open to work.</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>CAND_0005649</t>
+          <t>CAND_0093912</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -2145,19 +2145,19 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>0.8212</t>
+          <t>0.7582</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Acceptable but not standout: Senior Data Scientist at Sarvam AI (7.4 YOE); JD-aligned skills: Fine-tuning LLMs, Weaviate. Gaps: 90-day notice period.</t>
+          <t>Acceptable but not standout: Senior Data Scientist at Razorpay (5.3 YOE); JD-aligned skills: Milvus, Embeddings, Vector Search. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>CAND_0092245</t>
+          <t>CAND_0092255</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -2167,19 +2167,19 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>0.8205</t>
+          <t>0.7570</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Mixed signals: Senior Data Scientist at Ola (4.1 YOE); JD-aligned skills: Embeddings, FAISS, Qdrant. Gaps: under half of JD must-have skills covered.</t>
+          <t>Mixed signals: ML Engineer at InMobi (5.2 YOE); JD-aligned skills: Weaviate, OpenSearch, Vector Search. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>CAND_0055992</t>
+          <t>CAND_0010257</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -2189,19 +2189,19 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>0.8191</t>
+          <t>0.7560</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>JD overlap is thin: AI Engineer at CRED (16.9 YOE); JD-aligned skills: FAISS, OpenSearch, Embeddings. Gaps: experience above target band for this role.</t>
+          <t>JD overlap is thin: Senior Data Scientist at Google (6.5 YOE); JD-aligned skills: Milvus, Python, OpenSearch. Gaps: 120-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>CAND_0005538</t>
+          <t>CAND_0099269</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -2211,19 +2211,19 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>0.8165</t>
+          <t>0.7559</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Moderate fit: Senior AI Engineer at Adobe (5.9 YOE); JD-aligned skills: Python. Gaps: only 1 core JD skill matched; 90-day notice period.</t>
+          <t>Moderate fit: Data Scientist at BYJU'S (5.5 YOE); JD-aligned skills: Elasticsearch, Python, NLP. Gaps: 120-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>CAND_0002037</t>
+          <t>CAND_0021836</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -2233,19 +2233,19 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>0.8119</t>
+          <t>0.7532</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Partial alignment: ML Engineer at Locobuzz (5.5 YOE); JD-aligned skills: Fine-tuning LLMs, Milvus, Pinecone. Gaps: not flagged open to work.</t>
+          <t>Partial alignment: ML Engineer at CRED (6.5 YOE); JD-aligned skills: Vector Search, Elasticsearch, NLP. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>CAND_0099269</t>
+          <t>CAND_0032179</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -2255,19 +2255,19 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>0.8091</t>
+          <t>0.7530</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Acceptable but not standout: Data Scientist at BYJU'S (5.5 YOE); JD-aligned skills: Elasticsearch, Python, NLP. Gaps: 120-day notice period.</t>
+          <t>Acceptable but not standout: Computer Vision Engineer at InMobi (6.4 YOE); JD-aligned skills: Vector Search, Weaviate, Python. Gaps: not flagged open to work.</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>CAND_0041669</t>
+          <t>CAND_0060054</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -2277,19 +2277,19 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>0.8089</t>
+          <t>0.7522</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Mixed signals: Recommendation Systems Engineer at CRED (8.0 YOE); JD-aligned skills: FAISS, Milvus, Weaviate. Gaps: under half of JD must-have skills covered.</t>
+          <t>Mixed signals: AI Engineer at Mad Street Den (6.4 YOE); JD-aligned skills: Weaviate, FAISS, Elasticsearch. Gaps: not flagged open to work.</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>CAND_0094759</t>
+          <t>CAND_0005311</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -2299,19 +2299,19 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>0.8073</t>
+          <t>0.7501</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>JD overlap is thin: Lead AI Engineer at Meta (8.6 YOE); JD-aligned skills: Qdrant, Fine-tuning LLMs, Vector Search. Gaps: low recruiter response rate; not flagged open to work.</t>
+          <t>JD overlap is thin: AI Research Engineer at Aganitha (5.7 YOE); JD-aligned skills: Qdrant, Fine-tuning LLMs, NLP. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>CAND_0060054</t>
+          <t>CAND_0054123</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -2321,19 +2321,19 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>0.8066</t>
+          <t>0.7495</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Moderate fit: AI Engineer at Mad Street Den (6.4 YOE); JD-aligned skills: Weaviate, FAISS, Elasticsearch. Gaps: not flagged open to work.</t>
+          <t>Moderate fit: Applied ML Engineer at Meta (4.7 YOE); JD-aligned skills: Python, Weaviate, Qdrant. Gaps: not flagged open to work.</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>CAND_0069232</t>
+          <t>CAND_0027691</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -2343,19 +2343,19 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>0.8057</t>
+          <t>0.7487</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Partial alignment: ML Engineer at Yellow.ai (6.3 YOE); JD-aligned skills: Pinecone, NLP, Python. Gaps: 120-day notice period; not flagged open to work.</t>
+          <t>Partial alignment: NLP Engineer at Haptik (6.5 YOE); JD-aligned skills: Weaviate, Embeddings, Python. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>CAND_0065277</t>
+          <t>CAND_0011432</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -2365,19 +2365,19 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>0.8049</t>
+          <t>0.7483</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Acceptable but not standout: Computer Vision Engineer at Aganitha (6.3 YOE); JD-aligned skills: Vector Search, Milvus, Fine-tuning LLMs. Gaps: under half of JD must-have skills covered.</t>
+          <t>Acceptable but not standout: Senior Data Scientist at Amazon (7.6 YOE); JD-aligned skills: OpenSearch, Elasticsearch. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>CAND_0006418</t>
+          <t>CAND_0065878</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -2387,19 +2387,19 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>0.8037</t>
+          <t>0.7478</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Mixed signals: Machine Learning Engineer at Verloop.io (5.7 YOE); JD-aligned skills: Embeddings, Weaviate, Elasticsearch. Gaps: under half of JD must-have skills covered.</t>
+          <t>Mixed signals: Senior Data Scientist at Niramai (7.8 YOE); JD-aligned skills: Vector Search, Fine-tuning LLMs. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>CAND_0064904</t>
+          <t>CAND_0037980</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -2409,19 +2409,19 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>0.8031</t>
+          <t>0.7474</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>JD overlap is thin: AI Engineer at LinkedIn (4.9 YOE); JD-aligned skills: Embeddings, Elasticsearch, LLMs. Gaps: 90-day notice period.</t>
+          <t>JD overlap is thin: Senior Applied Scientist at Niramai (9.0 YOE); JD-aligned skills: NLP. Gaps: only 1 core JD skill matched.</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>CAND_0027723</t>
+          <t>CAND_0007009</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -2431,19 +2431,19 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>0.8023</t>
+          <t>0.7463</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Lower-tier shortlist entry — ML Engineer at Wysa (4.2 YOE); JD-aligned skills: Vector Search, NLP, Elasticsearch. Key gaps: weak secondary signals vs higher ranks.</t>
+          <t>Lower-tier shortlist entry — Recommendation Systems Engineer at Wysa (7.9 YOE); JD-aligned skills: Weaviate, Python, Embeddings. Key gaps: weak secondary signals vs higher ranks.</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>CAND_0061550</t>
+          <t>CAND_0001819</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -2453,19 +2453,19 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>0.8023</t>
+          <t>0.7460</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Lower-tier shortlist entry — ML Engineer at Infosys (5.3 YOE); JD-aligned skills: Sentence Transformers. Key gaps: only 1 core JD skill matched.</t>
+          <t>Lower-tier shortlist entry — ML Engineer at Genpact AI (4.4 YOE); JD-aligned skills: Weaviate, NLP. Key gaps: weak secondary signals vs higher ranks.</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>CAND_0001707</t>
+          <t>CAND_0046064</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -2475,19 +2475,19 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>0.8019</t>
+          <t>0.7457</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Lower-tier shortlist entry — Data Scientist at Vedantu (5.6 YOE); JD-aligned skills: Sentence Transformers, FAISS, Weaviate. Key gaps: 90-day notice period.</t>
+          <t>Lower-tier shortlist entry — Senior NLP Engineer at Salesforce (8.9 YOE); JD-aligned skills: Python, Pinecone, OpenSearch. Key gaps: weak secondary signals vs higher ranks.</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>CAND_0005477</t>
+          <t>CAND_0028793</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2497,19 +2497,19 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>0.8012</t>
+          <t>0.7455</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Lower-tier shortlist entry — ML Engineer at Zomato (6.2 YOE); JD-aligned skills: OpenSearch. Key gaps: only 1 core JD skill matched.</t>
+          <t>Lower-tier shortlist entry — Search Engineer at Google (7.2 YOE); JD-aligned skills: Embeddings, NLP. Key gaps: 120-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>CAND_0013536</t>
+          <t>CAND_0071939</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -2519,19 +2519,19 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>0.8009</t>
+          <t>0.7439</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Lower-tier shortlist entry — Applied ML Engineer at Haptik (14.1 YOE); JD-aligned skills: LLMs, NLP, Embeddings. Key gaps: 90-day notice period; experience above target band for this role.</t>
+          <t>Lower-tier shortlist entry — Data Scientist at Krutrim (6.4 YOE); JD-aligned skills: Elasticsearch, OpenSearch, Embeddings. Key gaps: weak secondary signals vs higher ranks.</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>CAND_0015057</t>
+          <t>CAND_0005260</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -2541,19 +2541,19 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>0.7999</t>
+          <t>0.7437</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Lower-tier shortlist entry — ML Engineer at Meesho (4.6 YOE); JD-aligned skills: Sentence Transformers, Vector Search, Embeddings. Key gaps: 90-day notice period.</t>
+          <t>Lower-tier shortlist entry — Senior NLP Engineer at Netflix (5.2 YOE); JD-aligned skills: Python, NLP, Embeddings. Key gaps: not flagged open to work.</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>CAND_0030348</t>
+          <t>CAND_0006418</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -2563,19 +2563,19 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>0.7992</t>
+          <t>0.7435</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Lower-tier shortlist entry — Machine Learning Engineer at BYJU'S (4.5 YOE); JD-aligned skills: Embeddings, Vector Search, Elasticsearch. Key gaps: weak secondary signals vs higher ranks.</t>
+          <t>Lower-tier shortlist entry — Machine Learning Engineer at Verloop.io (5.7 YOE); JD-aligned skills: Embeddings, Weaviate, Elasticsearch. Key gaps: weak secondary signals vs higher ranks.</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>CAND_0060538</t>
+          <t>CAND_0039754</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -2585,19 +2585,19 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>0.7983</t>
+          <t>0.7432</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Lower-tier shortlist entry — ML Engineer at Verloop.io (5.2 YOE); JD-aligned skills: OpenSearch, Embeddings, Milvus. Key gaps: 90-day notice period.</t>
+          <t>Lower-tier shortlist entry — Senior Applied Scientist at Meta (16.2 YOE); JD-aligned skills: Fine-tuning LLMs, Qdrant, NLP. Key gaps: experience above target band for this role.</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>CAND_0049615</t>
+          <t>CAND_0073982</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -2607,19 +2607,19 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>0.7961</t>
+          <t>0.7428</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Lower-tier shortlist entry — ML Engineer at Krutrim (5.1 YOE); JD-aligned skills: NLP, Pinecone. Key gaps: weak secondary signals vs higher ranks.</t>
+          <t>Lower-tier shortlist entry — Data Scientist at Dream11 (7.0 YOE); JD-aligned skills: Sentence Transformers, Qdrant, FAISS. Key gaps: weak secondary signals vs higher ranks.</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>CAND_0019159</t>
+          <t>CAND_0091899</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -2629,12 +2629,12 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>0.7956</t>
+          <t>0.7424</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Lower-tier shortlist entry — ML Engineer at Genpact AI (6.1 YOE); JD-aligned skills: Vector Search, Qdrant, Sentence Transformers. Key gaps: not flagged open to work.</t>
+          <t>Lower-tier shortlist entry — Senior Software Engineer (ML) at PhonePe (5.8 YOE); JD-aligned skills: Sentence Transformers, FAISS, NLP. Key gaps: not flagged open to work.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: regenerate submission after post-review upgrade
</commit_message>
<xml_diff>
--- a/submission.xlsx
+++ b/submission.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D101"/>
+  <dimension ref="A1:E101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -434,6 +434,11 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
+          <t>join_probability</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
           <t>reasoning</t>
         </is>
       </c>
@@ -441,7 +446,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>CAND_0080766</t>
+          <t>CAND_0018499</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -451,19 +456,24 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>0.9107</t>
+          <t>1.2336</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Rank 1: Staff Machine Learning Engineer at Salesforce (8.8 YOE); JD-aligned skills: Elasticsearch, OpenSearch, Python. Top-tier composite score across career, skills, and availability. Counterfactual: ranks on career trajectory and assessed depth over keyword coverage (4/20 listed must-haves), aligning with the JD anti-keyword-stuffing guidance.</t>
+          <t>0.6132</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Rank 1: Senior Machine Learning Engineer at Zomato (7.2 YOE); JD-aligned skills: Weaviate, Pinecone, Information Retrieval. Top-tier composite score across career, skills, and availability. Counterfactual: ranks on career trajectory and assessed depth over keyword coverage (5/20 listed must-haves), aligning with the JD anti-keyword-stuffing guidance. Join probability: 61%.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>CAND_0006567</t>
+          <t>CAND_0088025</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -473,19 +483,24 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>0.9058</t>
+          <t>1.2187</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Rank 2: Senior AI Engineer at Meta (7.9 YOE); JD-aligned skills: NLP, Python. Top-tier composite score across career, skills, and availability. Counterfactual: ranks on career trajectory and assessed depth over keyword coverage (2/20 listed must-haves), aligning with the JD anti-keyword-stuffing guidance.</t>
+          <t>0.5411</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Rank 2: Staff Machine Learning Engineer at Yellow.ai (8.6 YOE); JD-aligned skills: Pinecone, LLMs, Elasticsearch. Top-tier composite score across career, skills, and availability. Minor note: 90-day notice period. Join probability: 54%.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>CAND_0068351</t>
+          <t>CAND_0071974</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -495,19 +510,24 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>0.8977</t>
+          <t>1.2065</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Rank 3: Lead AI Engineer at Sarvam AI (6.4 YOE); JD-aligned skills: Qdrant, Elasticsearch, Python. Top-tier composite score across career, skills, and availability. Counterfactual: ranks on career trajectory and assessed depth over keyword coverage (4/20 listed must-haves), aligning with the JD anti-keyword-stuffing guidance.</t>
+          <t>0.3414</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Rank 3: Senior AI Engineer at Netflix (7.8 YOE); JD-aligned skills: Weaviate, Pinecone, Information Retrieval. Top-tier composite score across career, skills, and availability. Counterfactual: ranks on career trajectory and assessed depth over keyword coverage (7/20 listed must-haves), aligning with the JD anti-keyword-stuffing guidance. Join probability: 34%; low engagement signals.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>CAND_0077337</t>
+          <t>CAND_0068351</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -517,19 +537,24 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>0.8977</t>
+          <t>1.1986</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Rank 4: Staff Machine Learning Engineer at Paytm (7.0 YOE); JD-aligned skills: Pinecone, LLMs, Qdrant. Top-tier composite score across career, skills, and availability. Counterfactual: ranks on career trajectory and assessed depth over keyword coverage (6/20 listed must-haves), aligning with the JD anti-keyword-stuffing guidance.</t>
+          <t>0.4040</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Rank 4: Lead AI Engineer at Sarvam AI (6.4 YOE); JD-aligned skills: pgvector, Qdrant, Elasticsearch. Top-tier composite score across career, skills, and availability. Counterfactual: ranks on career trajectory and assessed depth over keyword coverage (7/20 listed must-haves), aligning with the JD anti-keyword-stuffing guidance. Join probability: 40%.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CAND_0096142</t>
+          <t>CAND_0081846</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -539,19 +564,24 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>0.8938</t>
+          <t>1.1861</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Rank 5: Applied ML Engineer at upGrad (5.0 YOE); JD-aligned skills: Weaviate, Pinecone, Python. Top-tier composite score across career, skills, and availability. Minor note: 120-day notice period.</t>
+          <t>0.4803</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Rank 5: Lead AI Engineer at Razorpay (6.7 YOE); JD-aligned skills: Information Retrieval, pgvector, Elasticsearch. Top-tier composite score across career, skills, and availability. Counterfactual: ranks on career trajectory and assessed depth over keyword coverage (7/20 listed must-haves), aligning with the JD anti-keyword-stuffing guidance. Join probability: 48%.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>CAND_0018499</t>
+          <t>CAND_0002025</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -561,19 +591,24 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>0.8901</t>
+          <t>1.1708</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Strong match — Senior Machine Learning Engineer at Zomato (7.2 YOE); JD-aligned skills: Weaviate, Pinecone, Milvus.</t>
+          <t>0.3912</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Strong match — Senior AI Engineer at Apple (5.9 YOE); JD-aligned skills: FAISS, OpenSearch, Weaviate. Join probability: 39%.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>CAND_0071974</t>
+          <t>CAND_0046525</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -583,19 +618,24 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>0.8893</t>
+          <t>1.1683</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Strong match — Senior AI Engineer at Netflix (7.8 YOE); JD-aligned skills: Weaviate, Pinecone, Qdrant.</t>
+          <t>0.3574</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Strong match — Senior Machine Learning Engineer at Genpact AI (6.1 YOE); JD-aligned skills: Elasticsearch, Information Retrieval, LLMs. Join probability: 36%.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>CAND_0002025</t>
+          <t>CAND_0077337</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -605,19 +645,24 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>0.8831</t>
+          <t>1.1645</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Strong match — Senior AI Engineer at Apple (5.9 YOE); JD-aligned skills: FAISS, OpenSearch, Weaviate.</t>
+          <t>0.4883</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Strong match — Staff Machine Learning Engineer at Paytm (7.0 YOE); JD-aligned skills: pgvector, Pinecone, Information Retrieval. Join probability: 49%.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>CAND_0081846</t>
+          <t>CAND_0055905</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -627,19 +672,24 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>0.8778</t>
+          <t>1.1445</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Strong match — Lead AI Engineer at Razorpay (6.7 YOE); JD-aligned skills: Elasticsearch, Vector Search, Python.</t>
+          <t>0.6870</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Strong match — Senior Machine Learning Engineer at Flipkart (8.1 YOE); JD-aligned skills: Elasticsearch, Python, LLMs. Join probability: 69%.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>CAND_0088025</t>
+          <t>CAND_0080766</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -649,19 +699,24 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>0.8769</t>
+          <t>1.1382</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Strong match — Staff Machine Learning Engineer at Yellow.ai (8.6 YOE); JD-aligned skills: Pinecone, LLMs, Elasticsearch. Watch: 90-day notice period.</t>
+          <t>0.4625</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Strong match — Staff Machine Learning Engineer at Salesforce (8.8 YOE); JD-aligned skills: Information Retrieval Systems, Elasticsearch, Natural Language Processing. Join probability: 46%.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>CAND_0038368</t>
+          <t>CAND_0006567</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -671,19 +726,24 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>0.8690</t>
+          <t>1.1293</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Strong match — ML Engineer at PhonePe (5.4 YOE); JD-aligned skills: Embeddings, FAISS, NLP.</t>
+          <t>0.6079</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Strong match — Senior AI Engineer at Meta (7.9 YOE); JD-aligned skills: Vector Representations, NLP, Python. Join probability: 61%.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>CAND_0046525</t>
+          <t>CAND_0050454</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -693,19 +753,24 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>0.8658</t>
+          <t>1.1031</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Strong match — Senior Machine Learning Engineer at Genpact AI (6.1 YOE); JD-aligned skills: Elasticsearch, LLMs, NLP.</t>
+          <t>0.3504</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Strong match — AI Engineer at Rephrase.ai (6.8 YOE); JD-aligned skills: Fine-tuning LLMs, FAISS, Qdrant. Join probability: 35%.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>CAND_0039383</t>
+          <t>CAND_0083879</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -715,19 +780,24 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>0.8585</t>
+          <t>1.1019</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Strong match — Applied ML Engineer at Meesho (7.1 YOE); JD-aligned skills: FAISS, NLP, Vector Search. Watch: 90-day notice period.</t>
+          <t>0.5950</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Strong match — Machine Learning Engineer at Ola (7.1 YOE); JD-aligned skills: Fine-tuning LLMs, Milvus, Sentence Transformers. Join probability: 60%.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>CAND_0087630</t>
+          <t>CAND_0018094</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -737,12 +807,17 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>0.8576</t>
+          <t>1.1014</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Strong match — AI Engineer at Vedantu (7.2 YOE); JD-aligned skills: Elasticsearch, NLP, Embeddings.</t>
+          <t>0.4428</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Strong match — ML Engineer at Mad Street Den (5.2 YOE); JD-aligned skills: Pinecone, Information Retrieval, Fine-tuning LLMs. Join probability: 44%.</t>
         </is>
       </c>
     </row>
@@ -759,19 +834,24 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>0.8566</t>
+          <t>1.0990</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Strong match — AI Engineer at PolicyBazaar (7.7 YOE); JD-aligned skills: Vector Search, OpenSearch, Qdrant.</t>
+          <t>0.2252</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Strong match — AI Engineer at PolicyBazaar (7.7 YOE); JD-aligned skills: Vector Search, OpenSearch, Qdrant. Join probability: 23%; low engagement signals.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>CAND_0044855</t>
+          <t>CAND_0049538</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -781,19 +861,24 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>0.8553</t>
+          <t>1.0933</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Strong match — Senior Data Scientist at Flipkart (6.6 YOE); JD-aligned skills: OpenSearch, Pinecone, Vector Search.</t>
+          <t>0.3362</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Strong match — Applied ML Engineer at Saarthi.ai (5.8 YOE); JD-aligned skills: OpenSearch, Vector Search, Milvus. Join probability: 34%; low engagement signals.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>CAND_0061257</t>
+          <t>CAND_0087630</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -803,19 +888,24 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>0.8551</t>
+          <t>1.0927</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Strong match — Staff Machine Learning Engineer at LinkedIn (8.0 YOE); JD-aligned skills: Python. Watch: only 1 core JD skill matched.</t>
+          <t>0.3940</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Strong match — AI Engineer at Vedantu (7.2 YOE); JD-aligned skills: Elasticsearch, pgvector, NLP. Join probability: 39%.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>CAND_0045250</t>
+          <t>CAND_0086022</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -825,19 +915,24 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>0.8527</t>
+          <t>1.0912</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Strong match — Applied ML Engineer at Rephrase.ai (6.6 YOE); JD-aligned skills: Sentence Transformers, Milvus, Embeddings.</t>
+          <t>0.3683</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Strong match — Senior Applied Scientist at Sarvam AI (5.3 YOE); JD-aligned skills: Vector Search, pgvector, Fine-tuning LLMs. Join probability: 37%.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>CAND_0050454</t>
+          <t>CAND_0016163</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -847,19 +942,24 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>0.8443</t>
+          <t>1.0899</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Strong match — AI Engineer at Rephrase.ai (6.8 YOE); JD-aligned skills: Fine-tuning LLMs, FAISS, Qdrant.</t>
+          <t>0.2905</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Strong match — Applied ML Engineer at Dream11 (6.7 YOE); JD-aligned skills: Weaviate, Embeddings, pgvector. Watch: 120-day notice period. Join probability: 29%; long notice.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>CAND_0020350</t>
+          <t>CAND_0005649</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -869,19 +969,24 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>0.8423</t>
+          <t>1.0870</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Strong match — AI Engineer at Zoho (5.8 YOE); JD-aligned skills: NLP, LLMs, FAISS.</t>
+          <t>0.5162</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Strong match — Senior Data Scientist at Sarvam AI (7.4 YOE); JD-aligned skills: Fine-tuning LLMs, Weaviate, Information Retrieval. Watch: 90-day notice period. Join probability: 52%.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>CAND_0042029</t>
+          <t>CAND_0030031</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -891,19 +996,24 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>0.8406</t>
+          <t>1.0786</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Solid profile: Senior Data Scientist at Flipkart (6.5 YOE); JD-aligned skills: NLP, Elasticsearch, Embeddings.</t>
+          <t>0.3445</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Solid profile: AI Engineer at Microsoft (5.7 YOE); JD-aligned skills: Information Retrieval, Python, NLP.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>CAND_0068811</t>
+          <t>CAND_0096142</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -913,19 +1023,24 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>0.8385</t>
+          <t>1.0786</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Good fit with caveats: Applied ML Engineer at Freshworks (8.0 YOE); JD-aligned skills: Vector Search, Qdrant, Embeddings.</t>
+          <t>0.2486</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Good fit with caveats: Applied ML Engineer at upGrad (5.0 YOE); JD-aligned skills: Weaviate, Pinecone, Python. Concerns: 120-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>CAND_0086022</t>
+          <t>CAND_0081852</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -935,19 +1050,24 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>0.8342</t>
+          <t>1.0778</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Competitive candidate: Senior Applied Scientist at Sarvam AI (5.3 YOE); JD-aligned skills: Vector Search, Fine-tuning LLMs, Elasticsearch.</t>
+          <t>0.2331</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Competitive candidate: Senior Data Scientist at Mad Street Den (5.9 YOE); JD-aligned skills: Milvus, pgvector, Weaviate.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>CAND_0047721</t>
+          <t>CAND_0039383</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -957,19 +1077,24 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>0.8322</t>
+          <t>1.0766</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Meets several JD signals: Senior Data Scientist at Microsoft (7.0 YOE); JD-aligned skills: Milvus, FAISS, Qdrant. Concerns: 90-day notice period.</t>
+          <t>0.5155</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Meets several JD signals: Applied ML Engineer at Meesho (7.1 YOE); JD-aligned skills: FAISS, NLP, Vector Search. Concerns: 90-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>CAND_0030031</t>
+          <t>CAND_0058688</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -979,19 +1104,24 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>0.8310</t>
+          <t>1.0750</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Solid profile: AI Engineer at Microsoft (5.7 YOE); JD-aligned skills: Python, NLP, Sentence Transformers.</t>
+          <t>0.7268</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Solid profile: AI Engineer at Vedantu (6.7 YOE); JD-aligned skills: Embeddings, Information Retrieval, Milvus.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>CAND_0090584</t>
+          <t>CAND_0020877</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1001,19 +1131,24 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>0.8287</t>
+          <t>1.0749</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Good fit with caveats: ML Engineer at Flipkart (5.1 YOE); JD-aligned skills: Fine-tuning LLMs, OpenSearch, FAISS. Concerns: 120-day notice period.</t>
+          <t>0.3909</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Good fit with caveats: Applied ML Engineer at CRED (5.1 YOE); JD-aligned skills: Elasticsearch, OpenSearch, Information Retrieval.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>CAND_0032216</t>
+          <t>CAND_0020350</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1023,19 +1158,24 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>0.8275</t>
+          <t>1.0743</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Competitive candidate: ML Engineer at upGrad (6.1 YOE); JD-aligned skills: Qdrant, Sentence Transformers, Vector Search.</t>
+          <t>0.3210</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Competitive candidate: AI Engineer at Zoho (5.8 YOE); JD-aligned skills: NLP, LLMs, FAISS.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>CAND_0037944</t>
+          <t>CAND_0042029</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1045,19 +1185,24 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>0.8271</t>
+          <t>1.0721</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Meets several JD signals: Senior Data Scientist at Vedantu (4.9 YOE); JD-aligned skills: Vector Search, OpenSearch, Embeddings.</t>
+          <t>0.4840</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Meets several JD signals: Senior Data Scientist at Flipkart (6.5 YOE); JD-aligned skills: NLP, Elasticsearch, Embeddings.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>CAND_0075574</t>
+          <t>CAND_0044855</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1067,19 +1212,24 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>0.8261</t>
+          <t>1.0706</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Solid profile: Machine Learning Engineer at Haptik (5.7 YOE); JD-aligned skills: Weaviate, OpenSearch, Qdrant.</t>
+          <t>0.3723</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Solid profile: Senior Data Scientist at Flipkart (6.6 YOE); JD-aligned skills: OpenSearch, Information Retrieval, Pinecone.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>CAND_0049538</t>
+          <t>CAND_0046064</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1089,19 +1239,24 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>0.8252</t>
+          <t>1.0691</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Good fit with caveats: Applied ML Engineer at Saarthi.ai (5.8 YOE); JD-aligned skills: OpenSearch, Vector Search, Milvus.</t>
+          <t>0.3780</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Good fit with caveats: Senior NLP Engineer at Salesforce (8.9 YOE); JD-aligned skills: Python, Pinecone, OpenSearch.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>CAND_0003841</t>
+          <t>CAND_0061257</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1111,19 +1266,24 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>0.8204</t>
+          <t>1.0681</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Competitive candidate: ML Engineer at Tech Mahindra (5.0 YOE); JD-aligned skills: Pinecone, Fine-tuning LLMs, Sentence Transformers.</t>
+          <t>0.3969</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Competitive candidate: Staff Machine Learning Engineer at LinkedIn (8.0 YOE); JD-aligned skills: Information Retrieval Systems, Python, Vector Representations.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>CAND_0020877</t>
+          <t>CAND_0079387</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1133,12 +1293,17 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>0.8197</t>
+          <t>1.0675</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Meets several JD signals: Applied ML Engineer at CRED (5.1 YOE); JD-aligned skills: Elasticsearch, OpenSearch, Weaviate.</t>
+          <t>0.4465</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Meets several JD signals: AI Engineer at Microsoft (6.9 YOE); JD-aligned skills: Python, Sentence Transformers, Vector Search.</t>
         </is>
       </c>
     </row>
@@ -1155,10 +1320,15 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>0.8196</t>
+          <t>1.0657</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
+        <is>
+          <t>0.3534</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
         <is>
           <t>Solid profile: Applied ML Engineer at Zoho (6.8 YOE); JD-aligned skills: NLP, Vector Search, Sentence Transformers.</t>
         </is>
@@ -1167,7 +1337,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>CAND_0037566</t>
+          <t>CAND_0093193</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1177,19 +1347,24 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>0.8188</t>
+          <t>1.0652</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Good fit with caveats: Machine Learning Engineer at LinkedIn (6.9 YOE); JD-aligned skills: Pinecone, NLP, LLMs.</t>
+          <t>0.4352</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Good fit with caveats: Senior Machine Learning Engineer at Niramai (7.9 YOE); JD-aligned skills: Text Encoders, Vector Representations, Qdrant.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>CAND_0079387</t>
+          <t>CAND_0045250</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1199,19 +1374,24 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>0.8185</t>
+          <t>1.0643</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Competitive candidate: AI Engineer at Microsoft (6.9 YOE); JD-aligned skills: Python, Sentence Transformers, Vector Search.</t>
+          <t>0.3580</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Competitive candidate: Applied ML Engineer at Rephrase.ai (6.6 YOE); JD-aligned skills: Sentence Transformers, Milvus, Embeddings.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>CAND_0098217</t>
+          <t>CAND_0003841</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1221,19 +1401,24 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>0.8171</t>
+          <t>1.0641</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Meets several JD signals: ML Engineer at Glance (6.4 YOE); JD-aligned skills: FAISS, Pinecone.</t>
+          <t>0.3402</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Meets several JD signals: ML Engineer at Tech Mahindra (5.0 YOE); JD-aligned skills: Pinecone, Fine-tuning LLMs, Sentence Transformers.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>CAND_0099806</t>
+          <t>CAND_0047721</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1243,19 +1428,24 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>0.8155</t>
+          <t>1.0600</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Solid profile: AI Engineer at Mad Street Den (4.6 YOE); JD-aligned skills: FAISS, Embeddings, Sentence Transformers.</t>
+          <t>0.1736</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Solid profile: Senior Data Scientist at Microsoft (7.0 YOE); JD-aligned skills: Milvus, Information Retrieval, FAISS. Concerns: 90-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>CAND_0055905</t>
+          <t>CAND_0042100</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1265,19 +1455,24 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>0.8149</t>
+          <t>1.0570</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Good fit with caveats: Senior Machine Learning Engineer at Flipkart (8.1 YOE); JD-aligned skills: Elasticsearch, Python, LLMs.</t>
+          <t>0.2536</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Good fit with caveats: Machine Learning Engineer at Freshworks (7.3 YOE); JD-aligned skills: Elasticsearch, Fine-tuning LLMs, Pinecone. Concerns: 90-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>CAND_0051004</t>
+          <t>CAND_0051292</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1287,19 +1482,24 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>0.8145</t>
+          <t>1.0558</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Competitive candidate: Senior Data Scientist at CRED (4.7 YOE); JD-aligned skills: Embeddings, Qdrant, Fine-tuning LLMs.</t>
+          <t>0.4013</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Competitive candidate: Applied ML Engineer at Freshworks (5.2 YOE); JD-aligned skills: pgvector, FAISS, LLMs.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>CAND_0018094</t>
+          <t>CAND_0038368</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1309,19 +1509,24 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>0.8120</t>
+          <t>1.0531</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Meets several JD signals: ML Engineer at Mad Street Den (5.2 YOE); JD-aligned skills: Pinecone, Fine-tuning LLMs.</t>
+          <t>0.4347</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Meets several JD signals: ML Engineer at PhonePe (5.4 YOE); JD-aligned skills: Embeddings, FAISS, NLP.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>CAND_0081852</t>
+          <t>CAND_0037566</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1331,19 +1536,24 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>0.8110</t>
+          <t>1.0519</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Solid profile: Senior Data Scientist at Mad Street Den (5.9 YOE); JD-aligned skills: Milvus, Weaviate, Vector Search.</t>
+          <t>0.5752</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Solid profile: Machine Learning Engineer at LinkedIn (6.9 YOE); JD-aligned skills: Pinecone, NLP, LLMs.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>CAND_0083879</t>
+          <t>CAND_0051004</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1353,19 +1563,24 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>0.8058</t>
+          <t>1.0514</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Good fit with caveats: Machine Learning Engineer at Ola (7.1 YOE); JD-aligned skills: Fine-tuning LLMs, Milvus, Sentence Transformers.</t>
+          <t>0.5405</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Good fit with caveats: Senior Data Scientist at CRED (4.7 YOE); JD-aligned skills: Embeddings, Qdrant, Fine-tuning LLMs.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>CAND_0058688</t>
+          <t>CAND_0069905</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1375,19 +1590,24 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>0.7999</t>
+          <t>1.0513</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Competitive candidate: AI Engineer at Vedantu (6.7 YOE); JD-aligned skills: Embeddings, Milvus.</t>
+          <t>0.3358</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Competitive candidate: Applied ML Engineer at Sarvam AI (6.6 YOE); JD-aligned skills: Sentence Transformers, Python, Weaviate. Concerns: 90-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>CAND_0079284</t>
+          <t>CAND_0055992</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1397,19 +1617,24 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>0.7976</t>
+          <t>1.0510</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Meets several JD signals: Machine Learning Engineer at Google (4.9 YOE); JD-aligned skills: Qdrant, Fine-tuning LLMs, Elasticsearch.</t>
+          <t>0.5850</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Meets several JD signals: AI Engineer at CRED (16.9 YOE); JD-aligned skills: Information Retrieval, FAISS, OpenSearch.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>CAND_0041669</t>
+          <t>CAND_0068811</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -1419,19 +1644,24 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>0.7936</t>
+          <t>1.0494</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Solid profile: Recommendation Systems Engineer at CRED (8.0 YOE); JD-aligned skills: FAISS, Milvus, Weaviate.</t>
+          <t>0.4651</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Solid profile: Applied ML Engineer at Freshworks (8.0 YOE); JD-aligned skills: Vector Search, Qdrant, Embeddings.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>CAND_0076482</t>
+          <t>CAND_0093912</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -1441,19 +1671,24 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>0.7909</t>
+          <t>1.0480</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Good fit with caveats: ML Engineer at Flipkart (6.6 YOE); JD-aligned skills: OpenSearch, Pinecone, Embeddings.</t>
+          <t>0.4763</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Good fit with caveats: Senior Data Scientist at Razorpay (5.3 YOE); JD-aligned skills: Milvus, Embeddings, Vector Search.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>CAND_0009691</t>
+          <t>CAND_0099806</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -1463,19 +1698,24 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>0.7893</t>
+          <t>1.0479</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Competitive candidate: Applied ML Engineer at LinkedIn (6.2 YOE); JD-aligned skills: Fine-tuning LLMs, Pinecone, Sentence Transformers. Concerns: 120-day notice period.</t>
+          <t>0.3301</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Competitive candidate: AI Engineer at Mad Street Den (4.6 YOE); JD-aligned skills: pgvector, FAISS, Embeddings.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>CAND_0095528</t>
+          <t>CAND_0078002</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1485,19 +1725,24 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>0.7892</t>
+          <t>1.0469</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Meets several JD signals: Senior Data Scientist at Netflix (5.3 YOE); JD-aligned skills: OpenSearch, Vector Search, Qdrant.</t>
+          <t>0.2974</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Meets several JD signals: Machine Learning Engineer at Meta (6.3 YOE); JD-aligned skills: pgvector, NLP, Weaviate.</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>CAND_0052328</t>
+          <t>CAND_0010257</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -1507,19 +1752,24 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>0.7883</t>
+          <t>1.0458</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Solid profile: Recommendation Systems Engineer at Amazon (6.5 YOE); JD-aligned skills: OpenSearch, Fine-tuning LLMs, Vector Search.</t>
+          <t>0.3313</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Solid profile: Senior Data Scientist at Google (6.5 YOE); JD-aligned skills: Milvus, Python, OpenSearch. Concerns: 120-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>CAND_0079064</t>
+          <t>CAND_0065878</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -1529,19 +1779,24 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>0.7866</t>
+          <t>1.0430</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Good fit with caveats: Senior Data Scientist at Niramai (5.2 YOE); JD-aligned skills: OpenSearch, NLP, Fine-tuning LLMs. Concerns: 120-day notice period.</t>
+          <t>0.2450</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Good fit with caveats: Senior Data Scientist at Niramai (7.8 YOE); JD-aligned skills: pgvector, Vector Search, Fine-tuning LLMs.</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>CAND_0040178</t>
+          <t>CAND_0032216</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -1551,19 +1806,24 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>0.7854</t>
+          <t>1.0428</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Moderate fit: ML Engineer at Meesho (5.0 YOE); JD-aligned skills: Weaviate, Fine-tuning LLMs, Vector Search. Gaps: under half of JD must-have skills covered.</t>
+          <t>0.2743</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Moderate fit: ML Engineer at upGrad (6.1 YOE); JD-aligned skills: Information Retrieval, Qdrant, Sentence Transformers. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>CAND_0010149</t>
+          <t>CAND_0005260</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -1573,19 +1833,24 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>0.7850</t>
+          <t>1.0401</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Partial alignment: ML Engineer at Glance (6.9 YOE); JD-aligned skills: Milvus, Vector Search, Elasticsearch. Gaps: 90-day notice period.</t>
+          <t>0.4814</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Partial alignment: Senior NLP Engineer at Netflix (5.2 YOE); JD-aligned skills: Information Retrieval, Python, NLP. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>CAND_0005649</t>
+          <t>CAND_0025923</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -1595,19 +1860,24 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>0.7836</t>
+          <t>1.0385</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Acceptable but not standout: Senior Data Scientist at Sarvam AI (7.4 YOE); JD-aligned skills: Fine-tuning LLMs, Weaviate. Gaps: 90-day notice period.</t>
+          <t>0.2891</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Acceptable but not standout: Senior Software Engineer (ML) at HCL (5.0 YOE); JD-aligned skills: pgvector, Qdrant, Pinecone. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>CAND_0055992</t>
+          <t>CAND_0075574</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -1617,19 +1887,24 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>0.7833</t>
+          <t>1.0377</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Mixed signals: AI Engineer at CRED (16.9 YOE); JD-aligned skills: FAISS, OpenSearch, Embeddings. Gaps: experience above target band for this role.</t>
+          <t>0.4170</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Mixed signals: Machine Learning Engineer at Haptik (5.7 YOE); JD-aligned skills: pgvector, Weaviate, OpenSearch. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>CAND_0015582</t>
+          <t>CAND_0005538</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -1639,19 +1914,24 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>0.7831</t>
+          <t>1.0374</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>JD overlap is thin: ML Engineer at Genpact AI (4.4 YOE); JD-aligned skills: Qdrant, Sentence Transformers, Embeddings. Gaps: 120-day notice period.</t>
+          <t>0.4072</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>JD overlap is thin: Senior AI Engineer at Adobe (5.9 YOE); JD-aligned skills: Vector Representations, Python, Information Retrieval Systems. Gaps: 90-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>CAND_0061550</t>
+          <t>CAND_0079064</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -1661,19 +1941,24 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>0.7799</t>
+          <t>1.0358</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Moderate fit: ML Engineer at Infosys (5.3 YOE); JD-aligned skills: Sentence Transformers. Gaps: only 1 core JD skill matched.</t>
+          <t>0.2563</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Moderate fit: Senior Data Scientist at Niramai (5.2 YOE); JD-aligned skills: OpenSearch, NLP, Fine-tuning LLMs. Gaps: 120-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>CAND_0051292</t>
+          <t>CAND_0015528</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -1683,19 +1968,24 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>0.7768</t>
+          <t>1.0352</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Partial alignment: Applied ML Engineer at Freshworks (5.2 YOE); JD-aligned skills: FAISS, LLMs, Vector Search. Gaps: under half of JD must-have skills covered.</t>
+          <t>0.3246</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Partial alignment: Applied ML Engineer at Krutrim (7.4 YOE); JD-aligned skills: Weaviate, pgvector, Information Retrieval. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>CAND_0074735</t>
+          <t>CAND_0067866</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -1705,19 +1995,24 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>0.7764</t>
+          <t>1.0323</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Acceptable but not standout: Applied ML Engineer at Rephrase.ai (5.5 YOE); JD-aligned skills: Weaviate, Vector Search, Elasticsearch. Gaps: 90-day notice period.</t>
+          <t>0.3513</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Acceptable but not standout: Senior Software Engineer (ML) at Tech Mahindra (6.4 YOE); JD-aligned skills: Embeddings, pgvector, Elasticsearch. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>CAND_0015578</t>
+          <t>CAND_0074735</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -1727,19 +2022,24 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>0.7761</t>
+          <t>1.0312</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Mixed signals: AI Engineer at Zoho (5.4 YOE); JD-aligned skills: Embeddings, NLP, Sentence Transformers. Gaps: 90-day notice period.</t>
+          <t>0.4586</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Mixed signals: Applied ML Engineer at Rephrase.ai (5.5 YOE); JD-aligned skills: Weaviate, Information Retrieval, Vector Search. Gaps: 90-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>CAND_0016163</t>
+          <t>CAND_0079284</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -1749,19 +2049,24 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>0.7759</t>
+          <t>1.0303</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>JD overlap is thin: Applied ML Engineer at Dream11 (6.7 YOE); JD-aligned skills: Weaviate, Embeddings, Pinecone. Gaps: 120-day notice period.</t>
+          <t>0.2718</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>JD overlap is thin: Machine Learning Engineer at Google (4.9 YOE); JD-aligned skills: Qdrant, Fine-tuning LLMs, Elasticsearch. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>CAND_0018293</t>
+          <t>CAND_0090584</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -1771,19 +2076,24 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>0.7736</t>
+          <t>1.0302</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Moderate fit: Data Scientist at PharmEasy (5.6 YOE); JD-aligned skills: Weaviate. Gaps: only 1 core JD skill matched.</t>
+          <t>0.1637</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>Moderate fit: ML Engineer at Flipkart (5.1 YOE); JD-aligned skills: Fine-tuning LLMs, OpenSearch, FAISS. Gaps: 120-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>CAND_0069905</t>
+          <t>CAND_0011432</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -1793,19 +2103,24 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>0.7719</t>
+          <t>1.0296</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Partial alignment: Applied ML Engineer at Sarvam AI (6.6 YOE); JD-aligned skills: Sentence Transformers, Python, Weaviate. Gaps: 90-day notice period.</t>
+          <t>0.5534</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>Partial alignment: Senior Data Scientist at Amazon (7.6 YOE); JD-aligned skills: OpenSearch, pgvector, Elasticsearch. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>CAND_0089552</t>
+          <t>CAND_0061550</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -1815,19 +2130,24 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>0.7705</t>
+          <t>1.0285</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Acceptable but not standout: Machine Learning Engineer at Netflix (6.0 YOE); JD-aligned skills: Weaviate, Qdrant, Vector Search. Gaps: 120-day notice period.</t>
+          <t>0.3313</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>Acceptable but not standout: ML Engineer at Infosys (5.3 YOE); JD-aligned skills: pgvector, Sentence Transformers. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>CAND_0067866</t>
+          <t>CAND_0011687</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -1837,19 +2157,24 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>0.7699</t>
+          <t>1.0254</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Mixed signals: Senior Software Engineer (ML) at Tech Mahindra (6.4 YOE); JD-aligned skills: Embeddings, Elasticsearch, Qdrant. Gaps: under half of JD must-have skills covered.</t>
+          <t>0.5094</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>Mixed signals: Senior NLP Engineer at Niramai (7.8 YOE); JD-aligned skills: OpenSearch, FAISS, Embeddings. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>CAND_0048166</t>
+          <t>CAND_0028793</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -1859,19 +2184,24 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>0.7697</t>
+          <t>1.0230</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>JD overlap is thin: ML Engineer at Aganitha (5.2 YOE); JD-aligned skills: Pinecone, Milvus, Qdrant. Gaps: under half of JD must-have skills covered.</t>
+          <t>0.2941</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>JD overlap is thin: Search Engineer at Google (7.2 YOE); JD-aligned skills: Embeddings, Information Retrieval, pgvector. Gaps: 120-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>CAND_0042100</t>
+          <t>CAND_0048166</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -1881,19 +2211,24 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>0.7689</t>
+          <t>1.0214</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Moderate fit: Machine Learning Engineer at Freshworks (7.3 YOE); JD-aligned skills: Elasticsearch, Fine-tuning LLMs, Pinecone. Gaps: 90-day notice period.</t>
+          <t>0.4054</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>Moderate fit: ML Engineer at Aganitha (5.2 YOE); JD-aligned skills: Pinecone, Milvus, Qdrant. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>CAND_0050876</t>
+          <t>CAND_0093547</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -1903,19 +2238,24 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>0.7682</t>
+          <t>1.0188</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Partial alignment: Applied ML Engineer at Freshworks (6.0 YOE); JD-aligned skills: Qdrant, FAISS, OpenSearch. Gaps: 90-day notice period.</t>
+          <t>0.3710</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>Partial alignment: Senior Machine Learning Engineer at PhonePe (2.9 YOE); JD-aligned skills: LLMs, Python, Milvus. Gaps: below typical senior YOE band for this JD.</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>CAND_0091909</t>
+          <t>CAND_0076482</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -1925,19 +2265,24 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>0.7668</t>
+          <t>1.0173</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Acceptable but not standout: Machine Learning Engineer at Rephrase.ai (6.9 YOE); JD-aligned skills: LLMs, Pinecone, Qdrant. Gaps: under half of JD must-have skills covered.</t>
+          <t>0.5553</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>Acceptable but not standout: ML Engineer at Flipkart (6.6 YOE); JD-aligned skills: OpenSearch, Pinecone, pgvector. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>CAND_0065514</t>
+          <t>CAND_0040178</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -1947,19 +2292,24 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>0.7666</t>
+          <t>1.0161</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Mixed signals: ML Engineer at Genpact AI (6.6 YOE); JD-aligned skills: Vector Search, Pinecone, Elasticsearch. Gaps: 90-day notice period.</t>
+          <t>0.3303</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>Mixed signals: ML Engineer at Meesho (5.0 YOE); JD-aligned skills: Weaviate, Fine-tuning LLMs, Vector Search. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>CAND_0010541</t>
+          <t>CAND_0060054</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -1969,19 +2319,24 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>0.7664</t>
+          <t>1.0155</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>JD overlap is thin: AI Research Engineer at Wysa (6.2 YOE); JD-aligned skills: Pinecone, Weaviate, Python. Gaps: under half of JD must-have skills covered.</t>
+          <t>0.3416</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>JD overlap is thin: AI Engineer at Mad Street Den (6.4 YOE); JD-aligned skills: Weaviate, FAISS, Elasticsearch. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>CAND_0018549</t>
+          <t>CAND_0024878</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -1991,19 +2346,24 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>0.7661</t>
+          <t>1.0126</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Moderate fit: Recommendation Systems Engineer at Uber (6.8 YOE); JD-aligned skills: Weaviate, Elasticsearch, Qdrant. Gaps: under half of JD must-have skills covered.</t>
+          <t>0.4462</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>Moderate fit: AI Specialist at HCL (5.7 YOE); JD-aligned skills: pgvector, Elasticsearch, NLP. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>CAND_0066999</t>
+          <t>CAND_0008425</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -2013,19 +2373,24 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>0.7656</t>
+          <t>1.0111</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Partial alignment: Recommendation Systems Engineer at Microsoft (5.9 YOE); JD-aligned skills: OpenSearch, FAISS, LLMs. Gaps: under half of JD must-have skills covered.</t>
+          <t>0.2436</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>Partial alignment: Senior NLP Engineer at Ola (7.8 YOE); JD-aligned skills: Qdrant, pgvector, Sentence Transformers. Gaps: 90-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>CAND_0070398</t>
+          <t>CAND_0036121</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -2035,19 +2400,24 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>0.7649</t>
+          <t>1.0109</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Acceptable but not standout: Machine Learning Engineer at Genpact AI (7.2 YOE); JD-aligned skills: FAISS, Embeddings, Python. Gaps: 120-day notice period.</t>
+          <t>0.3242</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>Acceptable but not standout: ML Engineer at Wysa (5.2 YOE); JD-aligned skills: Embeddings, Vector Search, Information Retrieval. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>CAND_0017093</t>
+          <t>CAND_0027691</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -2057,19 +2427,24 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>0.7648</t>
+          <t>1.0104</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Mixed signals: ML Engineer at Zoho (5.9 YOE); JD-aligned skills: LLMs, Embeddings. Gaps: under half of JD must-have skills covered.</t>
+          <t>0.4306</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>Mixed signals: NLP Engineer at Haptik (6.5 YOE); JD-aligned skills: Weaviate, Embeddings, Python. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>CAND_0092245</t>
+          <t>CAND_0037980</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -2079,19 +2454,24 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>0.7646</t>
+          <t>1.0099</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>JD overlap is thin: Senior Data Scientist at Ola (4.1 YOE); JD-aligned skills: Embeddings, FAISS, Qdrant. Gaps: under half of JD must-have skills covered.</t>
+          <t>0.7550</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>JD overlap is thin: Senior Applied Scientist at Niramai (9.0 YOE); JD-aligned skills: NLP, Text Encoders, pgvector. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>CAND_0093193</t>
+          <t>CAND_0096104</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -2101,19 +2481,24 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>0.7644</t>
+          <t>1.0086</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Moderate fit: Senior Machine Learning Engineer at Niramai (7.9 YOE); JD-aligned skills: Qdrant, OpenSearch. Gaps: under half of JD must-have skills covered.</t>
+          <t>0.5401</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>Moderate fit: AI Specialist at Yellow.ai (7.0 YOE); JD-aligned skills: Pinecone. Gaps: only 1 core JD skill matched.</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>CAND_0002037</t>
+          <t>CAND_0001819</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -2123,19 +2508,24 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>0.7638</t>
+          <t>1.0074</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Partial alignment: ML Engineer at Locobuzz (5.5 YOE); JD-aligned skills: Fine-tuning LLMs, Milvus, Pinecone. Gaps: not flagged open to work.</t>
+          <t>0.3603</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>Partial alignment: ML Engineer at Genpact AI (4.4 YOE); JD-aligned skills: Weaviate, pgvector, NLP. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>CAND_0093912</t>
+          <t>CAND_0052328</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -2145,19 +2535,24 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>0.7582</t>
+          <t>1.0063</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Acceptable but not standout: Senior Data Scientist at Razorpay (5.3 YOE); JD-aligned skills: Milvus, Embeddings, Vector Search. Gaps: under half of JD must-have skills covered.</t>
+          <t>0.5090</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>Acceptable but not standout: Recommendation Systems Engineer at Amazon (6.5 YOE); JD-aligned skills: OpenSearch, Fine-tuning LLMs, Vector Search. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>CAND_0092255</t>
+          <t>CAND_0030348</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -2167,19 +2562,24 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>0.7570</t>
+          <t>1.0047</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Mixed signals: ML Engineer at InMobi (5.2 YOE); JD-aligned skills: Weaviate, OpenSearch, Vector Search. Gaps: under half of JD must-have skills covered.</t>
+          <t>0.3735</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>Mixed signals: Machine Learning Engineer at BYJU'S (4.5 YOE); JD-aligned skills: Embeddings, Vector Search, Elasticsearch. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>CAND_0010257</t>
+          <t>CAND_0009691</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -2189,19 +2589,24 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>0.7560</t>
+          <t>1.0023</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>JD overlap is thin: Senior Data Scientist at Google (6.5 YOE); JD-aligned skills: Milvus, Python, OpenSearch. Gaps: 120-day notice period.</t>
+          <t>0.1214</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>JD overlap is thin: Applied ML Engineer at LinkedIn (6.2 YOE); JD-aligned skills: Fine-tuning LLMs, Pinecone, Sentence Transformers. Gaps: 120-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>CAND_0099269</t>
+          <t>CAND_0019288</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -2211,19 +2616,24 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>0.7559</t>
+          <t>1.0018</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Moderate fit: Data Scientist at BYJU'S (5.5 YOE); JD-aligned skills: Elasticsearch, Python, NLP. Gaps: 120-day notice period.</t>
+          <t>0.3846</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>Moderate fit: AI Research Engineer at Paytm (5.7 YOE); JD-aligned skills: pgvector, FAISS, OpenSearch. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>CAND_0021836</t>
+          <t>CAND_0002793</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -2233,19 +2643,24 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>0.7532</t>
+          <t>1.0014</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Partial alignment: ML Engineer at CRED (6.5 YOE); JD-aligned skills: Vector Search, Elasticsearch, NLP. Gaps: under half of JD must-have skills covered.</t>
+          <t>0.3997</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>Partial alignment: AI Specialist at Meesho (5.5 YOE); JD-aligned skills: pgvector, Information Retrieval, FAISS. Gaps: not flagged open to work.</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>CAND_0032179</t>
+          <t>CAND_0043637</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -2255,19 +2670,24 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>0.7530</t>
+          <t>0.9985</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Acceptable but not standout: Computer Vision Engineer at InMobi (6.4 YOE); JD-aligned skills: Vector Search, Weaviate, Python. Gaps: not flagged open to work.</t>
+          <t>0.4329</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>Acceptable but not standout: Junior ML Engineer at Rephrase.ai (5.5 YOE); JD-aligned skills: Milvus, pgvector. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>CAND_0060054</t>
+          <t>CAND_0091534</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -2277,19 +2697,24 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>0.7522</t>
+          <t>0.9982</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Mixed signals: AI Engineer at Mad Street Den (6.4 YOE); JD-aligned skills: Weaviate, FAISS, Elasticsearch. Gaps: not flagged open to work.</t>
+          <t>0.2365</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>Mixed signals: AI Engineer at Flipkart (16.6 YOE); JD-aligned skills: Qdrant, Sentence Transformers. Gaps: experience above target band for this role; not flagged open to work.</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>CAND_0005311</t>
+          <t>CAND_0070398</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -2299,19 +2724,24 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>0.7501</t>
+          <t>0.9974</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>JD overlap is thin: AI Research Engineer at Aganitha (5.7 YOE); JD-aligned skills: Qdrant, Fine-tuning LLMs, NLP. Gaps: under half of JD must-have skills covered.</t>
+          <t>0.2060</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>JD overlap is thin: Machine Learning Engineer at Genpact AI (7.2 YOE); JD-aligned skills: FAISS, Embeddings, Python. Gaps: 120-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>CAND_0054123</t>
+          <t>CAND_0015578</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -2321,19 +2751,24 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>0.7495</t>
+          <t>0.9968</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Moderate fit: Applied ML Engineer at Meta (4.7 YOE); JD-aligned skills: Python, Weaviate, Qdrant. Gaps: not flagged open to work.</t>
+          <t>0.1397</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>Moderate fit: AI Engineer at Zoho (5.4 YOE); JD-aligned skills: Embeddings, NLP, Sentence Transformers. Gaps: 90-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>CAND_0027691</t>
+          <t>CAND_0010541</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -2343,19 +2778,24 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>0.7487</t>
+          <t>0.9965</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Partial alignment: NLP Engineer at Haptik (6.5 YOE); JD-aligned skills: Weaviate, Embeddings, Python. Gaps: under half of JD must-have skills covered.</t>
+          <t>0.5800</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>Partial alignment: AI Research Engineer at Wysa (6.2 YOE); JD-aligned skills: Pinecone, Weaviate, Python. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>CAND_0011432</t>
+          <t>CAND_0065195</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -2365,19 +2805,24 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>0.7483</t>
+          <t>0.9964</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Acceptable but not standout: Senior Data Scientist at Amazon (7.6 YOE); JD-aligned skills: OpenSearch, Elasticsearch. Gaps: under half of JD must-have skills covered.</t>
+          <t>0.3492</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>Acceptable but not standout: Search Engineer at CRED (5.1 YOE); JD-aligned skills: LLMs, Elasticsearch, Qdrant. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>CAND_0065878</t>
+          <t>CAND_0037944</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -2387,19 +2832,24 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>0.7478</t>
+          <t>0.9956</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Mixed signals: Senior Data Scientist at Niramai (7.8 YOE); JD-aligned skills: Vector Search, Fine-tuning LLMs. Gaps: under half of JD must-have skills covered.</t>
+          <t>0.2490</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>Mixed signals: Senior Data Scientist at Vedantu (4.9 YOE); JD-aligned skills: Vector Search, OpenSearch, Embeddings. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>CAND_0037980</t>
+          <t>CAND_0093474</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -2409,19 +2859,24 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>0.7474</t>
+          <t>0.9916</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>JD overlap is thin: Senior Applied Scientist at Niramai (9.0 YOE); JD-aligned skills: NLP. Gaps: only 1 core JD skill matched.</t>
+          <t>0.4226</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>JD overlap is thin: Senior Software Engineer (ML) at Wipro (5.3 YOE); JD-aligned skills: Vector Search, Qdrant, FAISS. Gaps: 90-day notice period; not flagged open to work.</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>CAND_0007009</t>
+          <t>CAND_0039754</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -2431,19 +2886,24 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>0.7463</t>
+          <t>0.9907</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Lower-tier shortlist entry — Recommendation Systems Engineer at Wysa (7.9 YOE); JD-aligned skills: Weaviate, Python, Embeddings. Key gaps: weak secondary signals vs higher ranks.</t>
+          <t>0.5509</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>Lower-tier shortlist entry — Senior Applied Scientist at Meta (16.2 YOE); JD-aligned skills: Fine-tuning LLMs, Qdrant, NLP. Key gaps: experience above target band for this role.</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>CAND_0001819</t>
+          <t>CAND_0003791</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -2453,19 +2913,24 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>0.7460</t>
+          <t>0.9905</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Lower-tier shortlist entry — ML Engineer at Genpact AI (4.4 YOE); JD-aligned skills: Weaviate, NLP. Key gaps: weak secondary signals vs higher ranks.</t>
+          <t>0.4776</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>Lower-tier shortlist entry — ML Engineer at Meesho (6.6 YOE); JD-aligned skills: LLMs, pgvector, Python. Key gaps: weak secondary signals vs higher ranks.</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>CAND_0046064</t>
+          <t>CAND_0001661</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -2475,19 +2940,24 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>0.7457</t>
+          <t>0.9903</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Lower-tier shortlist entry — Senior NLP Engineer at Salesforce (8.9 YOE); JD-aligned skills: Python, Pinecone, OpenSearch. Key gaps: weak secondary signals vs higher ranks.</t>
+          <t>0.3461</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>Lower-tier shortlist entry — Senior Data Engineer at Cognizant (7.8 YOE); JD-aligned skills: Vector Search. Key gaps: only 1 core JD skill matched.</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>CAND_0028793</t>
+          <t>CAND_0007460</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2497,19 +2967,24 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>0.7455</t>
+          <t>0.9899</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Lower-tier shortlist entry — Search Engineer at Google (7.2 YOE); JD-aligned skills: Embeddings, NLP. Key gaps: 120-day notice period.</t>
+          <t>0.2260</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>Lower-tier shortlist entry — AI Engineer at Salesforce (4.7 YOE); JD-aligned skills: Embeddings, Weaviate, Information Retrieval. Key gaps: 120-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>CAND_0071939</t>
+          <t>CAND_0041669</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -2519,19 +2994,24 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>0.7439</t>
+          <t>0.9892</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Lower-tier shortlist entry — Data Scientist at Krutrim (6.4 YOE); JD-aligned skills: Elasticsearch, OpenSearch, Embeddings. Key gaps: weak secondary signals vs higher ranks.</t>
+          <t>0.6806</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>Lower-tier shortlist entry — Recommendation Systems Engineer at CRED (8.0 YOE); JD-aligned skills: FAISS, Milvus, Weaviate. Key gaps: weak secondary signals vs higher ranks.</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>CAND_0005260</t>
+          <t>CAND_0050876</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -2541,19 +3021,24 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>0.7437</t>
+          <t>0.9892</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Lower-tier shortlist entry — Senior NLP Engineer at Netflix (5.2 YOE); JD-aligned skills: Python, NLP, Embeddings. Key gaps: not flagged open to work.</t>
+          <t>0.4323</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>Lower-tier shortlist entry — Applied ML Engineer at Freshworks (6.0 YOE); JD-aligned skills: Qdrant, FAISS, OpenSearch. Key gaps: 90-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>CAND_0006418</t>
+          <t>CAND_0081086</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -2563,19 +3048,24 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>0.7435</t>
+          <t>0.9892</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Lower-tier shortlist entry — Machine Learning Engineer at Verloop.io (5.7 YOE); JD-aligned skills: Embeddings, Weaviate, Elasticsearch. Key gaps: weak secondary signals vs higher ranks.</t>
+          <t>0.2245</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>Lower-tier shortlist entry — AI Specialist at Observe.AI (5.2 YOE); JD-aligned skills: pgvector, Weaviate, Embeddings. Key gaps: weak secondary signals vs higher ranks.</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>CAND_0039754</t>
+          <t>CAND_0013665</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -2585,19 +3075,24 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>0.7432</t>
+          <t>0.9890</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Lower-tier shortlist entry — Senior Applied Scientist at Meta (16.2 YOE); JD-aligned skills: Fine-tuning LLMs, Qdrant, NLP. Key gaps: experience above target band for this role.</t>
+          <t>0.2424</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>Lower-tier shortlist entry — Senior Software Engineer (ML) at InMobi (5.2 YOE); JD-aligned skills: Qdrant, Embeddings. Key gaps: not flagged open to work.</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>CAND_0073982</t>
+          <t>CAND_0080465</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -2607,19 +3102,24 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>0.7428</t>
+          <t>0.9887</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Lower-tier shortlist entry — Data Scientist at Dream11 (7.0 YOE); JD-aligned skills: Sentence Transformers, Qdrant, FAISS. Key gaps: weak secondary signals vs higher ranks.</t>
+          <t>0.2782</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>Lower-tier shortlist entry — ML Engineer at Meesho (4.2 YOE); JD-aligned skills: Milvus, Qdrant. Key gaps: 90-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>CAND_0091899</t>
+          <t>CAND_0094759</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -2629,12 +3129,17 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>0.7424</t>
+          <t>0.9874</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Lower-tier shortlist entry — Senior Software Engineer (ML) at PhonePe (5.8 YOE); JD-aligned skills: Sentence Transformers, FAISS, NLP. Key gaps: not flagged open to work.</t>
+          <t>0.2923</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>Lower-tier shortlist entry — Lead AI Engineer at Meta (8.6 YOE); JD-aligned skills: Qdrant, Fine-tuning LLMs, Vector Search. Key gaps: low recruiter response rate; not flagged open to work.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
regenerate submission with bounded scores
</commit_message>
<xml_diff>
--- a/submission.xlsx
+++ b/submission.xlsx
@@ -446,7 +446,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>CAND_0018499</t>
+          <t>CAND_0001819</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -456,24 +456,24 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>1.2336</t>
+          <t>1.0000</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>0.6132</t>
+          <t>0.3603</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Rank 1: Senior Machine Learning Engineer at Zomato (7.2 YOE); JD-aligned skills: Weaviate, Pinecone, Information Retrieval. Top-tier composite score across career, skills, and availability. Counterfactual: ranks on career trajectory and assessed depth over keyword coverage (5/20 listed must-haves), aligning with the JD anti-keyword-stuffing guidance. Join probability: 61%.</t>
+          <t>Rank 1: ML Engineer at Genpact AI (4.4 YOE); JD-aligned skills: Weaviate, pgvector, NLP. Top-tier composite score across career, skills, and availability. Counterfactual: ranks on career trajectory and assessed depth over keyword coverage (3/20 listed must-haves), aligning with the JD anti-keyword-stuffing guidance. Join probability: 36%.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>CAND_0088025</t>
+          <t>CAND_0002025</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -483,24 +483,24 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>1.2187</t>
+          <t>1.0000</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>0.5411</t>
+          <t>0.3912</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Rank 2: Staff Machine Learning Engineer at Yellow.ai (8.6 YOE); JD-aligned skills: Pinecone, LLMs, Elasticsearch. Top-tier composite score across career, skills, and availability. Minor note: 90-day notice period. Join probability: 54%.</t>
+          <t>Rank 2: Senior AI Engineer at Apple (5.9 YOE); JD-aligned skills: FAISS, OpenSearch, Weaviate. Top-tier composite score across career, skills, and availability. Counterfactual: ranks on career trajectory and assessed depth over keyword coverage (8/20 listed must-haves), aligning with the JD anti-keyword-stuffing guidance. Join probability: 39%.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>CAND_0071974</t>
+          <t>CAND_0002793</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -510,24 +510,24 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>1.2065</t>
+          <t>1.0000</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>0.3414</t>
+          <t>0.3997</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Rank 3: Senior AI Engineer at Netflix (7.8 YOE); JD-aligned skills: Weaviate, Pinecone, Information Retrieval. Top-tier composite score across career, skills, and availability. Counterfactual: ranks on career trajectory and assessed depth over keyword coverage (7/20 listed must-haves), aligning with the JD anti-keyword-stuffing guidance. Join probability: 34%; low engagement signals.</t>
+          <t>Rank 3: AI Specialist at Meesho (5.5 YOE); JD-aligned skills: pgvector, Information Retrieval, FAISS. Top-tier composite score across career, skills, and availability. Counterfactual: ranks on career trajectory and assessed depth over keyword coverage (3/20 listed must-haves), aligning with the JD anti-keyword-stuffing guidance. Join probability: 40%.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>CAND_0068351</t>
+          <t>CAND_0003841</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -537,24 +537,24 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>1.1986</t>
+          <t>1.0000</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>0.4040</t>
+          <t>0.3402</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Rank 4: Lead AI Engineer at Sarvam AI (6.4 YOE); JD-aligned skills: pgvector, Qdrant, Elasticsearch. Top-tier composite score across career, skills, and availability. Counterfactual: ranks on career trajectory and assessed depth over keyword coverage (7/20 listed must-haves), aligning with the JD anti-keyword-stuffing guidance. Join probability: 40%.</t>
+          <t>Rank 4: ML Engineer at Tech Mahindra (5.0 YOE); JD-aligned skills: Pinecone, Fine-tuning LLMs, Sentence Transformers. Top-tier composite score across career, skills, and availability. Counterfactual: ranks on career trajectory and assessed depth over keyword coverage (3/20 listed must-haves), aligning with the JD anti-keyword-stuffing guidance. Join probability: 34%; low engagement signals.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CAND_0081846</t>
+          <t>CAND_0005260</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -564,24 +564,24 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>1.1861</t>
+          <t>1.0000</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>0.4803</t>
+          <t>0.4814</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Rank 5: Lead AI Engineer at Razorpay (6.7 YOE); JD-aligned skills: Information Retrieval, pgvector, Elasticsearch. Top-tier composite score across career, skills, and availability. Counterfactual: ranks on career trajectory and assessed depth over keyword coverage (7/20 listed must-haves), aligning with the JD anti-keyword-stuffing guidance. Join probability: 48%.</t>
+          <t>Rank 5: Senior NLP Engineer at Netflix (5.2 YOE); JD-aligned skills: Information Retrieval, Python, NLP. Top-tier composite score across career, skills, and availability. Counterfactual: ranks on career trajectory and assessed depth over keyword coverage (5/20 listed must-haves), aligning with the JD anti-keyword-stuffing guidance. Join probability: 48%.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>CAND_0002025</t>
+          <t>CAND_0005538</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -591,24 +591,24 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>1.1708</t>
+          <t>1.0000</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>0.3912</t>
+          <t>0.4072</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Strong match — Senior AI Engineer at Apple (5.9 YOE); JD-aligned skills: FAISS, OpenSearch, Weaviate. Join probability: 39%.</t>
+          <t>Strong match — Senior AI Engineer at Adobe (5.9 YOE); JD-aligned skills: Vector Representations, Python, Information Retrieval Systems. Watch: 90-day notice period. Join probability: 41%.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>CAND_0046525</t>
+          <t>CAND_0005649</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -618,24 +618,24 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>1.1683</t>
+          <t>1.0000</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>0.3574</t>
+          <t>0.5162</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Strong match — Senior Machine Learning Engineer at Genpact AI (6.1 YOE); JD-aligned skills: Elasticsearch, Information Retrieval, LLMs. Join probability: 36%.</t>
+          <t>Strong match — Senior Data Scientist at Sarvam AI (7.4 YOE); JD-aligned skills: Fine-tuning LLMs, Weaviate, Information Retrieval. Watch: 90-day notice period. Join probability: 52%.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>CAND_0077337</t>
+          <t>CAND_0006567</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -645,24 +645,24 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>1.1645</t>
+          <t>1.0000</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>0.4883</t>
+          <t>0.6079</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Strong match — Staff Machine Learning Engineer at Paytm (7.0 YOE); JD-aligned skills: pgvector, Pinecone, Information Retrieval. Join probability: 49%.</t>
+          <t>Strong match — Senior AI Engineer at Meta (7.9 YOE); JD-aligned skills: Vector Representations, NLP, Python. Join probability: 61%.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>CAND_0055905</t>
+          <t>CAND_0008425</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -672,24 +672,24 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>1.1445</t>
+          <t>1.0000</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>0.6870</t>
+          <t>0.2436</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Strong match — Senior Machine Learning Engineer at Flipkart (8.1 YOE); JD-aligned skills: Elasticsearch, Python, LLMs. Join probability: 69%.</t>
+          <t>Strong match — Senior NLP Engineer at Ola (7.8 YOE); JD-aligned skills: Qdrant, pgvector, Sentence Transformers. Watch: 90-day notice period. Join probability: 24%; low engagement signals.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>CAND_0080766</t>
+          <t>CAND_0009691</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -699,24 +699,24 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>1.1382</t>
+          <t>1.0000</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>0.4625</t>
+          <t>0.1214</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Strong match — Staff Machine Learning Engineer at Salesforce (8.8 YOE); JD-aligned skills: Information Retrieval Systems, Elasticsearch, Natural Language Processing. Join probability: 46%.</t>
+          <t>Strong match — Applied ML Engineer at LinkedIn (6.2 YOE); JD-aligned skills: Fine-tuning LLMs, Pinecone, Sentence Transformers. Watch: 120-day notice period. Join probability: 12%; long notice.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>CAND_0006567</t>
+          <t>CAND_0010257</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -726,24 +726,24 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>1.1293</t>
+          <t>1.0000</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>0.6079</t>
+          <t>0.3313</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Strong match — Senior AI Engineer at Meta (7.9 YOE); JD-aligned skills: Vector Representations, NLP, Python. Join probability: 61%.</t>
+          <t>Strong match — Senior Data Scientist at Google (6.5 YOE); JD-aligned skills: Milvus, Python, OpenSearch. Watch: 120-day notice period. Join probability: 33%; long notice.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>CAND_0050454</t>
+          <t>CAND_0011432</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -753,24 +753,24 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>1.1031</t>
+          <t>1.0000</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>0.3504</t>
+          <t>0.5534</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Strong match — AI Engineer at Rephrase.ai (6.8 YOE); JD-aligned skills: Fine-tuning LLMs, FAISS, Qdrant. Join probability: 35%.</t>
+          <t>Strong match — Senior Data Scientist at Amazon (7.6 YOE); JD-aligned skills: OpenSearch, pgvector, Elasticsearch. Join probability: 55%.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>CAND_0083879</t>
+          <t>CAND_0011687</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -780,24 +780,24 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>1.1019</t>
+          <t>1.0000</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>0.5950</t>
+          <t>0.5094</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Strong match — Machine Learning Engineer at Ola (7.1 YOE); JD-aligned skills: Fine-tuning LLMs, Milvus, Sentence Transformers. Join probability: 60%.</t>
+          <t>Strong match — Senior NLP Engineer at Niramai (7.8 YOE); JD-aligned skills: OpenSearch, FAISS, Embeddings. Join probability: 51%.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>CAND_0018094</t>
+          <t>CAND_0015528</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -807,24 +807,24 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>1.1014</t>
+          <t>1.0000</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>0.4428</t>
+          <t>0.3246</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Strong match — ML Engineer at Mad Street Den (5.2 YOE); JD-aligned skills: Pinecone, Information Retrieval, Fine-tuning LLMs. Join probability: 44%.</t>
+          <t>Strong match — Applied ML Engineer at Krutrim (7.4 YOE); JD-aligned skills: Weaviate, pgvector, Information Retrieval. Join probability: 32%; low engagement signals.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>CAND_0044222</t>
+          <t>CAND_0016163</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -834,24 +834,24 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>1.0990</t>
+          <t>1.0000</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>0.2252</t>
+          <t>0.2905</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Strong match — AI Engineer at PolicyBazaar (7.7 YOE); JD-aligned skills: Vector Search, OpenSearch, Qdrant. Join probability: 23%; low engagement signals.</t>
+          <t>Strong match — Applied ML Engineer at Dream11 (6.7 YOE); JD-aligned skills: Weaviate, Embeddings, pgvector. Watch: 120-day notice period. Join probability: 29%; long notice.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>CAND_0049538</t>
+          <t>CAND_0018094</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -861,24 +861,24 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>1.0933</t>
+          <t>1.0000</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>0.3362</t>
+          <t>0.4428</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Strong match — Applied ML Engineer at Saarthi.ai (5.8 YOE); JD-aligned skills: OpenSearch, Vector Search, Milvus. Join probability: 34%; low engagement signals.</t>
+          <t>Strong match — ML Engineer at Mad Street Den (5.2 YOE); JD-aligned skills: Pinecone, Information Retrieval, Fine-tuning LLMs. Join probability: 44%.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>CAND_0087630</t>
+          <t>CAND_0018499</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -888,24 +888,24 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>1.0927</t>
+          <t>1.0000</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>0.3940</t>
+          <t>0.6132</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Strong match — AI Engineer at Vedantu (7.2 YOE); JD-aligned skills: Elasticsearch, pgvector, NLP. Join probability: 39%.</t>
+          <t>Strong match — Senior Machine Learning Engineer at Zomato (7.2 YOE); JD-aligned skills: Weaviate, Pinecone, Information Retrieval. Join probability: 61%.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>CAND_0086022</t>
+          <t>CAND_0019288</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -915,24 +915,24 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>1.0912</t>
+          <t>1.0000</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>0.3683</t>
+          <t>0.3846</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Strong match — Senior Applied Scientist at Sarvam AI (5.3 YOE); JD-aligned skills: Vector Search, pgvector, Fine-tuning LLMs. Join probability: 37%.</t>
+          <t>Strong match — AI Research Engineer at Paytm (5.7 YOE); JD-aligned skills: pgvector, FAISS, OpenSearch. Join probability: 38%.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>CAND_0016163</t>
+          <t>CAND_0020350</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -942,24 +942,24 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>1.0899</t>
+          <t>1.0000</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>0.2905</t>
+          <t>0.3210</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Strong match — Applied ML Engineer at Dream11 (6.7 YOE); JD-aligned skills: Weaviate, Embeddings, pgvector. Watch: 120-day notice period. Join probability: 29%; long notice.</t>
+          <t>Strong match — AI Engineer at Zoho (5.8 YOE); JD-aligned skills: NLP, LLMs, FAISS. Join probability: 32%; low engagement signals.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>CAND_0005649</t>
+          <t>CAND_0020877</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -969,24 +969,24 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>1.0870</t>
+          <t>1.0000</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>0.5162</t>
+          <t>0.3909</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Strong match — Senior Data Scientist at Sarvam AI (7.4 YOE); JD-aligned skills: Fine-tuning LLMs, Weaviate, Information Retrieval. Watch: 90-day notice period. Join probability: 52%.</t>
+          <t>Strong match — Applied ML Engineer at CRED (5.1 YOE); JD-aligned skills: Elasticsearch, OpenSearch, Information Retrieval. Join probability: 39%.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>CAND_0030031</t>
+          <t>CAND_0024878</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -996,24 +996,24 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>1.0786</t>
+          <t>1.0000</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>0.3445</t>
+          <t>0.4462</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Solid profile: AI Engineer at Microsoft (5.7 YOE); JD-aligned skills: Information Retrieval, Python, NLP.</t>
+          <t>Solid profile: AI Specialist at HCL (5.7 YOE); JD-aligned skills: pgvector, Elasticsearch, NLP.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>CAND_0096142</t>
+          <t>CAND_0025923</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1023,24 +1023,24 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>1.0786</t>
+          <t>1.0000</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>0.2486</t>
+          <t>0.2891</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Good fit with caveats: Applied ML Engineer at upGrad (5.0 YOE); JD-aligned skills: Weaviate, Pinecone, Python. Concerns: 120-day notice period.</t>
+          <t>Good fit with caveats: Senior Software Engineer (ML) at HCL (5.0 YOE); JD-aligned skills: pgvector, Qdrant, Pinecone.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>CAND_0081852</t>
+          <t>CAND_0027691</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1050,24 +1050,24 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>1.0778</t>
+          <t>1.0000</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>0.2331</t>
+          <t>0.4306</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Competitive candidate: Senior Data Scientist at Mad Street Den (5.9 YOE); JD-aligned skills: Milvus, pgvector, Weaviate.</t>
+          <t>Competitive candidate: NLP Engineer at Haptik (6.5 YOE); JD-aligned skills: Weaviate, Embeddings, Python.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>CAND_0039383</t>
+          <t>CAND_0028793</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1077,24 +1077,24 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>1.0766</t>
+          <t>1.0000</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>0.5155</t>
+          <t>0.2941</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Meets several JD signals: Applied ML Engineer at Meesho (7.1 YOE); JD-aligned skills: FAISS, NLP, Vector Search. Concerns: 90-day notice period.</t>
+          <t>Meets several JD signals: Search Engineer at Google (7.2 YOE); JD-aligned skills: Embeddings, Information Retrieval, pgvector. Concerns: 120-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>CAND_0058688</t>
+          <t>CAND_0030031</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1104,24 +1104,24 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>1.0750</t>
+          <t>1.0000</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>0.7268</t>
+          <t>0.3445</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Solid profile: AI Engineer at Vedantu (6.7 YOE); JD-aligned skills: Embeddings, Information Retrieval, Milvus.</t>
+          <t>Solid profile: AI Engineer at Microsoft (5.7 YOE); JD-aligned skills: Information Retrieval, Python, NLP.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>CAND_0020877</t>
+          <t>CAND_0030348</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1131,24 +1131,24 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>1.0749</t>
+          <t>1.0000</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>0.3909</t>
+          <t>0.3735</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Good fit with caveats: Applied ML Engineer at CRED (5.1 YOE); JD-aligned skills: Elasticsearch, OpenSearch, Information Retrieval.</t>
+          <t>Good fit with caveats: Machine Learning Engineer at BYJU'S (4.5 YOE); JD-aligned skills: Embeddings, Vector Search, Elasticsearch.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>CAND_0020350</t>
+          <t>CAND_0032216</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1158,24 +1158,24 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>1.0743</t>
+          <t>1.0000</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>0.3210</t>
+          <t>0.2743</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Competitive candidate: AI Engineer at Zoho (5.8 YOE); JD-aligned skills: NLP, LLMs, FAISS.</t>
+          <t>Competitive candidate: ML Engineer at upGrad (6.1 YOE); JD-aligned skills: Information Retrieval, Qdrant, Sentence Transformers.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>CAND_0042029</t>
+          <t>CAND_0036121</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1185,24 +1185,24 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>1.0721</t>
+          <t>1.0000</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>0.4840</t>
+          <t>0.3242</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Meets several JD signals: Senior Data Scientist at Flipkart (6.5 YOE); JD-aligned skills: NLP, Elasticsearch, Embeddings.</t>
+          <t>Meets several JD signals: ML Engineer at Wysa (5.2 YOE); JD-aligned skills: Embeddings, Vector Search, Information Retrieval.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>CAND_0044855</t>
+          <t>CAND_0037566</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1212,24 +1212,24 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>1.0706</t>
+          <t>1.0000</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>0.3723</t>
+          <t>0.5752</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Solid profile: Senior Data Scientist at Flipkart (6.6 YOE); JD-aligned skills: OpenSearch, Information Retrieval, Pinecone.</t>
+          <t>Solid profile: Machine Learning Engineer at LinkedIn (6.9 YOE); JD-aligned skills: Pinecone, NLP, LLMs.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>CAND_0046064</t>
+          <t>CAND_0037980</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1239,24 +1239,24 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>1.0691</t>
+          <t>1.0000</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>0.3780</t>
+          <t>0.7550</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Good fit with caveats: Senior NLP Engineer at Salesforce (8.9 YOE); JD-aligned skills: Python, Pinecone, OpenSearch.</t>
+          <t>Good fit with caveats: Senior Applied Scientist at Niramai (9.0 YOE); JD-aligned skills: NLP, Text Encoders, pgvector.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>CAND_0061257</t>
+          <t>CAND_0038368</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1266,24 +1266,24 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>1.0681</t>
+          <t>1.0000</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>0.3969</t>
+          <t>0.4347</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Competitive candidate: Staff Machine Learning Engineer at LinkedIn (8.0 YOE); JD-aligned skills: Information Retrieval Systems, Python, Vector Representations.</t>
+          <t>Competitive candidate: ML Engineer at PhonePe (5.4 YOE); JD-aligned skills: Embeddings, FAISS, NLP.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>CAND_0079387</t>
+          <t>CAND_0039383</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1293,24 +1293,24 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>1.0675</t>
+          <t>1.0000</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>0.4465</t>
+          <t>0.5155</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Meets several JD signals: AI Engineer at Microsoft (6.9 YOE); JD-aligned skills: Python, Sentence Transformers, Vector Search.</t>
+          <t>Meets several JD signals: Applied ML Engineer at Meesho (7.1 YOE); JD-aligned skills: FAISS, NLP, Vector Search. Concerns: 90-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>CAND_0043228</t>
+          <t>CAND_0040178</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1320,24 +1320,24 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>1.0657</t>
+          <t>1.0000</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>0.3534</t>
+          <t>0.3303</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Solid profile: Applied ML Engineer at Zoho (6.8 YOE); JD-aligned skills: NLP, Vector Search, Sentence Transformers.</t>
+          <t>Solid profile: ML Engineer at Meesho (5.0 YOE); JD-aligned skills: Weaviate, Fine-tuning LLMs, Vector Search.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>CAND_0093193</t>
+          <t>CAND_0042029</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1347,24 +1347,24 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>1.0652</t>
+          <t>1.0000</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>0.4352</t>
+          <t>0.4840</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Good fit with caveats: Senior Machine Learning Engineer at Niramai (7.9 YOE); JD-aligned skills: Text Encoders, Vector Representations, Qdrant.</t>
+          <t>Good fit with caveats: Senior Data Scientist at Flipkart (6.5 YOE); JD-aligned skills: NLP, Elasticsearch, Embeddings.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>CAND_0045250</t>
+          <t>CAND_0042100</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1374,24 +1374,24 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>1.0643</t>
+          <t>1.0000</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>0.3580</t>
+          <t>0.2536</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Competitive candidate: Applied ML Engineer at Rephrase.ai (6.6 YOE); JD-aligned skills: Sentence Transformers, Milvus, Embeddings.</t>
+          <t>Competitive candidate: Machine Learning Engineer at Freshworks (7.3 YOE); JD-aligned skills: Elasticsearch, Fine-tuning LLMs, Pinecone. Concerns: 90-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>CAND_0003841</t>
+          <t>CAND_0043228</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1401,24 +1401,24 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>1.0641</t>
+          <t>1.0000</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>0.3402</t>
+          <t>0.3534</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Meets several JD signals: ML Engineer at Tech Mahindra (5.0 YOE); JD-aligned skills: Pinecone, Fine-tuning LLMs, Sentence Transformers.</t>
+          <t>Meets several JD signals: Applied ML Engineer at Zoho (6.8 YOE); JD-aligned skills: NLP, Vector Search, Sentence Transformers.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>CAND_0047721</t>
+          <t>CAND_0044222</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1428,24 +1428,24 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>1.0600</t>
+          <t>1.0000</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>0.1736</t>
+          <t>0.2252</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Solid profile: Senior Data Scientist at Microsoft (7.0 YOE); JD-aligned skills: Milvus, Information Retrieval, FAISS. Concerns: 90-day notice period.</t>
+          <t>Solid profile: AI Engineer at PolicyBazaar (7.7 YOE); JD-aligned skills: Vector Search, OpenSearch, Qdrant.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>CAND_0042100</t>
+          <t>CAND_0044855</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1455,24 +1455,24 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>1.0570</t>
+          <t>1.0000</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>0.2536</t>
+          <t>0.3723</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Good fit with caveats: Machine Learning Engineer at Freshworks (7.3 YOE); JD-aligned skills: Elasticsearch, Fine-tuning LLMs, Pinecone. Concerns: 90-day notice period.</t>
+          <t>Good fit with caveats: Senior Data Scientist at Flipkart (6.6 YOE); JD-aligned skills: OpenSearch, Information Retrieval, Pinecone.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>CAND_0051292</t>
+          <t>CAND_0045250</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1482,24 +1482,24 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>1.0558</t>
+          <t>1.0000</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>0.4013</t>
+          <t>0.3580</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Competitive candidate: Applied ML Engineer at Freshworks (5.2 YOE); JD-aligned skills: pgvector, FAISS, LLMs.</t>
+          <t>Competitive candidate: Applied ML Engineer at Rephrase.ai (6.6 YOE); JD-aligned skills: Sentence Transformers, Milvus, Embeddings.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>CAND_0038368</t>
+          <t>CAND_0046064</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1509,24 +1509,24 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>1.0531</t>
+          <t>1.0000</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>0.4347</t>
+          <t>0.3780</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Meets several JD signals: ML Engineer at PhonePe (5.4 YOE); JD-aligned skills: Embeddings, FAISS, NLP.</t>
+          <t>Meets several JD signals: Senior NLP Engineer at Salesforce (8.9 YOE); JD-aligned skills: Python, Pinecone, OpenSearch.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>CAND_0037566</t>
+          <t>CAND_0046525</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1536,24 +1536,24 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>1.0519</t>
+          <t>1.0000</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>0.5752</t>
+          <t>0.3574</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Solid profile: Machine Learning Engineer at LinkedIn (6.9 YOE); JD-aligned skills: Pinecone, NLP, LLMs.</t>
+          <t>Solid profile: Senior Machine Learning Engineer at Genpact AI (6.1 YOE); JD-aligned skills: Elasticsearch, Information Retrieval, LLMs.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>CAND_0051004</t>
+          <t>CAND_0047721</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1563,24 +1563,24 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>1.0514</t>
+          <t>1.0000</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>0.5405</t>
+          <t>0.1736</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Good fit with caveats: Senior Data Scientist at CRED (4.7 YOE); JD-aligned skills: Embeddings, Qdrant, Fine-tuning LLMs.</t>
+          <t>Good fit with caveats: Senior Data Scientist at Microsoft (7.0 YOE); JD-aligned skills: Milvus, Information Retrieval, FAISS. Concerns: 90-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>CAND_0069905</t>
+          <t>CAND_0048166</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1590,24 +1590,24 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>1.0513</t>
+          <t>1.0000</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>0.3358</t>
+          <t>0.4054</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Competitive candidate: Applied ML Engineer at Sarvam AI (6.6 YOE); JD-aligned skills: Sentence Transformers, Python, Weaviate. Concerns: 90-day notice period.</t>
+          <t>Competitive candidate: ML Engineer at Aganitha (5.2 YOE); JD-aligned skills: Pinecone, Milvus, Qdrant.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>CAND_0055992</t>
+          <t>CAND_0049538</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1617,24 +1617,24 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>1.0510</t>
+          <t>1.0000</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>0.5850</t>
+          <t>0.3362</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Meets several JD signals: AI Engineer at CRED (16.9 YOE); JD-aligned skills: Information Retrieval, FAISS, OpenSearch.</t>
+          <t>Meets several JD signals: Applied ML Engineer at Saarthi.ai (5.8 YOE); JD-aligned skills: OpenSearch, Vector Search, Milvus.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>CAND_0068811</t>
+          <t>CAND_0050454</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -1644,24 +1644,24 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>1.0494</t>
+          <t>1.0000</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>0.4651</t>
+          <t>0.3504</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Solid profile: Applied ML Engineer at Freshworks (8.0 YOE); JD-aligned skills: Vector Search, Qdrant, Embeddings.</t>
+          <t>Solid profile: AI Engineer at Rephrase.ai (6.8 YOE); JD-aligned skills: Fine-tuning LLMs, FAISS, Qdrant.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>CAND_0093912</t>
+          <t>CAND_0051004</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -1671,24 +1671,24 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>1.0480</t>
+          <t>1.0000</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>0.4763</t>
+          <t>0.5405</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Good fit with caveats: Senior Data Scientist at Razorpay (5.3 YOE); JD-aligned skills: Milvus, Embeddings, Vector Search.</t>
+          <t>Good fit with caveats: Senior Data Scientist at CRED (4.7 YOE); JD-aligned skills: Embeddings, Qdrant, Fine-tuning LLMs.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>CAND_0099806</t>
+          <t>CAND_0051292</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -1698,24 +1698,24 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>1.0479</t>
+          <t>1.0000</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>0.3301</t>
+          <t>0.4013</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Competitive candidate: AI Engineer at Mad Street Den (4.6 YOE); JD-aligned skills: pgvector, FAISS, Embeddings.</t>
+          <t>Competitive candidate: Applied ML Engineer at Freshworks (5.2 YOE); JD-aligned skills: pgvector, FAISS, LLMs.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>CAND_0078002</t>
+          <t>CAND_0052328</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1725,24 +1725,24 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>1.0469</t>
+          <t>1.0000</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>0.2974</t>
+          <t>0.5090</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Meets several JD signals: Machine Learning Engineer at Meta (6.3 YOE); JD-aligned skills: pgvector, NLP, Weaviate.</t>
+          <t>Meets several JD signals: Recommendation Systems Engineer at Amazon (6.5 YOE); JD-aligned skills: OpenSearch, Fine-tuning LLMs, Vector Search.</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>CAND_0010257</t>
+          <t>CAND_0055905</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -1752,24 +1752,24 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>1.0458</t>
+          <t>1.0000</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>0.3313</t>
+          <t>0.6870</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Solid profile: Senior Data Scientist at Google (6.5 YOE); JD-aligned skills: Milvus, Python, OpenSearch. Concerns: 120-day notice period.</t>
+          <t>Solid profile: Senior Machine Learning Engineer at Flipkart (8.1 YOE); JD-aligned skills: Elasticsearch, Python, LLMs.</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>CAND_0065878</t>
+          <t>CAND_0055992</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -1779,24 +1779,24 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>1.0430</t>
+          <t>1.0000</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>0.2450</t>
+          <t>0.5850</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Good fit with caveats: Senior Data Scientist at Niramai (7.8 YOE); JD-aligned skills: pgvector, Vector Search, Fine-tuning LLMs.</t>
+          <t>Good fit with caveats: AI Engineer at CRED (16.9 YOE); JD-aligned skills: Information Retrieval, FAISS, OpenSearch.</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>CAND_0032216</t>
+          <t>CAND_0058688</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -1806,24 +1806,24 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>1.0428</t>
+          <t>1.0000</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>0.2743</t>
+          <t>0.7268</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Moderate fit: ML Engineer at upGrad (6.1 YOE); JD-aligned skills: Information Retrieval, Qdrant, Sentence Transformers. Gaps: under half of JD must-have skills covered.</t>
+          <t>Moderate fit: AI Engineer at Vedantu (6.7 YOE); JD-aligned skills: Embeddings, Information Retrieval, Milvus. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>CAND_0005260</t>
+          <t>CAND_0060054</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -1833,24 +1833,24 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>1.0401</t>
+          <t>1.0000</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>0.4814</t>
+          <t>0.3416</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Partial alignment: Senior NLP Engineer at Netflix (5.2 YOE); JD-aligned skills: Information Retrieval, Python, NLP. Gaps: under half of JD must-have skills covered.</t>
+          <t>Partial alignment: AI Engineer at Mad Street Den (6.4 YOE); JD-aligned skills: Weaviate, FAISS, Elasticsearch. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>CAND_0025923</t>
+          <t>CAND_0061257</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -1860,24 +1860,24 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>1.0385</t>
+          <t>1.0000</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>0.2891</t>
+          <t>0.3969</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Acceptable but not standout: Senior Software Engineer (ML) at HCL (5.0 YOE); JD-aligned skills: pgvector, Qdrant, Pinecone. Gaps: under half of JD must-have skills covered.</t>
+          <t>Acceptable but not standout: Staff Machine Learning Engineer at LinkedIn (8.0 YOE); JD-aligned skills: Information Retrieval Systems, Python, Vector Representations. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>CAND_0075574</t>
+          <t>CAND_0061550</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -1887,24 +1887,24 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>1.0377</t>
+          <t>1.0000</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>0.4170</t>
+          <t>0.3313</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Mixed signals: Machine Learning Engineer at Haptik (5.7 YOE); JD-aligned skills: pgvector, Weaviate, OpenSearch. Gaps: under half of JD must-have skills covered.</t>
+          <t>Mixed signals: ML Engineer at Infosys (5.3 YOE); JD-aligned skills: pgvector, Sentence Transformers. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>CAND_0005538</t>
+          <t>CAND_0065878</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -1914,24 +1914,24 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>1.0374</t>
+          <t>1.0000</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>0.4072</t>
+          <t>0.2450</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>JD overlap is thin: Senior AI Engineer at Adobe (5.9 YOE); JD-aligned skills: Vector Representations, Python, Information Retrieval Systems. Gaps: 90-day notice period.</t>
+          <t>JD overlap is thin: Senior Data Scientist at Niramai (7.8 YOE); JD-aligned skills: pgvector, Vector Search, Fine-tuning LLMs. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>CAND_0079064</t>
+          <t>CAND_0067866</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -1941,24 +1941,24 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>1.0358</t>
+          <t>1.0000</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>0.2563</t>
+          <t>0.3513</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Moderate fit: Senior Data Scientist at Niramai (5.2 YOE); JD-aligned skills: OpenSearch, NLP, Fine-tuning LLMs. Gaps: 120-day notice period.</t>
+          <t>Moderate fit: Senior Software Engineer (ML) at Tech Mahindra (6.4 YOE); JD-aligned skills: Embeddings, pgvector, Elasticsearch. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>CAND_0015528</t>
+          <t>CAND_0068351</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -1968,24 +1968,24 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>1.0352</t>
+          <t>1.0000</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>0.3246</t>
+          <t>0.4040</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Partial alignment: Applied ML Engineer at Krutrim (7.4 YOE); JD-aligned skills: Weaviate, pgvector, Information Retrieval. Gaps: under half of JD must-have skills covered.</t>
+          <t>Partial alignment: Lead AI Engineer at Sarvam AI (6.4 YOE); JD-aligned skills: pgvector, Qdrant, Elasticsearch. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>CAND_0067866</t>
+          <t>CAND_0068811</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -1995,24 +1995,24 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>1.0323</t>
+          <t>1.0000</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>0.3513</t>
+          <t>0.4651</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Acceptable but not standout: Senior Software Engineer (ML) at Tech Mahindra (6.4 YOE); JD-aligned skills: Embeddings, pgvector, Elasticsearch. Gaps: under half of JD must-have skills covered.</t>
+          <t>Acceptable but not standout: Applied ML Engineer at Freshworks (8.0 YOE); JD-aligned skills: Vector Search, Qdrant, Embeddings. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>CAND_0074735</t>
+          <t>CAND_0069905</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -2022,24 +2022,24 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>1.0312</t>
+          <t>1.0000</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>0.4586</t>
+          <t>0.3358</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Mixed signals: Applied ML Engineer at Rephrase.ai (5.5 YOE); JD-aligned skills: Weaviate, Information Retrieval, Vector Search. Gaps: 90-day notice period.</t>
+          <t>Mixed signals: Applied ML Engineer at Sarvam AI (6.6 YOE); JD-aligned skills: Sentence Transformers, Python, Weaviate. Gaps: 90-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>CAND_0079284</t>
+          <t>CAND_0071974</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -2049,24 +2049,24 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>1.0303</t>
+          <t>1.0000</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>0.2718</t>
+          <t>0.3414</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>JD overlap is thin: Machine Learning Engineer at Google (4.9 YOE); JD-aligned skills: Qdrant, Fine-tuning LLMs, Elasticsearch. Gaps: under half of JD must-have skills covered.</t>
+          <t>JD overlap is thin: Senior AI Engineer at Netflix (7.8 YOE); JD-aligned skills: Weaviate, Pinecone, Information Retrieval. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>CAND_0090584</t>
+          <t>CAND_0074735</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -2076,24 +2076,24 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>1.0302</t>
+          <t>1.0000</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>0.1637</t>
+          <t>0.4586</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Moderate fit: ML Engineer at Flipkart (5.1 YOE); JD-aligned skills: Fine-tuning LLMs, OpenSearch, FAISS. Gaps: 120-day notice period.</t>
+          <t>Moderate fit: Applied ML Engineer at Rephrase.ai (5.5 YOE); JD-aligned skills: Weaviate, Information Retrieval, Vector Search. Gaps: 90-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>CAND_0011432</t>
+          <t>CAND_0075574</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -2103,24 +2103,24 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>1.0296</t>
+          <t>1.0000</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>0.5534</t>
+          <t>0.4170</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Partial alignment: Senior Data Scientist at Amazon (7.6 YOE); JD-aligned skills: OpenSearch, pgvector, Elasticsearch. Gaps: under half of JD must-have skills covered.</t>
+          <t>Partial alignment: Machine Learning Engineer at Haptik (5.7 YOE); JD-aligned skills: pgvector, Weaviate, OpenSearch. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>CAND_0061550</t>
+          <t>CAND_0076482</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -2130,24 +2130,24 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>1.0285</t>
+          <t>1.0000</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>0.3313</t>
+          <t>0.5553</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Acceptable but not standout: ML Engineer at Infosys (5.3 YOE); JD-aligned skills: pgvector, Sentence Transformers. Gaps: under half of JD must-have skills covered.</t>
+          <t>Acceptable but not standout: ML Engineer at Flipkart (6.6 YOE); JD-aligned skills: OpenSearch, Pinecone, pgvector. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>CAND_0011687</t>
+          <t>CAND_0077337</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -2157,24 +2157,24 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>1.0254</t>
+          <t>1.0000</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>0.5094</t>
+          <t>0.4883</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Mixed signals: Senior NLP Engineer at Niramai (7.8 YOE); JD-aligned skills: OpenSearch, FAISS, Embeddings. Gaps: under half of JD must-have skills covered.</t>
+          <t>Mixed signals: Staff Machine Learning Engineer at Paytm (7.0 YOE); JD-aligned skills: pgvector, Pinecone, Information Retrieval. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>CAND_0028793</t>
+          <t>CAND_0078002</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -2184,24 +2184,24 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>1.0230</t>
+          <t>1.0000</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>0.2941</t>
+          <t>0.2974</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>JD overlap is thin: Search Engineer at Google (7.2 YOE); JD-aligned skills: Embeddings, Information Retrieval, pgvector. Gaps: 120-day notice period.</t>
+          <t>JD overlap is thin: Machine Learning Engineer at Meta (6.3 YOE); JD-aligned skills: pgvector, NLP, Weaviate. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>CAND_0048166</t>
+          <t>CAND_0079064</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -2211,24 +2211,24 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>1.0214</t>
+          <t>1.0000</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>0.4054</t>
+          <t>0.2563</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Moderate fit: ML Engineer at Aganitha (5.2 YOE); JD-aligned skills: Pinecone, Milvus, Qdrant. Gaps: under half of JD must-have skills covered.</t>
+          <t>Moderate fit: Senior Data Scientist at Niramai (5.2 YOE); JD-aligned skills: OpenSearch, NLP, Fine-tuning LLMs. Gaps: 120-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>CAND_0093547</t>
+          <t>CAND_0079284</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2238,24 +2238,24 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>1.0188</t>
+          <t>1.0000</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>0.3710</t>
+          <t>0.2718</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Partial alignment: Senior Machine Learning Engineer at PhonePe (2.9 YOE); JD-aligned skills: LLMs, Python, Milvus. Gaps: below typical senior YOE band for this JD.</t>
+          <t>Partial alignment: Machine Learning Engineer at Google (4.9 YOE); JD-aligned skills: Qdrant, Fine-tuning LLMs, Elasticsearch. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>CAND_0076482</t>
+          <t>CAND_0079387</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -2265,24 +2265,24 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>1.0173</t>
+          <t>1.0000</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>0.5553</t>
+          <t>0.4465</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Acceptable but not standout: ML Engineer at Flipkart (6.6 YOE); JD-aligned skills: OpenSearch, Pinecone, pgvector. Gaps: under half of JD must-have skills covered.</t>
+          <t>Acceptable but not standout: AI Engineer at Microsoft (6.9 YOE); JD-aligned skills: Python, Sentence Transformers, Vector Search. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>CAND_0040178</t>
+          <t>CAND_0080766</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -2292,24 +2292,24 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>1.0161</t>
+          <t>1.0000</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>0.3303</t>
+          <t>0.4625</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Mixed signals: ML Engineer at Meesho (5.0 YOE); JD-aligned skills: Weaviate, Fine-tuning LLMs, Vector Search. Gaps: under half of JD must-have skills covered.</t>
+          <t>Mixed signals: Staff Machine Learning Engineer at Salesforce (8.8 YOE); JD-aligned skills: Information Retrieval Systems, Elasticsearch, Natural Language Processing. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>CAND_0060054</t>
+          <t>CAND_0081846</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -2319,24 +2319,24 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>1.0155</t>
+          <t>1.0000</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>0.3416</t>
+          <t>0.4803</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>JD overlap is thin: AI Engineer at Mad Street Den (6.4 YOE); JD-aligned skills: Weaviate, FAISS, Elasticsearch. Gaps: under half of JD must-have skills covered.</t>
+          <t>JD overlap is thin: Lead AI Engineer at Razorpay (6.7 YOE); JD-aligned skills: Information Retrieval, pgvector, Elasticsearch. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>CAND_0024878</t>
+          <t>CAND_0081852</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -2346,24 +2346,24 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>1.0126</t>
+          <t>1.0000</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>0.4462</t>
+          <t>0.2331</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Moderate fit: AI Specialist at HCL (5.7 YOE); JD-aligned skills: pgvector, Elasticsearch, NLP. Gaps: under half of JD must-have skills covered.</t>
+          <t>Moderate fit: Senior Data Scientist at Mad Street Den (5.9 YOE); JD-aligned skills: Milvus, pgvector, Weaviate. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>CAND_0008425</t>
+          <t>CAND_0083879</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -2373,24 +2373,24 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>1.0111</t>
+          <t>1.0000</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>0.2436</t>
+          <t>0.5950</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Partial alignment: Senior NLP Engineer at Ola (7.8 YOE); JD-aligned skills: Qdrant, pgvector, Sentence Transformers. Gaps: 90-day notice period.</t>
+          <t>Partial alignment: Machine Learning Engineer at Ola (7.1 YOE); JD-aligned skills: Fine-tuning LLMs, Milvus, Sentence Transformers. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>CAND_0036121</t>
+          <t>CAND_0086022</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -2400,24 +2400,24 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>1.0109</t>
+          <t>1.0000</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>0.3242</t>
+          <t>0.3683</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Acceptable but not standout: ML Engineer at Wysa (5.2 YOE); JD-aligned skills: Embeddings, Vector Search, Information Retrieval. Gaps: under half of JD must-have skills covered.</t>
+          <t>Acceptable but not standout: Senior Applied Scientist at Sarvam AI (5.3 YOE); JD-aligned skills: Vector Search, pgvector, Fine-tuning LLMs. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>CAND_0027691</t>
+          <t>CAND_0087630</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -2427,24 +2427,24 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>1.0104</t>
+          <t>1.0000</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>0.4306</t>
+          <t>0.3940</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Mixed signals: NLP Engineer at Haptik (6.5 YOE); JD-aligned skills: Weaviate, Embeddings, Python. Gaps: under half of JD must-have skills covered.</t>
+          <t>Mixed signals: AI Engineer at Vedantu (7.2 YOE); JD-aligned skills: Elasticsearch, pgvector, NLP. Gaps: not flagged open to work.</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>CAND_0037980</t>
+          <t>CAND_0088025</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -2454,24 +2454,24 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>1.0099</t>
+          <t>1.0000</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>0.7550</t>
+          <t>0.5411</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>JD overlap is thin: Senior Applied Scientist at Niramai (9.0 YOE); JD-aligned skills: NLP, Text Encoders, pgvector. Gaps: under half of JD must-have skills covered.</t>
+          <t>JD overlap is thin: Staff Machine Learning Engineer at Yellow.ai (8.6 YOE); JD-aligned skills: Pinecone, LLMs, Elasticsearch. Gaps: 90-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>CAND_0096104</t>
+          <t>CAND_0090584</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -2481,24 +2481,24 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>1.0086</t>
+          <t>1.0000</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>0.5401</t>
+          <t>0.1637</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Moderate fit: AI Specialist at Yellow.ai (7.0 YOE); JD-aligned skills: Pinecone. Gaps: only 1 core JD skill matched.</t>
+          <t>Moderate fit: ML Engineer at Flipkart (5.1 YOE); JD-aligned skills: Fine-tuning LLMs, OpenSearch, FAISS. Gaps: 120-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>CAND_0001819</t>
+          <t>CAND_0093193</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -2508,24 +2508,24 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>1.0074</t>
+          <t>1.0000</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>0.3603</t>
+          <t>0.4352</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Partial alignment: ML Engineer at Genpact AI (4.4 YOE); JD-aligned skills: Weaviate, pgvector, NLP. Gaps: under half of JD must-have skills covered.</t>
+          <t>Partial alignment: Senior Machine Learning Engineer at Niramai (7.9 YOE); JD-aligned skills: Text Encoders, Vector Representations, Qdrant. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>CAND_0052328</t>
+          <t>CAND_0093547</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -2535,24 +2535,24 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>1.0063</t>
+          <t>1.0000</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>0.5090</t>
+          <t>0.3710</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Acceptable but not standout: Recommendation Systems Engineer at Amazon (6.5 YOE); JD-aligned skills: OpenSearch, Fine-tuning LLMs, Vector Search. Gaps: under half of JD must-have skills covered.</t>
+          <t>Acceptable but not standout: Senior Machine Learning Engineer at PhonePe (2.9 YOE); JD-aligned skills: LLMs, Python, Milvus. Gaps: below typical senior YOE band for this JD; not flagged open to work.</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>CAND_0030348</t>
+          <t>CAND_0093912</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -2562,24 +2562,24 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>1.0047</t>
+          <t>1.0000</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>0.3735</t>
+          <t>0.4763</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Mixed signals: Machine Learning Engineer at BYJU'S (4.5 YOE); JD-aligned skills: Embeddings, Vector Search, Elasticsearch. Gaps: under half of JD must-have skills covered.</t>
+          <t>Mixed signals: Senior Data Scientist at Razorpay (5.3 YOE); JD-aligned skills: Milvus, Embeddings, Vector Search. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>CAND_0009691</t>
+          <t>CAND_0096104</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -2589,24 +2589,24 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>1.0023</t>
+          <t>1.0000</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>0.1214</t>
+          <t>0.5401</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>JD overlap is thin: Applied ML Engineer at LinkedIn (6.2 YOE); JD-aligned skills: Fine-tuning LLMs, Pinecone, Sentence Transformers. Gaps: 120-day notice period.</t>
+          <t>JD overlap is thin: AI Specialist at Yellow.ai (7.0 YOE); JD-aligned skills: Pinecone. Gaps: only 1 core JD skill matched.</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>CAND_0019288</t>
+          <t>CAND_0096142</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -2616,24 +2616,24 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>1.0018</t>
+          <t>1.0000</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>0.3846</t>
+          <t>0.2486</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Moderate fit: AI Research Engineer at Paytm (5.7 YOE); JD-aligned skills: pgvector, FAISS, OpenSearch. Gaps: under half of JD must-have skills covered.</t>
+          <t>Moderate fit: Applied ML Engineer at upGrad (5.0 YOE); JD-aligned skills: Weaviate, Pinecone, Python. Gaps: 120-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>CAND_0002793</t>
+          <t>CAND_0099806</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -2643,17 +2643,17 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>1.0014</t>
+          <t>1.0000</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>0.3997</t>
+          <t>0.3301</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Partial alignment: AI Specialist at Meesho (5.5 YOE); JD-aligned skills: pgvector, Information Retrieval, FAISS. Gaps: not flagged open to work.</t>
+          <t>Partial alignment: AI Engineer at Mad Street Den (4.6 YOE); JD-aligned skills: pgvector, FAISS, Embeddings. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: industry-aware trajectory scoring (ADR-020)
Ship Fix 1 only: PRODUCT/SERVICES industry ratio in trajectory_scorer moves rank 1 to CAND_0018499 (Zomato). NDCG@10 0.3980, Recovery 3/4.

Fix 2 (duration-weighted embed) and Fix 3 (aspiration penalty) evaluated on full 100K and reverted due to NDCG regression.

Docs synced: README, methodology, walkthrough, runbook, ADR-020, CHANGELOG, metadata.
</commit_message>
<xml_diff>
--- a/submission.xlsx
+++ b/submission.xlsx
@@ -446,23 +446,27 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>CAND_0046525</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C2" t="n">
-        <v>1</v>
+          <t>CAND_0068351</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>1.0000</t>
+        </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>0.3574</t>
+          <t>0.4040</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Rank 1: Senior Machine Learning Engineer at Genpact AI (6.1 YOE); JD-aligned skills: Elasticsearch, Information Retrieval, LLMs. Top-tier composite score across career, skills, and availability. Counterfactual: ranks on career trajectory and assessed depth over keyword coverage (7/20 listed must-haves), aligning with the JD anti-keyword-stuffing guidance. Join probability: 36%.</t>
+          <t>Rank 1: Lead AI Engineer at Sarvam AI (6.4 YOE); JD-aligned skills: pgvector, Qdrant, Elasticsearch. Top-tier composite score across career, skills, and availability. Counterfactual: ranks on career trajectory and assessed depth over keyword coverage (7/20 listed must-haves), aligning with the JD anti-keyword-stuffing guidance. Join probability: 40%.</t>
         </is>
       </c>
     </row>
@@ -472,11 +476,15 @@
           <t>CAND_0018499</t>
         </is>
       </c>
-      <c r="B3" t="n">
-        <v>2</v>
-      </c>
-      <c r="C3" t="n">
-        <v>0.9999</v>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>0.9999</t>
+        </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -492,345 +500,405 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>CAND_0088025</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>3</v>
-      </c>
-      <c r="C4" t="n">
-        <v>0.9998</v>
+          <t>CAND_0071974</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>0.9998</t>
+        </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>0.5411</t>
+          <t>0.3414</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Rank 3: Staff Machine Learning Engineer at Yellow.ai (8.6 YOE); JD-aligned skills: Pinecone, LLMs, Elasticsearch. Top-tier composite score across career, skills, and availability. Minor note: 90-day notice period. Join probability: 54%.</t>
+          <t>Rank 3: Senior AI Engineer at Netflix (7.8 YOE); JD-aligned skills: Weaviate, Pinecone, Information Retrieval. Top-tier composite score across career, skills, and availability. Counterfactual: ranks on career trajectory and assessed depth over keyword coverage (7/20 listed must-haves), aligning with the JD anti-keyword-stuffing guidance. Join probability: 34%; low engagement signals.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>CAND_0002025</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>4</v>
-      </c>
-      <c r="C5" t="n">
-        <v>0.9997</v>
+          <t>CAND_0088025</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>0.9997</t>
+        </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>0.3912</t>
+          <t>0.5411</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Rank 4: Senior AI Engineer at Apple (5.9 YOE); JD-aligned skills: FAISS, OpenSearch, Weaviate. Top-tier composite score across career, skills, and availability. Counterfactual: ranks on career trajectory and assessed depth over keyword coverage (8/20 listed must-haves), aligning with the JD anti-keyword-stuffing guidance. Join probability: 39%.</t>
+          <t>Rank 4: Staff Machine Learning Engineer at Yellow.ai (8.6 YOE); JD-aligned skills: Pinecone, LLMs, Elasticsearch. Top-tier composite score across career, skills, and availability. Minor note: 90-day notice period. Join probability: 54%.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CAND_0081846</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>5</v>
-      </c>
-      <c r="C6" t="n">
-        <v>0.9996</v>
+          <t>CAND_0080766</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>0.9996</t>
+        </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>0.4803</t>
+          <t>0.4625</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Rank 5: Lead AI Engineer at Razorpay (6.7 YOE); JD-aligned skills: Information Retrieval, pgvector, Elasticsearch. Top-tier composite score across career, skills, and availability. Counterfactual: ranks on career trajectory and assessed depth over keyword coverage (7/20 listed must-haves), aligning with the JD anti-keyword-stuffing guidance. Join probability: 48%.</t>
+          <t>Rank 5: Staff Machine Learning Engineer at Salesforce (8.8 YOE); JD-aligned skills: Information Retrieval Systems, Elasticsearch, Natural Language Processing. Top-tier composite score across career, skills, and availability. Counterfactual: ranks on career trajectory and assessed depth over keyword coverage (6/20 listed must-haves), aligning with the JD anti-keyword-stuffing guidance. Join probability: 46%.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>CAND_0071974</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>6</v>
-      </c>
-      <c r="C7" t="n">
-        <v>0.9995000000000001</v>
+          <t>CAND_0077337</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>0.9995</t>
+        </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>0.3414</t>
+          <t>0.4883</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Strong match — Senior AI Engineer at Netflix (7.8 YOE); JD-aligned skills: Weaviate, Pinecone, Information Retrieval. Join probability: 34%; low engagement signals.</t>
+          <t>Strong match — Staff Machine Learning Engineer at Paytm (7.0 YOE); JD-aligned skills: pgvector, Pinecone, Information Retrieval. Join probability: 49%.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>CAND_0055905</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>7</v>
-      </c>
-      <c r="C8" t="n">
-        <v>0.9994</v>
+          <t>CAND_0018094</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>0.9994</t>
+        </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>0.6870</t>
+          <t>0.4428</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Strong match — Senior Machine Learning Engineer at Flipkart (8.1 YOE); JD-aligned skills: Elasticsearch, Python, LLMs. Join probability: 69%.</t>
+          <t>Strong match — ML Engineer at Mad Street Den (5.2 YOE); JD-aligned skills: Pinecone, Information Retrieval, Fine-tuning LLMs. Join probability: 44%.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>CAND_0077337</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>8</v>
-      </c>
-      <c r="C9" t="n">
-        <v>0.9993</v>
+          <t>CAND_0096142</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>0.9993</t>
+        </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>0.4883</t>
+          <t>0.2486</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Strong match — Staff Machine Learning Engineer at Paytm (7.0 YOE); JD-aligned skills: pgvector, Pinecone, Information Retrieval. Join probability: 49%.</t>
+          <t>Strong match — Applied ML Engineer at upGrad (5.0 YOE); JD-aligned skills: Weaviate, Pinecone, Python. Watch: 120-day notice period. Join probability: 25%; long notice.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>CAND_0050454</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
-        <v>9</v>
-      </c>
-      <c r="C10" t="n">
-        <v>0.9992</v>
+          <t>CAND_0081846</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>0.9992</t>
+        </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>0.3504</t>
+          <t>0.4803</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Strong match — AI Engineer at Rephrase.ai (6.8 YOE); JD-aligned skills: Fine-tuning LLMs, FAISS, Qdrant. Join probability: 35%.</t>
+          <t>Strong match — Lead AI Engineer at Razorpay (6.7 YOE); JD-aligned skills: Information Retrieval, pgvector, Elasticsearch. Join probability: 48%.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>CAND_0006567</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
-        <v>10</v>
-      </c>
-      <c r="C11" t="n">
-        <v>0.9991</v>
+          <t>CAND_0038368</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>0.9991</t>
+        </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>0.6079</t>
+          <t>0.4347</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Strong match — Senior AI Engineer at Meta (7.9 YOE); JD-aligned skills: Vector Representations, NLP, Python. Join probability: 61%.</t>
+          <t>Strong match — ML Engineer at PhonePe (5.4 YOE); JD-aligned skills: Embeddings, FAISS, NLP. Join probability: 43%.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>CAND_0044222</t>
-        </is>
-      </c>
-      <c r="B12" t="n">
-        <v>11</v>
-      </c>
-      <c r="C12" t="n">
-        <v>0.999</v>
+          <t>CAND_0039383</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>0.9990</t>
+        </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>0.2252</t>
+          <t>0.5155</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Strong match — AI Engineer at PolicyBazaar (7.7 YOE); JD-aligned skills: Vector Search, OpenSearch, Qdrant. Join probability: 23%; low engagement signals.</t>
+          <t>Strong match — Applied ML Engineer at Meesho (7.1 YOE); JD-aligned skills: FAISS, NLP, Vector Search. Watch: 90-day notice period. Join probability: 52%.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>CAND_0083879</t>
-        </is>
-      </c>
-      <c r="B13" t="n">
-        <v>12</v>
-      </c>
-      <c r="C13" t="n">
-        <v>0.9989</v>
+          <t>CAND_0044222</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>0.9989</t>
+        </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>0.5950</t>
+          <t>0.2252</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Strong match — Machine Learning Engineer at Ola (7.1 YOE); JD-aligned skills: Fine-tuning LLMs, Milvus, Sentence Transformers. Join probability: 60%.</t>
+          <t>Strong match — AI Engineer at PolicyBazaar (7.7 YOE); JD-aligned skills: Vector Search, OpenSearch, Qdrant. Join probability: 23%; low engagement signals.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>CAND_0049538</t>
-        </is>
-      </c>
-      <c r="B14" t="n">
-        <v>13</v>
-      </c>
-      <c r="C14" t="n">
-        <v>0.9988</v>
+          <t>CAND_0010149</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>0.9988</t>
+        </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>0.3362</t>
+          <t>0.2385</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Strong match — Applied ML Engineer at Saarthi.ai (5.8 YOE); JD-aligned skills: OpenSearch, Vector Search, Milvus. Join probability: 34%; low engagement signals.</t>
+          <t>Strong match — ML Engineer at Glance (6.9 YOE); JD-aligned skills: Milvus, Vector Search, Elasticsearch. Watch: 90-day notice period. Join probability: 24%; low engagement signals.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>CAND_0086022</t>
-        </is>
-      </c>
-      <c r="B15" t="n">
-        <v>14</v>
-      </c>
-      <c r="C15" t="n">
-        <v>0.9987</v>
+          <t>CAND_0002025</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>0.9987</t>
+        </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>0.3683</t>
+          <t>0.3912</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Strong match — Senior Applied Scientist at Sarvam AI (5.3 YOE); JD-aligned skills: Vector Search, pgvector, Fine-tuning LLMs. Join probability: 37%.</t>
+          <t>Strong match — Senior AI Engineer at Apple (5.9 YOE); JD-aligned skills: FAISS, OpenSearch, Weaviate. Join probability: 39%.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>CAND_0016163</t>
-        </is>
-      </c>
-      <c r="B16" t="n">
-        <v>15</v>
-      </c>
-      <c r="C16" t="n">
-        <v>0.9986</v>
+          <t>CAND_0030031</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>0.9986</t>
+        </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>0.2905</t>
+          <t>0.3445</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Strong match — Applied ML Engineer at Dream11 (6.7 YOE); JD-aligned skills: Weaviate, Embeddings, pgvector. Watch: 120-day notice period. Join probability: 29%; long notice.</t>
+          <t>Strong match — AI Engineer at Microsoft (5.7 YOE); JD-aligned skills: Information Retrieval, Python, NLP. Join probability: 34%; low engagement signals.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>CAND_0068351</t>
-        </is>
-      </c>
-      <c r="B17" t="n">
-        <v>16</v>
-      </c>
-      <c r="C17" t="n">
-        <v>0.9985000000000001</v>
+          <t>CAND_0006567</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>0.9985</t>
+        </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>0.4040</t>
+          <t>0.6079</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Strong match — Lead AI Engineer at Sarvam AI (6.4 YOE); JD-aligned skills: pgvector, Qdrant, Elasticsearch. Join probability: 40%.</t>
+          <t>Strong match — Senior AI Engineer at Meta (7.9 YOE); JD-aligned skills: Vector Representations, NLP, Python. Join probability: 61%.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>CAND_0005649</t>
-        </is>
-      </c>
-      <c r="B18" t="n">
-        <v>17</v>
-      </c>
-      <c r="C18" t="n">
-        <v>0.9984</v>
+          <t>CAND_0083879</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>0.9984</t>
+        </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>0.5162</t>
+          <t>0.5950</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Strong match — Senior Data Scientist at Sarvam AI (7.4 YOE); JD-aligned skills: Fine-tuning LLMs, Weaviate, Information Retrieval. Watch: 90-day notice period. Join probability: 52%.</t>
+          <t>Strong match — Machine Learning Engineer at Ola (7.1 YOE); JD-aligned skills: Fine-tuning LLMs, Milvus, Sentence Transformers. Join probability: 60%.</t>
         </is>
       </c>
     </row>
@@ -840,11 +908,15 @@
           <t>CAND_0087630</t>
         </is>
       </c>
-      <c r="B19" t="n">
-        <v>18</v>
-      </c>
-      <c r="C19" t="n">
-        <v>0.9983</v>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>0.9983</t>
+        </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
@@ -860,920 +932,1080 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>CAND_0018094</t>
-        </is>
-      </c>
-      <c r="B20" t="n">
-        <v>19</v>
-      </c>
-      <c r="C20" t="n">
-        <v>0.9982</v>
+          <t>CAND_0020877</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>0.9982</t>
+        </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>0.4428</t>
+          <t>0.3909</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Strong match — ML Engineer at Mad Street Den (5.2 YOE); JD-aligned skills: Pinecone, Information Retrieval, Fine-tuning LLMs. Join probability: 44%.</t>
+          <t>Strong match — Applied ML Engineer at CRED (5.1 YOE); JD-aligned skills: Elasticsearch, OpenSearch, Information Retrieval. Join probability: 39%.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>CAND_0030031</t>
-        </is>
-      </c>
-      <c r="B21" t="n">
-        <v>20</v>
-      </c>
-      <c r="C21" t="n">
-        <v>0.9981</v>
+          <t>CAND_0049538</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>0.9981</t>
+        </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>0.3445</t>
+          <t>0.3362</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Strong match — AI Engineer at Microsoft (5.7 YOE); JD-aligned skills: Information Retrieval, Python, NLP. Join probability: 34%; low engagement signals.</t>
+          <t>Strong match — Applied ML Engineer at Saarthi.ai (5.8 YOE); JD-aligned skills: OpenSearch, Vector Search, Milvus. Join probability: 34%; low engagement signals.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>CAND_0081852</t>
-        </is>
-      </c>
-      <c r="B22" t="n">
-        <v>21</v>
-      </c>
-      <c r="C22" t="n">
-        <v>0.998</v>
+          <t>CAND_0098217</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>0.9980</t>
+        </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>0.2331</t>
+          <t>0.5342</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Solid profile: Senior Data Scientist at Mad Street Den (5.9 YOE); JD-aligned skills: Milvus, pgvector, Weaviate.</t>
+          <t>Solid profile: ML Engineer at Glance (6.4 YOE); JD-aligned skills: FAISS, Pinecone.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>CAND_0039383</t>
-        </is>
-      </c>
-      <c r="B23" t="n">
-        <v>22</v>
-      </c>
-      <c r="C23" t="n">
-        <v>0.9979</v>
+          <t>CAND_0047721</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>0.9979</t>
+        </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>0.5155</t>
+          <t>0.1736</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Good fit with caveats: Applied ML Engineer at Meesho (7.1 YOE); JD-aligned skills: FAISS, NLP, Vector Search. Concerns: 90-day notice period.</t>
+          <t>Good fit with caveats: Senior Data Scientist at Microsoft (7.0 YOE); JD-aligned skills: Milvus, Information Retrieval, FAISS. Concerns: 90-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>CAND_0058688</t>
-        </is>
-      </c>
-      <c r="B24" t="n">
-        <v>23</v>
-      </c>
-      <c r="C24" t="n">
-        <v>0.9978</v>
+          <t>CAND_0005649</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>0.9978</t>
+        </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>0.7268</t>
+          <t>0.5162</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Competitive candidate: AI Engineer at Vedantu (6.7 YOE); JD-aligned skills: Embeddings, Information Retrieval, Milvus.</t>
+          <t>Competitive candidate: Senior Data Scientist at Sarvam AI (7.4 YOE); JD-aligned skills: Fine-tuning LLMs, Weaviate, Information Retrieval. Concerns: 90-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>CAND_0020877</t>
-        </is>
-      </c>
-      <c r="B25" t="n">
-        <v>24</v>
-      </c>
-      <c r="C25" t="n">
-        <v>0.9977</v>
+          <t>CAND_0061550</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>0.9977</t>
+        </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>0.3909</t>
+          <t>0.3313</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Meets several JD signals: Applied ML Engineer at CRED (5.1 YOE); JD-aligned skills: Elasticsearch, OpenSearch, Information Retrieval.</t>
+          <t>Meets several JD signals: ML Engineer at Infosys (5.3 YOE); JD-aligned skills: pgvector, Sentence Transformers.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>CAND_0020350</t>
-        </is>
-      </c>
-      <c r="B26" t="n">
-        <v>25</v>
-      </c>
-      <c r="C26" t="n">
-        <v>0.9976</v>
+          <t>CAND_0061257</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>0.9976</t>
+        </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>0.3210</t>
+          <t>0.3969</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Solid profile: AI Engineer at Zoho (5.8 YOE); JD-aligned skills: NLP, LLMs, FAISS.</t>
+          <t>Solid profile: Staff Machine Learning Engineer at LinkedIn (8.0 YOE); JD-aligned skills: Information Retrieval Systems, Python, Vector Representations.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>CAND_0042029</t>
-        </is>
-      </c>
-      <c r="B27" t="n">
-        <v>26</v>
-      </c>
-      <c r="C27" t="n">
-        <v>0.9975000000000001</v>
+          <t>CAND_0078002</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>0.9975</t>
+        </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>0.4840</t>
+          <t>0.2974</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Good fit with caveats: Senior Data Scientist at Flipkart (6.5 YOE); JD-aligned skills: NLP, Elasticsearch, Embeddings.</t>
+          <t>Good fit with caveats: Machine Learning Engineer at Meta (6.3 YOE); JD-aligned skills: pgvector, NLP, Weaviate.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>CAND_0044855</t>
-        </is>
-      </c>
-      <c r="B28" t="n">
-        <v>27</v>
-      </c>
-      <c r="C28" t="n">
-        <v>0.9974</v>
+          <t>CAND_0050454</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>0.9974</t>
+        </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>0.3723</t>
+          <t>0.3504</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Competitive candidate: Senior Data Scientist at Flipkart (6.6 YOE); JD-aligned skills: OpenSearch, Information Retrieval, Pinecone.</t>
+          <t>Competitive candidate: AI Engineer at Rephrase.ai (6.8 YOE); JD-aligned skills: Fine-tuning LLMs, FAISS, Qdrant.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>CAND_0046064</t>
-        </is>
-      </c>
-      <c r="B29" t="n">
-        <v>28</v>
-      </c>
-      <c r="C29" t="n">
-        <v>0.9973</v>
+          <t>CAND_0044855</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>0.9973</t>
+        </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>0.3780</t>
+          <t>0.3723</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Meets several JD signals: Senior NLP Engineer at Salesforce (8.9 YOE); JD-aligned skills: Python, Pinecone, OpenSearch.</t>
+          <t>Meets several JD signals: Senior Data Scientist at Flipkart (6.6 YOE); JD-aligned skills: OpenSearch, Information Retrieval, Pinecone.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>CAND_0079387</t>
-        </is>
-      </c>
-      <c r="B30" t="n">
-        <v>29</v>
-      </c>
-      <c r="C30" t="n">
-        <v>0.9972</v>
+          <t>CAND_0055905</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>0.9972</t>
+        </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>0.4465</t>
+          <t>0.6870</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Solid profile: AI Engineer at Microsoft (6.9 YOE); JD-aligned skills: Python, Sentence Transformers, Vector Search.</t>
+          <t>Solid profile: Senior Machine Learning Engineer at Flipkart (8.1 YOE); JD-aligned skills: Elasticsearch, Python, LLMs.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>CAND_0080766</t>
-        </is>
-      </c>
-      <c r="B31" t="n">
-        <v>30</v>
-      </c>
-      <c r="C31" t="n">
-        <v>0.9971</v>
+          <t>CAND_0043228</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>0.9971</t>
+        </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>0.4625</t>
+          <t>0.3534</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Good fit with caveats: Staff Machine Learning Engineer at Salesforce (8.8 YOE); JD-aligned skills: Information Retrieval Systems, Elasticsearch, Natural Language Processing.</t>
+          <t>Good fit with caveats: Applied ML Engineer at Zoho (6.8 YOE); JD-aligned skills: NLP, Vector Search, Sentence Transformers.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>CAND_0061257</t>
-        </is>
-      </c>
-      <c r="B32" t="n">
-        <v>31</v>
-      </c>
-      <c r="C32" t="n">
-        <v>0.997</v>
+          <t>CAND_0042029</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>0.9970</t>
+        </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>0.3969</t>
+          <t>0.4840</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Competitive candidate: Staff Machine Learning Engineer at LinkedIn (8.0 YOE); JD-aligned skills: Information Retrieval Systems, Python, Vector Representations.</t>
+          <t>Competitive candidate: Senior Data Scientist at Flipkart (6.5 YOE); JD-aligned skills: NLP, Elasticsearch, Embeddings.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>CAND_0043228</t>
-        </is>
-      </c>
-      <c r="B33" t="n">
-        <v>32</v>
-      </c>
-      <c r="C33" t="n">
-        <v>0.9969</v>
+          <t>CAND_0079387</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>0.9969</t>
+        </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>0.3534</t>
+          <t>0.4465</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Meets several JD signals: Applied ML Engineer at Zoho (6.8 YOE); JD-aligned skills: NLP, Vector Search, Sentence Transformers.</t>
+          <t>Meets several JD signals: AI Engineer at Microsoft (6.9 YOE); JD-aligned skills: Python, Sentence Transformers, Vector Search.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>CAND_0093193</t>
-        </is>
-      </c>
-      <c r="B34" t="n">
-        <v>33</v>
-      </c>
-      <c r="C34" t="n">
-        <v>0.9968</v>
+          <t>CAND_0032216</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>0.9968</t>
+        </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>0.4352</t>
+          <t>0.2743</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Solid profile: Senior Machine Learning Engineer at Niramai (7.9 YOE); JD-aligned skills: Text Encoders, Vector Representations, Qdrant.</t>
+          <t>Solid profile: ML Engineer at upGrad (6.1 YOE); JD-aligned skills: Information Retrieval, Qdrant, Sentence Transformers.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>CAND_0045250</t>
-        </is>
-      </c>
-      <c r="B35" t="n">
-        <v>34</v>
-      </c>
-      <c r="C35" t="n">
-        <v>0.9967</v>
+          <t>CAND_0037566</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>0.9967</t>
+        </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>0.3580</t>
+          <t>0.5752</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Good fit with caveats: Applied ML Engineer at Rephrase.ai (6.6 YOE); JD-aligned skills: Sentence Transformers, Milvus, Embeddings.</t>
+          <t>Good fit with caveats: Machine Learning Engineer at LinkedIn (6.9 YOE); JD-aligned skills: Pinecone, NLP, LLMs.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>CAND_0003841</t>
-        </is>
-      </c>
-      <c r="B36" t="n">
-        <v>35</v>
-      </c>
-      <c r="C36" t="n">
-        <v>0.9966</v>
+          <t>CAND_0016163</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>0.9966</t>
+        </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>0.3402</t>
+          <t>0.2905</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Competitive candidate: ML Engineer at Tech Mahindra (5.0 YOE); JD-aligned skills: Pinecone, Fine-tuning LLMs, Sentence Transformers.</t>
+          <t>Competitive candidate: Applied ML Engineer at Dream11 (6.7 YOE); JD-aligned skills: Weaviate, Embeddings, pgvector. Concerns: 120-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>CAND_0047721</t>
-        </is>
-      </c>
-      <c r="B37" t="n">
-        <v>36</v>
-      </c>
-      <c r="C37" t="n">
-        <v>0.9965000000000001</v>
+          <t>CAND_0042100</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>0.9965</t>
+        </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>0.1736</t>
+          <t>0.2536</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Meets several JD signals: Senior Data Scientist at Microsoft (7.0 YOE); JD-aligned skills: Milvus, Information Retrieval, FAISS. Concerns: 90-day notice period.</t>
+          <t>Meets several JD signals: Machine Learning Engineer at Freshworks (7.3 YOE); JD-aligned skills: Elasticsearch, Fine-tuning LLMs, Pinecone. Concerns: 90-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>CAND_0096142</t>
-        </is>
-      </c>
-      <c r="B38" t="n">
-        <v>37</v>
-      </c>
-      <c r="C38" t="n">
-        <v>0.9964</v>
+          <t>CAND_0090584</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>37</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>0.9964</t>
+        </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>0.2486</t>
+          <t>0.1637</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Solid profile: Applied ML Engineer at upGrad (5.0 YOE); JD-aligned skills: Weaviate, Pinecone, Python. Concerns: 120-day notice period.</t>
+          <t>Solid profile: ML Engineer at Flipkart (5.1 YOE); JD-aligned skills: Fine-tuning LLMs, OpenSearch, FAISS. Concerns: 120-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>CAND_0042100</t>
-        </is>
-      </c>
-      <c r="B39" t="n">
-        <v>38</v>
-      </c>
-      <c r="C39" t="n">
-        <v>0.9963</v>
+          <t>CAND_0081852</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>0.9963</t>
+        </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>0.2536</t>
+          <t>0.2331</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Good fit with caveats: Machine Learning Engineer at Freshworks (7.3 YOE); JD-aligned skills: Elasticsearch, Fine-tuning LLMs, Pinecone. Concerns: 90-day notice period.</t>
+          <t>Good fit with caveats: Senior Data Scientist at Mad Street Den (5.9 YOE); JD-aligned skills: Milvus, pgvector, Weaviate.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>CAND_0051292</t>
-        </is>
-      </c>
-      <c r="B40" t="n">
-        <v>39</v>
-      </c>
-      <c r="C40" t="n">
-        <v>0.9962</v>
+          <t>CAND_0045250</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>0.9962</t>
+        </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>0.4013</t>
+          <t>0.3580</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Competitive candidate: Applied ML Engineer at Freshworks (5.2 YOE); JD-aligned skills: pgvector, FAISS, LLMs.</t>
+          <t>Competitive candidate: Applied ML Engineer at Rephrase.ai (6.6 YOE); JD-aligned skills: Sentence Transformers, Milvus, Embeddings.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>CAND_0037566</t>
-        </is>
-      </c>
-      <c r="B41" t="n">
-        <v>40</v>
-      </c>
-      <c r="C41" t="n">
-        <v>0.9961</v>
+          <t>CAND_0093193</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>0.9961</t>
+        </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>0.5752</t>
+          <t>0.4352</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Meets several JD signals: Machine Learning Engineer at LinkedIn (6.9 YOE); JD-aligned skills: Pinecone, NLP, LLMs.</t>
+          <t>Meets several JD signals: Senior Machine Learning Engineer at Niramai (7.9 YOE); JD-aligned skills: Text Encoders, Vector Representations, Qdrant.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>CAND_0051004</t>
-        </is>
-      </c>
-      <c r="B42" t="n">
-        <v>41</v>
-      </c>
-      <c r="C42" t="n">
-        <v>0.996</v>
+          <t>CAND_0051292</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>41</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>0.9960</t>
+        </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>0.5405</t>
+          <t>0.4013</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Solid profile: Senior Data Scientist at CRED (4.7 YOE); JD-aligned skills: Embeddings, Qdrant, Fine-tuning LLMs.</t>
+          <t>Solid profile: Applied ML Engineer at Freshworks (5.2 YOE); JD-aligned skills: pgvector, FAISS, LLMs.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>CAND_0069905</t>
-        </is>
-      </c>
-      <c r="B43" t="n">
-        <v>42</v>
-      </c>
-      <c r="C43" t="n">
-        <v>0.9959</v>
+          <t>CAND_0076482</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>0.9959</t>
+        </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>0.3358</t>
+          <t>0.5553</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Good fit with caveats: Applied ML Engineer at Sarvam AI (6.6 YOE); JD-aligned skills: Sentence Transformers, Python, Weaviate. Concerns: 90-day notice period.</t>
+          <t>Good fit with caveats: ML Engineer at Flipkart (6.6 YOE); JD-aligned skills: OpenSearch, Pinecone, pgvector.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>CAND_0055992</t>
-        </is>
-      </c>
-      <c r="B44" t="n">
-        <v>43</v>
-      </c>
-      <c r="C44" t="n">
-        <v>0.9958</v>
+          <t>CAND_0079284</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>43</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>0.9958</t>
+        </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>0.5850</t>
+          <t>0.2718</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Competitive candidate: AI Engineer at CRED (16.9 YOE); JD-aligned skills: Information Retrieval, FAISS, OpenSearch.</t>
+          <t>Competitive candidate: Machine Learning Engineer at Google (4.9 YOE); JD-aligned skills: Qdrant, Fine-tuning LLMs, Elasticsearch.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>CAND_0068811</t>
-        </is>
-      </c>
-      <c r="B45" t="n">
-        <v>44</v>
-      </c>
-      <c r="C45" t="n">
-        <v>0.9957</v>
+          <t>CAND_0058688</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>0.9957</t>
+        </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>0.4651</t>
+          <t>0.7268</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Meets several JD signals: Applied ML Engineer at Freshworks (8.0 YOE); JD-aligned skills: Vector Search, Qdrant, Embeddings.</t>
+          <t>Meets several JD signals: AI Engineer at Vedantu (6.7 YOE); JD-aligned skills: Embeddings, Information Retrieval, Milvus.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>CAND_0093912</t>
-        </is>
-      </c>
-      <c r="B46" t="n">
-        <v>45</v>
-      </c>
-      <c r="C46" t="n">
-        <v>0.9956</v>
+          <t>CAND_0020350</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>0.9956</t>
+        </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>0.4763</t>
+          <t>0.3210</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Solid profile: Senior Data Scientist at Razorpay (5.3 YOE); JD-aligned skills: Milvus, Embeddings, Vector Search.</t>
+          <t>Solid profile: AI Engineer at Zoho (5.8 YOE); JD-aligned skills: NLP, LLMs, FAISS.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>CAND_0099806</t>
-        </is>
-      </c>
-      <c r="B47" t="n">
-        <v>46</v>
-      </c>
-      <c r="C47" t="n">
-        <v>0.9955000000000001</v>
+          <t>CAND_0068811</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>46</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>0.9955</t>
+        </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>0.3301</t>
+          <t>0.4651</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Good fit with caveats: AI Engineer at Mad Street Den (4.6 YOE); JD-aligned skills: pgvector, FAISS, Embeddings.</t>
+          <t>Good fit with caveats: Applied ML Engineer at Freshworks (8.0 YOE); JD-aligned skills: Vector Search, Qdrant, Embeddings.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>CAND_0078002</t>
-        </is>
-      </c>
-      <c r="B48" t="n">
-        <v>47</v>
-      </c>
-      <c r="C48" t="n">
-        <v>0.9954</v>
+          <t>CAND_0015528</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>47</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>0.9954</t>
+        </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>0.2974</t>
+          <t>0.3246</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Competitive candidate: Machine Learning Engineer at Meta (6.3 YOE); JD-aligned skills: pgvector, NLP, Weaviate.</t>
+          <t>Competitive candidate: Applied ML Engineer at Krutrim (7.4 YOE); JD-aligned skills: Weaviate, pgvector, Information Retrieval.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>CAND_0010257</t>
-        </is>
-      </c>
-      <c r="B49" t="n">
-        <v>48</v>
-      </c>
-      <c r="C49" t="n">
-        <v>0.9953</v>
+          <t>CAND_0075574</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>48</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>0.9953</t>
+        </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>0.3313</t>
+          <t>0.4170</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Meets several JD signals: Senior Data Scientist at Google (6.5 YOE); JD-aligned skills: Milvus, Python, OpenSearch. Concerns: 120-day notice period.</t>
+          <t>Meets several JD signals: Machine Learning Engineer at Haptik (5.7 YOE); JD-aligned skills: pgvector, Weaviate, OpenSearch.</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>CAND_0065878</t>
-        </is>
-      </c>
-      <c r="B50" t="n">
-        <v>49</v>
-      </c>
-      <c r="C50" t="n">
-        <v>0.9952</v>
+          <t>CAND_0052328</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>49</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>0.9952</t>
+        </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>0.2450</t>
+          <t>0.5090</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Solid profile: Senior Data Scientist at Niramai (7.8 YOE); JD-aligned skills: pgvector, Vector Search, Fine-tuning LLMs.</t>
+          <t>Solid profile: Recommendation Systems Engineer at Amazon (6.5 YOE); JD-aligned skills: OpenSearch, Fine-tuning LLMs, Vector Search.</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>CAND_0032216</t>
-        </is>
-      </c>
-      <c r="B51" t="n">
-        <v>50</v>
-      </c>
-      <c r="C51" t="n">
-        <v>0.9951</v>
+          <t>CAND_0040178</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>0.9951</t>
+        </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>0.2743</t>
+          <t>0.3303</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Good fit with caveats: ML Engineer at upGrad (6.1 YOE); JD-aligned skills: Information Retrieval, Qdrant, Sentence Transformers.</t>
+          <t>Good fit with caveats: ML Engineer at Meesho (5.0 YOE); JD-aligned skills: Weaviate, Fine-tuning LLMs, Vector Search.</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>CAND_0005260</t>
-        </is>
-      </c>
-      <c r="B52" t="n">
-        <v>51</v>
-      </c>
-      <c r="C52" t="n">
-        <v>0.995</v>
+          <t>CAND_0051004</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>51</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>0.9950</t>
+        </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>0.4814</t>
+          <t>0.5405</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Moderate fit: Senior NLP Engineer at Netflix (5.2 YOE); JD-aligned skills: Information Retrieval, Python, NLP. Gaps: under half of JD must-have skills covered.</t>
+          <t>Moderate fit: Senior Data Scientist at CRED (4.7 YOE); JD-aligned skills: Embeddings, Qdrant, Fine-tuning LLMs. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>CAND_0025923</t>
-        </is>
-      </c>
-      <c r="B53" t="n">
-        <v>52</v>
-      </c>
-      <c r="C53" t="n">
-        <v>0.9949</v>
+          <t>CAND_0079064</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>52</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>0.9949</t>
+        </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>0.2891</t>
+          <t>0.2563</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Partial alignment: Senior Software Engineer (ML) at HCL (5.0 YOE); JD-aligned skills: pgvector, Qdrant, Pinecone. Gaps: under half of JD must-have skills covered.</t>
+          <t>Partial alignment: Senior Data Scientist at Niramai (5.2 YOE); JD-aligned skills: OpenSearch, NLP, Fine-tuning LLMs. Gaps: 120-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>CAND_0075574</t>
-        </is>
-      </c>
-      <c r="B54" t="n">
-        <v>53</v>
-      </c>
-      <c r="C54" t="n">
-        <v>0.9948</v>
+          <t>CAND_0065878</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>53</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>0.9948</t>
+        </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>0.4170</t>
+          <t>0.2450</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Acceptable but not standout: Machine Learning Engineer at Haptik (5.7 YOE); JD-aligned skills: pgvector, Weaviate, OpenSearch. Gaps: under half of JD must-have skills covered.</t>
+          <t>Acceptable but not standout: Senior Data Scientist at Niramai (7.8 YOE); JD-aligned skills: pgvector, Vector Search, Fine-tuning LLMs. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>CAND_0038368</t>
-        </is>
-      </c>
-      <c r="B55" t="n">
-        <v>54</v>
-      </c>
-      <c r="C55" t="n">
-        <v>0.9947</v>
+          <t>CAND_0069905</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>54</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>0.9947</t>
+        </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>0.4347</t>
+          <t>0.3358</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Mixed signals: ML Engineer at PhonePe (5.4 YOE); JD-aligned skills: Embeddings, FAISS, NLP. Gaps: under half of JD must-have skills covered.</t>
+          <t>Mixed signals: Applied ML Engineer at Sarvam AI (6.6 YOE); JD-aligned skills: Sentence Transformers, Python, Weaviate. Gaps: 90-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>CAND_0005538</t>
-        </is>
-      </c>
-      <c r="B56" t="n">
-        <v>55</v>
-      </c>
-      <c r="C56" t="n">
-        <v>0.9946</v>
+          <t>CAND_0011432</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>0.9946</t>
+        </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>0.4072</t>
+          <t>0.5534</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>JD overlap is thin: Senior AI Engineer at Adobe (5.9 YOE); JD-aligned skills: Vector Representations, Python, Information Retrieval Systems. Gaps: 90-day notice period.</t>
+          <t>JD overlap is thin: Senior Data Scientist at Amazon (7.6 YOE); JD-aligned skills: OpenSearch, pgvector, Elasticsearch. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>CAND_0079064</t>
-        </is>
-      </c>
-      <c r="B57" t="n">
-        <v>56</v>
-      </c>
-      <c r="C57" t="n">
-        <v>0.9945000000000001</v>
+          <t>CAND_0036121</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>0.9945</t>
+        </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>0.2563</t>
+          <t>0.3242</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Moderate fit: Senior Data Scientist at Niramai (5.2 YOE); JD-aligned skills: OpenSearch, NLP, Fine-tuning LLMs. Gaps: 120-day notice period.</t>
+          <t>Moderate fit: ML Engineer at Wysa (5.2 YOE); JD-aligned skills: Embeddings, Vector Search, Information Retrieval. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>CAND_0015528</t>
-        </is>
-      </c>
-      <c r="B58" t="n">
-        <v>57</v>
-      </c>
-      <c r="C58" t="n">
-        <v>0.9944</v>
+          <t>CAND_0093912</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>57</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>0.9944</t>
+        </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>0.3246</t>
+          <t>0.4763</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Partial alignment: Applied ML Engineer at Krutrim (7.4 YOE); JD-aligned skills: Weaviate, pgvector, Information Retrieval. Gaps: under half of JD must-have skills covered.</t>
+          <t>Partial alignment: Senior Data Scientist at Razorpay (5.3 YOE); JD-aligned skills: Milvus, Embeddings, Vector Search. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>CAND_0067866</t>
-        </is>
-      </c>
-      <c r="B59" t="n">
-        <v>58</v>
-      </c>
-      <c r="C59" t="n">
-        <v>0.9943</v>
+          <t>CAND_0080465</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>58</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>0.9943</t>
+        </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>0.3513</t>
+          <t>0.2782</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Acceptable but not standout: Senior Software Engineer (ML) at Tech Mahindra (6.4 YOE); JD-aligned skills: Embeddings, pgvector, Elasticsearch. Gaps: under half of JD must-have skills covered.</t>
+          <t>Acceptable but not standout: ML Engineer at Meesho (4.2 YOE); JD-aligned skills: Milvus, Qdrant. Gaps: 90-day notice period.</t>
         </is>
       </c>
     </row>
@@ -1783,11 +2015,15 @@
           <t>CAND_0074735</t>
         </is>
       </c>
-      <c r="B60" t="n">
-        <v>59</v>
-      </c>
-      <c r="C60" t="n">
-        <v>0.9942</v>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>59</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>0.9942</t>
+        </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
@@ -1803,345 +2039,405 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>CAND_0079284</t>
-        </is>
-      </c>
-      <c r="B61" t="n">
-        <v>60</v>
-      </c>
-      <c r="C61" t="n">
-        <v>0.9941</v>
+          <t>CAND_0099806</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>0.9941</t>
+        </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>0.2718</t>
+          <t>0.3301</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>JD overlap is thin: Machine Learning Engineer at Google (4.9 YOE); JD-aligned skills: Qdrant, Fine-tuning LLMs, Elasticsearch. Gaps: under half of JD must-have skills covered.</t>
+          <t>JD overlap is thin: AI Engineer at Mad Street Den (4.6 YOE); JD-aligned skills: pgvector, FAISS, Embeddings. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>CAND_0090584</t>
-        </is>
-      </c>
-      <c r="B62" t="n">
-        <v>61</v>
-      </c>
-      <c r="C62" t="n">
-        <v>0.994</v>
+          <t>CAND_0039962</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>0.9940</t>
+        </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>0.1637</t>
+          <t>0.2509</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Moderate fit: ML Engineer at Flipkart (5.1 YOE); JD-aligned skills: Fine-tuning LLMs, OpenSearch, FAISS. Gaps: 120-day notice period.</t>
+          <t>Moderate fit: ML Engineer at Paytm (6.5 YOE); JD-aligned skills: Pinecone, LLMs. Gaps: 90-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>CAND_0011432</t>
-        </is>
-      </c>
-      <c r="B63" t="n">
-        <v>62</v>
-      </c>
-      <c r="C63" t="n">
-        <v>0.9939</v>
+          <t>CAND_0002120</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>62</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>0.9939</t>
+        </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>0.5534</t>
+          <t>0.3168</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Partial alignment: Senior Data Scientist at Amazon (7.6 YOE); JD-aligned skills: OpenSearch, pgvector, Elasticsearch. Gaps: under half of JD must-have skills covered.</t>
+          <t>Partial alignment: ML Engineer at HCL (6.5 YOE); JD-aligned skills: Information Retrieval, Pinecone, Embeddings. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>CAND_0061550</t>
-        </is>
-      </c>
-      <c r="B64" t="n">
-        <v>63</v>
-      </c>
-      <c r="C64" t="n">
-        <v>0.9938</v>
+          <t>CAND_0028793</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>63</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>0.9938</t>
+        </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>0.3313</t>
+          <t>0.2941</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Acceptable but not standout: ML Engineer at Infosys (5.3 YOE); JD-aligned skills: pgvector, Sentence Transformers. Gaps: under half of JD must-have skills covered.</t>
+          <t>Acceptable but not standout: Search Engineer at Google (7.2 YOE); JD-aligned skills: Embeddings, Information Retrieval, pgvector. Gaps: 120-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>CAND_0011687</t>
-        </is>
-      </c>
-      <c r="B65" t="n">
-        <v>64</v>
-      </c>
-      <c r="C65" t="n">
-        <v>0.9937</v>
+          <t>CAND_0005538</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>64</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>0.9937</t>
+        </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>0.5094</t>
+          <t>0.4072</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Mixed signals: Senior NLP Engineer at Niramai (7.8 YOE); JD-aligned skills: OpenSearch, FAISS, Embeddings. Gaps: under half of JD must-have skills covered.</t>
+          <t>Mixed signals: Senior AI Engineer at Adobe (5.9 YOE); JD-aligned skills: Vector Representations, Python, Information Retrieval Systems. Gaps: 90-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>CAND_0028793</t>
-        </is>
-      </c>
-      <c r="B66" t="n">
-        <v>65</v>
-      </c>
-      <c r="C66" t="n">
-        <v>0.9936</v>
+          <t>CAND_0011489</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>65</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>0.9936</t>
+        </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>0.2941</t>
+          <t>0.2839</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>JD overlap is thin: Search Engineer at Google (7.2 YOE); JD-aligned skills: Embeddings, Information Retrieval, pgvector. Gaps: 120-day notice period.</t>
+          <t>JD overlap is thin: ML Engineer at Glance (5.8 YOE); JD-aligned skills: pgvector, Embeddings, Python. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>CAND_0048166</t>
-        </is>
-      </c>
-      <c r="B67" t="n">
-        <v>66</v>
-      </c>
-      <c r="C67" t="n">
-        <v>0.9935</v>
+          <t>CAND_0003841</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>66</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>0.9935</t>
+        </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>0.4054</t>
+          <t>0.3402</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Moderate fit: ML Engineer at Aganitha (5.2 YOE); JD-aligned skills: Pinecone, Milvus, Qdrant. Gaps: under half of JD must-have skills covered.</t>
+          <t>Moderate fit: ML Engineer at Tech Mahindra (5.0 YOE); JD-aligned skills: Pinecone, Fine-tuning LLMs, Sentence Transformers. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>CAND_0093547</t>
-        </is>
-      </c>
-      <c r="B68" t="n">
-        <v>67</v>
-      </c>
-      <c r="C68" t="n">
-        <v>0.9933999999999999</v>
+          <t>CAND_0055992</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>67</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>0.9934</t>
+        </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>0.3710</t>
+          <t>0.5850</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Partial alignment: Senior Machine Learning Engineer at PhonePe (2.9 YOE); JD-aligned skills: LLMs, Python, Milvus. Gaps: below typical senior YOE band for this JD.</t>
+          <t>Partial alignment: AI Engineer at CRED (16.9 YOE); JD-aligned skills: Information Retrieval, FAISS, OpenSearch. Gaps: experience above target band for this role.</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>CAND_0076482</t>
-        </is>
-      </c>
-      <c r="B69" t="n">
-        <v>68</v>
-      </c>
-      <c r="C69" t="n">
-        <v>0.9933</v>
+          <t>CAND_0021836</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>0.9933</t>
+        </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>0.5553</t>
+          <t>0.4646</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Acceptable but not standout: ML Engineer at Flipkart (6.6 YOE); JD-aligned skills: OpenSearch, Pinecone, pgvector. Gaps: under half of JD must-have skills covered.</t>
+          <t>Acceptable but not standout: ML Engineer at CRED (6.5 YOE); JD-aligned skills: Vector Search, Elasticsearch, NLP. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>CAND_0040178</t>
-        </is>
-      </c>
-      <c r="B70" t="n">
-        <v>69</v>
-      </c>
-      <c r="C70" t="n">
-        <v>0.9932</v>
+          <t>CAND_0009691</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>69</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>0.9932</t>
+        </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>0.3303</t>
+          <t>0.1214</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Mixed signals: ML Engineer at Meesho (5.0 YOE); JD-aligned skills: Weaviate, Fine-tuning LLMs, Vector Search. Gaps: under half of JD must-have skills covered.</t>
+          <t>Mixed signals: Applied ML Engineer at LinkedIn (6.2 YOE); JD-aligned skills: Fine-tuning LLMs, Pinecone, Sentence Transformers. Gaps: 120-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>CAND_0060054</t>
-        </is>
-      </c>
-      <c r="B71" t="n">
-        <v>70</v>
-      </c>
-      <c r="C71" t="n">
-        <v>0.9931</v>
+          <t>CAND_0046525</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>0.9931</t>
+        </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>0.3416</t>
+          <t>0.3574</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>JD overlap is thin: AI Engineer at Mad Street Den (6.4 YOE); JD-aligned skills: Weaviate, FAISS, Elasticsearch. Gaps: under half of JD must-have skills covered.</t>
+          <t>JD overlap is thin: Senior Machine Learning Engineer at Genpact AI (6.1 YOE); JD-aligned skills: Elasticsearch, Information Retrieval, LLMs. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>CAND_0024878</t>
-        </is>
-      </c>
-      <c r="B72" t="n">
-        <v>71</v>
-      </c>
-      <c r="C72" t="n">
-        <v>0.993</v>
+          <t>CAND_0010257</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>71</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>0.9930</t>
+        </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>0.4462</t>
+          <t>0.3313</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Moderate fit: AI Specialist at HCL (5.7 YOE); JD-aligned skills: pgvector, Elasticsearch, NLP. Gaps: under half of JD must-have skills covered.</t>
+          <t>Moderate fit: Senior Data Scientist at Google (6.5 YOE); JD-aligned skills: Milvus, Python, OpenSearch. Gaps: 120-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>CAND_0008425</t>
-        </is>
-      </c>
-      <c r="B73" t="n">
-        <v>72</v>
-      </c>
-      <c r="C73" t="n">
-        <v>0.9929</v>
+          <t>CAND_0067866</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>0.9929</t>
+        </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>0.2436</t>
+          <t>0.3513</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Partial alignment: Senior NLP Engineer at Ola (7.8 YOE); JD-aligned skills: Qdrant, pgvector, Sentence Transformers. Gaps: 90-day notice period.</t>
+          <t>Partial alignment: Senior Software Engineer (ML) at Tech Mahindra (6.4 YOE); JD-aligned skills: Embeddings, pgvector, Elasticsearch. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>CAND_0036121</t>
-        </is>
-      </c>
-      <c r="B74" t="n">
-        <v>73</v>
-      </c>
-      <c r="C74" t="n">
-        <v>0.9928</v>
+          <t>CAND_0037944</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>73</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>0.9928</t>
+        </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>0.3242</t>
+          <t>0.2490</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Acceptable but not standout: ML Engineer at Wysa (5.2 YOE); JD-aligned skills: Embeddings, Vector Search, Information Retrieval. Gaps: under half of JD must-have skills covered.</t>
+          <t>Acceptable but not standout: Senior Data Scientist at Vedantu (4.9 YOE); JD-aligned skills: Vector Search, OpenSearch, Embeddings. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>CAND_0027691</t>
-        </is>
-      </c>
-      <c r="B75" t="n">
-        <v>74</v>
-      </c>
-      <c r="C75" t="n">
-        <v>0.9927</v>
+          <t>CAND_0086022</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>74</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>0.9927</t>
+        </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>0.4306</t>
+          <t>0.3683</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Mixed signals: NLP Engineer at Haptik (6.5 YOE); JD-aligned skills: Weaviate, Embeddings, Python. Gaps: under half of JD must-have skills covered.</t>
+          <t>Mixed signals: Senior Applied Scientist at Sarvam AI (5.3 YOE); JD-aligned skills: Vector Search, pgvector, Fine-tuning LLMs. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
@@ -2151,11 +2447,15 @@
           <t>CAND_0037980</t>
         </is>
       </c>
-      <c r="B76" t="n">
-        <v>75</v>
-      </c>
-      <c r="C76" t="n">
-        <v>0.9926</v>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>75</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>0.9926</t>
+        </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
@@ -2171,575 +2471,675 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>CAND_0096104</t>
-        </is>
-      </c>
-      <c r="B77" t="n">
-        <v>76</v>
-      </c>
-      <c r="C77" t="n">
-        <v>0.9925</v>
+          <t>CAND_0065514</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>76</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>0.9925</t>
+        </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>0.5401</t>
+          <t>0.2597</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Moderate fit: AI Specialist at Yellow.ai (7.0 YOE); JD-aligned skills: Pinecone. Gaps: only 1 core JD skill matched.</t>
+          <t>Moderate fit: ML Engineer at Genpact AI (6.6 YOE); JD-aligned skills: Vector Search, Pinecone, Elasticsearch. Gaps: 90-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>CAND_0001819</t>
-        </is>
-      </c>
-      <c r="B78" t="n">
-        <v>77</v>
-      </c>
-      <c r="C78" t="n">
-        <v>0.9923999999999999</v>
+          <t>CAND_0030348</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>77</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>0.9924</t>
+        </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>0.3603</t>
+          <t>0.3735</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Partial alignment: ML Engineer at Genpact AI (4.4 YOE); JD-aligned skills: Weaviate, pgvector, NLP. Gaps: under half of JD must-have skills covered.</t>
+          <t>Partial alignment: Machine Learning Engineer at BYJU'S (4.5 YOE); JD-aligned skills: Embeddings, Vector Search, Elasticsearch. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>CAND_0052328</t>
-        </is>
-      </c>
-      <c r="B79" t="n">
-        <v>78</v>
-      </c>
-      <c r="C79" t="n">
-        <v>0.9923</v>
+          <t>CAND_0070398</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>78</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>0.9923</t>
+        </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>0.5090</t>
+          <t>0.2060</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Acceptable but not standout: Recommendation Systems Engineer at Amazon (6.5 YOE); JD-aligned skills: OpenSearch, Fine-tuning LLMs, Vector Search. Gaps: under half of JD must-have skills covered.</t>
+          <t>Acceptable but not standout: Machine Learning Engineer at Genpact AI (7.2 YOE); JD-aligned skills: FAISS, Embeddings, Python. Gaps: 120-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>CAND_0030348</t>
-        </is>
-      </c>
-      <c r="B80" t="n">
-        <v>79</v>
-      </c>
-      <c r="C80" t="n">
-        <v>0.9922</v>
+          <t>CAND_0017178</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>79</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>0.9922</t>
+        </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>0.3735</t>
+          <t>0.4976</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Mixed signals: Machine Learning Engineer at BYJU'S (4.5 YOE); JD-aligned skills: Embeddings, Vector Search, Elasticsearch. Gaps: under half of JD must-have skills covered.</t>
+          <t>Mixed signals: ML Engineer at Swiggy (4.2 YOE); JD-aligned skills: pgvector, Information Retrieval. Gaps: not flagged open to work.</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>CAND_0009691</t>
-        </is>
-      </c>
-      <c r="B81" t="n">
-        <v>80</v>
-      </c>
-      <c r="C81" t="n">
-        <v>0.9921</v>
+          <t>CAND_0001819</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>80</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>0.9921</t>
+        </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>0.1214</t>
+          <t>0.3603</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>JD overlap is thin: Applied ML Engineer at LinkedIn (6.2 YOE); JD-aligned skills: Fine-tuning LLMs, Pinecone, Sentence Transformers. Gaps: 120-day notice period.</t>
+          <t>JD overlap is thin: ML Engineer at Genpact AI (4.4 YOE); JD-aligned skills: Weaviate, pgvector, NLP. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>CAND_0019288</t>
-        </is>
-      </c>
-      <c r="B82" t="n">
-        <v>81</v>
-      </c>
-      <c r="C82" t="n">
-        <v>0.992</v>
+          <t>CAND_0015578</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>81</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>0.9920</t>
+        </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>0.3846</t>
+          <t>0.1397</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Moderate fit: AI Research Engineer at Paytm (5.7 YOE); JD-aligned skills: pgvector, FAISS, OpenSearch. Gaps: under half of JD must-have skills covered.</t>
+          <t>Moderate fit: AI Engineer at Zoho (5.4 YOE); JD-aligned skills: Embeddings, NLP, Sentence Transformers. Gaps: 90-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>CAND_0002793</t>
-        </is>
-      </c>
-      <c r="B83" t="n">
-        <v>82</v>
-      </c>
-      <c r="C83" t="n">
-        <v>0.9919</v>
+          <t>CAND_0033445</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>82</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>0.9919</t>
+        </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>0.3997</t>
+          <t>0.2922</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Partial alignment: AI Specialist at Meesho (5.5 YOE); JD-aligned skills: pgvector, Information Retrieval, FAISS. Gaps: not flagged open to work.</t>
+          <t>Partial alignment: ML Engineer at Vedantu (6.8 YOE); JD-aligned skills: Information Retrieval, pgvector. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>CAND_0043637</t>
-        </is>
-      </c>
-      <c r="B84" t="n">
-        <v>83</v>
-      </c>
-      <c r="C84" t="n">
-        <v>0.9918</v>
+          <t>CAND_0018293</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>83</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>0.9918</t>
+        </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>0.4329</t>
+          <t>0.5647</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Acceptable but not standout: Junior ML Engineer at Rephrase.ai (5.5 YOE); JD-aligned skills: Milvus, pgvector. Gaps: under half of JD must-have skills covered.</t>
+          <t>Acceptable but not standout: Data Scientist at PharmEasy (5.6 YOE); JD-aligned skills: Weaviate, Information Retrieval, pgvector. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>CAND_0091534</t>
-        </is>
-      </c>
-      <c r="B85" t="n">
-        <v>84</v>
-      </c>
-      <c r="C85" t="n">
-        <v>0.9917</v>
+          <t>CAND_0049615</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>84</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>0.9917</t>
+        </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>0.2365</t>
+          <t>0.2597</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Mixed signals: AI Engineer at Flipkart (16.6 YOE); JD-aligned skills: Qdrant, Sentence Transformers. Gaps: experience above target band for this role; not flagged open to work.</t>
+          <t>Mixed signals: ML Engineer at Krutrim (5.1 YOE); JD-aligned skills: NLP, Pinecone. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>CAND_0070398</t>
-        </is>
-      </c>
-      <c r="B86" t="n">
-        <v>85</v>
-      </c>
-      <c r="C86" t="n">
-        <v>0.9916</v>
+          <t>CAND_0017093</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>85</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>0.9916</t>
+        </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>0.2060</t>
+          <t>0.2136</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>JD overlap is thin: Machine Learning Engineer at Genpact AI (7.2 YOE); JD-aligned skills: FAISS, Embeddings, Python. Gaps: 120-day notice period.</t>
+          <t>JD overlap is thin: ML Engineer at Zoho (5.9 YOE); JD-aligned skills: LLMs, Embeddings, pgvector. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>CAND_0015578</t>
-        </is>
-      </c>
-      <c r="B87" t="n">
-        <v>86</v>
-      </c>
-      <c r="C87" t="n">
-        <v>0.9915</v>
+          <t>CAND_0050876</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>86</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>0.9915</t>
+        </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>0.1397</t>
+          <t>0.4323</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Moderate fit: AI Engineer at Zoho (5.4 YOE); JD-aligned skills: Embeddings, NLP, Sentence Transformers. Gaps: 90-day notice period.</t>
+          <t>Moderate fit: Applied ML Engineer at Freshworks (6.0 YOE); JD-aligned skills: Qdrant, FAISS, OpenSearch. Gaps: 90-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>CAND_0010541</t>
-        </is>
-      </c>
-      <c r="B88" t="n">
-        <v>87</v>
-      </c>
-      <c r="C88" t="n">
-        <v>0.9913999999999999</v>
+          <t>CAND_0041669</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>87</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>0.9914</t>
+        </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>0.5800</t>
+          <t>0.6806</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Partial alignment: AI Research Engineer at Wysa (6.2 YOE); JD-aligned skills: Pinecone, Weaviate, Python. Gaps: under half of JD must-have skills covered.</t>
+          <t>Partial alignment: Recommendation Systems Engineer at CRED (8.0 YOE); JD-aligned skills: FAISS, Milvus, Weaviate. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>CAND_0065195</t>
-        </is>
-      </c>
-      <c r="B89" t="n">
-        <v>88</v>
-      </c>
-      <c r="C89" t="n">
-        <v>0.9913</v>
+          <t>CAND_0027691</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>88</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>0.9913</t>
+        </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>0.3492</t>
+          <t>0.4306</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>Acceptable but not standout: Search Engineer at CRED (5.1 YOE); JD-aligned skills: LLMs, Elasticsearch, Qdrant. Gaps: under half of JD must-have skills covered.</t>
+          <t>Acceptable but not standout: NLP Engineer at Haptik (6.5 YOE); JD-aligned skills: Weaviate, Embeddings, Python. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>CAND_0037944</t>
-        </is>
-      </c>
-      <c r="B90" t="n">
-        <v>89</v>
-      </c>
-      <c r="C90" t="n">
-        <v>0.9912</v>
+          <t>CAND_0002037</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>89</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>0.9912</t>
+        </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>0.2490</t>
+          <t>0.1905</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Mixed signals: Senior Data Scientist at Vedantu (4.9 YOE); JD-aligned skills: Vector Search, OpenSearch, Embeddings. Gaps: under half of JD must-have skills covered.</t>
+          <t>Mixed signals: ML Engineer at Locobuzz (5.5 YOE); JD-aligned skills: Fine-tuning LLMs, pgvector, Milvus. Gaps: not flagged open to work.</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>CAND_0093474</t>
-        </is>
-      </c>
-      <c r="B91" t="n">
-        <v>90</v>
-      </c>
-      <c r="C91" t="n">
-        <v>0.9911</v>
+          <t>CAND_0066376</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>90</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>0.9911</t>
+        </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>0.4226</t>
+          <t>0.2674</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>JD overlap is thin: Senior Software Engineer (ML) at Wipro (5.3 YOE); JD-aligned skills: Vector Search, Qdrant, FAISS. Gaps: 90-day notice period; not flagged open to work.</t>
+          <t>JD overlap is thin: Applied ML Engineer at Dream11 (5.7 YOE); JD-aligned skills: LLMs, Fine-tuning LLMs, NLP. Gaps: 90-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>CAND_0039754</t>
-        </is>
-      </c>
-      <c r="B92" t="n">
-        <v>91</v>
-      </c>
-      <c r="C92" t="n">
-        <v>0.991</v>
+          <t>CAND_0048166</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>91</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>0.9910</t>
+        </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>0.5509</t>
+          <t>0.4054</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>Lower-tier shortlist entry — Senior Applied Scientist at Meta (16.2 YOE); JD-aligned skills: Fine-tuning LLMs, Qdrant, NLP. Key gaps: experience above target band for this role.</t>
+          <t>Lower-tier shortlist entry — ML Engineer at Aganitha (5.2 YOE); JD-aligned skills: Pinecone, Milvus, Qdrant. Key gaps: not flagged open to work.</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>CAND_0003791</t>
-        </is>
-      </c>
-      <c r="B93" t="n">
-        <v>92</v>
-      </c>
-      <c r="C93" t="n">
-        <v>0.9909</v>
+          <t>CAND_0062561</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>92</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>0.9909</t>
+        </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>0.4776</t>
+          <t>0.3470</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>Lower-tier shortlist entry — ML Engineer at Meesho (6.6 YOE); JD-aligned skills: LLMs, pgvector, Python. Key gaps: weak secondary signals vs higher ranks.</t>
+          <t>Lower-tier shortlist entry — ML Engineer at Razorpay (5.9 YOE); JD-aligned skills: Information Retrieval, Weaviate. Key gaps: weak secondary signals vs higher ranks.</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>CAND_0001661</t>
-        </is>
-      </c>
-      <c r="B94" t="n">
-        <v>93</v>
-      </c>
-      <c r="C94" t="n">
-        <v>0.9908</v>
+          <t>CAND_0035653</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>93</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>0.9908</t>
+        </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>0.3461</t>
+          <t>0.4419</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>Lower-tier shortlist entry — Senior Data Engineer at Cognizant (7.8 YOE); JD-aligned skills: Vector Search. Key gaps: only 1 core JD skill matched.</t>
+          <t>Lower-tier shortlist entry — Data Scientist at Swiggy (5.6 YOE); JD-aligned skills: OpenSearch, Vector Search, Fine-tuning LLMs. Key gaps: weak secondary signals vs higher ranks.</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>CAND_0007460</t>
-        </is>
-      </c>
-      <c r="B95" t="n">
-        <v>94</v>
-      </c>
-      <c r="C95" t="n">
-        <v>0.9907</v>
+          <t>CAND_0056940</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>94</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>0.9907</t>
+        </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>0.2260</t>
+          <t>0.2882</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>Lower-tier shortlist entry — AI Engineer at Salesforce (4.7 YOE); JD-aligned skills: Embeddings, Weaviate, Information Retrieval. Key gaps: 120-day notice period.</t>
+          <t>Lower-tier shortlist entry — Backend Engineer at Zomato (7.4 YOE); JD-aligned skills: pgvector. Key gaps: only 1 core JD skill matched.</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>CAND_0041669</t>
-        </is>
-      </c>
-      <c r="B96" t="n">
-        <v>95</v>
-      </c>
-      <c r="C96" t="n">
-        <v>0.9906</v>
+          <t>CAND_0032515</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>95</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>0.9906</t>
+        </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>0.6806</t>
+          <t>0.3727</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>Lower-tier shortlist entry — Recommendation Systems Engineer at CRED (8.0 YOE); JD-aligned skills: FAISS, Milvus, Weaviate. Key gaps: weak secondary signals vs higher ranks.</t>
+          <t>Lower-tier shortlist entry — Machine Learning Engineer at PharmEasy (5.1 YOE); JD-aligned skills: Milvus, Vector Search, Fine-tuning LLMs. Key gaps: not flagged open to work.</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>CAND_0050876</t>
-        </is>
-      </c>
-      <c r="B97" t="n">
-        <v>96</v>
-      </c>
-      <c r="C97" t="n">
-        <v>0.9905</v>
+          <t>CAND_0053605</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>96</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>0.9905</t>
+        </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>0.4323</t>
+          <t>0.6824</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>Lower-tier shortlist entry — Applied ML Engineer at Freshworks (6.0 YOE); JD-aligned skills: Qdrant, FAISS, OpenSearch. Key gaps: 90-day notice period.</t>
+          <t>Lower-tier shortlist entry — Senior Software Engineer (ML) at Verloop.io (6.9 YOE); JD-aligned skills: pgvector. Key gaps: only 1 core JD skill matched.</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>CAND_0081086</t>
-        </is>
-      </c>
-      <c r="B98" t="n">
-        <v>97</v>
-      </c>
-      <c r="C98" t="n">
-        <v>0.9903999999999999</v>
+          <t>CAND_0092255</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>97</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>0.9904</t>
+        </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>0.2245</t>
+          <t>0.2741</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>Lower-tier shortlist entry — AI Specialist at Observe.AI (5.2 YOE); JD-aligned skills: pgvector, Weaviate, Embeddings. Key gaps: weak secondary signals vs higher ranks.</t>
+          <t>Lower-tier shortlist entry — ML Engineer at InMobi (5.2 YOE); JD-aligned skills: Weaviate, OpenSearch, Vector Search. Key gaps: weak secondary signals vs higher ranks.</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>CAND_0013665</t>
-        </is>
-      </c>
-      <c r="B99" t="n">
-        <v>98</v>
-      </c>
-      <c r="C99" t="n">
-        <v>0.9903</v>
+          <t>CAND_0082489</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>98</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>0.9903</t>
+        </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>0.2424</t>
+          <t>0.2325</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>Lower-tier shortlist entry — Senior Software Engineer (ML) at InMobi (5.2 YOE); JD-aligned skills: Qdrant, Embeddings. Key gaps: not flagged open to work.</t>
+          <t>Lower-tier shortlist entry — ML Engineer at InMobi (5.3 YOE); JD-aligned skills: Weaviate. Key gaps: only 1 core JD skill matched; 90-day notice period; not flagged open to work.</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>CAND_0080465</t>
-        </is>
-      </c>
-      <c r="B100" t="n">
-        <v>99</v>
-      </c>
-      <c r="C100" t="n">
-        <v>0.9902</v>
+          <t>CAND_0098288</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>99</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>0.9902</t>
+        </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>0.2782</t>
+          <t>0.4556</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>Lower-tier shortlist entry — ML Engineer at Meesho (4.2 YOE); JD-aligned skills: Milvus, Qdrant. Key gaps: 90-day notice period.</t>
+          <t>Lower-tier shortlist entry — Junior ML Engineer at Vedantu (6.7 YOE); JD-aligned skills: Information Retrieval, NLP, pgvector. Key gaps: weak secondary signals vs higher ranks.</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>CAND_0094759</t>
-        </is>
-      </c>
-      <c r="B101" t="n">
-        <v>100</v>
-      </c>
-      <c r="C101" t="n">
-        <v>0.9901</v>
+          <t>CAND_0091909</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>0.9901</t>
+        </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>0.2923</t>
+          <t>0.1949</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>Lower-tier shortlist entry — Lead AI Engineer at Meta (8.6 YOE); JD-aligned skills: Qdrant, Fine-tuning LLMs, Vector Search. Key gaps: low recruiter response rate; not flagged open to work.</t>
+          <t>Lower-tier shortlist entry — Machine Learning Engineer at Rephrase.ai (6.9 YOE); JD-aligned skills: LLMs, Pinecone, Qdrant. Key gaps: weak secondary signals vs higher ranks.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: regenerate submission from full 100k fix1 run
</commit_message>
<xml_diff>
--- a/submission.xlsx
+++ b/submission.xlsx
@@ -446,7 +446,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>CAND_0068351</t>
+          <t>CAND_0018499</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -461,19 +461,19 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>0.4040</t>
+          <t>0.6132</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Rank 1: Lead AI Engineer at Sarvam AI (6.4 YOE); JD-aligned skills: pgvector, Qdrant, Elasticsearch. Top-tier composite score across career, skills, and availability. Counterfactual: ranks on career trajectory and assessed depth over keyword coverage (7/20 listed must-haves), aligning with the JD anti-keyword-stuffing guidance. Join probability: 40%.</t>
+          <t>Rank 1: Senior Machine Learning Engineer at Zomato (7.2 YOE); JD-aligned skills: Weaviate, Pinecone, Information Retrieval. Top-tier composite score across career, skills, and availability. Counterfactual: ranks on career trajectory and assessed depth over keyword coverage (5/20 listed must-haves), aligning with the JD anti-keyword-stuffing guidance. Join probability: 61%.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>CAND_0018499</t>
+          <t>CAND_0088025</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -488,19 +488,19 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>0.6132</t>
+          <t>0.5411</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Rank 2: Senior Machine Learning Engineer at Zomato (7.2 YOE); JD-aligned skills: Weaviate, Pinecone, Information Retrieval. Top-tier composite score across career, skills, and availability. Counterfactual: ranks on career trajectory and assessed depth over keyword coverage (5/20 listed must-haves), aligning with the JD anti-keyword-stuffing guidance. Join probability: 61%.</t>
+          <t>Rank 2: Staff Machine Learning Engineer at Yellow.ai (8.6 YOE); JD-aligned skills: Pinecone, LLMs, Elasticsearch. Top-tier composite score across career, skills, and availability. Minor note: 90-day notice period. Join probability: 54%.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>CAND_0071974</t>
+          <t>CAND_0002025</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -515,19 +515,19 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>0.3414</t>
+          <t>0.3912</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Rank 3: Senior AI Engineer at Netflix (7.8 YOE); JD-aligned skills: Weaviate, Pinecone, Information Retrieval. Top-tier composite score across career, skills, and availability. Counterfactual: ranks on career trajectory and assessed depth over keyword coverage (7/20 listed must-haves), aligning with the JD anti-keyword-stuffing guidance. Join probability: 34%; low engagement signals.</t>
+          <t>Rank 3: Senior AI Engineer at Apple (5.9 YOE); JD-aligned skills: FAISS, OpenSearch, Weaviate. Top-tier composite score across career, skills, and availability. Counterfactual: ranks on career trajectory and assessed depth over keyword coverage (8/20 listed must-haves), aligning with the JD anti-keyword-stuffing guidance. Join probability: 39%.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>CAND_0088025</t>
+          <t>CAND_0081846</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -542,19 +542,19 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>0.5411</t>
+          <t>0.4803</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Rank 4: Staff Machine Learning Engineer at Yellow.ai (8.6 YOE); JD-aligned skills: Pinecone, LLMs, Elasticsearch. Top-tier composite score across career, skills, and availability. Minor note: 90-day notice period. Join probability: 54%.</t>
+          <t>Rank 4: Lead AI Engineer at Razorpay (6.7 YOE); JD-aligned skills: Information Retrieval, pgvector, Elasticsearch. Top-tier composite score across career, skills, and availability. Counterfactual: ranks on career trajectory and assessed depth over keyword coverage (7/20 listed must-haves), aligning with the JD anti-keyword-stuffing guidance. Join probability: 48%.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CAND_0080766</t>
+          <t>CAND_0071974</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -569,19 +569,19 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>0.4625</t>
+          <t>0.3414</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Rank 5: Staff Machine Learning Engineer at Salesforce (8.8 YOE); JD-aligned skills: Information Retrieval Systems, Elasticsearch, Natural Language Processing. Top-tier composite score across career, skills, and availability. Counterfactual: ranks on career trajectory and assessed depth over keyword coverage (6/20 listed must-haves), aligning with the JD anti-keyword-stuffing guidance. Join probability: 46%.</t>
+          <t>Rank 5: Senior AI Engineer at Netflix (7.8 YOE); JD-aligned skills: Weaviate, Pinecone, Information Retrieval. Top-tier composite score across career, skills, and availability. Counterfactual: ranks on career trajectory and assessed depth over keyword coverage (7/20 listed must-haves), aligning with the JD anti-keyword-stuffing guidance. Join probability: 34%; low engagement signals.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>CAND_0077337</t>
+          <t>CAND_0046525</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -596,19 +596,19 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>0.4883</t>
+          <t>0.3574</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Strong match — Staff Machine Learning Engineer at Paytm (7.0 YOE); JD-aligned skills: pgvector, Pinecone, Information Retrieval. Join probability: 49%.</t>
+          <t>Strong match — Senior Machine Learning Engineer at Genpact AI (6.1 YOE); JD-aligned skills: Elasticsearch, Information Retrieval, LLMs. Join probability: 36%.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>CAND_0018094</t>
+          <t>CAND_0055905</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -623,19 +623,19 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>0.4428</t>
+          <t>0.6870</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Strong match — ML Engineer at Mad Street Den (5.2 YOE); JD-aligned skills: Pinecone, Information Retrieval, Fine-tuning LLMs. Join probability: 44%.</t>
+          <t>Strong match — Senior Machine Learning Engineer at Flipkart (8.1 YOE); JD-aligned skills: Elasticsearch, Python, LLMs. Join probability: 69%.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>CAND_0096142</t>
+          <t>CAND_0077337</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -650,19 +650,19 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>0.2486</t>
+          <t>0.4883</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Strong match — Applied ML Engineer at upGrad (5.0 YOE); JD-aligned skills: Weaviate, Pinecone, Python. Watch: 120-day notice period. Join probability: 25%; long notice.</t>
+          <t>Strong match — Staff Machine Learning Engineer at Paytm (7.0 YOE); JD-aligned skills: pgvector, Pinecone, Information Retrieval. Join probability: 49%.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>CAND_0081846</t>
+          <t>CAND_0050454</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -677,19 +677,19 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>0.4803</t>
+          <t>0.3504</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Strong match — Lead AI Engineer at Razorpay (6.7 YOE); JD-aligned skills: Information Retrieval, pgvector, Elasticsearch. Join probability: 48%.</t>
+          <t>Strong match — AI Engineer at Rephrase.ai (6.8 YOE); JD-aligned skills: Fine-tuning LLMs, FAISS, Qdrant. Join probability: 35%.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>CAND_0038368</t>
+          <t>CAND_0006567</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -704,19 +704,19 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>0.4347</t>
+          <t>0.6079</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Strong match — ML Engineer at PhonePe (5.4 YOE); JD-aligned skills: Embeddings, FAISS, NLP. Join probability: 43%.</t>
+          <t>Strong match — Senior AI Engineer at Meta (7.9 YOE); JD-aligned skills: Vector Representations, NLP, Python. Join probability: 61%.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>CAND_0039383</t>
+          <t>CAND_0044222</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -731,19 +731,19 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>0.5155</t>
+          <t>0.2252</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Strong match — Applied ML Engineer at Meesho (7.1 YOE); JD-aligned skills: FAISS, NLP, Vector Search. Watch: 90-day notice period. Join probability: 52%.</t>
+          <t>Strong match — AI Engineer at PolicyBazaar (7.7 YOE); JD-aligned skills: Vector Search, OpenSearch, Qdrant. Join probability: 23%; low engagement signals.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>CAND_0044222</t>
+          <t>CAND_0083879</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -758,19 +758,19 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>0.2252</t>
+          <t>0.5950</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Strong match — AI Engineer at PolicyBazaar (7.7 YOE); JD-aligned skills: Vector Search, OpenSearch, Qdrant. Join probability: 23%; low engagement signals.</t>
+          <t>Strong match — Machine Learning Engineer at Ola (7.1 YOE); JD-aligned skills: Fine-tuning LLMs, Milvus, Sentence Transformers. Join probability: 60%.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>CAND_0010149</t>
+          <t>CAND_0086022</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -785,19 +785,19 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>0.2385</t>
+          <t>0.3683</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Strong match — ML Engineer at Glance (6.9 YOE); JD-aligned skills: Milvus, Vector Search, Elasticsearch. Watch: 90-day notice period. Join probability: 24%; low engagement signals.</t>
+          <t>Strong match — Senior Applied Scientist at Sarvam AI (5.3 YOE); JD-aligned skills: Vector Search, pgvector, Fine-tuning LLMs. Join probability: 37%.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>CAND_0002025</t>
+          <t>CAND_0016163</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -812,19 +812,19 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>0.3912</t>
+          <t>0.2905</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Strong match — Senior AI Engineer at Apple (5.9 YOE); JD-aligned skills: FAISS, OpenSearch, Weaviate. Join probability: 39%.</t>
+          <t>Strong match — Applied ML Engineer at Dream11 (6.7 YOE); JD-aligned skills: Weaviate, Embeddings, pgvector. Watch: 120-day notice period. Join probability: 29%; long notice.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>CAND_0030031</t>
+          <t>CAND_0049538</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -839,19 +839,19 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>0.3445</t>
+          <t>0.3362</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Strong match — AI Engineer at Microsoft (5.7 YOE); JD-aligned skills: Information Retrieval, Python, NLP. Join probability: 34%; low engagement signals.</t>
+          <t>Strong match — Applied ML Engineer at Saarthi.ai (5.8 YOE); JD-aligned skills: OpenSearch, Vector Search, Milvus. Join probability: 34%; low engagement signals.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>CAND_0006567</t>
+          <t>CAND_0005649</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -866,19 +866,19 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>0.6079</t>
+          <t>0.5162</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Strong match — Senior AI Engineer at Meta (7.9 YOE); JD-aligned skills: Vector Representations, NLP, Python. Join probability: 61%.</t>
+          <t>Strong match — Senior Data Scientist at Sarvam AI (7.4 YOE); JD-aligned skills: Fine-tuning LLMs, Weaviate, Information Retrieval. Watch: 90-day notice period. Join probability: 52%.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>CAND_0083879</t>
+          <t>CAND_0068351</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -893,12 +893,12 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>0.5950</t>
+          <t>0.4040</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Strong match — Machine Learning Engineer at Ola (7.1 YOE); JD-aligned skills: Fine-tuning LLMs, Milvus, Sentence Transformers. Join probability: 60%.</t>
+          <t>Strong match — Lead AI Engineer at Sarvam AI (6.4 YOE); JD-aligned skills: pgvector, Qdrant, Elasticsearch. Join probability: 40%.</t>
         </is>
       </c>
     </row>
@@ -932,7 +932,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>CAND_0020877</t>
+          <t>CAND_0030031</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -947,19 +947,19 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>0.3909</t>
+          <t>0.3445</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Strong match — Applied ML Engineer at CRED (5.1 YOE); JD-aligned skills: Elasticsearch, OpenSearch, Information Retrieval. Join probability: 39%.</t>
+          <t>Strong match — AI Engineer at Microsoft (5.7 YOE); JD-aligned skills: Information Retrieval, Python, NLP. Join probability: 34%; low engagement signals.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>CAND_0049538</t>
+          <t>CAND_0018094</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -974,19 +974,19 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>0.3362</t>
+          <t>0.4428</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Strong match — Applied ML Engineer at Saarthi.ai (5.8 YOE); JD-aligned skills: OpenSearch, Vector Search, Milvus. Join probability: 34%; low engagement signals.</t>
+          <t>Strong match — ML Engineer at Mad Street Den (5.2 YOE); JD-aligned skills: Pinecone, Information Retrieval, Fine-tuning LLMs. Join probability: 44%.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>CAND_0098217</t>
+          <t>CAND_0081852</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1001,19 +1001,19 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>0.5342</t>
+          <t>0.2331</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Solid profile: ML Engineer at Glance (6.4 YOE); JD-aligned skills: FAISS, Pinecone.</t>
+          <t>Solid profile: Senior Data Scientist at Mad Street Den (5.9 YOE); JD-aligned skills: Milvus, pgvector, Weaviate.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>CAND_0047721</t>
+          <t>CAND_0039383</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1028,19 +1028,19 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>0.1736</t>
+          <t>0.5155</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Good fit with caveats: Senior Data Scientist at Microsoft (7.0 YOE); JD-aligned skills: Milvus, Information Retrieval, FAISS. Concerns: 90-day notice period.</t>
+          <t>Good fit with caveats: Applied ML Engineer at Meesho (7.1 YOE); JD-aligned skills: FAISS, NLP, Vector Search. Concerns: 90-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>CAND_0005649</t>
+          <t>CAND_0058688</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1055,19 +1055,19 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>0.5162</t>
+          <t>0.7268</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Competitive candidate: Senior Data Scientist at Sarvam AI (7.4 YOE); JD-aligned skills: Fine-tuning LLMs, Weaviate, Information Retrieval. Concerns: 90-day notice period.</t>
+          <t>Competitive candidate: AI Engineer at Vedantu (6.7 YOE); JD-aligned skills: Embeddings, Information Retrieval, Milvus.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>CAND_0061550</t>
+          <t>CAND_0020877</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1082,19 +1082,19 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>0.3313</t>
+          <t>0.3909</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Meets several JD signals: ML Engineer at Infosys (5.3 YOE); JD-aligned skills: pgvector, Sentence Transformers.</t>
+          <t>Meets several JD signals: Applied ML Engineer at CRED (5.1 YOE); JD-aligned skills: Elasticsearch, OpenSearch, Information Retrieval.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>CAND_0061257</t>
+          <t>CAND_0020350</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1109,19 +1109,19 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>0.3969</t>
+          <t>0.3210</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Solid profile: Staff Machine Learning Engineer at LinkedIn (8.0 YOE); JD-aligned skills: Information Retrieval Systems, Python, Vector Representations.</t>
+          <t>Solid profile: AI Engineer at Zoho (5.8 YOE); JD-aligned skills: NLP, LLMs, FAISS.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>CAND_0078002</t>
+          <t>CAND_0042029</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1136,19 +1136,19 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>0.2974</t>
+          <t>0.4840</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Good fit with caveats: Machine Learning Engineer at Meta (6.3 YOE); JD-aligned skills: pgvector, NLP, Weaviate.</t>
+          <t>Good fit with caveats: Senior Data Scientist at Flipkart (6.5 YOE); JD-aligned skills: NLP, Elasticsearch, Embeddings.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>CAND_0050454</t>
+          <t>CAND_0044855</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1163,19 +1163,19 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>0.3504</t>
+          <t>0.3723</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Competitive candidate: AI Engineer at Rephrase.ai (6.8 YOE); JD-aligned skills: Fine-tuning LLMs, FAISS, Qdrant.</t>
+          <t>Competitive candidate: Senior Data Scientist at Flipkart (6.6 YOE); JD-aligned skills: OpenSearch, Information Retrieval, Pinecone.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>CAND_0044855</t>
+          <t>CAND_0046064</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1190,19 +1190,19 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>0.3723</t>
+          <t>0.3780</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Meets several JD signals: Senior Data Scientist at Flipkart (6.6 YOE); JD-aligned skills: OpenSearch, Information Retrieval, Pinecone.</t>
+          <t>Meets several JD signals: Senior NLP Engineer at Salesforce (8.9 YOE); JD-aligned skills: Python, Pinecone, OpenSearch.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>CAND_0055905</t>
+          <t>CAND_0079387</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1217,12 +1217,12 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>0.6870</t>
+          <t>0.4465</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Solid profile: Senior Machine Learning Engineer at Flipkart (8.1 YOE); JD-aligned skills: Elasticsearch, Python, LLMs.</t>
+          <t>Solid profile: AI Engineer at Microsoft (6.9 YOE); JD-aligned skills: Python, Sentence Transformers, Vector Search.</t>
         </is>
       </c>
     </row>
@@ -1256,7 +1256,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>CAND_0042029</t>
+          <t>CAND_0045250</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1271,19 +1271,19 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>0.4840</t>
+          <t>0.3580</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Competitive candidate: Senior Data Scientist at Flipkart (6.5 YOE); JD-aligned skills: NLP, Elasticsearch, Embeddings.</t>
+          <t>Competitive candidate: Applied ML Engineer at Rephrase.ai (6.6 YOE); JD-aligned skills: Sentence Transformers, Milvus, Embeddings.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>CAND_0079387</t>
+          <t>CAND_0093193</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1298,19 +1298,19 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>0.4465</t>
+          <t>0.4352</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Meets several JD signals: AI Engineer at Microsoft (6.9 YOE); JD-aligned skills: Python, Sentence Transformers, Vector Search.</t>
+          <t>Meets several JD signals: Senior Machine Learning Engineer at Niramai (7.9 YOE); JD-aligned skills: Text Encoders, Vector Representations, Qdrant.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>CAND_0032216</t>
+          <t>CAND_0080766</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1325,19 +1325,19 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>0.2743</t>
+          <t>0.4625</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Solid profile: ML Engineer at upGrad (6.1 YOE); JD-aligned skills: Information Retrieval, Qdrant, Sentence Transformers.</t>
+          <t>Solid profile: Staff Machine Learning Engineer at Salesforce (8.8 YOE); JD-aligned skills: Information Retrieval Systems, Elasticsearch, Natural Language Processing.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>CAND_0037566</t>
+          <t>CAND_0061257</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1352,19 +1352,19 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>0.5752</t>
+          <t>0.3969</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Good fit with caveats: Machine Learning Engineer at LinkedIn (6.9 YOE); JD-aligned skills: Pinecone, NLP, LLMs.</t>
+          <t>Good fit with caveats: Staff Machine Learning Engineer at LinkedIn (8.0 YOE); JD-aligned skills: Information Retrieval Systems, Python, Vector Representations.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>CAND_0016163</t>
+          <t>CAND_0047721</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1379,12 +1379,12 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>0.2905</t>
+          <t>0.1736</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Competitive candidate: Applied ML Engineer at Dream11 (6.7 YOE); JD-aligned skills: Weaviate, Embeddings, pgvector. Concerns: 120-day notice period.</t>
+          <t>Competitive candidate: Senior Data Scientist at Microsoft (7.0 YOE); JD-aligned skills: Milvus, Information Retrieval, FAISS. Concerns: 90-day notice period.</t>
         </is>
       </c>
     </row>
@@ -1418,7 +1418,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>CAND_0090584</t>
+          <t>CAND_0051292</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1433,19 +1433,19 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>0.1637</t>
+          <t>0.4013</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Solid profile: ML Engineer at Flipkart (5.1 YOE); JD-aligned skills: Fine-tuning LLMs, OpenSearch, FAISS. Concerns: 120-day notice period.</t>
+          <t>Solid profile: Applied ML Engineer at Freshworks (5.2 YOE); JD-aligned skills: pgvector, FAISS, LLMs.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>CAND_0081852</t>
+          <t>CAND_0096142</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1460,19 +1460,19 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>0.2331</t>
+          <t>0.2486</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Good fit with caveats: Senior Data Scientist at Mad Street Den (5.9 YOE); JD-aligned skills: Milvus, pgvector, Weaviate.</t>
+          <t>Good fit with caveats: Applied ML Engineer at upGrad (5.0 YOE); JD-aligned skills: Weaviate, Pinecone, Python. Concerns: 120-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>CAND_0045250</t>
+          <t>CAND_0037566</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1487,19 +1487,19 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>0.3580</t>
+          <t>0.5752</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Competitive candidate: Applied ML Engineer at Rephrase.ai (6.6 YOE); JD-aligned skills: Sentence Transformers, Milvus, Embeddings.</t>
+          <t>Competitive candidate: Machine Learning Engineer at LinkedIn (6.9 YOE); JD-aligned skills: Pinecone, NLP, LLMs.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>CAND_0093193</t>
+          <t>CAND_0051004</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1514,19 +1514,19 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>0.4352</t>
+          <t>0.5405</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Meets several JD signals: Senior Machine Learning Engineer at Niramai (7.9 YOE); JD-aligned skills: Text Encoders, Vector Representations, Qdrant.</t>
+          <t>Meets several JD signals: Senior Data Scientist at CRED (4.7 YOE); JD-aligned skills: Embeddings, Qdrant, Fine-tuning LLMs.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>CAND_0051292</t>
+          <t>CAND_0069905</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1541,19 +1541,19 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>0.4013</t>
+          <t>0.3358</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Solid profile: Applied ML Engineer at Freshworks (5.2 YOE); JD-aligned skills: pgvector, FAISS, LLMs.</t>
+          <t>Solid profile: Applied ML Engineer at Sarvam AI (6.6 YOE); JD-aligned skills: Sentence Transformers, Python, Weaviate. Concerns: 90-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>CAND_0076482</t>
+          <t>CAND_0055992</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1568,19 +1568,19 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>0.5553</t>
+          <t>0.5850</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Good fit with caveats: ML Engineer at Flipkart (6.6 YOE); JD-aligned skills: OpenSearch, Pinecone, pgvector.</t>
+          <t>Good fit with caveats: AI Engineer at CRED (16.9 YOE); JD-aligned skills: Information Retrieval, FAISS, OpenSearch.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>CAND_0079284</t>
+          <t>CAND_0068811</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1595,19 +1595,19 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>0.2718</t>
+          <t>0.4651</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Competitive candidate: Machine Learning Engineer at Google (4.9 YOE); JD-aligned skills: Qdrant, Fine-tuning LLMs, Elasticsearch.</t>
+          <t>Competitive candidate: Applied ML Engineer at Freshworks (8.0 YOE); JD-aligned skills: Vector Search, Qdrant, Embeddings.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>CAND_0058688</t>
+          <t>CAND_0093912</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1622,19 +1622,19 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>0.7268</t>
+          <t>0.4763</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Meets several JD signals: AI Engineer at Vedantu (6.7 YOE); JD-aligned skills: Embeddings, Information Retrieval, Milvus.</t>
+          <t>Meets several JD signals: Senior Data Scientist at Razorpay (5.3 YOE); JD-aligned skills: Milvus, Embeddings, Vector Search.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>CAND_0020350</t>
+          <t>CAND_0099806</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -1649,19 +1649,19 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>0.3210</t>
+          <t>0.3301</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Solid profile: AI Engineer at Zoho (5.8 YOE); JD-aligned skills: NLP, LLMs, FAISS.</t>
+          <t>Solid profile: AI Engineer at Mad Street Den (4.6 YOE); JD-aligned skills: pgvector, FAISS, Embeddings.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>CAND_0068811</t>
+          <t>CAND_0010257</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -1676,19 +1676,19 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>0.4651</t>
+          <t>0.3313</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Good fit with caveats: Applied ML Engineer at Freshworks (8.0 YOE); JD-aligned skills: Vector Search, Qdrant, Embeddings.</t>
+          <t>Good fit with caveats: Senior Data Scientist at Google (6.5 YOE); JD-aligned skills: Milvus, Python, OpenSearch. Concerns: 120-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>CAND_0015528</t>
+          <t>CAND_0065878</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -1703,19 +1703,19 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>0.3246</t>
+          <t>0.2450</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Competitive candidate: Applied ML Engineer at Krutrim (7.4 YOE); JD-aligned skills: Weaviate, pgvector, Information Retrieval.</t>
+          <t>Competitive candidate: Senior Data Scientist at Niramai (7.8 YOE); JD-aligned skills: pgvector, Vector Search, Fine-tuning LLMs.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>CAND_0075574</t>
+          <t>CAND_0032216</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1730,19 +1730,19 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>0.4170</t>
+          <t>0.2743</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Meets several JD signals: Machine Learning Engineer at Haptik (5.7 YOE); JD-aligned skills: pgvector, Weaviate, OpenSearch.</t>
+          <t>Meets several JD signals: ML Engineer at upGrad (6.1 YOE); JD-aligned skills: Information Retrieval, Qdrant, Sentence Transformers.</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>CAND_0052328</t>
+          <t>CAND_0078002</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -1757,19 +1757,19 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>0.5090</t>
+          <t>0.2974</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Solid profile: Recommendation Systems Engineer at Amazon (6.5 YOE); JD-aligned skills: OpenSearch, Fine-tuning LLMs, Vector Search.</t>
+          <t>Solid profile: Machine Learning Engineer at Meta (6.3 YOE); JD-aligned skills: pgvector, NLP, Weaviate.</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>CAND_0040178</t>
+          <t>CAND_0005260</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -1784,19 +1784,19 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>0.3303</t>
+          <t>0.4814</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Good fit with caveats: ML Engineer at Meesho (5.0 YOE); JD-aligned skills: Weaviate, Fine-tuning LLMs, Vector Search.</t>
+          <t>Good fit with caveats: Senior NLP Engineer at Netflix (5.2 YOE); JD-aligned skills: Information Retrieval, Python, NLP.</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>CAND_0051004</t>
+          <t>CAND_0075574</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -1811,19 +1811,19 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>0.5405</t>
+          <t>0.4170</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Moderate fit: Senior Data Scientist at CRED (4.7 YOE); JD-aligned skills: Embeddings, Qdrant, Fine-tuning LLMs. Gaps: under half of JD must-have skills covered.</t>
+          <t>Moderate fit: Machine Learning Engineer at Haptik (5.7 YOE); JD-aligned skills: pgvector, Weaviate, OpenSearch. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>CAND_0079064</t>
+          <t>CAND_0005538</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -1838,19 +1838,19 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>0.2563</t>
+          <t>0.4072</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Partial alignment: Senior Data Scientist at Niramai (5.2 YOE); JD-aligned skills: OpenSearch, NLP, Fine-tuning LLMs. Gaps: 120-day notice period.</t>
+          <t>Partial alignment: Senior AI Engineer at Adobe (5.9 YOE); JD-aligned skills: Vector Representations, Python, Information Retrieval Systems. Gaps: 90-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>CAND_0065878</t>
+          <t>CAND_0079064</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -1865,19 +1865,19 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>0.2450</t>
+          <t>0.2563</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Acceptable but not standout: Senior Data Scientist at Niramai (7.8 YOE); JD-aligned skills: pgvector, Vector Search, Fine-tuning LLMs. Gaps: under half of JD must-have skills covered.</t>
+          <t>Acceptable but not standout: Senior Data Scientist at Niramai (5.2 YOE); JD-aligned skills: OpenSearch, NLP, Fine-tuning LLMs. Gaps: 120-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>CAND_0069905</t>
+          <t>CAND_0015528</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -1892,19 +1892,19 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>0.3358</t>
+          <t>0.3246</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Mixed signals: Applied ML Engineer at Sarvam AI (6.6 YOE); JD-aligned skills: Sentence Transformers, Python, Weaviate. Gaps: 90-day notice period.</t>
+          <t>Mixed signals: Applied ML Engineer at Krutrim (7.4 YOE); JD-aligned skills: Weaviate, pgvector, Information Retrieval. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>CAND_0011432</t>
+          <t>CAND_0038368</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -1919,19 +1919,19 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>0.5534</t>
+          <t>0.4347</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>JD overlap is thin: Senior Data Scientist at Amazon (7.6 YOE); JD-aligned skills: OpenSearch, pgvector, Elasticsearch. Gaps: under half of JD must-have skills covered.</t>
+          <t>JD overlap is thin: ML Engineer at PhonePe (5.4 YOE); JD-aligned skills: Embeddings, FAISS, NLP. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>CAND_0036121</t>
+          <t>CAND_0074735</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -1946,19 +1946,19 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>0.3242</t>
+          <t>0.4586</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Moderate fit: ML Engineer at Wysa (5.2 YOE); JD-aligned skills: Embeddings, Vector Search, Information Retrieval. Gaps: under half of JD must-have skills covered.</t>
+          <t>Moderate fit: Applied ML Engineer at Rephrase.ai (5.5 YOE); JD-aligned skills: Weaviate, Information Retrieval, Vector Search. Gaps: 90-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>CAND_0093912</t>
+          <t>CAND_0079284</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -1973,19 +1973,19 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>0.4763</t>
+          <t>0.2718</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Partial alignment: Senior Data Scientist at Razorpay (5.3 YOE); JD-aligned skills: Milvus, Embeddings, Vector Search. Gaps: under half of JD must-have skills covered.</t>
+          <t>Partial alignment: Machine Learning Engineer at Google (4.9 YOE); JD-aligned skills: Qdrant, Fine-tuning LLMs, Elasticsearch. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>CAND_0080465</t>
+          <t>CAND_0011432</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -2000,19 +2000,19 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>0.2782</t>
+          <t>0.5534</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Acceptable but not standout: ML Engineer at Meesho (4.2 YOE); JD-aligned skills: Milvus, Qdrant. Gaps: 90-day notice period.</t>
+          <t>Acceptable but not standout: Senior Data Scientist at Amazon (7.6 YOE); JD-aligned skills: OpenSearch, pgvector, Elasticsearch. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>CAND_0074735</t>
+          <t>CAND_0067866</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -2027,19 +2027,19 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>0.4586</t>
+          <t>0.3513</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Mixed signals: Applied ML Engineer at Rephrase.ai (5.5 YOE); JD-aligned skills: Weaviate, Information Retrieval, Vector Search. Gaps: 90-day notice period.</t>
+          <t>Mixed signals: Senior Software Engineer (ML) at Tech Mahindra (6.4 YOE); JD-aligned skills: Embeddings, pgvector, Elasticsearch. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>CAND_0099806</t>
+          <t>CAND_0090584</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -2054,19 +2054,19 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>0.3301</t>
+          <t>0.1637</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>JD overlap is thin: AI Engineer at Mad Street Den (4.6 YOE); JD-aligned skills: pgvector, FAISS, Embeddings. Gaps: under half of JD must-have skills covered.</t>
+          <t>JD overlap is thin: ML Engineer at Flipkart (5.1 YOE); JD-aligned skills: Fine-tuning LLMs, OpenSearch, FAISS. Gaps: 120-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>CAND_0039962</t>
+          <t>CAND_0011687</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -2081,19 +2081,19 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>0.2509</t>
+          <t>0.5094</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Moderate fit: ML Engineer at Paytm (6.5 YOE); JD-aligned skills: Pinecone, LLMs. Gaps: 90-day notice period.</t>
+          <t>Moderate fit: Senior NLP Engineer at Niramai (7.8 YOE); JD-aligned skills: OpenSearch, FAISS, Embeddings. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>CAND_0002120</t>
+          <t>CAND_0061550</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -2108,12 +2108,12 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>0.3168</t>
+          <t>0.3313</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Partial alignment: ML Engineer at HCL (6.5 YOE); JD-aligned skills: Information Retrieval, Pinecone, Embeddings. Gaps: under half of JD must-have skills covered.</t>
+          <t>Partial alignment: ML Engineer at Infosys (5.3 YOE); JD-aligned skills: pgvector, Sentence Transformers. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
@@ -2147,7 +2147,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>CAND_0005538</t>
+          <t>CAND_0048166</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -2162,19 +2162,19 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>0.4072</t>
+          <t>0.4054</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Mixed signals: Senior AI Engineer at Adobe (5.9 YOE); JD-aligned skills: Vector Representations, Python, Information Retrieval Systems. Gaps: 90-day notice period.</t>
+          <t>Mixed signals: ML Engineer at Aganitha (5.2 YOE); JD-aligned skills: Pinecone, Milvus, Qdrant. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>CAND_0011489</t>
+          <t>CAND_0093547</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -2189,19 +2189,19 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>0.2839</t>
+          <t>0.3710</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>JD overlap is thin: ML Engineer at Glance (5.8 YOE); JD-aligned skills: pgvector, Embeddings, Python. Gaps: under half of JD must-have skills covered.</t>
+          <t>JD overlap is thin: Senior Machine Learning Engineer at PhonePe (2.9 YOE); JD-aligned skills: LLMs, Python, Milvus. Gaps: below typical senior YOE band for this JD.</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>CAND_0003841</t>
+          <t>CAND_0076482</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -2216,19 +2216,19 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>0.3402</t>
+          <t>0.5553</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Moderate fit: ML Engineer at Tech Mahindra (5.0 YOE); JD-aligned skills: Pinecone, Fine-tuning LLMs, Sentence Transformers. Gaps: under half of JD must-have skills covered.</t>
+          <t>Moderate fit: ML Engineer at Flipkart (6.6 YOE); JD-aligned skills: OpenSearch, Pinecone, pgvector. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>CAND_0055992</t>
+          <t>CAND_0040178</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2243,19 +2243,19 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>0.5850</t>
+          <t>0.3303</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Partial alignment: AI Engineer at CRED (16.9 YOE); JD-aligned skills: Information Retrieval, FAISS, OpenSearch. Gaps: experience above target band for this role.</t>
+          <t>Partial alignment: ML Engineer at Meesho (5.0 YOE); JD-aligned skills: Weaviate, Fine-tuning LLMs, Vector Search. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>CAND_0021836</t>
+          <t>CAND_0060054</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -2270,19 +2270,19 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>0.4646</t>
+          <t>0.3416</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Acceptable but not standout: ML Engineer at CRED (6.5 YOE); JD-aligned skills: Vector Search, Elasticsearch, NLP. Gaps: under half of JD must-have skills covered.</t>
+          <t>Acceptable but not standout: AI Engineer at Mad Street Den (6.4 YOE); JD-aligned skills: Weaviate, FAISS, Elasticsearch. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>CAND_0009691</t>
+          <t>CAND_0003841</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -2297,19 +2297,19 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>0.1214</t>
+          <t>0.3402</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Mixed signals: Applied ML Engineer at LinkedIn (6.2 YOE); JD-aligned skills: Fine-tuning LLMs, Pinecone, Sentence Transformers. Gaps: 120-day notice period.</t>
+          <t>Mixed signals: ML Engineer at Tech Mahindra (5.0 YOE); JD-aligned skills: Pinecone, Fine-tuning LLMs, Sentence Transformers. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>CAND_0046525</t>
+          <t>CAND_0008425</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -2324,19 +2324,19 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>0.3574</t>
+          <t>0.2436</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>JD overlap is thin: Senior Machine Learning Engineer at Genpact AI (6.1 YOE); JD-aligned skills: Elasticsearch, Information Retrieval, LLMs. Gaps: under half of JD must-have skills covered.</t>
+          <t>JD overlap is thin: Senior NLP Engineer at Ola (7.8 YOE); JD-aligned skills: Qdrant, pgvector, Sentence Transformers. Gaps: 90-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>CAND_0010257</t>
+          <t>CAND_0027691</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -2351,19 +2351,19 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>0.3313</t>
+          <t>0.4306</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Moderate fit: Senior Data Scientist at Google (6.5 YOE); JD-aligned skills: Milvus, Python, OpenSearch. Gaps: 120-day notice period.</t>
+          <t>Moderate fit: NLP Engineer at Haptik (6.5 YOE); JD-aligned skills: Weaviate, Embeddings, Python. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>CAND_0067866</t>
+          <t>CAND_0037980</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -2378,19 +2378,19 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>0.3513</t>
+          <t>0.7550</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Partial alignment: Senior Software Engineer (ML) at Tech Mahindra (6.4 YOE); JD-aligned skills: Embeddings, pgvector, Elasticsearch. Gaps: under half of JD must-have skills covered.</t>
+          <t>Partial alignment: Senior Applied Scientist at Niramai (9.0 YOE); JD-aligned skills: NLP, Text Encoders, pgvector. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>CAND_0037944</t>
+          <t>CAND_0096104</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -2405,19 +2405,19 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>0.2490</t>
+          <t>0.5401</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Acceptable but not standout: Senior Data Scientist at Vedantu (4.9 YOE); JD-aligned skills: Vector Search, OpenSearch, Embeddings. Gaps: under half of JD must-have skills covered.</t>
+          <t>Acceptable but not standout: AI Specialist at Yellow.ai (7.0 YOE); JD-aligned skills: Pinecone. Gaps: only 1 core JD skill matched.</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>CAND_0086022</t>
+          <t>CAND_0024878</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -2432,19 +2432,19 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>0.3683</t>
+          <t>0.4462</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Mixed signals: Senior Applied Scientist at Sarvam AI (5.3 YOE); JD-aligned skills: Vector Search, pgvector, Fine-tuning LLMs. Gaps: under half of JD must-have skills covered.</t>
+          <t>Mixed signals: AI Specialist at HCL (5.7 YOE); JD-aligned skills: pgvector, Elasticsearch, NLP. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>CAND_0037980</t>
+          <t>CAND_0001819</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -2459,19 +2459,19 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>0.7550</t>
+          <t>0.3603</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>JD overlap is thin: Senior Applied Scientist at Niramai (9.0 YOE); JD-aligned skills: NLP, Text Encoders, pgvector. Gaps: under half of JD must-have skills covered.</t>
+          <t>JD overlap is thin: ML Engineer at Genpact AI (4.4 YOE); JD-aligned skills: Weaviate, pgvector, NLP. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>CAND_0065514</t>
+          <t>CAND_0036121</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -2486,19 +2486,19 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>0.2597</t>
+          <t>0.3242</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Moderate fit: ML Engineer at Genpact AI (6.6 YOE); JD-aligned skills: Vector Search, Pinecone, Elasticsearch. Gaps: 90-day notice period.</t>
+          <t>Moderate fit: ML Engineer at Wysa (5.2 YOE); JD-aligned skills: Embeddings, Vector Search, Information Retrieval. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>CAND_0030348</t>
+          <t>CAND_0052328</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -2513,19 +2513,19 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>0.3735</t>
+          <t>0.5090</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Partial alignment: Machine Learning Engineer at BYJU'S (4.5 YOE); JD-aligned skills: Embeddings, Vector Search, Elasticsearch. Gaps: under half of JD must-have skills covered.</t>
+          <t>Partial alignment: Recommendation Systems Engineer at Amazon (6.5 YOE); JD-aligned skills: OpenSearch, Fine-tuning LLMs, Vector Search. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>CAND_0070398</t>
+          <t>CAND_0030348</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -2540,19 +2540,19 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>0.2060</t>
+          <t>0.3735</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Acceptable but not standout: Machine Learning Engineer at Genpact AI (7.2 YOE); JD-aligned skills: FAISS, Embeddings, Python. Gaps: 120-day notice period.</t>
+          <t>Acceptable but not standout: Machine Learning Engineer at BYJU'S (4.5 YOE); JD-aligned skills: Embeddings, Vector Search, Elasticsearch. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>CAND_0017178</t>
+          <t>CAND_0019288</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -2567,19 +2567,19 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>0.4976</t>
+          <t>0.3846</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Mixed signals: ML Engineer at Swiggy (4.2 YOE); JD-aligned skills: pgvector, Information Retrieval. Gaps: not flagged open to work.</t>
+          <t>Mixed signals: AI Research Engineer at Paytm (5.7 YOE); JD-aligned skills: pgvector, FAISS, OpenSearch. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>CAND_0001819</t>
+          <t>CAND_0002793</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -2594,19 +2594,19 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>0.3603</t>
+          <t>0.3997</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>JD overlap is thin: ML Engineer at Genpact AI (4.4 YOE); JD-aligned skills: Weaviate, pgvector, NLP. Gaps: under half of JD must-have skills covered.</t>
+          <t>JD overlap is thin: AI Specialist at Meesho (5.5 YOE); JD-aligned skills: pgvector, Information Retrieval, FAISS. Gaps: not flagged open to work.</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>CAND_0015578</t>
+          <t>CAND_0043637</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -2621,19 +2621,19 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>0.1397</t>
+          <t>0.4329</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Moderate fit: AI Engineer at Zoho (5.4 YOE); JD-aligned skills: Embeddings, NLP, Sentence Transformers. Gaps: 90-day notice period.</t>
+          <t>Moderate fit: Junior ML Engineer at Rephrase.ai (5.5 YOE); JD-aligned skills: Milvus, pgvector. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>CAND_0033445</t>
+          <t>CAND_0009691</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -2648,19 +2648,19 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>0.2922</t>
+          <t>0.1214</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Partial alignment: ML Engineer at Vedantu (6.8 YOE); JD-aligned skills: Information Retrieval, pgvector. Gaps: under half of JD must-have skills covered.</t>
+          <t>Partial alignment: Applied ML Engineer at LinkedIn (6.2 YOE); JD-aligned skills: Fine-tuning LLMs, Pinecone, Sentence Transformers. Gaps: 120-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>CAND_0018293</t>
+          <t>CAND_0091534</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -2675,19 +2675,19 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>0.5647</t>
+          <t>0.2365</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Acceptable but not standout: Data Scientist at PharmEasy (5.6 YOE); JD-aligned skills: Weaviate, Information Retrieval, pgvector. Gaps: under half of JD must-have skills covered.</t>
+          <t>Acceptable but not standout: AI Engineer at Flipkart (16.6 YOE); JD-aligned skills: Qdrant, Sentence Transformers. Gaps: experience above target band for this role; not flagged open to work.</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>CAND_0049615</t>
+          <t>CAND_0010541</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -2702,19 +2702,19 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>0.2597</t>
+          <t>0.5800</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Mixed signals: ML Engineer at Krutrim (5.1 YOE); JD-aligned skills: NLP, Pinecone. Gaps: under half of JD must-have skills covered.</t>
+          <t>Mixed signals: AI Research Engineer at Wysa (6.2 YOE); JD-aligned skills: Pinecone, Weaviate, Python. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>CAND_0017093</t>
+          <t>CAND_0065195</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -2729,19 +2729,19 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>0.2136</t>
+          <t>0.3492</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>JD overlap is thin: ML Engineer at Zoho (5.9 YOE); JD-aligned skills: LLMs, Embeddings, pgvector. Gaps: under half of JD must-have skills covered.</t>
+          <t>JD overlap is thin: Search Engineer at CRED (5.1 YOE); JD-aligned skills: LLMs, Elasticsearch, Qdrant. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>CAND_0050876</t>
+          <t>CAND_0015578</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -2756,19 +2756,19 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>0.4323</t>
+          <t>0.1397</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Moderate fit: Applied ML Engineer at Freshworks (6.0 YOE); JD-aligned skills: Qdrant, FAISS, OpenSearch. Gaps: 90-day notice period.</t>
+          <t>Moderate fit: AI Engineer at Zoho (5.4 YOE); JD-aligned skills: Embeddings, NLP, Sentence Transformers. Gaps: 90-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>CAND_0041669</t>
+          <t>CAND_0037944</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -2783,19 +2783,19 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>0.6806</t>
+          <t>0.2490</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Partial alignment: Recommendation Systems Engineer at CRED (8.0 YOE); JD-aligned skills: FAISS, Milvus, Weaviate. Gaps: under half of JD must-have skills covered.</t>
+          <t>Partial alignment: Senior Data Scientist at Vedantu (4.9 YOE); JD-aligned skills: Vector Search, OpenSearch, Embeddings. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>CAND_0027691</t>
+          <t>CAND_0070398</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -2810,19 +2810,19 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>0.4306</t>
+          <t>0.2060</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>Acceptable but not standout: NLP Engineer at Haptik (6.5 YOE); JD-aligned skills: Weaviate, Embeddings, Python. Gaps: under half of JD must-have skills covered.</t>
+          <t>Acceptable but not standout: Machine Learning Engineer at Genpact AI (7.2 YOE); JD-aligned skills: FAISS, Embeddings, Python. Gaps: 120-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>CAND_0002037</t>
+          <t>CAND_0039754</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -2837,19 +2837,19 @@
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>0.1905</t>
+          <t>0.5509</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Mixed signals: ML Engineer at Locobuzz (5.5 YOE); JD-aligned skills: Fine-tuning LLMs, pgvector, Milvus. Gaps: not flagged open to work.</t>
+          <t>Mixed signals: Senior Applied Scientist at Meta (16.2 YOE); JD-aligned skills: Fine-tuning LLMs, Qdrant, NLP. Gaps: experience above target band for this role.</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>CAND_0066376</t>
+          <t>CAND_0003791</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -2864,19 +2864,19 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>0.2674</t>
+          <t>0.4776</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>JD overlap is thin: Applied ML Engineer at Dream11 (5.7 YOE); JD-aligned skills: LLMs, Fine-tuning LLMs, NLP. Gaps: 90-day notice period.</t>
+          <t>JD overlap is thin: ML Engineer at Meesho (6.6 YOE); JD-aligned skills: LLMs, pgvector, Python. Gaps: under half of JD must-have skills covered.</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>CAND_0048166</t>
+          <t>CAND_0007460</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -2891,19 +2891,19 @@
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>0.4054</t>
+          <t>0.2260</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>Lower-tier shortlist entry — ML Engineer at Aganitha (5.2 YOE); JD-aligned skills: Pinecone, Milvus, Qdrant. Key gaps: not flagged open to work.</t>
+          <t>Lower-tier shortlist entry — AI Engineer at Salesforce (4.7 YOE); JD-aligned skills: Embeddings, Weaviate, Information Retrieval. Key gaps: 120-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>CAND_0062561</t>
+          <t>CAND_0041669</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -2918,19 +2918,19 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>0.3470</t>
+          <t>0.6806</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>Lower-tier shortlist entry — ML Engineer at Razorpay (5.9 YOE); JD-aligned skills: Information Retrieval, Weaviate. Key gaps: weak secondary signals vs higher ranks.</t>
+          <t>Lower-tier shortlist entry — Recommendation Systems Engineer at CRED (8.0 YOE); JD-aligned skills: FAISS, Milvus, Weaviate. Key gaps: weak secondary signals vs higher ranks.</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>CAND_0035653</t>
+          <t>CAND_0081086</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -2945,19 +2945,19 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>0.4419</t>
+          <t>0.2245</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>Lower-tier shortlist entry — Data Scientist at Swiggy (5.6 YOE); JD-aligned skills: OpenSearch, Vector Search, Fine-tuning LLMs. Key gaps: weak secondary signals vs higher ranks.</t>
+          <t>Lower-tier shortlist entry — AI Specialist at Observe.AI (5.2 YOE); JD-aligned skills: pgvector, Weaviate, Embeddings. Key gaps: weak secondary signals vs higher ranks.</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>CAND_0056940</t>
+          <t>CAND_0050876</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2972,19 +2972,19 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>0.2882</t>
+          <t>0.4323</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>Lower-tier shortlist entry — Backend Engineer at Zomato (7.4 YOE); JD-aligned skills: pgvector. Key gaps: only 1 core JD skill matched.</t>
+          <t>Lower-tier shortlist entry — Applied ML Engineer at Freshworks (6.0 YOE); JD-aligned skills: Qdrant, FAISS, OpenSearch. Key gaps: 90-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>CAND_0032515</t>
+          <t>CAND_0013665</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -2999,19 +2999,19 @@
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>0.3727</t>
+          <t>0.2424</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>Lower-tier shortlist entry — Machine Learning Engineer at PharmEasy (5.1 YOE); JD-aligned skills: Milvus, Vector Search, Fine-tuning LLMs. Key gaps: not flagged open to work.</t>
+          <t>Lower-tier shortlist entry — Senior Software Engineer (ML) at InMobi (5.2 YOE); JD-aligned skills: Qdrant, Embeddings. Key gaps: not flagged open to work.</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>CAND_0053605</t>
+          <t>CAND_0080465</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -3026,19 +3026,19 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>0.6824</t>
+          <t>0.2782</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>Lower-tier shortlist entry — Senior Software Engineer (ML) at Verloop.io (6.9 YOE); JD-aligned skills: pgvector. Key gaps: only 1 core JD skill matched.</t>
+          <t>Lower-tier shortlist entry — ML Engineer at Meesho (4.2 YOE); JD-aligned skills: Milvus, Qdrant. Key gaps: 90-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>CAND_0092255</t>
+          <t>CAND_0025923</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -3053,19 +3053,19 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>0.2741</t>
+          <t>0.2891</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>Lower-tier shortlist entry — ML Engineer at InMobi (5.2 YOE); JD-aligned skills: Weaviate, OpenSearch, Vector Search. Key gaps: weak secondary signals vs higher ranks.</t>
+          <t>Lower-tier shortlist entry — Senior Software Engineer (ML) at HCL (5.0 YOE); JD-aligned skills: pgvector, Qdrant, Pinecone. Key gaps: not flagged open to work.</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>CAND_0082489</t>
+          <t>CAND_0093474</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -3080,19 +3080,19 @@
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>0.2325</t>
+          <t>0.4226</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>Lower-tier shortlist entry — ML Engineer at InMobi (5.3 YOE); JD-aligned skills: Weaviate. Key gaps: only 1 core JD skill matched; 90-day notice period; not flagged open to work.</t>
+          <t>Lower-tier shortlist entry — Senior Software Engineer (ML) at Wipro (5.3 YOE); JD-aligned skills: Vector Search, Qdrant, FAISS. Key gaps: 90-day notice period; not flagged open to work.</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>CAND_0098288</t>
+          <t>CAND_0094759</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -3107,19 +3107,19 @@
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>0.4556</t>
+          <t>0.2923</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>Lower-tier shortlist entry — Junior ML Engineer at Vedantu (6.7 YOE); JD-aligned skills: Information Retrieval, NLP, pgvector. Key gaps: weak secondary signals vs higher ranks.</t>
+          <t>Lower-tier shortlist entry — Lead AI Engineer at Meta (8.6 YOE); JD-aligned skills: Qdrant, Fine-tuning LLMs, Vector Search. Key gaps: low recruiter response rate; not flagged open to work.</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>CAND_0091909</t>
+          <t>CAND_0010149</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -3134,12 +3134,12 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>0.1949</t>
+          <t>0.2385</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>Lower-tier shortlist entry — Machine Learning Engineer at Rephrase.ai (6.9 YOE); JD-aligned skills: LLMs, Pinecone, Qdrant. Key gaps: weak secondary signals vs higher ranks.</t>
+          <t>Lower-tier shortlist entry — ML Engineer at Glance (6.9 YOE); JD-aligned skills: Milvus, Vector Search, Elasticsearch. Key gaps: 90-day notice period.</t>
         </is>
       </c>
     </row>

</xml_diff>